<commit_message>
minor cleanup and typo fixes
</commit_message>
<xml_diff>
--- a/Jupyter/Wedge/wedge_data_2026-03-25.xlsx
+++ b/Jupyter/Wedge/wedge_data_2026-03-25.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\patri\projects\emma-openmc\Jupyter\Wedge\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C3F34BDA-AD99-4B40-AB8C-3C4A43F6D461}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{100225AE-D78B-42E7-A4DA-1A50FD7EF77D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="17496" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -4257,15 +4257,15 @@
   <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>12</xdr:col>
-      <xdr:colOff>255270</xdr:colOff>
+      <xdr:colOff>132179</xdr:colOff>
       <xdr:row>19</xdr:row>
-      <xdr:rowOff>68580</xdr:rowOff>
+      <xdr:rowOff>56857</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>19</xdr:col>
-      <xdr:colOff>560070</xdr:colOff>
+      <xdr:colOff>436979</xdr:colOff>
       <xdr:row>34</xdr:row>
-      <xdr:rowOff>68580</xdr:rowOff>
+      <xdr:rowOff>56857</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
@@ -6348,6 +6348,7 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <drawing r:id="rId1"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
+  <drawing r:id="rId2"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
biso add fixes for prism_hcpb.py
</commit_message>
<xml_diff>
--- a/Jupyter/Wedge/wedge_data_2026-03-25.xlsx
+++ b/Jupyter/Wedge/wedge_data_2026-03-25.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\patri\projects\emma-openmc\Jupyter\Wedge\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{100225AE-D78B-42E7-A4DA-1A50FD7EF77D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D92552F5-14F5-4602-8D22-687681DBA2D8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="17496" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -274,41 +274,53 @@
           </c:marker>
           <c:xVal>
             <c:numRef>
-              <c:f>'Sheet 1'!$A$23:$A$33</c:f>
+              <c:f>'Sheet 1'!$A$27:$A$41</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="11"/>
+                <c:ptCount val="15"/>
                 <c:pt idx="0">
                   <c:v>0.1</c:v>
                 </c:pt>
                 <c:pt idx="1">
+                  <c:v>0.5</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>1.5</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>10</c:v>
+                </c:pt>
+                <c:pt idx="4">
                   <c:v>15</c:v>
                 </c:pt>
-                <c:pt idx="2">
+                <c:pt idx="5">
                   <c:v>30</c:v>
                 </c:pt>
-                <c:pt idx="3">
+                <c:pt idx="6">
                   <c:v>60</c:v>
                 </c:pt>
-                <c:pt idx="4">
+                <c:pt idx="7">
                   <c:v>90</c:v>
                 </c:pt>
-                <c:pt idx="5">
+                <c:pt idx="8">
+                  <c:v>100</c:v>
+                </c:pt>
+                <c:pt idx="9">
                   <c:v>120</c:v>
                 </c:pt>
-                <c:pt idx="6">
+                <c:pt idx="10">
                   <c:v>150</c:v>
                 </c:pt>
-                <c:pt idx="7">
+                <c:pt idx="11">
                   <c:v>250</c:v>
                 </c:pt>
-                <c:pt idx="8">
+                <c:pt idx="12">
                   <c:v>500</c:v>
                 </c:pt>
-                <c:pt idx="9">
+                <c:pt idx="13">
                   <c:v>750</c:v>
                 </c:pt>
-                <c:pt idx="10">
+                <c:pt idx="14">
                   <c:v>1000</c:v>
                 </c:pt>
               </c:numCache>
@@ -316,42 +328,42 @@
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>'Sheet 1'!$F$23:$F$33</c:f>
+              <c:f>'Sheet 1'!$F$27:$F$41</c:f>
               <c:numCache>
                 <c:formatCode>0.000000</c:formatCode>
-                <c:ptCount val="11"/>
+                <c:ptCount val="15"/>
                 <c:pt idx="0">
-                  <c:v>0.60767258302427063</c:v>
-                </c:pt>
-                <c:pt idx="1">
-                  <c:v>0.65530071246920629</c:v>
-                </c:pt>
-                <c:pt idx="2">
-                  <c:v>0.67754280833532643</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>0.7150760468910391</c:v>
+                  <c:v>0.90095484884115951</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>0.74349815634063066</c:v>
+                  <c:v>0.98605362776739691</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>0.76438369871068157</c:v>
+                  <c:v>0.98894298080377097</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>0.78725904477144404</c:v>
+                  <c:v>0.99045126110744741</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>0.83345315481177829</c:v>
-                </c:pt>
-                <c:pt idx="8">
-                  <c:v>0.88203918971975193</c:v>
+                  <c:v>1.0286907074262921</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>0.89495763249258353</c:v>
+                  <c:v>1.0109751026946947</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>0.8942179214729904</c:v>
+                  <c:v>1.0514992257935214</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>1.0588139493303126</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>1.0670379652207234</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>1.0821051236786146</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>1.0789515024556622</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -390,41 +402,53 @@
           </c:marker>
           <c:xVal>
             <c:numRef>
-              <c:f>'Sheet 1'!$A$23:$A$33</c:f>
+              <c:f>'Sheet 1'!$A$27:$A$41</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="11"/>
+                <c:ptCount val="15"/>
                 <c:pt idx="0">
                   <c:v>0.1</c:v>
                 </c:pt>
                 <c:pt idx="1">
+                  <c:v>0.5</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>1.5</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>10</c:v>
+                </c:pt>
+                <c:pt idx="4">
                   <c:v>15</c:v>
                 </c:pt>
-                <c:pt idx="2">
+                <c:pt idx="5">
                   <c:v>30</c:v>
                 </c:pt>
-                <c:pt idx="3">
+                <c:pt idx="6">
                   <c:v>60</c:v>
                 </c:pt>
-                <c:pt idx="4">
+                <c:pt idx="7">
                   <c:v>90</c:v>
                 </c:pt>
-                <c:pt idx="5">
+                <c:pt idx="8">
+                  <c:v>100</c:v>
+                </c:pt>
+                <c:pt idx="9">
                   <c:v>120</c:v>
                 </c:pt>
-                <c:pt idx="6">
+                <c:pt idx="10">
                   <c:v>150</c:v>
                 </c:pt>
-                <c:pt idx="7">
+                <c:pt idx="11">
                   <c:v>250</c:v>
                 </c:pt>
-                <c:pt idx="8">
+                <c:pt idx="12">
                   <c:v>500</c:v>
                 </c:pt>
-                <c:pt idx="9">
+                <c:pt idx="13">
                   <c:v>750</c:v>
                 </c:pt>
-                <c:pt idx="10">
+                <c:pt idx="14">
                   <c:v>1000</c:v>
                 </c:pt>
               </c:numCache>
@@ -432,42 +456,42 @@
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>'Sheet 1'!$K$23:$K$33</c:f>
+              <c:f>'Sheet 1'!$K$27:$K$41</c:f>
               <c:numCache>
                 <c:formatCode>0.000000</c:formatCode>
-                <c:ptCount val="11"/>
+                <c:ptCount val="15"/>
                 <c:pt idx="0">
-                  <c:v>0.77519648206887304</c:v>
-                </c:pt>
-                <c:pt idx="1">
-                  <c:v>0.80083243056645892</c:v>
-                </c:pt>
-                <c:pt idx="2">
-                  <c:v>0.81914690706968962</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>0.82656078378953657</c:v>
+                  <c:v>1.0035506001332684</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>0.84465973083032153</c:v>
+                  <c:v>1.0779572449118415</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>0.8509612295329948</c:v>
+                  <c:v>1.0206668727246053</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>0.86330946178656565</c:v>
+                  <c:v>1.0298609475740441</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>0.88204852071416562</c:v>
-                </c:pt>
-                <c:pt idx="8">
-                  <c:v>0.90265799625796272</c:v>
+                  <c:v>1.0714308642620487</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>0.90631014559227674</c:v>
+                  <c:v>1.0452657339217364</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>0.90335830122978089</c:v>
+                  <c:v>1.0670489493344424</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>1.0639924185567</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>1.0846944326462025</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>1.0956277405879706</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>1.0707528532565391</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -826,84 +850,108 @@
           </c:trendline>
           <c:xVal>
             <c:numRef>
-              <c:f>'Sheet 1'!$A$6:$A$16</c:f>
+              <c:f>'Sheet 1'!$A$6:$A$20</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="11"/>
+                <c:ptCount val="15"/>
                 <c:pt idx="0">
                   <c:v>0.1</c:v>
                 </c:pt>
                 <c:pt idx="1">
+                  <c:v>0.5</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>1.5</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>10</c:v>
+                </c:pt>
+                <c:pt idx="4">
                   <c:v>15</c:v>
                 </c:pt>
-                <c:pt idx="2">
+                <c:pt idx="5">
                   <c:v>30</c:v>
                 </c:pt>
-                <c:pt idx="3">
+                <c:pt idx="6">
                   <c:v>60</c:v>
                 </c:pt>
-                <c:pt idx="4">
+                <c:pt idx="7">
                   <c:v>90</c:v>
                 </c:pt>
-                <c:pt idx="5">
+                <c:pt idx="8">
+                  <c:v>100</c:v>
+                </c:pt>
+                <c:pt idx="9">
                   <c:v>120</c:v>
                 </c:pt>
-                <c:pt idx="6">
+                <c:pt idx="10">
                   <c:v>150</c:v>
                 </c:pt>
-                <c:pt idx="7">
+                <c:pt idx="11">
                   <c:v>250</c:v>
                 </c:pt>
-                <c:pt idx="8">
+                <c:pt idx="12">
                   <c:v>500</c:v>
                 </c:pt>
-                <c:pt idx="9">
+                <c:pt idx="13">
                   <c:v>750</c:v>
                 </c:pt>
-                <c:pt idx="10">
-                  <c:v>1000</c:v>
+                <c:pt idx="14">
+                  <c:v>999.99</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>'Sheet 1'!$F$6:$F$16</c:f>
+              <c:f>'Sheet 1'!$F$6:$F$20</c:f>
               <c:numCache>
                 <c:formatCode>0.000000</c:formatCode>
-                <c:ptCount val="11"/>
+                <c:ptCount val="15"/>
                 <c:pt idx="0">
-                  <c:v>1.0005581562381762</c:v>
+                  <c:v>1.0120583199660715</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>1.0026743854359832</c:v>
+                  <c:v>0.98723674640081305</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>1.0021589302375784</c:v>
+                  <c:v>0.97352011835670349</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>1.0049611638314022</c:v>
+                  <c:v>0.98670947182667379</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>1.007997543080646</c:v>
+                  <c:v>1.0274179661023068</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>1.0068066975783474</c:v>
+                  <c:v>0.9995818870330847</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>1.0105439212957481</c:v>
+                  <c:v>1.0035538292803527</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>1.0160375172429779</c:v>
+                  <c:v>1.0225693897940391</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>1.0277465853256991</c:v>
+                  <c:v>1.0133855529616367</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>1.0410308363977838</c:v>
+                  <c:v>1.0168926589087053</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>1.0542808874235223</c:v>
+                  <c:v>1.0023371440138709</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>0.99143857028386306</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>0.99628894469879192</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>1.0133076136706871</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>0.98894242420015732</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -993,84 +1041,96 @@
           </c:trendline>
           <c:xVal>
             <c:numRef>
-              <c:f>'Sheet 1'!$A$6:$A$16</c:f>
+              <c:f>'Sheet 1'!$A$6:$A$20</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="11"/>
+                <c:ptCount val="15"/>
                 <c:pt idx="0">
                   <c:v>0.1</c:v>
                 </c:pt>
                 <c:pt idx="1">
+                  <c:v>0.5</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>1.5</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>10</c:v>
+                </c:pt>
+                <c:pt idx="4">
                   <c:v>15</c:v>
                 </c:pt>
-                <c:pt idx="2">
+                <c:pt idx="5">
                   <c:v>30</c:v>
                 </c:pt>
-                <c:pt idx="3">
+                <c:pt idx="6">
                   <c:v>60</c:v>
                 </c:pt>
-                <c:pt idx="4">
+                <c:pt idx="7">
                   <c:v>90</c:v>
                 </c:pt>
-                <c:pt idx="5">
+                <c:pt idx="8">
+                  <c:v>100</c:v>
+                </c:pt>
+                <c:pt idx="9">
                   <c:v>120</c:v>
                 </c:pt>
-                <c:pt idx="6">
+                <c:pt idx="10">
                   <c:v>150</c:v>
                 </c:pt>
-                <c:pt idx="7">
+                <c:pt idx="11">
                   <c:v>250</c:v>
                 </c:pt>
-                <c:pt idx="8">
+                <c:pt idx="12">
                   <c:v>500</c:v>
                 </c:pt>
-                <c:pt idx="9">
+                <c:pt idx="13">
                   <c:v>750</c:v>
                 </c:pt>
-                <c:pt idx="10">
-                  <c:v>1000</c:v>
+                <c:pt idx="14">
+                  <c:v>999.99</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>'Sheet 1'!$K$6:$K$16</c:f>
+              <c:f>'Sheet 1'!$K$6:$K$20</c:f>
               <c:numCache>
                 <c:formatCode>0.000000</c:formatCode>
-                <c:ptCount val="11"/>
+                <c:ptCount val="15"/>
                 <c:pt idx="0">
-                  <c:v>1.0003878283273324</c:v>
-                </c:pt>
-                <c:pt idx="1">
-                  <c:v>1.0027368257083531</c:v>
-                </c:pt>
-                <c:pt idx="2">
-                  <c:v>1.002132645867061</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>1.004473547867506</c:v>
+                  <c:v>1.0124595607074192</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>1.0073888101001607</c:v>
+                  <c:v>1.0246126531897757</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>1.0081526090820587</c:v>
+                  <c:v>0.99123212311197628</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>1.010816520529382</c:v>
+                  <c:v>1.0019803232436455</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>1.0129844821876621</c:v>
-                </c:pt>
-                <c:pt idx="8">
-                  <c:v>1.0286922566821892</c:v>
+                  <c:v>1.0235838898658773</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>1.0410106462729396</c:v>
+                  <c:v>0.99238859087523068</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>1.0574321213036151</c:v>
+                  <c:v>1.0068419602917082</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>1.0041778550412717</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>1.0147327958753034</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>1.0192489706741765</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>0.9824392574158276</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1355,7 +1415,7 @@
           <c:order val="0"/>
           <c:tx>
             <c:strRef>
-              <c:f>'Sheet 1'!$F$57</c:f>
+              <c:f>'Sheet 1'!$F$65</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -1388,7 +1448,7 @@
           </c:marker>
           <c:xVal>
             <c:numRef>
-              <c:f>'Sheet 1'!$A$58:$A$68</c:f>
+              <c:f>'Sheet 1'!$A$66:$A$76</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="11"/>
@@ -1430,7 +1490,7 @@
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>'Sheet 1'!$F$58:$F$68</c:f>
+              <c:f>'Sheet 1'!$F$66:$F$76</c:f>
               <c:numCache>
                 <c:formatCode>0.000000</c:formatCode>
                 <c:ptCount val="11"/>
@@ -1719,7 +1779,7 @@
           <c:order val="0"/>
           <c:tx>
             <c:strRef>
-              <c:f>'Sheet 1'!$F$40</c:f>
+              <c:f>'Sheet 1'!$F$48</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -1752,7 +1812,7 @@
           </c:marker>
           <c:xVal>
             <c:numRef>
-              <c:f>'Sheet 1'!$A$41:$A$51</c:f>
+              <c:f>'Sheet 1'!$A$49:$A$59</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="11"/>
@@ -1794,7 +1854,7 @@
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>'Sheet 1'!$F$41:$F$51</c:f>
+              <c:f>'Sheet 1'!$F$49:$F$59</c:f>
               <c:numCache>
                 <c:formatCode>0.000000</c:formatCode>
                 <c:ptCount val="11"/>
@@ -4258,13 +4318,13 @@
     <xdr:from>
       <xdr:col>12</xdr:col>
       <xdr:colOff>132179</xdr:colOff>
-      <xdr:row>19</xdr:row>
+      <xdr:row>23</xdr:row>
       <xdr:rowOff>56857</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>19</xdr:col>
       <xdr:colOff>436979</xdr:colOff>
-      <xdr:row>34</xdr:row>
+      <xdr:row>42</xdr:row>
       <xdr:rowOff>56857</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
@@ -4300,7 +4360,7 @@
     <xdr:to>
       <xdr:col>19</xdr:col>
       <xdr:colOff>605790</xdr:colOff>
-      <xdr:row>15</xdr:row>
+      <xdr:row>19</xdr:row>
       <xdr:rowOff>99060</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
@@ -4330,13 +4390,13 @@
     <xdr:from>
       <xdr:col>11</xdr:col>
       <xdr:colOff>868680</xdr:colOff>
-      <xdr:row>53</xdr:row>
+      <xdr:row>61</xdr:row>
       <xdr:rowOff>76200</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>19</xdr:col>
       <xdr:colOff>198120</xdr:colOff>
-      <xdr:row>68</xdr:row>
+      <xdr:row>76</xdr:row>
       <xdr:rowOff>76200</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
@@ -4366,13 +4426,13 @@
     <xdr:from>
       <xdr:col>11</xdr:col>
       <xdr:colOff>929640</xdr:colOff>
-      <xdr:row>37</xdr:row>
+      <xdr:row>45</xdr:row>
       <xdr:rowOff>7620</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>19</xdr:col>
       <xdr:colOff>259080</xdr:colOff>
-      <xdr:row>52</xdr:row>
+      <xdr:row>60</xdr:row>
       <xdr:rowOff>7620</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
@@ -4664,7 +4724,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C22416C2-1180-4450-A3B0-0B08DD9AEC85}">
-  <dimension ref="A1:L68"/>
+  <dimension ref="A1:L76"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="12.33203125" customWidth="1"/>
@@ -4769,1579 +4829,1774 @@
         <v>1.40420707746021</v>
       </c>
       <c r="D6">
-        <v>1.3831224644600999</v>
+        <v>1.3686193553583801</v>
       </c>
       <c r="E6">
-        <v>1.3838944628918</v>
+        <v>1.38512260545705</v>
       </c>
       <c r="F6" s="10">
         <f>E6/D6</f>
-        <v>1.0005581562381762</v>
+        <v>1.0120583199660715</v>
       </c>
       <c r="G6" s="4"/>
       <c r="H6">
         <v>1.4043892076542099</v>
       </c>
       <c r="I6">
-        <v>1.38336349245063</v>
+        <v>1.3681177802680899</v>
       </c>
       <c r="J6">
-        <v>1.3838999999999999</v>
+        <v>1.3851639268062399</v>
       </c>
       <c r="K6" s="10">
         <f>J6/I6</f>
-        <v>1.0003878283273324</v>
+        <v>1.0124595607074192</v>
       </c>
       <c r="L6" s="10"/>
     </row>
-    <row r="7" spans="1:12" s="4" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="4">
-        <v>15</v>
+    <row r="7" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A7">
+        <v>0.5</v>
       </c>
       <c r="B7" s="5"/>
-      <c r="C7" s="4">
-        <v>1.3978225806626601</v>
-      </c>
       <c r="D7">
-        <v>1.37702734478371</v>
+        <v>1.3922831524096599</v>
       </c>
       <c r="E7">
-        <v>1.3807100466595501</v>
-      </c>
-      <c r="F7" s="11">
-        <f t="shared" ref="F7:F16" si="0">E7/D7</f>
-        <v>1.0026743854359832</v>
-      </c>
-      <c r="H7" s="4">
-        <v>1.3977474767840601</v>
-      </c>
+        <v>1.37451308945358</v>
+      </c>
+      <c r="F7" s="10">
+        <f t="shared" ref="F7:F20" si="0">E7/D7</f>
+        <v>0.98723674640081305</v>
+      </c>
+      <c r="G7" s="4"/>
       <c r="I7">
-        <v>1.3757277802121</v>
+        <v>1.3884228746446901</v>
       </c>
       <c r="J7">
-        <v>1.3794929073686799</v>
-      </c>
-      <c r="K7" s="11">
-        <f t="shared" ref="K7:K16" si="1">J7/I7</f>
-        <v>1.0027368257083531</v>
-      </c>
-      <c r="L7" s="11"/>
+        <v>1.3739233641712201</v>
+      </c>
+      <c r="K7" s="10"/>
+      <c r="L7" s="10"/>
     </row>
     <row r="8" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A8">
-        <v>30</v>
+        <v>1.5</v>
       </c>
       <c r="B8" s="5"/>
-      <c r="C8">
-        <v>1.3935791421766499</v>
-      </c>
       <c r="D8">
-        <v>1.3755520515803401</v>
+        <v>1.4141178954362701</v>
       </c>
       <c r="E8">
-        <v>1.37852177249786</v>
+        <v>1.3766722209354501</v>
       </c>
       <c r="F8" s="10">
         <f t="shared" si="0"/>
-        <v>1.0021589302375784</v>
+        <v>0.97352011835670349</v>
       </c>
       <c r="G8" s="4"/>
-      <c r="H8">
-        <v>1.3923333952149399</v>
-      </c>
       <c r="I8">
-        <v>1.3733520244906201</v>
+        <v>1.4147283449213399</v>
       </c>
       <c r="J8">
-        <v>1.3762808980096699</v>
-      </c>
-      <c r="K8" s="10">
-        <f t="shared" si="1"/>
-        <v>1.002132645867061</v>
-      </c>
+        <v>1.3760578260651899</v>
+      </c>
+      <c r="K8" s="10"/>
       <c r="L8" s="10"/>
     </row>
-    <row r="9" spans="1:12" s="4" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="4">
-        <v>60</v>
+    <row r="9" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A9">
+        <v>10</v>
       </c>
       <c r="B9" s="5"/>
-      <c r="C9" s="4">
-        <v>1.38536063754419</v>
-      </c>
       <c r="D9">
-        <v>1.3645310546268701</v>
+        <v>1.4052374449883001</v>
       </c>
       <c r="E9">
-        <v>1.37130071674191</v>
-      </c>
-      <c r="F9" s="11">
+        <v>1.38656109713547</v>
+      </c>
+      <c r="F9" s="10">
         <f t="shared" si="0"/>
-        <v>1.0049611638314022</v>
-      </c>
-      <c r="H9" s="4">
-        <v>1.3811147115786999</v>
-      </c>
+        <v>0.98670947182667379</v>
+      </c>
+      <c r="G9" s="4"/>
       <c r="I9">
-        <v>1.36149933832843</v>
+        <v>1.3952787310994501</v>
       </c>
       <c r="J9">
-        <v>1.3675900707900199</v>
-      </c>
-      <c r="K9" s="11">
-        <f t="shared" si="1"/>
-        <v>1.004473547867506</v>
-      </c>
-      <c r="L9" s="11"/>
+        <v>1.3887518550334099</v>
+      </c>
+      <c r="K9" s="10"/>
+      <c r="L9" s="10"/>
     </row>
-    <row r="10" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:12" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A10">
-        <v>90</v>
+        <v>15</v>
       </c>
       <c r="B10" s="5"/>
-      <c r="C10">
-        <v>1.37856347972413</v>
+      <c r="C10" s="4">
+        <v>1.3978225806626601</v>
       </c>
       <c r="D10">
-        <v>1.3579435428314801</v>
+        <v>1.3588321367490299</v>
       </c>
       <c r="E10">
-        <v>1.3688037548163601</v>
+        <v>1.3960885502131399</v>
       </c>
       <c r="F10" s="10">
         <f t="shared" si="0"/>
-        <v>1.007997543080646</v>
-      </c>
-      <c r="G10" s="4"/>
-      <c r="H10">
-        <v>1.3698685473168299</v>
+        <v>1.0274179661023068</v>
+      </c>
+      <c r="H10" s="4">
+        <v>1.3977474767840601</v>
       </c>
       <c r="I10">
-        <v>1.35117281876724</v>
+        <v>1.36086238814935</v>
       </c>
       <c r="J10">
-        <v>1.3611563781376099</v>
-      </c>
-      <c r="K10" s="10">
+        <v>1.3943568221478799</v>
+      </c>
+      <c r="K10" s="11">
+        <f t="shared" ref="K10:K20" si="1">J10/I10</f>
+        <v>1.0246126531897757</v>
+      </c>
+      <c r="L10" s="11"/>
+    </row>
+    <row r="11" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A11">
+        <v>30</v>
+      </c>
+      <c r="B11" s="5"/>
+      <c r="C11">
+        <v>1.3935791421766499</v>
+      </c>
+      <c r="D11">
+        <v>1.38084479180245</v>
+      </c>
+      <c r="E11">
+        <v>1.3802674426896999</v>
+      </c>
+      <c r="F11" s="10">
+        <f t="shared" si="0"/>
+        <v>0.9995818870330847</v>
+      </c>
+      <c r="G11" s="4"/>
+      <c r="H11">
+        <v>1.3923333952149399</v>
+      </c>
+      <c r="I11">
+        <v>1.3852911212816701</v>
+      </c>
+      <c r="J11">
+        <v>1.3731450592762</v>
+      </c>
+      <c r="K11" s="10">
         <f t="shared" si="1"/>
-        <v>1.0073888101001607</v>
-      </c>
-      <c r="L10" s="10"/>
+        <v>0.99123212311197628</v>
+      </c>
+      <c r="L11" s="10"/>
     </row>
-    <row r="11" spans="1:12" s="4" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="4">
-        <v>120</v>
-      </c>
-      <c r="B11" s="5"/>
-      <c r="C11" s="4">
-        <v>1.3699400435562701</v>
-      </c>
-      <c r="D11">
-        <v>1.3501528303570001</v>
-      </c>
-      <c r="E11">
-        <v>1.35934291235779</v>
-      </c>
-      <c r="F11" s="11">
-        <f t="shared" si="0"/>
-        <v>1.0068066975783474</v>
-      </c>
-      <c r="H11" s="4">
-        <v>1.35986137171571</v>
-      </c>
-      <c r="I11">
-        <v>1.3415734947956099</v>
-      </c>
-      <c r="J11">
-        <v>1.35251081905353</v>
-      </c>
-      <c r="K11" s="11">
-        <f t="shared" si="1"/>
-        <v>1.0081526090820587</v>
-      </c>
-      <c r="L11" s="11"/>
-    </row>
-    <row r="12" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:12" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A12">
-        <v>150</v>
+        <v>60</v>
       </c>
       <c r="B12" s="5"/>
-      <c r="C12">
-        <v>1.3618779251700099</v>
+      <c r="C12" s="4">
+        <v>1.38536063754419</v>
       </c>
       <c r="D12">
-        <v>1.3433447133374901</v>
+        <v>1.35391575819657</v>
       </c>
       <c r="E12">
-        <v>1.35750883426798</v>
+        <v>1.35872734366118</v>
       </c>
       <c r="F12" s="10">
         <f t="shared" si="0"/>
-        <v>1.0105439212957481</v>
-      </c>
-      <c r="G12" s="4"/>
-      <c r="H12">
-        <v>1.34863286309854</v>
+        <v>1.0035538292803527</v>
+      </c>
+      <c r="H12" s="4">
+        <v>1.3811147115786999</v>
       </c>
       <c r="I12">
-        <v>1.3311196421075699</v>
+        <v>1.3558315843768101</v>
       </c>
       <c r="J12">
-        <v>1.34551772504349</v>
-      </c>
-      <c r="K12" s="10">
+        <v>1.35851656917782</v>
+      </c>
+      <c r="K12" s="11">
         <f t="shared" si="1"/>
-        <v>1.010816520529382</v>
-      </c>
-      <c r="L12" s="10"/>
+        <v>1.0019803232436455</v>
+      </c>
+      <c r="L12" s="11"/>
     </row>
-    <row r="13" spans="1:12" s="4" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="4">
-        <v>250</v>
+    <row r="13" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A13">
+        <v>90</v>
       </c>
       <c r="B13" s="5"/>
-      <c r="C13" s="4">
-        <v>1.34128105403747</v>
+      <c r="C13">
+        <v>1.37856347972413</v>
       </c>
       <c r="D13">
-        <v>1.3183641537176001</v>
+        <v>1.3540665504448699</v>
       </c>
       <c r="E13">
-        <v>1.33950744156537</v>
-      </c>
-      <c r="F13" s="11">
+        <v>1.3846270062289301</v>
+      </c>
+      <c r="F13" s="10">
         <f t="shared" si="0"/>
-        <v>1.0160375172429779</v>
-      </c>
-      <c r="H13" s="4">
-        <v>1.31869938927708</v>
+        <v>1.0225693897940391</v>
+      </c>
+      <c r="G13" s="4"/>
+      <c r="H13">
+        <v>1.3698685473168299</v>
       </c>
       <c r="I13">
-        <v>1.3013234683263499</v>
+        <v>1.34423803647162</v>
       </c>
       <c r="J13">
-        <v>1.31822047972122</v>
-      </c>
-      <c r="K13" s="11">
+        <v>1.37594039827729</v>
+      </c>
+      <c r="K13" s="10">
         <f t="shared" si="1"/>
-        <v>1.0129844821876621</v>
-      </c>
-      <c r="L13" s="11"/>
+        <v>1.0235838898658773</v>
+      </c>
+      <c r="L13" s="10"/>
     </row>
     <row r="14" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A14">
-        <v>500</v>
+        <v>100</v>
       </c>
       <c r="B14" s="5"/>
-      <c r="C14">
-        <v>1.2896852557910301</v>
-      </c>
       <c r="D14">
-        <v>1.2700267746399601</v>
+        <v>1.3565730983264299</v>
       </c>
       <c r="E14">
-        <v>1.30526568090843</v>
+        <v>1.37473157938041</v>
       </c>
       <c r="F14" s="10">
         <f t="shared" si="0"/>
-        <v>1.0277465853256991</v>
+        <v>1.0133855529616367</v>
       </c>
       <c r="G14" s="4"/>
-      <c r="H14">
-        <v>1.24433347413396</v>
-      </c>
       <c r="I14">
-        <v>1.2338069312922</v>
+        <v>1.3294388930292</v>
       </c>
       <c r="J14">
-        <v>1.2692076364611</v>
-      </c>
-      <c r="K14" s="10">
-        <f t="shared" si="1"/>
-        <v>1.0286922566821892</v>
-      </c>
+        <v>1.3730626322350199</v>
+      </c>
+      <c r="K14" s="10"/>
       <c r="L14" s="10"/>
     </row>
     <row r="15" spans="1:12" s="4" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="4">
-        <v>750</v>
+      <c r="A15">
+        <v>120</v>
       </c>
       <c r="B15" s="5"/>
       <c r="C15" s="4">
-        <v>1.24225887840578</v>
+        <v>1.3699400435562701</v>
       </c>
       <c r="D15">
-        <v>1.2232055342510899</v>
+        <v>1.34077916991197</v>
       </c>
       <c r="E15">
-        <v>1.27339468040781</v>
-      </c>
-      <c r="F15" s="11">
+        <v>1.3634284951011899</v>
+      </c>
+      <c r="F15" s="10">
         <f t="shared" si="0"/>
-        <v>1.0410308363977838</v>
+        <v>1.0168926589087053</v>
       </c>
       <c r="H15" s="4">
-        <v>1.1765306054398399</v>
+        <v>1.35986137171571</v>
       </c>
       <c r="I15">
-        <v>1.1709175184150999</v>
+        <v>1.35581073898229</v>
       </c>
       <c r="J15">
-        <v>1.21893760257761</v>
+        <v>1.34549110875214</v>
       </c>
       <c r="K15" s="11">
         <f t="shared" si="1"/>
-        <v>1.0410106462729396</v>
+        <v>0.99238859087523068</v>
       </c>
       <c r="L15" s="11"/>
     </row>
     <row r="16" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A16">
-        <v>1000</v>
+        <v>150</v>
       </c>
       <c r="B16" s="5"/>
       <c r="C16">
-        <v>1.1938794039418501</v>
+        <v>1.3618779251700099</v>
       </c>
       <c r="D16">
-        <v>1.1763723210775801</v>
+        <v>1.3628583617894401</v>
       </c>
       <c r="E16">
-        <v>1.2402268546061399</v>
+        <v>1.3660435580514501</v>
       </c>
       <c r="F16" s="10">
         <f t="shared" si="0"/>
-        <v>1.0542808874235223</v>
+        <v>1.0023371440138709</v>
       </c>
       <c r="G16" s="4"/>
       <c r="H16">
-        <v>1.1108715265371401</v>
+        <v>1.34863286309854</v>
       </c>
       <c r="I16">
-        <v>1.10875726262634</v>
+        <v>1.34642475596859</v>
       </c>
       <c r="J16">
-        <v>1.17243554422976</v>
+        <v>1.3556369406847</v>
       </c>
       <c r="K16" s="10">
         <f t="shared" si="1"/>
-        <v>1.0574321213036151</v>
+        <v>1.0068419602917082</v>
       </c>
       <c r="L16" s="10"/>
     </row>
+    <row r="17" spans="1:12" s="4" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A17">
+        <v>250</v>
+      </c>
+      <c r="B17" s="5"/>
+      <c r="C17" s="4">
+        <v>1.34128105403747</v>
+      </c>
+      <c r="D17">
+        <v>1.31238054231434</v>
+      </c>
+      <c r="E17">
+        <v>1.30114468854049</v>
+      </c>
+      <c r="F17" s="10">
+        <f t="shared" si="0"/>
+        <v>0.99143857028386306</v>
+      </c>
+      <c r="H17" s="4">
+        <v>1.31869938927708</v>
+      </c>
+      <c r="I17">
+        <v>1.2854468687873799</v>
+      </c>
+      <c r="J17">
+        <v>1.2908172794684301</v>
+      </c>
+      <c r="K17" s="11">
+        <f t="shared" si="1"/>
+        <v>1.0041778550412717</v>
+      </c>
+      <c r="L17" s="11"/>
+    </row>
+    <row r="18" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A18">
+        <v>500</v>
+      </c>
+      <c r="B18" s="5"/>
+      <c r="C18">
+        <v>1.2896852557910301</v>
+      </c>
+      <c r="D18">
+        <v>1.27106900787611</v>
+      </c>
+      <c r="E18">
+        <v>1.2663520004962301</v>
+      </c>
+      <c r="F18" s="10">
+        <f t="shared" si="0"/>
+        <v>0.99628894469879192</v>
+      </c>
+      <c r="G18" s="4"/>
+      <c r="H18">
+        <v>1.24433347413396</v>
+      </c>
+      <c r="I18">
+        <v>1.24215702849295</v>
+      </c>
+      <c r="J18">
+        <v>1.26045747443881</v>
+      </c>
+      <c r="K18" s="10">
+        <f t="shared" si="1"/>
+        <v>1.0147327958753034</v>
+      </c>
+      <c r="L18" s="10"/>
+    </row>
+    <row r="19" spans="1:12" s="4" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A19">
+        <v>750</v>
+      </c>
+      <c r="B19" s="5"/>
+      <c r="C19" s="4">
+        <v>1.24225887840578</v>
+      </c>
+      <c r="D19">
+        <v>1.2502327359779</v>
+      </c>
+      <c r="E19">
+        <v>1.26687035022674</v>
+      </c>
+      <c r="F19" s="10">
+        <f t="shared" si="0"/>
+        <v>1.0133076136706871</v>
+      </c>
+      <c r="H19" s="4">
+        <v>1.1765306054398399</v>
+      </c>
+      <c r="I19">
+        <v>1.20261020085431</v>
+      </c>
+      <c r="J19">
+        <v>1.2257592093430201</v>
+      </c>
+      <c r="K19" s="11">
+        <f t="shared" si="1"/>
+        <v>1.0192489706741765</v>
+      </c>
+      <c r="L19" s="11"/>
+    </row>
     <row r="20" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="C20" s="12" t="s">
-        <v>5</v>
-      </c>
-      <c r="D20" s="12"/>
-      <c r="E20" s="13"/>
-      <c r="F20" s="13"/>
-      <c r="H20" s="2"/>
-      <c r="I20" s="2"/>
-      <c r="J20" s="2"/>
-      <c r="K20" s="2"/>
-    </row>
-    <row r="21" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="C21" s="3" t="s">
-        <v>4</v>
-      </c>
-      <c r="D21" s="3"/>
-      <c r="E21" s="9"/>
-      <c r="F21" s="3"/>
-      <c r="H21" s="3" t="s">
-        <v>3</v>
-      </c>
-      <c r="I21" s="3"/>
-      <c r="J21" s="9"/>
-      <c r="K21" s="9"/>
-      <c r="L21" s="3"/>
-    </row>
-    <row r="22" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A22" s="6" t="s">
-        <v>0</v>
-      </c>
-      <c r="B22" s="6"/>
-      <c r="C22" s="6" t="s">
-        <v>1</v>
-      </c>
-      <c r="D22" s="6" t="s">
-        <v>7</v>
-      </c>
-      <c r="E22" s="6" t="s">
-        <v>6</v>
-      </c>
-      <c r="F22" s="7" t="s">
-        <v>8</v>
-      </c>
-      <c r="G22" s="8"/>
-      <c r="H22" s="6" t="s">
-        <v>1</v>
-      </c>
-      <c r="I22" s="6" t="s">
-        <v>7</v>
-      </c>
-      <c r="J22" s="6" t="s">
-        <v>6</v>
-      </c>
-      <c r="K22" s="7" t="s">
-        <v>8</v>
-      </c>
-      <c r="L22" s="7"/>
-    </row>
-    <row r="23" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A23">
-        <v>0.1</v>
-      </c>
-      <c r="B23" s="5"/>
-      <c r="C23" s="2">
-        <v>3.52725672373683E-5</v>
-      </c>
-      <c r="D23" s="2">
-        <v>3.4352992727381499E-5</v>
-      </c>
-      <c r="E23" s="2">
-        <v>2.0875371825261901E-5</v>
-      </c>
-      <c r="F23" s="10">
-        <f>E23/D23</f>
-        <v>0.60767258302427063</v>
-      </c>
-      <c r="G23" s="4"/>
-      <c r="H23" s="2">
-        <v>3.2364516810043102E-5</v>
-      </c>
-      <c r="I23" s="2">
-        <v>3.0077664875068999E-5</v>
-      </c>
-      <c r="J23" s="2">
-        <v>2.3316099999999999E-5</v>
-      </c>
-      <c r="K23" s="10">
-        <f>J23/I23</f>
-        <v>0.77519648206887304</v>
-      </c>
-      <c r="L23" s="10"/>
+      <c r="A20">
+        <v>999.99</v>
+      </c>
+      <c r="B20" s="5"/>
+      <c r="C20">
+        <v>1.1938794039418501</v>
+      </c>
+      <c r="D20">
+        <v>1.2216766905077201</v>
+      </c>
+      <c r="E20">
+        <v>1.20816790789953</v>
+      </c>
+      <c r="F20" s="10">
+        <f t="shared" si="0"/>
+        <v>0.98894242420015732</v>
+      </c>
+      <c r="G20" s="4"/>
+      <c r="H20">
+        <v>1.1108715265371401</v>
+      </c>
+      <c r="I20">
+        <v>1.1553240194424299</v>
+      </c>
+      <c r="J20">
+        <v>1.13503567173569</v>
+      </c>
+      <c r="K20" s="10">
+        <f t="shared" si="1"/>
+        <v>0.9824392574158276</v>
+      </c>
+      <c r="L20" s="10"/>
     </row>
     <row r="24" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A24" s="4">
-        <v>15</v>
-      </c>
-      <c r="B24" s="5"/>
-      <c r="C24" s="5">
-        <v>5.02535867346246E-3</v>
-      </c>
-      <c r="D24">
-        <v>4.8415021318079796E-3</v>
-      </c>
-      <c r="E24">
-        <v>3.1726397963949501E-3</v>
-      </c>
-      <c r="F24" s="11">
-        <f t="shared" ref="F24:F33" si="2">E24/D24</f>
-        <v>0.65530071246920629</v>
-      </c>
-      <c r="G24" s="4"/>
-      <c r="H24">
-        <v>4.7442437671726999E-3</v>
-      </c>
-      <c r="I24">
-        <v>4.41670217006298E-3</v>
-      </c>
-      <c r="J24">
-        <v>3.5370383339396899E-3</v>
-      </c>
-      <c r="K24" s="11">
-        <f t="shared" ref="K24:K33" si="3">J24/I24</f>
-        <v>0.80083243056645892</v>
-      </c>
-      <c r="L24" s="11"/>
+      <c r="C24" s="12" t="s">
+        <v>5</v>
+      </c>
+      <c r="D24" s="12"/>
+      <c r="E24" s="13"/>
+      <c r="F24" s="13"/>
+      <c r="H24" s="2"/>
+      <c r="I24" s="2"/>
+      <c r="J24" s="2"/>
+      <c r="K24" s="2"/>
     </row>
     <row r="25" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A25">
-        <v>30</v>
-      </c>
-      <c r="B25" s="5"/>
-      <c r="C25" s="2">
-        <v>9.6096776712520909E-3</v>
-      </c>
-      <c r="D25">
-        <v>9.3736870838320892E-3</v>
-      </c>
-      <c r="E25">
-        <v>6.3510742712361698E-3</v>
-      </c>
-      <c r="F25" s="10">
-        <f t="shared" si="2"/>
-        <v>0.67754280833532643</v>
-      </c>
-      <c r="G25" s="4"/>
-      <c r="H25">
-        <v>9.3381817414101998E-3</v>
-      </c>
-      <c r="I25">
-        <v>8.6773810916228808E-3</v>
-      </c>
-      <c r="J25">
-        <v>7.1080498826678901E-3</v>
-      </c>
-      <c r="K25" s="10">
-        <f t="shared" si="3"/>
-        <v>0.81914690706968962</v>
-      </c>
-      <c r="L25" s="10"/>
+      <c r="C25" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="D25" s="3"/>
+      <c r="E25" s="9"/>
+      <c r="F25" s="3"/>
+      <c r="H25" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="I25" s="3"/>
+      <c r="J25" s="9"/>
+      <c r="K25" s="9"/>
+      <c r="L25" s="3"/>
     </row>
     <row r="26" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A26" s="4">
-        <v>60</v>
-      </c>
-      <c r="B26" s="5"/>
-      <c r="C26" s="5">
-        <v>1.7956202904139199E-2</v>
-      </c>
-      <c r="D26">
-        <v>1.7499246818678899E-2</v>
-      </c>
-      <c r="E26">
-        <v>1.25132922386715E-2</v>
-      </c>
-      <c r="F26" s="11">
-        <f t="shared" si="2"/>
-        <v>0.7150760468910391</v>
-      </c>
-      <c r="G26" s="4"/>
-      <c r="H26">
-        <v>1.8093633576609602E-2</v>
-      </c>
-      <c r="I26">
-        <v>1.6825678983851101E-2</v>
-      </c>
-      <c r="J26">
-        <v>1.39074464086831E-2</v>
-      </c>
-      <c r="K26" s="11">
-        <f t="shared" si="3"/>
-        <v>0.82656078378953657</v>
-      </c>
-      <c r="L26" s="11"/>
+      <c r="A26" s="6" t="s">
+        <v>0</v>
+      </c>
+      <c r="B26" s="6"/>
+      <c r="C26" s="6" t="s">
+        <v>1</v>
+      </c>
+      <c r="D26" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="E26" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="F26" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="G26" s="8"/>
+      <c r="H26" s="6" t="s">
+        <v>1</v>
+      </c>
+      <c r="I26" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="J26" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="K26" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="L26" s="7"/>
     </row>
     <row r="27" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A27">
-        <v>90</v>
+        <v>0.1</v>
       </c>
       <c r="B27" s="5"/>
       <c r="C27" s="2">
-        <v>2.54716677488637E-2</v>
+        <v>3.52725672373683E-5</v>
       </c>
       <c r="D27">
-        <v>2.48286557998008E-2</v>
+        <v>3.2314434653956498E-4</v>
       </c>
       <c r="E27">
-        <v>1.8460059811568001E-2</v>
+        <v>2.9113846589042902E-4</v>
       </c>
       <c r="F27" s="10">
-        <f t="shared" si="2"/>
-        <v>0.74349815634063066</v>
+        <f>E27/D27</f>
+        <v>0.90095484884115951</v>
       </c>
       <c r="G27" s="4"/>
-      <c r="H27">
-        <v>2.63480432958439E-2</v>
+      <c r="H27" s="2">
+        <v>3.2364516810043102E-5</v>
       </c>
       <c r="I27">
-        <v>2.45310107988954E-2</v>
+        <v>2.8864520587018101E-4</v>
       </c>
       <c r="J27">
-        <v>2.0720356978390701E-2</v>
+        <v>2.8967006957661098E-4</v>
       </c>
       <c r="K27" s="10">
-        <f t="shared" si="3"/>
-        <v>0.84465973083032153</v>
+        <f>J27/I27</f>
+        <v>1.0035506001332684</v>
       </c>
       <c r="L27" s="10"/>
     </row>
     <row r="28" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A28" s="4">
-        <v>120</v>
+      <c r="A28">
+        <v>0.5</v>
       </c>
       <c r="B28" s="5"/>
-      <c r="C28" s="5">
-        <v>3.2417642839879697E-2</v>
-      </c>
+      <c r="C28" s="2"/>
       <c r="D28">
-        <v>3.1708222423746601E-2</v>
+        <v>1.63531469505055E-3</v>
       </c>
       <c r="E28">
-        <v>2.4237248335804401E-2</v>
-      </c>
-      <c r="F28" s="11">
-        <f t="shared" si="2"/>
-        <v>0.76438369871068157</v>
-      </c>
+        <v>1.5602327945626699E-3</v>
+      </c>
+      <c r="F28" s="10"/>
       <c r="G28" s="4"/>
-      <c r="H28">
-        <v>3.4169678168819703E-2</v>
-      </c>
+      <c r="H28" s="2"/>
       <c r="I28">
-        <v>3.2010350694294497E-2</v>
+        <v>1.4624167995472899E-3</v>
       </c>
       <c r="J28">
-        <v>2.7239567384599199E-2</v>
-      </c>
-      <c r="K28" s="11">
-        <f t="shared" si="3"/>
-        <v>0.8509612295329948</v>
-      </c>
-      <c r="L28" s="11"/>
+        <v>1.55376135488548E-3</v>
+      </c>
+      <c r="K28" s="10"/>
+      <c r="L28" s="10"/>
     </row>
     <row r="29" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A29">
-        <v>150</v>
+        <v>1.5</v>
       </c>
       <c r="B29" s="5"/>
-      <c r="C29" s="2">
-        <v>3.9055212834252402E-2</v>
-      </c>
+      <c r="C29" s="2"/>
       <c r="D29">
-        <v>3.8101638451620401E-2</v>
+        <v>5.0200091937920499E-3</v>
       </c>
       <c r="E29">
-        <v>2.9995859491649599E-2</v>
-      </c>
-      <c r="F29" s="10">
-        <f t="shared" si="2"/>
-        <v>0.78725904477144404</v>
-      </c>
+        <v>4.4418725803358596E-3</v>
+      </c>
+      <c r="F29" s="10"/>
       <c r="G29" s="4"/>
-      <c r="H29">
-        <v>4.1796462699614498E-2</v>
-      </c>
+      <c r="H29" s="2"/>
       <c r="I29">
-        <v>3.8938267233086299E-2</v>
+        <v>4.4120832608900004E-3</v>
       </c>
       <c r="J29">
-        <v>3.3615774527897199E-2</v>
-      </c>
-      <c r="K29" s="10">
-        <f t="shared" si="3"/>
-        <v>0.86330946178656565</v>
-      </c>
+        <v>4.3968622699160501E-3</v>
+      </c>
+      <c r="K29" s="10"/>
       <c r="L29" s="10"/>
     </row>
     <row r="30" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A30" s="4">
-        <v>250</v>
+      <c r="A30">
+        <v>10</v>
       </c>
       <c r="B30" s="5"/>
-      <c r="C30" s="5">
-        <v>5.8983323870902299E-2</v>
-      </c>
+      <c r="C30" s="2"/>
       <c r="D30">
-        <v>5.7845592896108598E-2</v>
+        <v>3.2233154188020502E-2</v>
       </c>
       <c r="E30">
-        <v>4.8211591891219499E-2</v>
-      </c>
-      <c r="F30" s="11">
-        <f t="shared" si="2"/>
-        <v>0.83345315481177829</v>
-      </c>
+        <v>3.1830960117675798E-2</v>
+      </c>
+      <c r="F30" s="10"/>
       <c r="G30" s="4"/>
-      <c r="H30">
-        <v>6.5796691976300697E-2</v>
-      </c>
+      <c r="H30" s="2"/>
       <c r="I30">
-        <v>6.12659256159543E-2</v>
+        <v>2.9294700126228299E-2</v>
       </c>
       <c r="J30">
-        <v>5.4039519059736599E-2</v>
-      </c>
-      <c r="K30" s="11">
-        <f t="shared" si="3"/>
-        <v>0.88204852071416562</v>
-      </c>
-      <c r="L30" s="11"/>
+        <v>2.9963416156383201E-2</v>
+      </c>
+      <c r="K30" s="10"/>
+      <c r="L30" s="10"/>
     </row>
     <row r="31" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A31">
-        <v>500</v>
+      <c r="A31" s="4">
+        <v>15</v>
       </c>
       <c r="B31" s="5"/>
-      <c r="C31" s="2">
-        <v>0.103595084893309</v>
+      <c r="C31" s="5">
+        <v>5.02535867346246E-3</v>
       </c>
       <c r="D31">
-        <v>0.101681976801287</v>
+        <v>4.8083671005010903E-2</v>
       </c>
       <c r="E31">
-        <v>8.9687488426909795E-2</v>
-      </c>
-      <c r="F31" s="10">
-        <f t="shared" si="2"/>
-        <v>0.88203918971975193</v>
+        <v>4.7413078230864998E-2</v>
+      </c>
+      <c r="F31" s="11">
+        <f t="shared" ref="F31:F41" si="2">E31/D31</f>
+        <v>0.98605362776739691</v>
       </c>
       <c r="G31" s="4"/>
       <c r="H31">
-        <v>0.11839645185777101</v>
+        <v>4.7442437671726999E-3</v>
       </c>
       <c r="I31">
-        <v>0.111333610679465</v>
+        <v>4.28280907778881E-2</v>
       </c>
       <c r="J31">
-        <v>0.10049617393209</v>
-      </c>
-      <c r="K31" s="10">
-        <f t="shared" si="3"/>
-        <v>0.90265799625796272</v>
-      </c>
-      <c r="L31" s="10"/>
+        <v>4.61668507397665E-2</v>
+      </c>
+      <c r="K31" s="11">
+        <f t="shared" ref="K31:K41" si="3">J31/I31</f>
+        <v>1.0779572449118415</v>
+      </c>
+      <c r="L31" s="11"/>
     </row>
     <row r="32" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A32" s="4">
-        <v>750</v>
+      <c r="A32">
+        <v>30</v>
       </c>
       <c r="B32" s="5"/>
-      <c r="C32" s="5">
-        <v>0.14519436153500101</v>
+      <c r="C32" s="2">
+        <v>9.6096776712520909E-3</v>
       </c>
       <c r="D32">
-        <v>0.142175529915751</v>
+        <v>9.5891818868841697E-2</v>
       </c>
       <c r="E32">
-        <v>0.127241075651779</v>
-      </c>
-      <c r="F32" s="11">
+        <v>9.4831541186847598E-2</v>
+      </c>
+      <c r="F32" s="10">
         <f t="shared" si="2"/>
-        <v>0.89495763249258353</v>
+        <v>0.98894298080377097</v>
       </c>
       <c r="G32" s="4"/>
       <c r="H32">
-        <v>0.165934052581929</v>
+        <v>9.3381817414101998E-3</v>
       </c>
       <c r="I32">
-        <v>0.15627146301212599</v>
+        <v>8.7192700810209606E-2</v>
       </c>
       <c r="J32">
-        <v>0.14163041239443799</v>
-      </c>
-      <c r="K32" s="11">
+        <v>8.8994701260368805E-2</v>
+      </c>
+      <c r="K32" s="10">
         <f t="shared" si="3"/>
-        <v>0.90631014559227674</v>
-      </c>
-      <c r="L32" s="11"/>
+        <v>1.0206668727246053</v>
+      </c>
+      <c r="L32" s="10"/>
     </row>
     <row r="33" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A33">
-        <v>1000</v>
+      <c r="A33" s="4">
+        <v>60</v>
       </c>
       <c r="B33" s="5"/>
-      <c r="C33" s="2">
-        <v>0.185920101577397</v>
+      <c r="C33" s="5">
+        <v>1.7956202904139199E-2</v>
       </c>
       <c r="D33">
-        <v>0.18161105406700601</v>
+        <v>0.18310601049282599</v>
       </c>
       <c r="E33">
-        <v>0.16239985928431699</v>
-      </c>
-      <c r="F33" s="10">
+        <v>0.18135757900897301</v>
+      </c>
+      <c r="F33" s="11">
         <f t="shared" si="2"/>
-        <v>0.8942179214729904</v>
+        <v>0.99045126110744741</v>
       </c>
       <c r="G33" s="4"/>
       <c r="H33">
-        <v>0.211237572970251</v>
+        <v>1.8093633576609602E-2</v>
       </c>
       <c r="I33">
-        <v>0.197961811715788</v>
+        <v>0.168976390095402</v>
       </c>
       <c r="J33">
-        <v>0.17883044593994399</v>
-      </c>
-      <c r="K33" s="10">
+        <v>0.17402218522129201</v>
+      </c>
+      <c r="K33" s="11">
         <f t="shared" si="3"/>
-        <v>0.90335830122978089</v>
-      </c>
-      <c r="L33" s="10"/>
+        <v>1.0298609475740441</v>
+      </c>
+      <c r="L33" s="11"/>
+    </row>
+    <row r="34" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A34">
+        <v>90</v>
+      </c>
+      <c r="B34" s="5"/>
+      <c r="C34" s="2">
+        <v>2.54716677488637E-2</v>
+      </c>
+      <c r="D34">
+        <v>0.27052609093888302</v>
+      </c>
+      <c r="E34">
+        <v>0.27828767586518899</v>
+      </c>
+      <c r="F34" s="10">
+        <f t="shared" si="2"/>
+        <v>1.0286907074262921</v>
+      </c>
+      <c r="G34" s="4"/>
+      <c r="H34">
+        <v>2.63480432958439E-2</v>
+      </c>
+      <c r="I34">
+        <v>0.25226765578979399</v>
+      </c>
+      <c r="J34">
+        <v>0.27028735246822</v>
+      </c>
+      <c r="K34" s="10">
+        <f t="shared" si="3"/>
+        <v>1.0714308642620487</v>
+      </c>
+      <c r="L34" s="10"/>
+    </row>
+    <row r="35" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A35" s="4">
+        <v>100</v>
+      </c>
+      <c r="B35" s="5"/>
+      <c r="C35" s="2"/>
+      <c r="D35">
+        <v>0.29782820153673201</v>
+      </c>
+      <c r="E35">
+        <v>0.31219673881320298</v>
+      </c>
+      <c r="F35" s="10"/>
+      <c r="G35" s="4"/>
+      <c r="I35">
+        <v>0.27710332040764002</v>
+      </c>
+      <c r="J35">
+        <v>0.29733056001795299</v>
+      </c>
+      <c r="K35" s="10"/>
+      <c r="L35" s="10"/>
+    </row>
+    <row r="36" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A36" s="4">
+        <v>120</v>
+      </c>
+      <c r="B36" s="5"/>
+      <c r="C36" s="5">
+        <v>3.2417642839879697E-2</v>
+      </c>
+      <c r="D36">
+        <v>0.35933558625490702</v>
+      </c>
+      <c r="E36">
+        <v>0.36327933121591299</v>
+      </c>
+      <c r="F36" s="11">
+        <f t="shared" si="2"/>
+        <v>1.0109751026946947</v>
+      </c>
+      <c r="G36" s="4"/>
+      <c r="H36">
+        <v>3.4169678168819703E-2</v>
+      </c>
+      <c r="I36">
+        <v>0.33488526020133202</v>
+      </c>
+      <c r="J36">
+        <v>0.350044087283917</v>
+      </c>
+      <c r="K36" s="11">
+        <f t="shared" si="3"/>
+        <v>1.0452657339217364</v>
+      </c>
+      <c r="L36" s="11"/>
     </row>
     <row r="37" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="C37" s="1" t="s">
-        <v>9</v>
-      </c>
+      <c r="A37">
+        <v>150</v>
+      </c>
+      <c r="B37" s="5"/>
+      <c r="C37" s="2">
+        <v>3.9055212834252402E-2</v>
+      </c>
+      <c r="D37">
+        <v>0.440983559195115</v>
+      </c>
+      <c r="E37">
+        <v>0.46369387108133497</v>
+      </c>
+      <c r="F37" s="10">
+        <f t="shared" si="2"/>
+        <v>1.0514992257935214</v>
+      </c>
+      <c r="G37" s="4"/>
+      <c r="H37">
+        <v>4.1796462699614498E-2</v>
+      </c>
+      <c r="I37">
+        <v>0.41421243624474702</v>
+      </c>
+      <c r="J37">
+        <v>0.44198494489621698</v>
+      </c>
+      <c r="K37" s="10">
+        <f t="shared" si="3"/>
+        <v>1.0670489493344424</v>
+      </c>
+      <c r="L37" s="10"/>
     </row>
     <row r="38" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="C38" s="14" t="s">
-        <v>2</v>
-      </c>
-      <c r="D38" s="14"/>
-      <c r="E38" s="15"/>
-      <c r="H38" s="2"/>
-      <c r="I38" s="2"/>
-      <c r="J38" s="2"/>
-      <c r="K38" s="2"/>
+      <c r="A38" s="4">
+        <v>250</v>
+      </c>
+      <c r="B38" s="5"/>
+      <c r="C38" s="5">
+        <v>5.8983323870902299E-2</v>
+      </c>
+      <c r="D38">
+        <v>0.69943129650860603</v>
+      </c>
+      <c r="E38">
+        <v>0.74056761334149801</v>
+      </c>
+      <c r="F38" s="11">
+        <f t="shared" si="2"/>
+        <v>1.0588139493303126</v>
+      </c>
+      <c r="G38" s="4"/>
+      <c r="H38">
+        <v>6.5796691976300697E-2</v>
+      </c>
+      <c r="I38">
+        <v>0.66184301157104197</v>
+      </c>
+      <c r="J38">
+        <v>0.70419594658632301</v>
+      </c>
+      <c r="K38" s="11">
+        <f t="shared" si="3"/>
+        <v>1.0639924185567</v>
+      </c>
+      <c r="L38" s="11"/>
     </row>
     <row r="39" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="C39" s="3" t="s">
-        <v>4</v>
-      </c>
-      <c r="D39" s="3"/>
-      <c r="E39" s="9"/>
-      <c r="F39" s="3"/>
-      <c r="H39" s="3" t="s">
-        <v>3</v>
-      </c>
-      <c r="I39" s="3"/>
-      <c r="J39" s="9"/>
-      <c r="K39" s="9"/>
+      <c r="A39">
+        <v>500</v>
+      </c>
+      <c r="B39" s="5"/>
+      <c r="C39" s="2">
+        <v>0.103595084893309</v>
+      </c>
+      <c r="D39">
+        <v>1.3176141318230901</v>
+      </c>
+      <c r="E39">
+        <v>1.4059443021665801</v>
+      </c>
+      <c r="F39" s="10">
+        <f t="shared" si="2"/>
+        <v>1.0670379652207234</v>
+      </c>
+      <c r="G39" s="4"/>
+      <c r="H39">
+        <v>0.11839645185777101</v>
+      </c>
+      <c r="I39">
+        <v>1.25292933313</v>
+      </c>
+      <c r="J39">
+        <v>1.3590454721452301</v>
+      </c>
+      <c r="K39" s="10">
+        <f t="shared" si="3"/>
+        <v>1.0846944326462025</v>
+      </c>
+      <c r="L39" s="10"/>
     </row>
     <row r="40" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A40" s="6" t="s">
-        <v>0</v>
-      </c>
-      <c r="B40" s="6"/>
-      <c r="C40" s="6" t="s">
-        <v>1</v>
-      </c>
-      <c r="D40" s="6" t="s">
-        <v>7</v>
-      </c>
-      <c r="E40" s="6" t="s">
-        <v>6</v>
-      </c>
-      <c r="F40" s="7" t="s">
-        <v>8</v>
-      </c>
-      <c r="G40" s="8"/>
-      <c r="H40" s="6" t="s">
-        <v>1</v>
-      </c>
-      <c r="I40" s="6" t="s">
-        <v>7</v>
-      </c>
-      <c r="J40" s="6" t="s">
-        <v>6</v>
-      </c>
-      <c r="K40" s="7" t="s">
-        <v>8</v>
-      </c>
+      <c r="A40" s="4">
+        <v>750</v>
+      </c>
+      <c r="B40" s="5"/>
+      <c r="C40" s="5">
+        <v>0.14519436153500101</v>
+      </c>
+      <c r="D40">
+        <v>1.9175894049158899</v>
+      </c>
+      <c r="E40">
+        <v>2.0750333201713098</v>
+      </c>
+      <c r="F40" s="11">
+        <f t="shared" si="2"/>
+        <v>1.0821051236786146</v>
+      </c>
+      <c r="G40" s="4"/>
+      <c r="H40">
+        <v>0.165934052581929</v>
+      </c>
+      <c r="I40">
+        <v>1.8041504774598101</v>
+      </c>
+      <c r="J40">
+        <v>1.9766773113</v>
+      </c>
+      <c r="K40" s="11">
+        <f t="shared" si="3"/>
+        <v>1.0956277405879706</v>
+      </c>
+      <c r="L40" s="11"/>
     </row>
     <row r="41" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A41">
-        <v>0.1</v>
+        <v>1000</v>
       </c>
       <c r="B41" s="5"/>
-      <c r="C41">
-        <v>1.38755773111088</v>
+      <c r="C41" s="2">
+        <v>0.185920101577397</v>
       </c>
       <c r="D41">
-        <v>1.3354353849754901</v>
+        <v>2.4565650146404598</v>
       </c>
       <c r="E41">
-        <v>1.33571066860882</v>
+        <v>2.6505145134263399</v>
       </c>
       <c r="F41" s="10">
-        <f>E41/D41</f>
-        <v>1.0002061377408649</v>
+        <f t="shared" si="2"/>
+        <v>1.0789515024556622</v>
       </c>
       <c r="G41" s="4"/>
+      <c r="H41">
+        <v>0.211237572970251</v>
+      </c>
       <c r="I41">
-        <v>1.3355902411931799</v>
+        <v>2.3142913460731198</v>
       </c>
       <c r="J41">
-        <v>1.33570664006712</v>
+        <v>2.4780340620747099</v>
       </c>
       <c r="K41" s="10">
-        <f>J41/I41</f>
-        <v>1.0000871516355467</v>
-      </c>
-    </row>
-    <row r="42" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A42" s="4">
-        <v>15</v>
-      </c>
-      <c r="B42" s="5"/>
-      <c r="C42">
-        <v>1.38409520401011</v>
-      </c>
-      <c r="D42">
-        <v>1.3305745989353699</v>
-      </c>
-      <c r="E42">
-        <v>1.3291243406104201</v>
-      </c>
-      <c r="F42" s="11">
-        <f t="shared" ref="F42:F51" si="4">E42/D42</f>
-        <v>0.99891005109663888</v>
-      </c>
-      <c r="G42" s="4"/>
-      <c r="H42" s="4"/>
-      <c r="I42">
-        <v>1.3283272840070699</v>
-      </c>
-      <c r="J42">
-        <v>1.32707241565139</v>
-      </c>
-      <c r="K42" s="11">
-        <f t="shared" ref="K42:K51" si="5">J42/I42</f>
-        <v>0.99905530182900826</v>
-      </c>
-    </row>
-    <row r="43" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A43">
-        <v>30</v>
-      </c>
-      <c r="B43" s="5"/>
-      <c r="C43">
-        <v>1.3811622398640599</v>
-      </c>
-      <c r="D43">
-        <v>1.3310144038562199</v>
-      </c>
-      <c r="E43">
-        <v>1.3285615218559801</v>
-      </c>
-      <c r="F43" s="10">
-        <f t="shared" si="4"/>
-        <v>0.99815713339154455</v>
-      </c>
-      <c r="G43" s="4"/>
-      <c r="I43">
-        <v>1.32510611680532</v>
-      </c>
-      <c r="J43">
-        <v>1.3232823680411001</v>
-      </c>
-      <c r="K43" s="10">
-        <f t="shared" si="5"/>
-        <v>0.9986236960639675</v>
-      </c>
-    </row>
-    <row r="44" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A44" s="4">
-        <v>60</v>
-      </c>
-      <c r="B44" s="5"/>
-      <c r="C44">
-        <v>1.37486493369789</v>
-      </c>
-      <c r="D44">
-        <v>1.32588118290715</v>
-      </c>
-      <c r="E44">
-        <v>1.3260681746726899</v>
-      </c>
-      <c r="F44" s="11">
-        <f t="shared" si="4"/>
-        <v>1.0001410320682957</v>
-      </c>
-      <c r="G44" s="4"/>
-      <c r="H44" s="4"/>
-      <c r="I44">
-        <v>1.3187223856414001</v>
-      </c>
-      <c r="J44">
-        <v>1.31770759949175</v>
-      </c>
-      <c r="K44" s="11">
-        <f t="shared" si="5"/>
-        <v>0.99923047780131791</v>
-      </c>
+        <f t="shared" si="3"/>
+        <v>1.0707528532565391</v>
+      </c>
+      <c r="L41" s="10"/>
     </row>
     <row r="45" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A45">
-        <v>90</v>
-      </c>
-      <c r="B45" s="5"/>
-      <c r="C45">
-        <v>1.36350384779266</v>
-      </c>
-      <c r="D45">
-        <v>1.3250331310758601</v>
-      </c>
-      <c r="E45">
-        <v>1.32283704671966</v>
-      </c>
-      <c r="F45" s="10">
-        <f t="shared" si="4"/>
-        <v>0.99834261928649515</v>
-      </c>
-      <c r="G45" s="4"/>
-      <c r="I45">
-        <v>1.3124798292895099</v>
-      </c>
-      <c r="J45">
-        <v>1.3112535491322701</v>
-      </c>
-      <c r="K45" s="10">
-        <f t="shared" si="5"/>
-        <v>0.99906567694994319</v>
+      <c r="C45" s="1" t="s">
+        <v>9</v>
       </c>
     </row>
     <row r="46" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A46" s="4">
-        <v>120</v>
-      </c>
-      <c r="B46" s="5"/>
-      <c r="C46">
-        <v>1.3571706170428599</v>
-      </c>
-      <c r="D46">
-        <v>1.3186752377537301</v>
-      </c>
-      <c r="E46">
-        <v>1.31925522687803</v>
-      </c>
-      <c r="F46" s="11">
-        <f t="shared" si="4"/>
-        <v>1.000439827114133</v>
-      </c>
-      <c r="G46" s="4"/>
-      <c r="H46" s="4"/>
-      <c r="I46">
-        <v>1.3033297752905399</v>
-      </c>
-      <c r="J46">
-        <v>1.3019564075099299</v>
-      </c>
-      <c r="K46" s="11">
-        <f t="shared" si="5"/>
-        <v>0.99894626225330896</v>
-      </c>
+      <c r="C46" s="14" t="s">
+        <v>2</v>
+      </c>
+      <c r="D46" s="14"/>
+      <c r="E46" s="15"/>
+      <c r="H46" s="2"/>
+      <c r="I46" s="2"/>
+      <c r="J46" s="2"/>
+      <c r="K46" s="2"/>
     </row>
     <row r="47" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A47">
-        <v>150</v>
-      </c>
-      <c r="B47" s="5"/>
-      <c r="C47">
-        <v>1.35109721915133</v>
-      </c>
-      <c r="D47">
-        <v>1.3162252475838401</v>
-      </c>
-      <c r="E47">
-        <v>1.3162028531863199</v>
-      </c>
-      <c r="F47" s="10">
-        <f t="shared" si="4"/>
-        <v>0.99998298589275558</v>
-      </c>
-      <c r="G47" s="4"/>
-      <c r="I47">
-        <v>1.29663015170481</v>
-      </c>
-      <c r="J47">
-        <v>1.2969552292914901</v>
-      </c>
-      <c r="K47" s="10">
-        <f t="shared" si="5"/>
-        <v>1.0002507095691495</v>
-      </c>
+      <c r="C47" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="D47" s="3"/>
+      <c r="E47" s="9"/>
+      <c r="F47" s="3"/>
+      <c r="H47" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="I47" s="3"/>
+      <c r="J47" s="9"/>
+      <c r="K47" s="9"/>
     </row>
     <row r="48" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A48" s="4">
-        <v>250</v>
-      </c>
-      <c r="B48" s="5"/>
-      <c r="C48">
-        <v>1.32844051248484</v>
-      </c>
-      <c r="D48">
-        <v>1.30260068538983</v>
-      </c>
-      <c r="E48">
-        <v>1.3066950650451801</v>
-      </c>
-      <c r="F48" s="11">
-        <f t="shared" si="4"/>
-        <v>1.0031432346852518</v>
-      </c>
-      <c r="G48" s="4"/>
-      <c r="H48" s="4"/>
-      <c r="I48">
-        <v>1.2708609670523101</v>
-      </c>
-      <c r="J48">
-        <v>1.27351639583336</v>
-      </c>
-      <c r="K48" s="11">
-        <f t="shared" si="5"/>
-        <v>1.0020894722946829</v>
+      <c r="A48" s="6" t="s">
+        <v>0</v>
+      </c>
+      <c r="B48" s="6"/>
+      <c r="C48" s="6" t="s">
+        <v>1</v>
+      </c>
+      <c r="D48" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="E48" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="F48" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="G48" s="8"/>
+      <c r="H48" s="6" t="s">
+        <v>1</v>
+      </c>
+      <c r="I48" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="J48" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="K48" s="7" t="s">
+        <v>8</v>
       </c>
     </row>
     <row r="49" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A49">
-        <v>500</v>
+        <v>0.1</v>
       </c>
       <c r="B49" s="5"/>
       <c r="C49">
-        <v>1.26939305918802</v>
+        <v>1.38755773111088</v>
       </c>
       <c r="D49">
-        <v>1.26652819252339</v>
+        <v>1.3354353849754901</v>
       </c>
       <c r="E49">
-        <v>1.2763205188269799</v>
+        <v>1.33571066860882</v>
       </c>
       <c r="F49" s="10">
-        <f t="shared" si="4"/>
-        <v>1.0077316291586689</v>
+        <f>E49/D49</f>
+        <v>1.0002061377408649</v>
       </c>
       <c r="G49" s="4"/>
       <c r="I49">
-        <v>1.2073775660257999</v>
+        <v>1.3355902411931799</v>
       </c>
       <c r="J49">
-        <v>1.2155197343022801</v>
+        <v>1.33570664006712</v>
       </c>
       <c r="K49" s="10">
-        <f t="shared" si="5"/>
-        <v>1.0067436802749954</v>
+        <f>J49/I49</f>
+        <v>1.0000871516355467</v>
       </c>
     </row>
     <row r="50" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A50" s="4">
-        <v>750</v>
+        <v>15</v>
       </c>
       <c r="B50" s="5"/>
       <c r="C50">
-        <v>1.2146497361047901</v>
+        <v>1.38409520401011</v>
       </c>
       <c r="D50">
-        <v>1.2257285387942201</v>
+        <v>1.3305745989353699</v>
       </c>
       <c r="E50">
-        <v>1.2402498141564899</v>
+        <v>1.3291243406104201</v>
       </c>
       <c r="F50" s="11">
-        <f t="shared" si="4"/>
-        <v>1.0118470565893447</v>
+        <f t="shared" ref="F50:F59" si="4">E50/D50</f>
+        <v>0.99891005109663888</v>
       </c>
       <c r="G50" s="4"/>
       <c r="H50" s="4"/>
       <c r="I50">
-        <v>1.1403490012176101</v>
+        <v>1.3283272840070699</v>
       </c>
       <c r="J50">
-        <v>1.15185236456864</v>
+        <v>1.32707241565139</v>
       </c>
       <c r="K50" s="11">
-        <f t="shared" si="5"/>
-        <v>1.0100875813796892</v>
+        <f t="shared" ref="K50:K59" si="5">J50/I50</f>
+        <v>0.99905530182900826</v>
       </c>
     </row>
     <row r="51" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A51">
-        <v>1000</v>
+        <v>30</v>
       </c>
       <c r="B51" s="5"/>
       <c r="C51">
-        <v>1.1436421352186501</v>
+        <v>1.3811622398640599</v>
       </c>
       <c r="D51">
-        <v>1.1781818408587099</v>
+        <v>1.3310144038562199</v>
       </c>
       <c r="E51">
-        <v>1.19775360779693</v>
+        <v>1.3285615218559801</v>
       </c>
       <c r="F51" s="10">
         <f t="shared" si="4"/>
-        <v>1.0166118389025205</v>
+        <v>0.99815713339154455</v>
       </c>
       <c r="G51" s="4"/>
       <c r="I51">
-        <v>1.072078850564</v>
+        <v>1.32510611680532</v>
       </c>
       <c r="J51">
-        <v>1.0876143945201899</v>
+        <v>1.3232823680411001</v>
       </c>
       <c r="K51" s="10">
         <f t="shared" si="5"/>
-        <v>1.0144910460158942</v>
+        <v>0.9986236960639675</v>
+      </c>
+    </row>
+    <row r="52" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A52" s="4">
+        <v>60</v>
+      </c>
+      <c r="B52" s="5"/>
+      <c r="C52">
+        <v>1.37486493369789</v>
+      </c>
+      <c r="D52">
+        <v>1.32588118290715</v>
+      </c>
+      <c r="E52">
+        <v>1.3260681746726899</v>
+      </c>
+      <c r="F52" s="11">
+        <f t="shared" si="4"/>
+        <v>1.0001410320682957</v>
+      </c>
+      <c r="G52" s="4"/>
+      <c r="H52" s="4"/>
+      <c r="I52">
+        <v>1.3187223856414001</v>
+      </c>
+      <c r="J52">
+        <v>1.31770759949175</v>
+      </c>
+      <c r="K52" s="11">
+        <f t="shared" si="5"/>
+        <v>0.99923047780131791</v>
+      </c>
+    </row>
+    <row r="53" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A53">
+        <v>90</v>
+      </c>
+      <c r="B53" s="5"/>
+      <c r="C53">
+        <v>1.36350384779266</v>
+      </c>
+      <c r="D53">
+        <v>1.3250331310758601</v>
+      </c>
+      <c r="E53">
+        <v>1.32283704671966</v>
+      </c>
+      <c r="F53" s="10">
+        <f t="shared" si="4"/>
+        <v>0.99834261928649515</v>
+      </c>
+      <c r="G53" s="4"/>
+      <c r="I53">
+        <v>1.3124798292895099</v>
+      </c>
+      <c r="J53">
+        <v>1.3112535491322701</v>
+      </c>
+      <c r="K53" s="10">
+        <f t="shared" si="5"/>
+        <v>0.99906567694994319</v>
+      </c>
+    </row>
+    <row r="54" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A54" s="4">
+        <v>120</v>
+      </c>
+      <c r="B54" s="5"/>
+      <c r="C54">
+        <v>1.3571706170428599</v>
+      </c>
+      <c r="D54">
+        <v>1.3186752377537301</v>
+      </c>
+      <c r="E54">
+        <v>1.31925522687803</v>
+      </c>
+      <c r="F54" s="11">
+        <f t="shared" si="4"/>
+        <v>1.000439827114133</v>
+      </c>
+      <c r="G54" s="4"/>
+      <c r="H54" s="4"/>
+      <c r="I54">
+        <v>1.3033297752905399</v>
+      </c>
+      <c r="J54">
+        <v>1.3019564075099299</v>
+      </c>
+      <c r="K54" s="11">
+        <f t="shared" si="5"/>
+        <v>0.99894626225330896</v>
       </c>
     </row>
     <row r="55" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="C55" s="12" t="s">
-        <v>5</v>
-      </c>
-      <c r="D55" s="12"/>
-      <c r="E55" s="13"/>
-      <c r="F55" s="13"/>
-      <c r="H55" s="2"/>
-      <c r="I55" s="2"/>
-      <c r="J55" s="2"/>
-      <c r="K55" s="2"/>
+      <c r="A55">
+        <v>150</v>
+      </c>
+      <c r="B55" s="5"/>
+      <c r="C55">
+        <v>1.35109721915133</v>
+      </c>
+      <c r="D55">
+        <v>1.3162252475838401</v>
+      </c>
+      <c r="E55">
+        <v>1.3162028531863199</v>
+      </c>
+      <c r="F55" s="10">
+        <f t="shared" si="4"/>
+        <v>0.99998298589275558</v>
+      </c>
+      <c r="G55" s="4"/>
+      <c r="I55">
+        <v>1.29663015170481</v>
+      </c>
+      <c r="J55">
+        <v>1.2969552292914901</v>
+      </c>
+      <c r="K55" s="10">
+        <f t="shared" si="5"/>
+        <v>1.0002507095691495</v>
+      </c>
     </row>
     <row r="56" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="C56" s="3" t="s">
-        <v>4</v>
-      </c>
-      <c r="D56" s="3"/>
-      <c r="E56" s="9"/>
-      <c r="F56" s="3"/>
-      <c r="H56" s="3" t="s">
-        <v>3</v>
-      </c>
-      <c r="I56" s="3"/>
-      <c r="J56" s="9"/>
-      <c r="K56" s="9"/>
+      <c r="A56" s="4">
+        <v>250</v>
+      </c>
+      <c r="B56" s="5"/>
+      <c r="C56">
+        <v>1.32844051248484</v>
+      </c>
+      <c r="D56">
+        <v>1.30260068538983</v>
+      </c>
+      <c r="E56">
+        <v>1.3066950650451801</v>
+      </c>
+      <c r="F56" s="11">
+        <f t="shared" si="4"/>
+        <v>1.0031432346852518</v>
+      </c>
+      <c r="G56" s="4"/>
+      <c r="H56" s="4"/>
+      <c r="I56">
+        <v>1.2708609670523101</v>
+      </c>
+      <c r="J56">
+        <v>1.27351639583336</v>
+      </c>
+      <c r="K56" s="11">
+        <f t="shared" si="5"/>
+        <v>1.0020894722946829</v>
+      </c>
     </row>
     <row r="57" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A57" s="6" t="s">
-        <v>0</v>
-      </c>
-      <c r="B57" s="6"/>
-      <c r="C57" s="6" t="s">
-        <v>1</v>
-      </c>
-      <c r="D57" s="6" t="s">
-        <v>7</v>
-      </c>
-      <c r="E57" s="6" t="s">
-        <v>6</v>
-      </c>
-      <c r="F57" s="7" t="s">
-        <v>8</v>
-      </c>
-      <c r="G57" s="8"/>
-      <c r="H57" s="6" t="s">
-        <v>1</v>
-      </c>
-      <c r="I57" s="6" t="s">
-        <v>7</v>
-      </c>
-      <c r="J57" s="6" t="s">
-        <v>6</v>
-      </c>
-      <c r="K57" s="7" t="s">
-        <v>8</v>
+      <c r="A57">
+        <v>500</v>
+      </c>
+      <c r="B57" s="5"/>
+      <c r="C57">
+        <v>1.26939305918802</v>
+      </c>
+      <c r="D57">
+        <v>1.26652819252339</v>
+      </c>
+      <c r="E57">
+        <v>1.2763205188269799</v>
+      </c>
+      <c r="F57" s="10">
+        <f t="shared" si="4"/>
+        <v>1.0077316291586689</v>
+      </c>
+      <c r="G57" s="4"/>
+      <c r="I57">
+        <v>1.2073775660257999</v>
+      </c>
+      <c r="J57">
+        <v>1.2155197343022801</v>
+      </c>
+      <c r="K57" s="10">
+        <f t="shared" si="5"/>
+        <v>1.0067436802749954</v>
       </c>
     </row>
     <row r="58" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A58">
-        <v>0.1</v>
+      <c r="A58" s="4">
+        <v>750</v>
       </c>
       <c r="B58" s="5"/>
-      <c r="C58" s="2">
-        <v>2.0906018648200899E-5</v>
-      </c>
-      <c r="D58" s="2">
-        <v>2.0018619481595599E-5</v>
-      </c>
-      <c r="E58" s="2">
-        <v>2.04228717705638E-5</v>
-      </c>
-      <c r="F58" s="10">
-        <f>E58/D58</f>
-        <v>1.0201938145305103</v>
+      <c r="C58">
+        <v>1.2146497361047901</v>
+      </c>
+      <c r="D58">
+        <v>1.2257285387942201</v>
+      </c>
+      <c r="E58">
+        <v>1.2402498141564899</v>
+      </c>
+      <c r="F58" s="11">
+        <f t="shared" si="4"/>
+        <v>1.0118470565893447</v>
       </c>
       <c r="G58" s="4"/>
-      <c r="H58" s="2"/>
-      <c r="I58" s="2">
-        <v>2.4434932696069799E-5</v>
-      </c>
-      <c r="J58" s="2">
-        <v>2.5518609602937599E-5</v>
-      </c>
-      <c r="K58" s="10">
-        <f>J58/I58</f>
-        <v>1.0443494942403546</v>
+      <c r="H58" s="4"/>
+      <c r="I58">
+        <v>1.1403490012176101</v>
+      </c>
+      <c r="J58">
+        <v>1.15185236456864</v>
+      </c>
+      <c r="K58" s="11">
+        <f t="shared" si="5"/>
+        <v>1.0100875813796892</v>
       </c>
     </row>
     <row r="59" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A59" s="4">
-        <v>15</v>
+      <c r="A59">
+        <v>1000</v>
       </c>
       <c r="B59" s="5"/>
-      <c r="C59" s="2">
-        <v>3.1327203465188001E-3</v>
+      <c r="C59">
+        <v>1.1436421352186501</v>
       </c>
       <c r="D59">
-        <v>2.9966209956305001E-3</v>
+        <v>1.1781818408587099</v>
       </c>
       <c r="E59">
-        <v>3.14006419786265E-3</v>
-      </c>
-      <c r="F59" s="11">
-        <f t="shared" ref="F59:F68" si="6">E59/D59</f>
-        <v>1.0478683164942482</v>
+        <v>1.19775360779693</v>
+      </c>
+      <c r="F59" s="10">
+        <f t="shared" si="4"/>
+        <v>1.0166118389025205</v>
       </c>
       <c r="G59" s="4"/>
       <c r="I59">
-        <v>3.6561489620800698E-3</v>
+        <v>1.072078850564</v>
       </c>
       <c r="J59">
-        <v>3.8583728177792702E-3</v>
-      </c>
-      <c r="K59" s="11">
-        <f t="shared" ref="K59:K68" si="7">J59/I59</f>
-        <v>1.0553106172085915</v>
-      </c>
-    </row>
-    <row r="60" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A60">
-        <v>30</v>
-      </c>
-      <c r="B60" s="5"/>
-      <c r="C60" s="2">
-        <v>6.2691724987101998E-3</v>
-      </c>
-      <c r="D60">
-        <v>6.0122469256428399E-3</v>
-      </c>
-      <c r="E60">
-        <v>6.2971023902297701E-3</v>
-      </c>
-      <c r="F60" s="10">
-        <f t="shared" si="6"/>
-        <v>1.0473792025028101</v>
-      </c>
-      <c r="G60" s="4"/>
-      <c r="I60">
-        <v>7.3167786817070497E-3</v>
-      </c>
-      <c r="J60">
-        <v>7.7206053021012903E-3</v>
-      </c>
-      <c r="K60" s="10">
-        <f t="shared" si="7"/>
-        <v>1.0551918594181156</v>
-      </c>
-    </row>
-    <row r="61" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A61" s="4">
-        <v>60</v>
-      </c>
-      <c r="B61" s="5"/>
-      <c r="C61" s="2">
-        <v>1.2558983712415E-2</v>
-      </c>
-      <c r="D61">
-        <v>1.2036181905772299E-2</v>
-      </c>
-      <c r="E61">
-        <v>1.26843202591898E-2</v>
-      </c>
-      <c r="F61" s="11">
-        <f t="shared" si="6"/>
-        <v>1.053849165664958</v>
-      </c>
-      <c r="G61" s="4"/>
-      <c r="I61">
-        <v>1.4655010559957399E-2</v>
-      </c>
-      <c r="J61">
-        <v>1.54708347850845E-2</v>
-      </c>
-      <c r="K61" s="11">
-        <f t="shared" si="7"/>
-        <v>1.0556686207621178</v>
-      </c>
-    </row>
-    <row r="62" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A62">
-        <v>90</v>
-      </c>
-      <c r="B62" s="5"/>
-      <c r="C62" s="2">
-        <v>1.8782496824776201E-2</v>
-      </c>
-      <c r="D62">
-        <v>1.81922730031659E-2</v>
-      </c>
-      <c r="E62">
-        <v>1.9125340454343599E-2</v>
-      </c>
-      <c r="F62" s="10">
-        <f t="shared" si="6"/>
-        <v>1.051289217736306</v>
-      </c>
-      <c r="G62" s="4"/>
-      <c r="I62">
-        <v>2.20520227131588E-2</v>
-      </c>
-      <c r="J62">
-        <v>2.3279563002525702E-2</v>
-      </c>
-      <c r="K62" s="10">
-        <f t="shared" si="7"/>
-        <v>1.0556656550437167</v>
+        <v>1.0876143945201899</v>
+      </c>
+      <c r="K59" s="10">
+        <f t="shared" si="5"/>
+        <v>1.0144910460158942</v>
       </c>
     </row>
     <row r="63" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A63" s="4">
-        <v>120</v>
-      </c>
-      <c r="B63" s="5"/>
-      <c r="C63" s="2">
-        <v>2.51046376970986E-2</v>
-      </c>
-      <c r="D63">
-        <v>2.42950363565053E-2</v>
-      </c>
-      <c r="E63">
-        <v>2.55954016873969E-2</v>
-      </c>
-      <c r="F63" s="11">
-        <f t="shared" si="6"/>
-        <v>1.0535239096501048</v>
-      </c>
-      <c r="G63" s="4"/>
-      <c r="I63">
-        <v>2.9379142051595902E-2</v>
-      </c>
-      <c r="J63">
-        <v>3.0966693098777899E-2</v>
-      </c>
-      <c r="K63" s="11">
-        <f t="shared" si="7"/>
-        <v>1.0540366714723639</v>
-      </c>
+      <c r="C63" s="12" t="s">
+        <v>5</v>
+      </c>
+      <c r="D63" s="12"/>
+      <c r="E63" s="13"/>
+      <c r="F63" s="13"/>
+      <c r="H63" s="2"/>
+      <c r="I63" s="2"/>
+      <c r="J63" s="2"/>
+      <c r="K63" s="2"/>
     </row>
     <row r="64" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A64">
-        <v>150</v>
-      </c>
-      <c r="B64" s="5"/>
-      <c r="C64" s="2">
-        <v>3.1476119846668899E-2</v>
-      </c>
-      <c r="D64">
-        <v>3.0568379602756501E-2</v>
-      </c>
-      <c r="E64">
-        <v>3.2160454077141201E-2</v>
-      </c>
-      <c r="F64" s="10">
-        <f t="shared" si="6"/>
-        <v>1.0520823967470339</v>
-      </c>
-      <c r="G64" s="4"/>
-      <c r="I64">
-        <v>3.6804448452257998E-2</v>
-      </c>
-      <c r="J64">
-        <v>3.8844686371276298E-2</v>
-      </c>
-      <c r="K64" s="10">
-        <f t="shared" si="7"/>
-        <v>1.0554345467685748</v>
-      </c>
+      <c r="C64" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="D64" s="3"/>
+      <c r="E64" s="9"/>
+      <c r="F64" s="3"/>
+      <c r="H64" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="I64" s="3"/>
+      <c r="J64" s="9"/>
+      <c r="K64" s="9"/>
     </row>
     <row r="65" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A65" s="4">
-        <v>250</v>
-      </c>
-      <c r="B65" s="5"/>
-      <c r="C65" s="2">
-        <v>5.2878603388737497E-2</v>
-      </c>
-      <c r="D65">
-        <v>5.1688372196524002E-2</v>
-      </c>
-      <c r="E65">
-        <v>5.4514904682317102E-2</v>
-      </c>
-      <c r="F65" s="11">
-        <f t="shared" si="6"/>
-        <v>1.0546841071923558</v>
-      </c>
-      <c r="G65" s="4"/>
-      <c r="I65">
-        <v>6.1567552933483601E-2</v>
-      </c>
-      <c r="J65">
-        <v>6.4958585716827305E-2</v>
-      </c>
-      <c r="K65" s="11">
-        <f t="shared" si="7"/>
-        <v>1.0550782453057264</v>
+      <c r="A65" s="6" t="s">
+        <v>0</v>
+      </c>
+      <c r="B65" s="6"/>
+      <c r="C65" s="6" t="s">
+        <v>1</v>
+      </c>
+      <c r="D65" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="E65" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="F65" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="G65" s="8"/>
+      <c r="H65" s="6" t="s">
+        <v>1</v>
+      </c>
+      <c r="I65" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="J65" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="K65" s="7" t="s">
+        <v>8</v>
       </c>
     </row>
     <row r="66" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A66">
-        <v>500</v>
+        <v>0.1</v>
       </c>
       <c r="B66" s="5"/>
       <c r="C66" s="2">
-        <v>0.107716927588289</v>
-      </c>
-      <c r="D66">
-        <v>0.107312205249392</v>
-      </c>
-      <c r="E66">
-        <v>0.11284726504879</v>
+        <v>2.0906018648200899E-5</v>
+      </c>
+      <c r="D66" s="2">
+        <v>2.0018619481595599E-5</v>
+      </c>
+      <c r="E66" s="2">
+        <v>2.04228717705638E-5</v>
       </c>
       <c r="F66" s="10">
-        <f t="shared" si="6"/>
-        <v>1.0515790332193304</v>
+        <f>E66/D66</f>
+        <v>1.0201938145305103</v>
       </c>
       <c r="G66" s="4"/>
-      <c r="I66">
-        <v>0.124585487877085</v>
-      </c>
-      <c r="J66">
-        <v>0.13088073929294</v>
+      <c r="H66" s="2"/>
+      <c r="I66" s="2">
+        <v>2.4434932696069799E-5</v>
+      </c>
+      <c r="J66" s="2">
+        <v>2.5518609602937599E-5</v>
       </c>
       <c r="K66" s="10">
-        <f t="shared" si="7"/>
-        <v>1.0505295722890764</v>
+        <f>J66/I66</f>
+        <v>1.0443494942403546</v>
       </c>
     </row>
     <row r="67" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A67" s="4">
-        <v>750</v>
+        <v>15</v>
       </c>
       <c r="B67" s="5"/>
       <c r="C67" s="2">
-        <v>0.16515386445267599</v>
+        <v>3.1327203465188001E-3</v>
       </c>
       <c r="D67">
-        <v>0.166593474221475</v>
+        <v>2.9966209956305001E-3</v>
       </c>
       <c r="E67">
-        <v>0.17437302973664801</v>
+        <v>3.14006419786265E-3</v>
       </c>
       <c r="F67" s="11">
-        <f t="shared" si="6"/>
-        <v>1.0466978406658991</v>
+        <f t="shared" ref="F67:F76" si="6">E67/D67</f>
+        <v>1.0478683164942482</v>
       </c>
       <c r="G67" s="4"/>
       <c r="I67">
-        <v>0.188315720076114</v>
+        <v>3.6561489620800698E-3</v>
       </c>
       <c r="J67">
-        <v>0.19671890522285099</v>
+        <v>3.8583728177792702E-3</v>
       </c>
       <c r="K67" s="11">
-        <f t="shared" si="7"/>
-        <v>1.0446228554012409</v>
+        <f t="shared" ref="K67:K76" si="7">J67/I67</f>
+        <v>1.0553106172085915</v>
       </c>
     </row>
     <row r="68" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A68">
-        <v>1000</v>
+        <v>30</v>
       </c>
       <c r="B68" s="5"/>
       <c r="C68" s="2">
-        <v>0.22114304090137801</v>
+        <v>6.2691724987101998E-3</v>
       </c>
       <c r="D68">
-        <v>0.22843742858074301</v>
+        <v>6.0122469256428399E-3</v>
       </c>
       <c r="E68">
-        <v>0.23785710518924499</v>
+        <v>6.2971023902297701E-3</v>
       </c>
       <c r="F68" s="10">
         <f t="shared" si="6"/>
-        <v>1.0412352593312988</v>
+        <v>1.0473792025028101</v>
       </c>
       <c r="G68" s="4"/>
       <c r="I68">
+        <v>7.3167786817070497E-3</v>
+      </c>
+      <c r="J68">
+        <v>7.7206053021012903E-3</v>
+      </c>
+      <c r="K68" s="10">
+        <f t="shared" si="7"/>
+        <v>1.0551918594181156</v>
+      </c>
+    </row>
+    <row r="69" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A69" s="4">
+        <v>60</v>
+      </c>
+      <c r="B69" s="5"/>
+      <c r="C69" s="2">
+        <v>1.2558983712415E-2</v>
+      </c>
+      <c r="D69">
+        <v>1.2036181905772299E-2</v>
+      </c>
+      <c r="E69">
+        <v>1.26843202591898E-2</v>
+      </c>
+      <c r="F69" s="11">
+        <f t="shared" si="6"/>
+        <v>1.053849165664958</v>
+      </c>
+      <c r="G69" s="4"/>
+      <c r="I69">
+        <v>1.4655010559957399E-2</v>
+      </c>
+      <c r="J69">
+        <v>1.54708347850845E-2</v>
+      </c>
+      <c r="K69" s="11">
+        <f t="shared" si="7"/>
+        <v>1.0556686207621178</v>
+      </c>
+    </row>
+    <row r="70" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A70">
+        <v>90</v>
+      </c>
+      <c r="B70" s="5"/>
+      <c r="C70" s="2">
+        <v>1.8782496824776201E-2</v>
+      </c>
+      <c r="D70">
+        <v>1.81922730031659E-2</v>
+      </c>
+      <c r="E70">
+        <v>1.9125340454343599E-2</v>
+      </c>
+      <c r="F70" s="10">
+        <f t="shared" si="6"/>
+        <v>1.051289217736306</v>
+      </c>
+      <c r="G70" s="4"/>
+      <c r="I70">
+        <v>2.20520227131588E-2</v>
+      </c>
+      <c r="J70">
+        <v>2.3279563002525702E-2</v>
+      </c>
+      <c r="K70" s="10">
+        <f t="shared" si="7"/>
+        <v>1.0556656550437167</v>
+      </c>
+    </row>
+    <row r="71" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A71" s="4">
+        <v>120</v>
+      </c>
+      <c r="B71" s="5"/>
+      <c r="C71" s="2">
+        <v>2.51046376970986E-2</v>
+      </c>
+      <c r="D71">
+        <v>2.42950363565053E-2</v>
+      </c>
+      <c r="E71">
+        <v>2.55954016873969E-2</v>
+      </c>
+      <c r="F71" s="11">
+        <f t="shared" si="6"/>
+        <v>1.0535239096501048</v>
+      </c>
+      <c r="G71" s="4"/>
+      <c r="I71">
+        <v>2.9379142051595902E-2</v>
+      </c>
+      <c r="J71">
+        <v>3.0966693098777899E-2</v>
+      </c>
+      <c r="K71" s="11">
+        <f t="shared" si="7"/>
+        <v>1.0540366714723639</v>
+      </c>
+    </row>
+    <row r="72" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A72">
+        <v>150</v>
+      </c>
+      <c r="B72" s="5"/>
+      <c r="C72" s="2">
+        <v>3.1476119846668899E-2</v>
+      </c>
+      <c r="D72">
+        <v>3.0568379602756501E-2</v>
+      </c>
+      <c r="E72">
+        <v>3.2160454077141201E-2</v>
+      </c>
+      <c r="F72" s="10">
+        <f t="shared" si="6"/>
+        <v>1.0520823967470339</v>
+      </c>
+      <c r="G72" s="4"/>
+      <c r="I72">
+        <v>3.6804448452257998E-2</v>
+      </c>
+      <c r="J72">
+        <v>3.8844686371276298E-2</v>
+      </c>
+      <c r="K72" s="10">
+        <f t="shared" si="7"/>
+        <v>1.0554345467685748</v>
+      </c>
+    </row>
+    <row r="73" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A73" s="4">
+        <v>250</v>
+      </c>
+      <c r="B73" s="5"/>
+      <c r="C73" s="2">
+        <v>5.2878603388737497E-2</v>
+      </c>
+      <c r="D73">
+        <v>5.1688372196524002E-2</v>
+      </c>
+      <c r="E73">
+        <v>5.4514904682317102E-2</v>
+      </c>
+      <c r="F73" s="11">
+        <f t="shared" si="6"/>
+        <v>1.0546841071923558</v>
+      </c>
+      <c r="G73" s="4"/>
+      <c r="I73">
+        <v>6.1567552933483601E-2</v>
+      </c>
+      <c r="J73">
+        <v>6.4958585716827305E-2</v>
+      </c>
+      <c r="K73" s="11">
+        <f t="shared" si="7"/>
+        <v>1.0550782453057264</v>
+      </c>
+    </row>
+    <row r="74" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A74">
+        <v>500</v>
+      </c>
+      <c r="B74" s="5"/>
+      <c r="C74" s="2">
+        <v>0.107716927588289</v>
+      </c>
+      <c r="D74">
+        <v>0.107312205249392</v>
+      </c>
+      <c r="E74">
+        <v>0.11284726504879</v>
+      </c>
+      <c r="F74" s="10">
+        <f t="shared" si="6"/>
+        <v>1.0515790332193304</v>
+      </c>
+      <c r="G74" s="4"/>
+      <c r="I74">
+        <v>0.124585487877085</v>
+      </c>
+      <c r="J74">
+        <v>0.13088073929294</v>
+      </c>
+      <c r="K74" s="10">
+        <f t="shared" si="7"/>
+        <v>1.0505295722890764</v>
+      </c>
+    </row>
+    <row r="75" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A75" s="4">
+        <v>750</v>
+      </c>
+      <c r="B75" s="5"/>
+      <c r="C75" s="2">
+        <v>0.16515386445267599</v>
+      </c>
+      <c r="D75">
+        <v>0.166593474221475</v>
+      </c>
+      <c r="E75">
+        <v>0.17437302973664801</v>
+      </c>
+      <c r="F75" s="11">
+        <f t="shared" si="6"/>
+        <v>1.0466978406658991</v>
+      </c>
+      <c r="G75" s="4"/>
+      <c r="I75">
+        <v>0.188315720076114</v>
+      </c>
+      <c r="J75">
+        <v>0.19671890522285099</v>
+      </c>
+      <c r="K75" s="11">
+        <f t="shared" si="7"/>
+        <v>1.0446228554012409</v>
+      </c>
+    </row>
+    <row r="76" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A76">
+        <v>1000</v>
+      </c>
+      <c r="B76" s="5"/>
+      <c r="C76" s="2">
+        <v>0.22114304090137801</v>
+      </c>
+      <c r="D76">
+        <v>0.22843742858074301</v>
+      </c>
+      <c r="E76">
+        <v>0.23785710518924499</v>
+      </c>
+      <c r="F76" s="10">
+        <f t="shared" si="6"/>
+        <v>1.0412352593312988</v>
+      </c>
+      <c r="G76" s="4"/>
+      <c r="I76">
         <v>0.25212873564071397</v>
       </c>
-      <c r="J68">
+      <c r="J76">
         <v>0.26159631710660702</v>
       </c>
-      <c r="K68" s="10">
+      <c r="K76" s="10">
         <f t="shared" si="7"/>
         <v>1.0375505847908761</v>
       </c>

</xml_diff>

<commit_message>
dcll, hcpb prisms fixed, openmc running
</commit_message>
<xml_diff>
--- a/Jupyter/Wedge/wedge_data_2026-03-25.xlsx
+++ b/Jupyter/Wedge/wedge_data_2026-03-25.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\patri\projects\emma-openmc\Jupyter\Wedge\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D92552F5-14F5-4602-8D22-687681DBA2D8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7B184866-94F8-47FB-9604-EE9CD1C46C89}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="17496" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="49" uniqueCount="10">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="61" uniqueCount="11">
   <si>
     <t>Fertile kg/m3</t>
   </si>
@@ -67,14 +67,16 @@
   <si>
     <t>DCLL-Greta</t>
   </si>
+  <si>
+    <t>FISSILE PRODUCTION RATE ERROR PROPAGATION [ RXNS/SRC-N ]</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="2">
+  <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.000000"/>
-    <numFmt numFmtId="165" formatCode="0.000000000"/>
   </numFmts>
   <fonts count="6" x14ac:knownFonts="1">
     <font>
@@ -161,7 +163,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="11" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -178,8 +180,6 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="11" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="165" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
-    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -274,7 +274,7 @@
           </c:marker>
           <c:xVal>
             <c:numRef>
-              <c:f>'Sheet 1'!$A$27:$A$41</c:f>
+              <c:f>'Sheet 1'!$A$26:$A$40</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="15"/>
@@ -328,42 +328,54 @@
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>'Sheet 1'!$F$27:$F$41</c:f>
+              <c:f>'Sheet 1'!$F$26:$F$40</c:f>
               <c:numCache>
                 <c:formatCode>0.000000</c:formatCode>
                 <c:ptCount val="15"/>
                 <c:pt idx="0">
-                  <c:v>0.90095484884115951</c:v>
+                  <c:v>0.7274775745944605</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>0.64347975683918834</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>0.49583688440425344</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>0.66859607525333198</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>0.98605362776739691</c:v>
+                  <c:v>0.73291562987349301</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>0.98894298080377097</c:v>
+                  <c:v>0.74746751893992558</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>0.99045126110744741</c:v>
+                  <c:v>0.78627670393149318</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>1.0286907074262921</c:v>
+                  <c:v>0.87619376520123537</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>0.86809490045634352</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>1.0109751026946947</c:v>
+                  <c:v>0.79255474288640204</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>1.0514992257935214</c:v>
+                  <c:v>0.90551396638088599</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>1.0588139493303126</c:v>
+                  <c:v>0.92837643974491146</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>1.0670379652207234</c:v>
+                  <c:v>0.93787715524054671</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>1.0821051236786146</c:v>
+                  <c:v>1.0174259839976012</c:v>
                 </c:pt>
                 <c:pt idx="14">
-                  <c:v>1.0789515024556622</c:v>
+                  <c:v>1.0246283267351703</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -402,7 +414,7 @@
           </c:marker>
           <c:xVal>
             <c:numRef>
-              <c:f>'Sheet 1'!$A$27:$A$41</c:f>
+              <c:f>'Sheet 1'!$A$26:$A$40</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="15"/>
@@ -456,42 +468,54 @@
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>'Sheet 1'!$K$27:$K$41</c:f>
+              <c:f>'Sheet 1'!$K$26:$K$40</c:f>
               <c:numCache>
                 <c:formatCode>0.000000</c:formatCode>
                 <c:ptCount val="15"/>
                 <c:pt idx="0">
-                  <c:v>1.0035506001332684</c:v>
+                  <c:v>0.29264705217301878</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>1.3315375295667062</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>0.8971337860952534</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>0.86727127408207016</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>1.0779572449118415</c:v>
+                  <c:v>0.96019947785672299</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>1.0206668727246053</c:v>
+                  <c:v>0.82054207267800461</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>1.0298609475740441</c:v>
+                  <c:v>0.89620098412984728</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>1.0714308642620487</c:v>
+                  <c:v>0.99789498609321658</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>0.92546657383389286</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>1.0452657339217364</c:v>
+                  <c:v>0.95340718196328889</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>1.0670489493344424</c:v>
+                  <c:v>0.94899688560909901</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>1.0639924185567</c:v>
+                  <c:v>0.9624346474925255</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>1.0846944326462025</c:v>
+                  <c:v>1.0215461604572156</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>1.0956277405879706</c:v>
+                  <c:v>1.0753115641669349</c:v>
                 </c:pt>
                 <c:pt idx="14">
-                  <c:v>1.0707528532565391</c:v>
+                  <c:v>1.0025476893384362</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -850,7 +874,7 @@
           </c:trendline>
           <c:xVal>
             <c:numRef>
-              <c:f>'Sheet 1'!$A$6:$A$20</c:f>
+              <c:f>'Sheet 1'!$A$5:$A$19</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="15"/>
@@ -904,7 +928,7 @@
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>'Sheet 1'!$F$6:$F$20</c:f>
+              <c:f>'Sheet 1'!$F$5:$F$19</c:f>
               <c:numCache>
                 <c:formatCode>0.000000</c:formatCode>
                 <c:ptCount val="15"/>
@@ -1041,7 +1065,7 @@
           </c:trendline>
           <c:xVal>
             <c:numRef>
-              <c:f>'Sheet 1'!$A$6:$A$20</c:f>
+              <c:f>'Sheet 1'!$A$5:$A$19</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="15"/>
@@ -1095,13 +1119,22 @@
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>'Sheet 1'!$K$6:$K$20</c:f>
+              <c:f>'Sheet 1'!$K$5:$K$19</c:f>
               <c:numCache>
                 <c:formatCode>0.000000</c:formatCode>
                 <c:ptCount val="15"/>
                 <c:pt idx="0">
                   <c:v>1.0124595607074192</c:v>
                 </c:pt>
+                <c:pt idx="1">
+                  <c:v>0.98955684846579572</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>0.97266576371713243</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>0.99532217045916183</c:v>
+                </c:pt>
                 <c:pt idx="4">
                   <c:v>1.0246126531897757</c:v>
                 </c:pt>
@@ -1113,6 +1146,9 @@
                 </c:pt>
                 <c:pt idx="7">
                   <c:v>1.0235838898658773</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>1.0328136474978709</c:v>
                 </c:pt>
                 <c:pt idx="9">
                   <c:v>0.99238859087523068</c:v>
@@ -1456,34 +1492,34 @@
                   <c:v>0.1</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>15</c:v>
+                  <c:v>0.5</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>30</c:v>
+                  <c:v>1</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>60</c:v>
+                  <c:v>10</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>90</c:v>
+                  <c:v>25</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>120</c:v>
+                  <c:v>50</c:v>
                 </c:pt>
                 <c:pt idx="6">
+                  <c:v>75</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>100</c:v>
+                </c:pt>
+                <c:pt idx="8">
                   <c:v>150</c:v>
                 </c:pt>
-                <c:pt idx="7">
+                <c:pt idx="9">
                   <c:v>250</c:v>
                 </c:pt>
-                <c:pt idx="8">
+                <c:pt idx="10">
                   <c:v>500</c:v>
-                </c:pt>
-                <c:pt idx="9">
-                  <c:v>750</c:v>
-                </c:pt>
-                <c:pt idx="10">
-                  <c:v>1000</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1495,37 +1531,37 @@
                 <c:formatCode>0.000000</c:formatCode>
                 <c:ptCount val="11"/>
                 <c:pt idx="0">
-                  <c:v>1.0201938145305103</c:v>
+                  <c:v>0.98141967163352228</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>1.0478683164942482</c:v>
+                  <c:v>0.92802141334950694</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>1.0473792025028101</c:v>
+                  <c:v>1.0257080460192236</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>1.053849165664958</c:v>
+                  <c:v>1.0646127665011473</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>1.051289217736306</c:v>
+                  <c:v>1.0753237074121145</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>1.0535239096501048</c:v>
+                  <c:v>1.0422360763919929</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>1.0520823967470339</c:v>
+                  <c:v>1.0978441524727602</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>1.0546841071923558</c:v>
+                  <c:v>1.0378247495664441</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>1.0515790332193304</c:v>
+                  <c:v>1.0332088675177227</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>1.0466978406658991</c:v>
+                  <c:v>1.1033275421994369</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>1.0412352593312988</c:v>
+                  <c:v>1.0613255687481478</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1779,7 +1815,7 @@
           <c:order val="0"/>
           <c:tx>
             <c:strRef>
-              <c:f>'Sheet 1'!$F$48</c:f>
+              <c:f>'Sheet 1'!$F$47</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -1812,7 +1848,7 @@
           </c:marker>
           <c:xVal>
             <c:numRef>
-              <c:f>'Sheet 1'!$A$49:$A$59</c:f>
+              <c:f>'Sheet 1'!$A$48:$A$58</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="11"/>
@@ -1820,76 +1856,76 @@
                   <c:v>0.1</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>15</c:v>
+                  <c:v>0.5</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>30</c:v>
+                  <c:v>1</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>60</c:v>
+                  <c:v>10</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>90</c:v>
+                  <c:v>25</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>120</c:v>
+                  <c:v>50</c:v>
                 </c:pt>
                 <c:pt idx="6">
+                  <c:v>75</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>100</c:v>
+                </c:pt>
+                <c:pt idx="8">
                   <c:v>150</c:v>
                 </c:pt>
-                <c:pt idx="7">
+                <c:pt idx="9">
                   <c:v>250</c:v>
                 </c:pt>
-                <c:pt idx="8">
+                <c:pt idx="10">
                   <c:v>500</c:v>
-                </c:pt>
-                <c:pt idx="9">
-                  <c:v>750</c:v>
-                </c:pt>
-                <c:pt idx="10">
-                  <c:v>1000</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>'Sheet 1'!$F$49:$F$59</c:f>
+              <c:f>'Sheet 1'!$F$48:$F$58</c:f>
               <c:numCache>
                 <c:formatCode>0.000000</c:formatCode>
                 <c:ptCount val="11"/>
                 <c:pt idx="0">
-                  <c:v>1.0002061377408649</c:v>
+                  <c:v>0.9985035371420129</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0.99891005109663888</c:v>
+                  <c:v>0.98715209394887005</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>0.99815713339154455</c:v>
+                  <c:v>0.99284501043036377</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>1.0001410320682957</c:v>
+                  <c:v>1.0204895071175968</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>0.99834261928649515</c:v>
+                  <c:v>1.0049119467662411</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>1.000439827114133</c:v>
+                  <c:v>0.99460716116426584</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>0.99998298589275558</c:v>
+                  <c:v>1.0195310334465668</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>1.0031432346852518</c:v>
+                  <c:v>0.98333502299608533</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>1.0077316291586689</c:v>
+                  <c:v>0.98631763108404502</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>1.0118470565893447</c:v>
+                  <c:v>1.0290963972436542</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>1.0166118389025205</c:v>
+                  <c:v>0.99666881879093805</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -4318,13 +4354,13 @@
     <xdr:from>
       <xdr:col>12</xdr:col>
       <xdr:colOff>132179</xdr:colOff>
-      <xdr:row>23</xdr:row>
+      <xdr:row>22</xdr:row>
       <xdr:rowOff>56857</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>19</xdr:col>
       <xdr:colOff>436979</xdr:colOff>
-      <xdr:row>42</xdr:row>
+      <xdr:row>41</xdr:row>
       <xdr:rowOff>56857</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
@@ -4360,7 +4396,7 @@
     <xdr:to>
       <xdr:col>19</xdr:col>
       <xdr:colOff>605790</xdr:colOff>
-      <xdr:row>19</xdr:row>
+      <xdr:row>18</xdr:row>
       <xdr:rowOff>99060</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
@@ -4426,7 +4462,7 @@
     <xdr:from>
       <xdr:col>11</xdr:col>
       <xdr:colOff>929640</xdr:colOff>
-      <xdr:row>45</xdr:row>
+      <xdr:row>44</xdr:row>
       <xdr:rowOff>7620</xdr:rowOff>
     </xdr:from>
     <xdr:to>
@@ -4724,7 +4760,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C22416C2-1180-4450-A3B0-0B08DD9AEC85}">
-  <dimension ref="A1:L76"/>
+  <dimension ref="A1:L95"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="12.33203125" customWidth="1"/>
@@ -4802,1415 +4838,1515 @@
       <c r="L4" s="7"/>
     </row>
     <row r="5" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A5" s="8">
-        <v>0</v>
-      </c>
-      <c r="B5" s="8"/>
-      <c r="C5" s="16">
-        <f>1.38911+0.015389</f>
-        <v>1.4044990000000002</v>
-      </c>
-      <c r="D5" s="6"/>
-      <c r="E5" s="6"/>
-      <c r="F5" s="17"/>
-      <c r="G5" s="8"/>
-      <c r="H5" s="6"/>
-      <c r="I5" s="6"/>
-      <c r="J5" s="6"/>
-      <c r="K5" s="17"/>
-      <c r="L5" s="7"/>
+      <c r="A5">
+        <v>0.1</v>
+      </c>
+      <c r="B5" s="5"/>
+      <c r="C5">
+        <v>1.4063862998066801</v>
+      </c>
+      <c r="D5">
+        <v>1.3686193553583801</v>
+      </c>
+      <c r="E5">
+        <v>1.38512260545705</v>
+      </c>
+      <c r="F5" s="10">
+        <f>E5/D5</f>
+        <v>1.0120583199660715</v>
+      </c>
+      <c r="G5" s="4"/>
+      <c r="H5">
+        <v>1.4074651112049299</v>
+      </c>
+      <c r="I5">
+        <v>1.3681177802680899</v>
+      </c>
+      <c r="J5">
+        <v>1.3851639268062399</v>
+      </c>
+      <c r="K5" s="10">
+        <f>J5/I5</f>
+        <v>1.0124595607074192</v>
+      </c>
+      <c r="L5" s="10"/>
     </row>
     <row r="6" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A6">
-        <v>0.1</v>
+        <v>0.5</v>
       </c>
       <c r="B6" s="5"/>
       <c r="C6">
-        <v>1.40420707746021</v>
+        <v>1.4065448393936499</v>
       </c>
       <c r="D6">
-        <v>1.3686193553583801</v>
+        <v>1.3922831524096599</v>
       </c>
       <c r="E6">
-        <v>1.38512260545705</v>
+        <v>1.37451308945358</v>
       </c>
       <c r="F6" s="10">
-        <f>E6/D6</f>
-        <v>1.0120583199660715</v>
+        <f t="shared" ref="F6:F19" si="0">E6/D6</f>
+        <v>0.98723674640081305</v>
       </c>
       <c r="G6" s="4"/>
       <c r="H6">
-        <v>1.4043892076542099</v>
+        <v>1.4079920998080599</v>
       </c>
       <c r="I6">
-        <v>1.3681177802680899</v>
+        <v>1.3884228746446901</v>
       </c>
       <c r="J6">
-        <v>1.3851639268062399</v>
+        <v>1.3739233641712201</v>
       </c>
       <c r="K6" s="10">
-        <f>J6/I6</f>
-        <v>1.0124595607074192</v>
+        <f t="shared" ref="K6:K19" si="1">J6/I6</f>
+        <v>0.98955684846579572</v>
       </c>
       <c r="L6" s="10"/>
     </row>
     <row r="7" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A7">
-        <v>0.5</v>
+        <v>1.5</v>
       </c>
       <c r="B7" s="5"/>
+      <c r="C7">
+        <v>1.40593053429746</v>
+      </c>
       <c r="D7">
-        <v>1.3922831524096599</v>
+        <v>1.4141178954362701</v>
       </c>
       <c r="E7">
-        <v>1.37451308945358</v>
+        <v>1.3766722209354501</v>
       </c>
       <c r="F7" s="10">
-        <f t="shared" ref="F7:F20" si="0">E7/D7</f>
-        <v>0.98723674640081305</v>
+        <f t="shared" si="0"/>
+        <v>0.97352011835670349</v>
       </c>
       <c r="G7" s="4"/>
+      <c r="H7">
+        <v>1.4079445884292401</v>
+      </c>
       <c r="I7">
-        <v>1.3884228746446901</v>
+        <v>1.4147283449213399</v>
       </c>
       <c r="J7">
-        <v>1.3739233641712201</v>
-      </c>
-      <c r="K7" s="10"/>
+        <v>1.3760578260651899</v>
+      </c>
+      <c r="K7" s="10">
+        <f t="shared" si="1"/>
+        <v>0.97266576371713243</v>
+      </c>
       <c r="L7" s="10"/>
     </row>
     <row r="8" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A8">
-        <v>1.5</v>
+        <v>10</v>
       </c>
       <c r="B8" s="5"/>
+      <c r="C8">
+        <v>1.39838837861919</v>
+      </c>
       <c r="D8">
-        <v>1.4141178954362701</v>
+        <v>1.4052374449883001</v>
       </c>
       <c r="E8">
-        <v>1.3766722209354501</v>
+        <v>1.38656109713547</v>
       </c>
       <c r="F8" s="10">
         <f t="shared" si="0"/>
-        <v>0.97352011835670349</v>
+        <v>0.98670947182667379</v>
       </c>
       <c r="G8" s="4"/>
+      <c r="H8">
+        <v>1.4018754625880101</v>
+      </c>
       <c r="I8">
-        <v>1.4147283449213399</v>
+        <v>1.3952787310994501</v>
       </c>
       <c r="J8">
-        <v>1.3760578260651899</v>
-      </c>
-      <c r="K8" s="10"/>
+        <v>1.3887518550334099</v>
+      </c>
+      <c r="K8" s="10">
+        <f t="shared" si="1"/>
+        <v>0.99532217045916183</v>
+      </c>
       <c r="L8" s="10"/>
     </row>
-    <row r="9" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:12" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A9">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="B9" s="5"/>
+      <c r="C9">
+        <v>1.39742877901721</v>
+      </c>
       <c r="D9">
-        <v>1.4052374449883001</v>
+        <v>1.3588321367490299</v>
       </c>
       <c r="E9">
-        <v>1.38656109713547</v>
+        <v>1.3960885502131399</v>
       </c>
       <c r="F9" s="10">
         <f t="shared" si="0"/>
-        <v>0.98670947182667379</v>
-      </c>
-      <c r="G9" s="4"/>
+        <v>1.0274179661023068</v>
+      </c>
+      <c r="H9">
+        <v>1.4018991482118599</v>
+      </c>
       <c r="I9">
-        <v>1.3952787310994501</v>
+        <v>1.36086238814935</v>
       </c>
       <c r="J9">
-        <v>1.3887518550334099</v>
-      </c>
-      <c r="K9" s="10"/>
-      <c r="L9" s="10"/>
-    </row>
-    <row r="10" spans="1:12" s="4" customFormat="1" x14ac:dyDescent="0.3">
+        <v>1.3943568221478799</v>
+      </c>
+      <c r="K9" s="10">
+        <f t="shared" si="1"/>
+        <v>1.0246126531897757</v>
+      </c>
+      <c r="L9" s="11"/>
+    </row>
+    <row r="10" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A10">
-        <v>15</v>
+        <v>30</v>
       </c>
       <c r="B10" s="5"/>
-      <c r="C10" s="4">
-        <v>1.3978225806626601</v>
+      <c r="C10">
+        <v>1.3977734656963801</v>
       </c>
       <c r="D10">
-        <v>1.3588321367490299</v>
+        <v>1.38084479180245</v>
       </c>
       <c r="E10">
-        <v>1.3960885502131399</v>
+        <v>1.3802674426896999</v>
       </c>
       <c r="F10" s="10">
         <f t="shared" si="0"/>
-        <v>1.0274179661023068</v>
-      </c>
-      <c r="H10" s="4">
-        <v>1.3977474767840601</v>
+        <v>0.9995818870330847</v>
+      </c>
+      <c r="G10" s="4"/>
+      <c r="H10">
+        <v>1.3914317207496001</v>
       </c>
       <c r="I10">
-        <v>1.36086238814935</v>
+        <v>1.3852911212816701</v>
       </c>
       <c r="J10">
-        <v>1.3943568221478799</v>
-      </c>
-      <c r="K10" s="11">
-        <f t="shared" ref="K10:K20" si="1">J10/I10</f>
-        <v>1.0246126531897757</v>
-      </c>
-      <c r="L10" s="11"/>
-    </row>
-    <row r="11" spans="1:12" x14ac:dyDescent="0.3">
+        <v>1.3731450592762</v>
+      </c>
+      <c r="K10" s="10">
+        <f t="shared" si="1"/>
+        <v>0.99123212311197628</v>
+      </c>
+      <c r="L10" s="10"/>
+    </row>
+    <row r="11" spans="1:12" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A11">
-        <v>30</v>
+        <v>60</v>
       </c>
       <c r="B11" s="5"/>
       <c r="C11">
-        <v>1.3935791421766499</v>
+        <v>1.39314164652525</v>
       </c>
       <c r="D11">
-        <v>1.38084479180245</v>
+        <v>1.35391575819657</v>
       </c>
       <c r="E11">
-        <v>1.3802674426896999</v>
+        <v>1.35872734366118</v>
       </c>
       <c r="F11" s="10">
         <f t="shared" si="0"/>
-        <v>0.9995818870330847</v>
-      </c>
-      <c r="G11" s="4"/>
+        <v>1.0035538292803527</v>
+      </c>
       <c r="H11">
-        <v>1.3923333952149399</v>
+        <v>1.3881975250755401</v>
       </c>
       <c r="I11">
-        <v>1.3852911212816701</v>
+        <v>1.3558315843768101</v>
       </c>
       <c r="J11">
-        <v>1.3731450592762</v>
+        <v>1.35851656917782</v>
       </c>
       <c r="K11" s="10">
         <f t="shared" si="1"/>
-        <v>0.99123212311197628</v>
-      </c>
-      <c r="L11" s="10"/>
-    </row>
-    <row r="12" spans="1:12" s="4" customFormat="1" x14ac:dyDescent="0.3">
+        <v>1.0019803232436455</v>
+      </c>
+      <c r="L11" s="11"/>
+    </row>
+    <row r="12" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A12">
-        <v>60</v>
+        <v>90</v>
       </c>
       <c r="B12" s="5"/>
-      <c r="C12" s="4">
-        <v>1.38536063754419</v>
+      <c r="C12">
+        <v>1.3818447189929399</v>
       </c>
       <c r="D12">
-        <v>1.35391575819657</v>
+        <v>1.3540665504448699</v>
       </c>
       <c r="E12">
-        <v>1.35872734366118</v>
+        <v>1.3846270062289301</v>
       </c>
       <c r="F12" s="10">
         <f t="shared" si="0"/>
-        <v>1.0035538292803527</v>
-      </c>
-      <c r="H12" s="4">
-        <v>1.3811147115786999</v>
+        <v>1.0225693897940391</v>
+      </c>
+      <c r="G12" s="4"/>
+      <c r="H12">
+        <v>1.3733638983322201</v>
       </c>
       <c r="I12">
-        <v>1.3558315843768101</v>
+        <v>1.34423803647162</v>
       </c>
       <c r="J12">
-        <v>1.35851656917782</v>
-      </c>
-      <c r="K12" s="11">
+        <v>1.37594039827729</v>
+      </c>
+      <c r="K12" s="10">
         <f t="shared" si="1"/>
-        <v>1.0019803232436455</v>
-      </c>
-      <c r="L12" s="11"/>
+        <v>1.0235838898658773</v>
+      </c>
+      <c r="L12" s="10"/>
     </row>
     <row r="13" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A13">
-        <v>90</v>
+        <v>100</v>
       </c>
       <c r="B13" s="5"/>
       <c r="C13">
-        <v>1.37856347972413</v>
+        <v>1.37950613179578</v>
       </c>
       <c r="D13">
-        <v>1.3540665504448699</v>
+        <v>1.3565730983264299</v>
       </c>
       <c r="E13">
-        <v>1.3846270062289301</v>
+        <v>1.37473157938041</v>
       </c>
       <c r="F13" s="10">
         <f t="shared" si="0"/>
-        <v>1.0225693897940391</v>
+        <v>1.0133855529616367</v>
       </c>
       <c r="G13" s="4"/>
       <c r="H13">
-        <v>1.3698685473168299</v>
+        <v>1.3697423426526301</v>
       </c>
       <c r="I13">
-        <v>1.34423803647162</v>
+        <v>1.3294388930292</v>
       </c>
       <c r="J13">
-        <v>1.37594039827729</v>
+        <v>1.3730626322350199</v>
       </c>
       <c r="K13" s="10">
         <f t="shared" si="1"/>
-        <v>1.0235838898658773</v>
+        <v>1.0328136474978709</v>
       </c>
       <c r="L13" s="10"/>
     </row>
-    <row r="14" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:12" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A14">
-        <v>100</v>
+        <v>120</v>
       </c>
       <c r="B14" s="5"/>
+      <c r="C14">
+        <v>1.37505741757767</v>
+      </c>
       <c r="D14">
-        <v>1.3565730983264299</v>
+        <v>1.34077916991197</v>
       </c>
       <c r="E14">
-        <v>1.37473157938041</v>
+        <v>1.3634284951011899</v>
       </c>
       <c r="F14" s="10">
         <f t="shared" si="0"/>
-        <v>1.0133855529616367</v>
-      </c>
-      <c r="G14" s="4"/>
+        <v>1.0168926589087053</v>
+      </c>
+      <c r="H14">
+        <v>1.36267435359262</v>
+      </c>
       <c r="I14">
-        <v>1.3294388930292</v>
+        <v>1.35581073898229</v>
       </c>
       <c r="J14">
-        <v>1.3730626322350199</v>
-      </c>
-      <c r="K14" s="10"/>
-      <c r="L14" s="10"/>
-    </row>
-    <row r="15" spans="1:12" s="4" customFormat="1" x14ac:dyDescent="0.3">
+        <v>1.34549110875214</v>
+      </c>
+      <c r="K14" s="10">
+        <f t="shared" si="1"/>
+        <v>0.99238859087523068</v>
+      </c>
+      <c r="L14" s="11"/>
+    </row>
+    <row r="15" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A15">
-        <v>120</v>
+        <v>150</v>
       </c>
       <c r="B15" s="5"/>
-      <c r="C15" s="4">
-        <v>1.3699400435562701</v>
+      <c r="C15">
+        <v>1.3614670031018901</v>
       </c>
       <c r="D15">
-        <v>1.34077916991197</v>
+        <v>1.3628583617894401</v>
       </c>
       <c r="E15">
-        <v>1.3634284951011899</v>
+        <v>1.3660435580514501</v>
       </c>
       <c r="F15" s="10">
         <f t="shared" si="0"/>
-        <v>1.0168926589087053</v>
-      </c>
-      <c r="H15" s="4">
-        <v>1.35986137171571</v>
+        <v>1.0023371440138709</v>
+      </c>
+      <c r="G15" s="4"/>
+      <c r="H15">
+        <v>1.3561935884492</v>
       </c>
       <c r="I15">
-        <v>1.35581073898229</v>
+        <v>1.34642475596859</v>
       </c>
       <c r="J15">
-        <v>1.34549110875214</v>
-      </c>
-      <c r="K15" s="11">
+        <v>1.3556369406847</v>
+      </c>
+      <c r="K15" s="10">
         <f t="shared" si="1"/>
-        <v>0.99238859087523068</v>
-      </c>
-      <c r="L15" s="11"/>
-    </row>
-    <row r="16" spans="1:12" x14ac:dyDescent="0.3">
+        <v>1.0068419602917082</v>
+      </c>
+      <c r="L15" s="10"/>
+    </row>
+    <row r="16" spans="1:12" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A16">
-        <v>150</v>
+        <v>250</v>
       </c>
       <c r="B16" s="5"/>
       <c r="C16">
-        <v>1.3618779251700099</v>
+        <v>1.3422623387583901</v>
       </c>
       <c r="D16">
-        <v>1.3628583617894401</v>
+        <v>1.31238054231434</v>
       </c>
       <c r="E16">
-        <v>1.3660435580514501</v>
+        <v>1.30114468854049</v>
       </c>
       <c r="F16" s="10">
         <f t="shared" si="0"/>
-        <v>1.0023371440138709</v>
-      </c>
-      <c r="G16" s="4"/>
+        <v>0.99143857028386306</v>
+      </c>
       <c r="H16">
-        <v>1.34863286309854</v>
+        <v>1.3247863550055301</v>
       </c>
       <c r="I16">
-        <v>1.34642475596859</v>
+        <v>1.2854468687873799</v>
       </c>
       <c r="J16">
-        <v>1.3556369406847</v>
+        <v>1.2908172794684301</v>
       </c>
       <c r="K16" s="10">
         <f t="shared" si="1"/>
-        <v>1.0068419602917082</v>
-      </c>
-      <c r="L16" s="10"/>
-    </row>
-    <row r="17" spans="1:12" s="4" customFormat="1" x14ac:dyDescent="0.3">
+        <v>1.0041778550412717</v>
+      </c>
+      <c r="L16" s="11"/>
+    </row>
+    <row r="17" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A17">
-        <v>250</v>
+        <v>500</v>
       </c>
       <c r="B17" s="5"/>
-      <c r="C17" s="4">
-        <v>1.34128105403747</v>
+      <c r="C17">
+        <v>1.3014014859735601</v>
       </c>
       <c r="D17">
-        <v>1.31238054231434</v>
+        <v>1.27106900787611</v>
       </c>
       <c r="E17">
-        <v>1.30114468854049</v>
+        <v>1.2663520004962301</v>
       </c>
       <c r="F17" s="10">
         <f t="shared" si="0"/>
-        <v>0.99143857028386306</v>
-      </c>
-      <c r="H17" s="4">
-        <v>1.31869938927708</v>
+        <v>0.99628894469879192</v>
+      </c>
+      <c r="G17" s="4"/>
+      <c r="H17">
+        <v>1.26268865444005</v>
       </c>
       <c r="I17">
-        <v>1.2854468687873799</v>
+        <v>1.24215702849295</v>
       </c>
       <c r="J17">
-        <v>1.2908172794684301</v>
-      </c>
-      <c r="K17" s="11">
+        <v>1.26045747443881</v>
+      </c>
+      <c r="K17" s="10">
         <f t="shared" si="1"/>
-        <v>1.0041778550412717</v>
-      </c>
-      <c r="L17" s="11"/>
-    </row>
-    <row r="18" spans="1:12" x14ac:dyDescent="0.3">
+        <v>1.0147327958753034</v>
+      </c>
+      <c r="L17" s="10"/>
+    </row>
+    <row r="18" spans="1:12" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A18">
-        <v>500</v>
+        <v>750</v>
       </c>
       <c r="B18" s="5"/>
       <c r="C18">
-        <v>1.2896852557910301</v>
+        <v>1.2615551433943699</v>
       </c>
       <c r="D18">
-        <v>1.27106900787611</v>
+        <v>1.2502327359779</v>
       </c>
       <c r="E18">
-        <v>1.2663520004962301</v>
+        <v>1.26687035022674</v>
       </c>
       <c r="F18" s="10">
         <f t="shared" si="0"/>
-        <v>0.99628894469879192</v>
-      </c>
-      <c r="G18" s="4"/>
+        <v>1.0133076136706871</v>
+      </c>
       <c r="H18">
-        <v>1.24433347413396</v>
+        <v>1.2096572387659299</v>
       </c>
       <c r="I18">
-        <v>1.24215702849295</v>
+        <v>1.20261020085431</v>
       </c>
       <c r="J18">
-        <v>1.26045747443881</v>
+        <v>1.2257592093430201</v>
       </c>
       <c r="K18" s="10">
         <f t="shared" si="1"/>
-        <v>1.0147327958753034</v>
-      </c>
-      <c r="L18" s="10"/>
-    </row>
-    <row r="19" spans="1:12" s="4" customFormat="1" x14ac:dyDescent="0.3">
+        <v>1.0192489706741765</v>
+      </c>
+      <c r="L18" s="11"/>
+    </row>
+    <row r="19" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A19">
-        <v>750</v>
+        <v>999.99</v>
       </c>
       <c r="B19" s="5"/>
-      <c r="C19" s="4">
-        <v>1.24225887840578</v>
+      <c r="C19">
+        <v>1.2295679722156101</v>
       </c>
       <c r="D19">
-        <v>1.2502327359779</v>
+        <v>1.2216766905077201</v>
       </c>
       <c r="E19">
-        <v>1.26687035022674</v>
+        <v>1.20816790789953</v>
       </c>
       <c r="F19" s="10">
         <f t="shared" si="0"/>
-        <v>1.0133076136706871</v>
-      </c>
-      <c r="H19" s="4">
-        <v>1.1765306054398399</v>
+        <v>0.98894242420015732</v>
+      </c>
+      <c r="G19" s="4"/>
+      <c r="H19">
+        <v>1.15612158785918</v>
       </c>
       <c r="I19">
-        <v>1.20261020085431</v>
+        <v>1.1553240194424299</v>
       </c>
       <c r="J19">
-        <v>1.2257592093430201</v>
-      </c>
-      <c r="K19" s="11">
-        <f t="shared" si="1"/>
-        <v>1.0192489706741765</v>
-      </c>
-      <c r="L19" s="11"/>
-    </row>
-    <row r="20" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A20">
-        <v>999.99</v>
-      </c>
-      <c r="B20" s="5"/>
-      <c r="C20">
-        <v>1.1938794039418501</v>
-      </c>
-      <c r="D20">
-        <v>1.2216766905077201</v>
-      </c>
-      <c r="E20">
-        <v>1.20816790789953</v>
-      </c>
-      <c r="F20" s="10">
-        <f t="shared" si="0"/>
-        <v>0.98894242420015732</v>
-      </c>
-      <c r="G20" s="4"/>
-      <c r="H20">
-        <v>1.1108715265371401</v>
-      </c>
-      <c r="I20">
-        <v>1.1553240194424299</v>
-      </c>
-      <c r="J20">
         <v>1.13503567173569</v>
       </c>
-      <c r="K20" s="10">
+      <c r="K19" s="10">
         <f t="shared" si="1"/>
         <v>0.9824392574158276</v>
       </c>
-      <c r="L20" s="10"/>
+      <c r="L19" s="10"/>
+    </row>
+    <row r="23" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="C23" s="12" t="s">
+        <v>5</v>
+      </c>
+      <c r="D23" s="12"/>
+      <c r="E23" s="13"/>
+      <c r="F23" s="13"/>
+      <c r="H23" s="2"/>
+      <c r="I23" s="2"/>
+      <c r="J23" s="2"/>
+      <c r="K23" s="2"/>
     </row>
     <row r="24" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="C24" s="12" t="s">
-        <v>5</v>
-      </c>
-      <c r="D24" s="12"/>
-      <c r="E24" s="13"/>
-      <c r="F24" s="13"/>
-      <c r="H24" s="2"/>
-      <c r="I24" s="2"/>
-      <c r="J24" s="2"/>
-      <c r="K24" s="2"/>
+      <c r="C24" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="D24" s="3"/>
+      <c r="E24" s="9"/>
+      <c r="F24" s="3"/>
+      <c r="H24" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="I24" s="3"/>
+      <c r="J24" s="9"/>
+      <c r="K24" s="9"/>
+      <c r="L24" s="3"/>
     </row>
     <row r="25" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="C25" s="3" t="s">
-        <v>4</v>
-      </c>
-      <c r="D25" s="3"/>
-      <c r="E25" s="9"/>
-      <c r="F25" s="3"/>
-      <c r="H25" s="3" t="s">
-        <v>3</v>
-      </c>
-      <c r="I25" s="3"/>
-      <c r="J25" s="9"/>
-      <c r="K25" s="9"/>
-      <c r="L25" s="3"/>
+      <c r="A25" s="6" t="s">
+        <v>0</v>
+      </c>
+      <c r="B25" s="6"/>
+      <c r="C25" s="6" t="s">
+        <v>1</v>
+      </c>
+      <c r="D25" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="E25" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="F25" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="G25" s="8"/>
+      <c r="H25" s="6" t="s">
+        <v>1</v>
+      </c>
+      <c r="I25" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="J25" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="K25" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="L25" s="7"/>
     </row>
     <row r="26" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A26" s="6" t="s">
-        <v>0</v>
-      </c>
-      <c r="B26" s="6"/>
-      <c r="C26" s="6" t="s">
-        <v>1</v>
-      </c>
-      <c r="D26" s="6" t="s">
-        <v>7</v>
-      </c>
-      <c r="E26" s="6" t="s">
-        <v>6</v>
-      </c>
-      <c r="F26" s="7" t="s">
-        <v>8</v>
-      </c>
-      <c r="G26" s="8"/>
-      <c r="H26" s="6" t="s">
-        <v>1</v>
-      </c>
-      <c r="I26" s="6" t="s">
-        <v>7</v>
-      </c>
-      <c r="J26" s="6" t="s">
-        <v>6</v>
-      </c>
-      <c r="K26" s="7" t="s">
-        <v>8</v>
-      </c>
-      <c r="L26" s="7"/>
+      <c r="A26">
+        <v>0.1</v>
+      </c>
+      <c r="B26" s="5"/>
+      <c r="C26" s="2">
+        <v>3.53760968083747E-5</v>
+      </c>
+      <c r="D26" s="2">
+        <v>3.4283030439073703E-5</v>
+      </c>
+      <c r="E26" s="2">
+        <v>2.4940135833565399E-5</v>
+      </c>
+      <c r="F26" s="10">
+        <f>E26/D26</f>
+        <v>0.7274775745944605</v>
+      </c>
+      <c r="G26" s="4"/>
+      <c r="H26" s="2">
+        <v>3.2455422398815998E-5</v>
+      </c>
+      <c r="I26" s="2">
+        <v>3.06037506527904E-5</v>
+      </c>
+      <c r="J26" s="2">
+        <v>8.9560974139772096E-6</v>
+      </c>
+      <c r="K26" s="10">
+        <f>J26/I26</f>
+        <v>0.29264705217301878</v>
+      </c>
+      <c r="L26" s="10"/>
     </row>
     <row r="27" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A27">
-        <v>0.1</v>
+        <v>0.5</v>
       </c>
       <c r="B27" s="5"/>
-      <c r="C27" s="2">
-        <v>3.52725672373683E-5</v>
+      <c r="C27">
+        <v>1.769377952569E-4</v>
       </c>
       <c r="D27">
-        <v>3.2314434653956498E-4</v>
+        <v>1.7795710468822501E-4</v>
       </c>
       <c r="E27">
-        <v>2.9113846589042902E-4</v>
+        <v>1.1451179445258501E-4</v>
       </c>
       <c r="F27" s="10">
-        <f>E27/D27</f>
-        <v>0.90095484884115951</v>
+        <f t="shared" ref="F27:F40" si="2">E27/D27</f>
+        <v>0.64347975683918834</v>
       </c>
       <c r="G27" s="4"/>
-      <c r="H27" s="2">
-        <v>3.2364516810043102E-5</v>
+      <c r="H27">
+        <v>1.622082823178E-4</v>
       </c>
       <c r="I27">
-        <v>2.8864520587018101E-4</v>
+        <v>1.51128498783429E-4</v>
       </c>
       <c r="J27">
-        <v>2.8967006957661098E-4</v>
+        <v>2.0123326791721201E-4</v>
       </c>
       <c r="K27" s="10">
-        <f>J27/I27</f>
-        <v>1.0035506001332684</v>
+        <f t="shared" ref="K27:K40" si="3">J27/I27</f>
+        <v>1.3315375295667062</v>
       </c>
       <c r="L27" s="10"/>
     </row>
     <row r="28" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A28">
-        <v>0.5</v>
+        <v>1.5</v>
       </c>
       <c r="B28" s="5"/>
-      <c r="C28" s="2"/>
+      <c r="C28">
+        <v>5.2503514596129999E-4</v>
+      </c>
       <c r="D28">
-        <v>1.63531469505055E-3</v>
+        <v>5.6289187437775004E-4</v>
       </c>
       <c r="E28">
-        <v>1.5602327945626699E-3</v>
-      </c>
-      <c r="F28" s="10"/>
+        <v>2.79102553247934E-4</v>
+      </c>
+      <c r="F28" s="10">
+        <f t="shared" si="2"/>
+        <v>0.49583688440425344</v>
+      </c>
       <c r="G28" s="4"/>
-      <c r="H28" s="2"/>
+      <c r="H28">
+        <v>4.8498345014689998E-4</v>
+      </c>
       <c r="I28">
-        <v>1.4624167995472899E-3</v>
+        <v>4.4989314990682798E-4</v>
       </c>
       <c r="J28">
-        <v>1.55376135488548E-3</v>
-      </c>
-      <c r="K28" s="10"/>
+        <v>4.03614344914232E-4</v>
+      </c>
+      <c r="K28" s="10">
+        <f t="shared" si="3"/>
+        <v>0.8971337860952534</v>
+      </c>
       <c r="L28" s="10"/>
     </row>
     <row r="29" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A29">
-        <v>1.5</v>
+        <v>10</v>
       </c>
       <c r="B29" s="5"/>
-      <c r="C29" s="2"/>
+      <c r="C29">
+        <v>3.3839428456904001E-3</v>
+      </c>
       <c r="D29">
-        <v>5.0200091937920499E-3</v>
+        <v>3.3365070331695802E-3</v>
       </c>
       <c r="E29">
-        <v>4.4418725803358596E-3</v>
-      </c>
-      <c r="F29" s="10"/>
+        <v>2.2307755074323201E-3</v>
+      </c>
+      <c r="F29" s="10">
+        <f t="shared" si="2"/>
+        <v>0.66859607525333198</v>
+      </c>
       <c r="G29" s="4"/>
-      <c r="H29" s="2"/>
+      <c r="H29">
+        <v>3.1626406186310001E-3</v>
+      </c>
       <c r="I29">
-        <v>4.4120832608900004E-3</v>
+        <v>3.0155921421882699E-3</v>
       </c>
       <c r="J29">
-        <v>4.3968622699160501E-3</v>
-      </c>
-      <c r="K29" s="10"/>
+        <v>2.6153364392675002E-3</v>
+      </c>
+      <c r="K29" s="10">
+        <f t="shared" si="3"/>
+        <v>0.86727127408207016</v>
+      </c>
       <c r="L29" s="10"/>
     </row>
     <row r="30" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A30">
-        <v>10</v>
+      <c r="A30" s="4">
+        <v>15</v>
       </c>
       <c r="B30" s="5"/>
-      <c r="C30" s="2"/>
+      <c r="C30">
+        <v>4.9687340175238997E-3</v>
+      </c>
       <c r="D30">
-        <v>3.2233154188020502E-2</v>
+        <v>4.9536689812130401E-3</v>
       </c>
       <c r="E30">
-        <v>3.1830960117675798E-2</v>
-      </c>
-      <c r="F30" s="10"/>
+        <v>3.6306214215505398E-3</v>
+      </c>
+      <c r="F30" s="10">
+        <f t="shared" si="2"/>
+        <v>0.73291562987349301</v>
+      </c>
       <c r="G30" s="4"/>
-      <c r="H30" s="2"/>
+      <c r="H30">
+        <v>4.7034313826145001E-3</v>
+      </c>
       <c r="I30">
-        <v>2.9294700126228299E-2</v>
+        <v>4.2298917106053102E-3</v>
       </c>
       <c r="J30">
-        <v>2.9963416156383201E-2</v>
-      </c>
-      <c r="K30" s="10"/>
-      <c r="L30" s="10"/>
+        <v>4.0615398119136998E-3</v>
+      </c>
+      <c r="K30" s="10">
+        <f t="shared" si="3"/>
+        <v>0.96019947785672299</v>
+      </c>
+      <c r="L30" s="11"/>
     </row>
     <row r="31" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A31" s="4">
-        <v>15</v>
+      <c r="A31">
+        <v>30</v>
       </c>
       <c r="B31" s="5"/>
-      <c r="C31" s="5">
-        <v>5.02535867346246E-3</v>
+      <c r="C31">
+        <v>9.6668811570342003E-3</v>
       </c>
       <c r="D31">
-        <v>4.8083671005010903E-2</v>
+        <v>9.8049806314099101E-3</v>
       </c>
       <c r="E31">
-        <v>4.7413078230864998E-2</v>
-      </c>
-      <c r="F31" s="11">
-        <f t="shared" ref="F31:F41" si="2">E31/D31</f>
-        <v>0.98605362776739691</v>
+        <v>7.3289045458139902E-3</v>
+      </c>
+      <c r="F31" s="10">
+        <f t="shared" si="2"/>
+        <v>0.74746751893992558</v>
       </c>
       <c r="G31" s="4"/>
       <c r="H31">
-        <v>4.7442437671726999E-3</v>
+        <v>9.2377761797262006E-3</v>
       </c>
       <c r="I31">
-        <v>4.28280907778881E-2</v>
+        <v>8.8658994417866593E-3</v>
       </c>
       <c r="J31">
-        <v>4.61668507397665E-2</v>
-      </c>
-      <c r="K31" s="11">
-        <f t="shared" ref="K31:K41" si="3">J31/I31</f>
-        <v>1.0779572449118415</v>
-      </c>
-      <c r="L31" s="11"/>
+        <v>7.2748435041183898E-3</v>
+      </c>
+      <c r="K31" s="10">
+        <f t="shared" si="3"/>
+        <v>0.82054207267800461</v>
+      </c>
+      <c r="L31" s="10"/>
     </row>
     <row r="32" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A32">
-        <v>30</v>
+      <c r="A32" s="4">
+        <v>60</v>
       </c>
       <c r="B32" s="5"/>
-      <c r="C32" s="2">
-        <v>9.6096776712520909E-3</v>
+      <c r="C32">
+        <v>1.7647794082264599E-2</v>
       </c>
       <c r="D32">
-        <v>9.5891818868841697E-2</v>
+        <v>1.6929482364304901E-2</v>
       </c>
       <c r="E32">
-        <v>9.4831541186847598E-2</v>
+        <v>1.3311257592672E-2</v>
       </c>
       <c r="F32" s="10">
         <f t="shared" si="2"/>
-        <v>0.98894298080377097</v>
+        <v>0.78627670393149318</v>
       </c>
       <c r="G32" s="4"/>
       <c r="H32">
-        <v>9.3381817414101998E-3</v>
+        <v>1.79734898063151E-2</v>
       </c>
       <c r="I32">
-        <v>8.7192700810209606E-2</v>
+        <v>1.57606335049696E-2</v>
       </c>
       <c r="J32">
-        <v>8.8994701260368805E-2</v>
+        <v>1.41246952576636E-2</v>
       </c>
       <c r="K32" s="10">
         <f t="shared" si="3"/>
-        <v>1.0206668727246053</v>
-      </c>
-      <c r="L32" s="10"/>
+        <v>0.89620098412984728</v>
+      </c>
+      <c r="L32" s="11"/>
     </row>
     <row r="33" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A33" s="4">
-        <v>60</v>
+      <c r="A33">
+        <v>90</v>
       </c>
       <c r="B33" s="5"/>
-      <c r="C33" s="5">
-        <v>1.7956202904139199E-2</v>
+      <c r="C33">
+        <v>2.5054917938694E-2</v>
       </c>
       <c r="D33">
-        <v>0.18310601049282599</v>
+        <v>2.3458449507632401E-2</v>
       </c>
       <c r="E33">
-        <v>0.18135757900897301</v>
-      </c>
-      <c r="F33" s="11">
+        <v>2.05541471998755E-2</v>
+      </c>
+      <c r="F33" s="10">
         <f t="shared" si="2"/>
-        <v>0.99045126110744741</v>
+        <v>0.87619376520123537</v>
       </c>
       <c r="G33" s="4"/>
       <c r="H33">
-        <v>1.8093633576609602E-2</v>
+        <v>2.6164917465571601E-2</v>
       </c>
       <c r="I33">
-        <v>0.168976390095402</v>
+        <v>2.3818302176688601E-2</v>
       </c>
       <c r="J33">
-        <v>0.17402218522129201</v>
-      </c>
-      <c r="K33" s="11">
+        <v>2.3768164319370701E-2</v>
+      </c>
+      <c r="K33" s="10">
         <f t="shared" si="3"/>
-        <v>1.0298609475740441</v>
-      </c>
-      <c r="L33" s="11"/>
+        <v>0.99789498609321658</v>
+      </c>
+      <c r="L33" s="10"/>
     </row>
     <row r="34" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A34">
-        <v>90</v>
+      <c r="A34" s="4">
+        <v>100</v>
       </c>
       <c r="B34" s="5"/>
-      <c r="C34" s="2">
-        <v>2.54716677488637E-2</v>
+      <c r="C34">
+        <v>2.73242514617307E-2</v>
       </c>
       <c r="D34">
-        <v>0.27052609093888302</v>
+        <v>2.5947125661509699E-2</v>
       </c>
       <c r="E34">
-        <v>0.27828767586518899</v>
+        <v>2.2524567468256498E-2</v>
       </c>
       <c r="F34" s="10">
         <f t="shared" si="2"/>
-        <v>1.0286907074262921</v>
+        <v>0.86809490045634352</v>
       </c>
       <c r="G34" s="4"/>
       <c r="H34">
-        <v>2.63480432958439E-2</v>
+        <v>2.8758676699886999E-2</v>
       </c>
       <c r="I34">
-        <v>0.25226765578979399</v>
+        <v>2.6060698692637999E-2</v>
       </c>
       <c r="J34">
-        <v>0.27028735246822</v>
+        <v>2.41183055307931E-2</v>
       </c>
       <c r="K34" s="10">
         <f t="shared" si="3"/>
-        <v>1.0714308642620487</v>
+        <v>0.92546657383389286</v>
       </c>
       <c r="L34" s="10"/>
     </row>
     <row r="35" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A35" s="4">
-        <v>100</v>
+        <v>120</v>
       </c>
       <c r="B35" s="5"/>
-      <c r="C35" s="2"/>
+      <c r="C35">
+        <v>3.1756367537968302E-2</v>
+      </c>
       <c r="D35">
-        <v>0.29782820153673201</v>
+        <v>3.2193504593870201E-2</v>
       </c>
       <c r="E35">
-        <v>0.31219673881320298</v>
-      </c>
-      <c r="F35" s="10"/>
+        <v>2.5515114756006999E-2</v>
+      </c>
+      <c r="F35" s="10">
+        <f t="shared" si="2"/>
+        <v>0.79255474288640204</v>
+      </c>
       <c r="G35" s="4"/>
+      <c r="H35">
+        <v>3.3831181126573399E-2</v>
+      </c>
       <c r="I35">
-        <v>0.27710332040764002</v>
+        <v>3.0884672634417399E-2</v>
       </c>
       <c r="J35">
-        <v>0.29733056001795299</v>
-      </c>
-      <c r="K35" s="10"/>
-      <c r="L35" s="10"/>
+        <v>2.9445668702238598E-2</v>
+      </c>
+      <c r="K35" s="10">
+        <f t="shared" si="3"/>
+        <v>0.95340718196328889</v>
+      </c>
+      <c r="L35" s="11"/>
     </row>
     <row r="36" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A36" s="4">
-        <v>120</v>
+      <c r="A36">
+        <v>150</v>
       </c>
       <c r="B36" s="5"/>
-      <c r="C36" s="5">
-        <v>3.2417642839879697E-2</v>
+      <c r="C36">
+        <v>3.79760832406765E-2</v>
       </c>
       <c r="D36">
-        <v>0.35933558625490702</v>
+        <v>3.6337278414827603E-2</v>
       </c>
       <c r="E36">
-        <v>0.36327933121591299</v>
-      </c>
-      <c r="F36" s="11">
+        <v>3.2903913104897098E-2</v>
+      </c>
+      <c r="F36" s="10">
         <f t="shared" si="2"/>
-        <v>1.0109751026946947</v>
+        <v>0.90551396638088599</v>
       </c>
       <c r="G36" s="4"/>
       <c r="H36">
-        <v>3.4169678168819703E-2</v>
+        <v>4.0827391559504302E-2</v>
       </c>
       <c r="I36">
-        <v>0.33488526020133202</v>
+        <v>3.8123585674305099E-2</v>
       </c>
       <c r="J36">
-        <v>0.350044087283917</v>
-      </c>
-      <c r="K36" s="11">
+        <v>3.6179164073167201E-2</v>
+      </c>
+      <c r="K36" s="10">
         <f t="shared" si="3"/>
-        <v>1.0452657339217364</v>
-      </c>
-      <c r="L36" s="11"/>
+        <v>0.94899688560909901</v>
+      </c>
+      <c r="L36" s="10"/>
     </row>
     <row r="37" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A37">
-        <v>150</v>
+      <c r="A37" s="4">
+        <v>250</v>
       </c>
       <c r="B37" s="5"/>
-      <c r="C37" s="2">
-        <v>3.9055212834252402E-2</v>
+      <c r="C37">
+        <v>5.6477544791410803E-2</v>
       </c>
       <c r="D37">
-        <v>0.440983559195115</v>
+        <v>5.5465836690505303E-2</v>
       </c>
       <c r="E37">
-        <v>0.46369387108133497</v>
+        <v>5.1493175994203999E-2</v>
       </c>
       <c r="F37" s="10">
         <f t="shared" si="2"/>
-        <v>1.0514992257935214</v>
+        <v>0.92837643974491146</v>
       </c>
       <c r="G37" s="4"/>
       <c r="H37">
-        <v>4.1796462699614498E-2</v>
+        <v>6.2587066941841005E-2</v>
       </c>
       <c r="I37">
-        <v>0.41421243624474702</v>
+        <v>5.8814448863946898E-2</v>
       </c>
       <c r="J37">
-        <v>0.44198494489621698</v>
+        <v>5.6605063359839898E-2</v>
       </c>
       <c r="K37" s="10">
         <f t="shared" si="3"/>
-        <v>1.0670489493344424</v>
-      </c>
-      <c r="L37" s="10"/>
+        <v>0.9624346474925255</v>
+      </c>
+      <c r="L37" s="11"/>
     </row>
     <row r="38" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A38" s="4">
-        <v>250</v>
+      <c r="A38">
+        <v>500</v>
       </c>
       <c r="B38" s="5"/>
-      <c r="C38" s="5">
-        <v>5.8983323870902299E-2</v>
+      <c r="C38">
+        <v>9.6749839749360703E-2</v>
       </c>
       <c r="D38">
-        <v>0.69943129650860603</v>
+        <v>9.2698744321603202E-2</v>
       </c>
       <c r="E38">
-        <v>0.74056761334149801</v>
-      </c>
-      <c r="F38" s="11">
+        <v>8.6940034618715994E-2</v>
+      </c>
+      <c r="F38" s="10">
         <f t="shared" si="2"/>
-        <v>1.0588139493303126</v>
+        <v>0.93787715524054671</v>
       </c>
       <c r="G38" s="4"/>
       <c r="H38">
-        <v>6.5796691976300697E-2</v>
+        <v>0.10941310652236901</v>
       </c>
       <c r="I38">
-        <v>0.66184301157104197</v>
+        <v>0.101328636998795</v>
       </c>
       <c r="J38">
-        <v>0.70419594658632301</v>
-      </c>
-      <c r="K38" s="11">
+        <v>0.103511880070482</v>
+      </c>
+      <c r="K38" s="10">
         <f t="shared" si="3"/>
-        <v>1.0639924185567</v>
-      </c>
-      <c r="L38" s="11"/>
+        <v>1.0215461604572156</v>
+      </c>
+      <c r="L38" s="10"/>
     </row>
     <row r="39" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A39">
-        <v>500</v>
+      <c r="A39" s="4">
+        <v>750</v>
       </c>
       <c r="B39" s="5"/>
-      <c r="C39" s="2">
-        <v>0.103595084893309</v>
+      <c r="C39">
+        <v>0.12913289428404701</v>
       </c>
       <c r="D39">
-        <v>1.3176141318230901</v>
+        <v>0.12658460512460301</v>
       </c>
       <c r="E39">
-        <v>1.4059443021665801</v>
+        <v>0.128790466427847</v>
       </c>
       <c r="F39" s="10">
         <f t="shared" si="2"/>
-        <v>1.0670379652207234</v>
+        <v>1.0174259839976012</v>
       </c>
       <c r="G39" s="4"/>
       <c r="H39">
-        <v>0.11839645185777101</v>
+        <v>0.14632252761592299</v>
       </c>
       <c r="I39">
-        <v>1.25292933313</v>
+        <v>0.13858937862319001</v>
       </c>
       <c r="J39">
-        <v>1.3590454721452301</v>
+        <v>0.149026761504226</v>
       </c>
       <c r="K39" s="10">
         <f t="shared" si="3"/>
-        <v>1.0846944326462025</v>
-      </c>
-      <c r="L39" s="10"/>
+        <v>1.0753115641669349</v>
+      </c>
+      <c r="L39" s="11"/>
     </row>
     <row r="40" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A40" s="4">
-        <v>750</v>
+      <c r="A40">
+        <v>1000</v>
       </c>
       <c r="B40" s="5"/>
-      <c r="C40" s="5">
-        <v>0.14519436153500101</v>
+      <c r="C40">
+        <v>0.157828985100924</v>
       </c>
       <c r="D40">
-        <v>1.9175894049158899</v>
+        <v>0.15157133316674601</v>
       </c>
       <c r="E40">
-        <v>2.0750333201713098</v>
-      </c>
-      <c r="F40" s="11">
+        <v>0.15530428148366199</v>
+      </c>
+      <c r="F40" s="10">
         <f t="shared" si="2"/>
-        <v>1.0821051236786146</v>
+        <v>1.0246283267351703</v>
       </c>
       <c r="G40" s="4"/>
       <c r="H40">
-        <v>0.165934052581929</v>
+        <v>0.178362496787381</v>
       </c>
       <c r="I40">
-        <v>1.8041504774598101</v>
+        <v>0.17072801306535401</v>
       </c>
       <c r="J40">
-        <v>1.9766773113</v>
-      </c>
-      <c r="K40" s="11">
+        <v>0.17116297500401301</v>
+      </c>
+      <c r="K40" s="10">
         <f t="shared" si="3"/>
-        <v>1.0956277405879706</v>
-      </c>
-      <c r="L40" s="11"/>
-    </row>
-    <row r="41" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A41">
-        <v>1000</v>
-      </c>
-      <c r="B41" s="5"/>
-      <c r="C41" s="2">
-        <v>0.185920101577397</v>
-      </c>
-      <c r="D41">
-        <v>2.4565650146404598</v>
-      </c>
-      <c r="E41">
-        <v>2.6505145134263399</v>
-      </c>
-      <c r="F41" s="10">
-        <f t="shared" si="2"/>
-        <v>1.0789515024556622</v>
-      </c>
-      <c r="G41" s="4"/>
-      <c r="H41">
-        <v>0.211237572970251</v>
-      </c>
-      <c r="I41">
-        <v>2.3142913460731198</v>
-      </c>
-      <c r="J41">
-        <v>2.4780340620747099</v>
-      </c>
-      <c r="K41" s="10">
-        <f t="shared" si="3"/>
-        <v>1.0707528532565391</v>
-      </c>
-      <c r="L41" s="10"/>
+        <v>1.0025476893384362</v>
+      </c>
+      <c r="L40" s="10"/>
+    </row>
+    <row r="44" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="C44" s="1" t="s">
+        <v>9</v>
+      </c>
     </row>
     <row r="45" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="C45" s="1" t="s">
-        <v>9</v>
-      </c>
+      <c r="C45" s="14" t="s">
+        <v>2</v>
+      </c>
+      <c r="D45" s="14"/>
+      <c r="E45" s="15"/>
+      <c r="H45" s="2"/>
+      <c r="I45" s="2"/>
+      <c r="J45" s="2"/>
+      <c r="K45" s="2"/>
     </row>
     <row r="46" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="C46" s="14" t="s">
-        <v>2</v>
-      </c>
-      <c r="D46" s="14"/>
-      <c r="E46" s="15"/>
-      <c r="H46" s="2"/>
-      <c r="I46" s="2"/>
-      <c r="J46" s="2"/>
-      <c r="K46" s="2"/>
+      <c r="C46" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="D46" s="3"/>
+      <c r="E46" s="9"/>
+      <c r="F46" s="3"/>
+      <c r="H46" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="I46" s="3"/>
+      <c r="J46" s="9"/>
+      <c r="K46" s="9"/>
     </row>
     <row r="47" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="C47" s="3" t="s">
-        <v>4</v>
-      </c>
-      <c r="D47" s="3"/>
-      <c r="E47" s="9"/>
-      <c r="F47" s="3"/>
-      <c r="H47" s="3" t="s">
-        <v>3</v>
-      </c>
-      <c r="I47" s="3"/>
-      <c r="J47" s="9"/>
-      <c r="K47" s="9"/>
+      <c r="A47" s="6" t="s">
+        <v>0</v>
+      </c>
+      <c r="B47" s="6"/>
+      <c r="C47" s="6" t="s">
+        <v>1</v>
+      </c>
+      <c r="D47" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="E47" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="F47" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="G47" s="8"/>
+      <c r="H47" s="6" t="s">
+        <v>1</v>
+      </c>
+      <c r="I47" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="J47" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="K47" s="7" t="s">
+        <v>8</v>
+      </c>
     </row>
     <row r="48" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A48" s="6" t="s">
-        <v>0</v>
-      </c>
-      <c r="B48" s="6"/>
-      <c r="C48" s="6" t="s">
-        <v>1</v>
-      </c>
-      <c r="D48" s="6" t="s">
-        <v>7</v>
-      </c>
-      <c r="E48" s="6" t="s">
-        <v>6</v>
-      </c>
-      <c r="F48" s="7" t="s">
-        <v>8</v>
-      </c>
-      <c r="G48" s="8"/>
-      <c r="H48" s="6" t="s">
-        <v>1</v>
-      </c>
-      <c r="I48" s="6" t="s">
-        <v>7</v>
-      </c>
-      <c r="J48" s="6" t="s">
-        <v>6</v>
-      </c>
-      <c r="K48" s="7" t="s">
-        <v>8</v>
+      <c r="A48">
+        <v>0.1</v>
+      </c>
+      <c r="B48" s="5"/>
+      <c r="C48">
+        <v>1.38755773111088</v>
+      </c>
+      <c r="D48">
+        <v>1.33146077610654</v>
+      </c>
+      <c r="E48">
+        <v>1.3294682945082299</v>
+      </c>
+      <c r="F48" s="10">
+        <f>E48/D48</f>
+        <v>0.9985035371420129</v>
+      </c>
+      <c r="G48" s="4"/>
+      <c r="I48">
+        <v>1.33422182541257</v>
+      </c>
+      <c r="J48">
+        <v>1.3288821396550801</v>
+      </c>
+      <c r="K48" s="10">
+        <f>J48/I48</f>
+        <v>0.99599790255579224</v>
       </c>
     </row>
     <row r="49" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A49">
-        <v>0.1</v>
+        <v>0.5</v>
       </c>
       <c r="B49" s="5"/>
       <c r="C49">
-        <v>1.38755773111088</v>
+        <v>1.38409520401011</v>
       </c>
       <c r="D49">
-        <v>1.3354353849754901</v>
+        <v>1.35765661048369</v>
       </c>
       <c r="E49">
-        <v>1.33571066860882</v>
+        <v>1.3402135659025001</v>
       </c>
       <c r="F49" s="10">
-        <f>E49/D49</f>
-        <v>1.0002061377408649</v>
+        <f t="shared" ref="F49:F60" si="4">E49/D49</f>
+        <v>0.98715209394887005</v>
       </c>
       <c r="G49" s="4"/>
+      <c r="H49" s="4"/>
       <c r="I49">
-        <v>1.3355902411931799</v>
+        <v>1.3552315082948401</v>
       </c>
       <c r="J49">
-        <v>1.33570664006712</v>
-      </c>
-      <c r="K49" s="10">
-        <f>J49/I49</f>
-        <v>1.0000871516355467</v>
+        <v>1.34024384554322</v>
+      </c>
+      <c r="K49" s="11">
+        <f t="shared" ref="K49:K58" si="5">J49/I49</f>
+        <v>0.98894088378266998</v>
       </c>
     </row>
     <row r="50" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A50" s="4">
-        <v>15</v>
+      <c r="A50">
+        <v>1</v>
       </c>
       <c r="B50" s="5"/>
       <c r="C50">
-        <v>1.38409520401011</v>
+        <v>1.3811622398640599</v>
       </c>
       <c r="D50">
-        <v>1.3305745989353699</v>
+        <v>1.33903476392587</v>
       </c>
       <c r="E50">
-        <v>1.3291243406104201</v>
-      </c>
-      <c r="F50" s="11">
-        <f t="shared" ref="F50:F59" si="4">E50/D50</f>
-        <v>0.99891005109663888</v>
+        <v>1.3294539841566</v>
+      </c>
+      <c r="F50" s="10">
+        <f t="shared" si="4"/>
+        <v>0.99284501043036377</v>
       </c>
       <c r="G50" s="4"/>
-      <c r="H50" s="4"/>
       <c r="I50">
-        <v>1.3283272840070699</v>
+        <v>1.3461367977004299</v>
       </c>
       <c r="J50">
-        <v>1.32707241565139</v>
-      </c>
-      <c r="K50" s="11">
-        <f t="shared" ref="K50:K59" si="5">J50/I50</f>
-        <v>0.99905530182900826</v>
+        <v>1.32904261090945</v>
+      </c>
+      <c r="K50" s="10">
+        <f t="shared" si="5"/>
+        <v>0.98730130041747499</v>
       </c>
     </row>
     <row r="51" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A51">
-        <v>30</v>
+        <v>10</v>
       </c>
       <c r="B51" s="5"/>
       <c r="C51">
-        <v>1.3811622398640599</v>
+        <v>1.37486493369789</v>
       </c>
       <c r="D51">
-        <v>1.3310144038562199</v>
+        <v>1.31789010731641</v>
       </c>
       <c r="E51">
-        <v>1.3285615218559801</v>
+        <v>1.3448930260504799</v>
       </c>
       <c r="F51" s="10">
         <f t="shared" si="4"/>
-        <v>0.99815713339154455</v>
+        <v>1.0204895071175968</v>
       </c>
       <c r="G51" s="4"/>
+      <c r="H51" s="4"/>
       <c r="I51">
-        <v>1.32510611680532</v>
+        <v>1.31846450590491</v>
       </c>
       <c r="J51">
-        <v>1.3232823680411001</v>
-      </c>
-      <c r="K51" s="10">
+        <v>1.3511493506913199</v>
+      </c>
+      <c r="K51" s="11">
         <f t="shared" si="5"/>
-        <v>0.9986236960639675</v>
+        <v>1.0247900831914902</v>
       </c>
     </row>
     <row r="52" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A52" s="4">
-        <v>60</v>
+      <c r="A52">
+        <v>25</v>
       </c>
       <c r="B52" s="5"/>
       <c r="C52">
-        <v>1.37486493369789</v>
+        <v>1.36350384779266</v>
       </c>
       <c r="D52">
-        <v>1.32588118290715</v>
+        <v>1.32036564820574</v>
       </c>
       <c r="E52">
-        <v>1.3260681746726899</v>
-      </c>
-      <c r="F52" s="11">
+        <v>1.3268512139816999</v>
+      </c>
+      <c r="F52" s="10">
         <f t="shared" si="4"/>
-        <v>1.0001410320682957</v>
+        <v>1.0049119467662411</v>
       </c>
       <c r="G52" s="4"/>
-      <c r="H52" s="4"/>
       <c r="I52">
-        <v>1.3187223856414001</v>
+        <v>1.33152629750905</v>
       </c>
       <c r="J52">
-        <v>1.31770759949175</v>
-      </c>
-      <c r="K52" s="11">
+        <v>1.33015612015508</v>
+      </c>
+      <c r="K52" s="10">
         <f t="shared" si="5"/>
-        <v>0.99923047780131791</v>
+        <v>0.99897097236717491</v>
       </c>
     </row>
     <row r="53" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A53">
-        <v>90</v>
+        <v>50</v>
       </c>
       <c r="B53" s="5"/>
       <c r="C53">
-        <v>1.36350384779266</v>
+        <v>1.3571706170428599</v>
       </c>
       <c r="D53">
-        <v>1.3250331310758601</v>
+        <v>1.3197738196808499</v>
       </c>
       <c r="E53">
-        <v>1.32283704671966</v>
+        <v>1.3126564921716899</v>
       </c>
       <c r="F53" s="10">
         <f t="shared" si="4"/>
-        <v>0.99834261928649515</v>
+        <v>0.99460716116426584</v>
       </c>
       <c r="G53" s="4"/>
+      <c r="H53" s="4"/>
       <c r="I53">
-        <v>1.3124798292895099</v>
+        <v>1.32005527665466</v>
       </c>
       <c r="J53">
-        <v>1.3112535491322701</v>
-      </c>
-      <c r="K53" s="10">
+        <v>1.30244954906179</v>
+      </c>
+      <c r="K53" s="11">
         <f t="shared" si="5"/>
-        <v>0.99906567694994319</v>
+        <v>0.98666288608952257</v>
       </c>
     </row>
     <row r="54" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A54" s="4">
-        <v>120</v>
+      <c r="A54">
+        <v>75</v>
       </c>
       <c r="B54" s="5"/>
       <c r="C54">
-        <v>1.3571706170428599</v>
+        <v>1.35109721915133</v>
       </c>
       <c r="D54">
-        <v>1.3186752377537301</v>
+        <v>1.29935652652886</v>
       </c>
       <c r="E54">
-        <v>1.31925522687803</v>
-      </c>
-      <c r="F54" s="11">
+        <v>1.32473430230751</v>
+      </c>
+      <c r="F54" s="10">
         <f t="shared" si="4"/>
-        <v>1.000439827114133</v>
+        <v>1.0195310334465668</v>
       </c>
       <c r="G54" s="4"/>
-      <c r="H54" s="4"/>
       <c r="I54">
-        <v>1.3033297752905399</v>
+        <v>1.30908256842566</v>
       </c>
       <c r="J54">
-        <v>1.3019564075099299</v>
-      </c>
-      <c r="K54" s="11">
+        <v>1.30672475018709</v>
+      </c>
+      <c r="K54" s="10">
         <f t="shared" si="5"/>
-        <v>0.99894626225330896</v>
+        <v>0.99819887736996948</v>
       </c>
     </row>
     <row r="55" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A55">
-        <v>150</v>
+        <v>100</v>
       </c>
       <c r="B55" s="5"/>
       <c r="C55">
-        <v>1.35109721915133</v>
+        <v>1.32844051248484</v>
       </c>
       <c r="D55">
-        <v>1.3162252475838401</v>
+        <v>1.33910590256307</v>
       </c>
       <c r="E55">
-        <v>1.3162028531863199</v>
+        <v>1.3167897334910501</v>
       </c>
       <c r="F55" s="10">
         <f t="shared" si="4"/>
-        <v>0.99998298589275558</v>
+        <v>0.98333502299608533</v>
       </c>
       <c r="G55" s="4"/>
+      <c r="H55" s="4"/>
       <c r="I55">
-        <v>1.29663015170481</v>
+        <v>1.3171859836539099</v>
       </c>
       <c r="J55">
-        <v>1.2969552292914901</v>
-      </c>
-      <c r="K55" s="10">
+        <v>1.31060168409573</v>
+      </c>
+      <c r="K55" s="11">
         <f t="shared" si="5"/>
-        <v>1.0002507095691495</v>
+        <v>0.99500123775997451</v>
       </c>
     </row>
     <row r="56" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A56" s="4">
-        <v>250</v>
+      <c r="A56">
+        <v>150</v>
       </c>
       <c r="B56" s="5"/>
       <c r="C56">
-        <v>1.32844051248484</v>
+        <v>1.26939305918802</v>
       </c>
       <c r="D56">
-        <v>1.30260068538983</v>
+        <v>1.3346899335651701</v>
       </c>
       <c r="E56">
-        <v>1.3066950650451801</v>
-      </c>
-      <c r="F56" s="11">
+        <v>1.3164282135057199</v>
+      </c>
+      <c r="F56" s="10">
         <f t="shared" si="4"/>
-        <v>1.0031432346852518</v>
+        <v>0.98631763108404502</v>
       </c>
       <c r="G56" s="4"/>
-      <c r="H56" s="4"/>
       <c r="I56">
-        <v>1.2708609670523101</v>
+        <v>1.28924587434467</v>
       </c>
       <c r="J56">
-        <v>1.27351639583336</v>
-      </c>
-      <c r="K56" s="11">
+        <v>1.3011790803332</v>
+      </c>
+      <c r="K56" s="10">
         <f t="shared" si="5"/>
-        <v>1.0020894722946829</v>
+        <v>1.0092559582512495</v>
       </c>
     </row>
     <row r="57" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A57">
-        <v>500</v>
+        <v>250</v>
       </c>
       <c r="B57" s="5"/>
       <c r="C57">
-        <v>1.26939305918802</v>
+        <v>1.2146497361047901</v>
       </c>
       <c r="D57">
-        <v>1.26652819252339</v>
+        <v>1.29678717701069</v>
       </c>
       <c r="E57">
-        <v>1.2763205188269799</v>
+        <v>1.33451901185347</v>
       </c>
       <c r="F57" s="10">
         <f t="shared" si="4"/>
-        <v>1.0077316291586689</v>
+        <v>1.0290963972436542</v>
       </c>
       <c r="G57" s="4"/>
+      <c r="H57" s="4"/>
       <c r="I57">
-        <v>1.2073775660257999</v>
+        <v>1.2845821783281699</v>
       </c>
       <c r="J57">
-        <v>1.2155197343022801</v>
-      </c>
-      <c r="K57" s="10">
+        <v>1.27732476166037</v>
+      </c>
+      <c r="K57" s="11">
         <f t="shared" si="5"/>
-        <v>1.0067436802749954</v>
+        <v>0.99435036793267273</v>
       </c>
     </row>
     <row r="58" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A58" s="4">
-        <v>750</v>
+      <c r="A58">
+        <v>500</v>
       </c>
       <c r="B58" s="5"/>
       <c r="C58">
-        <v>1.2146497361047901</v>
+        <v>1.1436421352186501</v>
       </c>
       <c r="D58">
-        <v>1.2257285387942201</v>
+        <v>1.2662694099393199</v>
       </c>
       <c r="E58">
-        <v>1.2402498141564899</v>
-      </c>
-      <c r="F58" s="11">
+        <v>1.2620512370753201</v>
+      </c>
+      <c r="F58" s="10">
         <f t="shared" si="4"/>
-        <v>1.0118470565893447</v>
+        <v>0.99666881879093805</v>
       </c>
       <c r="G58" s="4"/>
-      <c r="H58" s="4"/>
       <c r="I58">
-        <v>1.1403490012176101</v>
+        <v>1.2051198250164299</v>
       </c>
       <c r="J58">
-        <v>1.15185236456864</v>
-      </c>
-      <c r="K58" s="11">
+        <v>1.19710463230099</v>
+      </c>
+      <c r="K58" s="10">
         <f t="shared" si="5"/>
-        <v>1.0100875813796892</v>
+        <v>0.99334904915755518</v>
       </c>
     </row>
     <row r="59" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A59">
-        <v>1000</v>
-      </c>
-      <c r="B59" s="5"/>
-      <c r="C59">
-        <v>1.1436421352186501</v>
+        <v>750</v>
       </c>
       <c r="D59">
-        <v>1.1781818408587099</v>
+        <v>1.23279071771682</v>
       </c>
       <c r="E59">
-        <v>1.19775360779693</v>
+        <v>1.23649350366719</v>
       </c>
       <c r="F59" s="10">
         <f t="shared" si="4"/>
-        <v>1.0166118389025205</v>
-      </c>
-      <c r="G59" s="4"/>
+        <v>1.0030035803296993</v>
+      </c>
       <c r="I59">
-        <v>1.072078850564</v>
+        <v>1.1807532343395699</v>
       </c>
       <c r="J59">
-        <v>1.0876143945201899</v>
-      </c>
-      <c r="K59" s="10">
-        <f t="shared" si="5"/>
-        <v>1.0144910460158942</v>
+        <v>1.1563239206929501</v>
+      </c>
+    </row>
+    <row r="60" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A60">
+        <v>999.99</v>
+      </c>
+      <c r="D60">
+        <v>1.1928852496040101</v>
+      </c>
+      <c r="E60">
+        <v>1.2106403902979499</v>
+      </c>
+      <c r="F60" s="10">
+        <f t="shared" si="4"/>
+        <v>1.0148841983751864</v>
+      </c>
+      <c r="I60">
+        <v>1.13357719050286</v>
+      </c>
+      <c r="J60">
+        <v>1.1342010761596699</v>
       </c>
     </row>
     <row r="63" spans="1:11" x14ac:dyDescent="0.3">
@@ -6279,326 +6415,794 @@
         <v>2.0906018648200899E-5</v>
       </c>
       <c r="D66" s="2">
-        <v>2.0018619481595599E-5</v>
+        <v>1.9785240862768899E-5</v>
       </c>
       <c r="E66" s="2">
-        <v>2.04228717705638E-5</v>
+        <v>1.9417624590728801E-5</v>
       </c>
       <c r="F66" s="10">
         <f>E66/D66</f>
-        <v>1.0201938145305103</v>
+        <v>0.98141967163352228</v>
       </c>
       <c r="G66" s="4"/>
       <c r="H66" s="2"/>
       <c r="I66" s="2">
-        <v>2.4434932696069799E-5</v>
+        <v>2.44555572729164E-5</v>
       </c>
       <c r="J66" s="2">
-        <v>2.5518609602937599E-5</v>
+        <v>2.3173152783100001E-5</v>
       </c>
       <c r="K66" s="10">
         <f>J66/I66</f>
-        <v>1.0443494942403546</v>
+        <v>0.94756183735642718</v>
       </c>
     </row>
     <row r="67" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A67" s="4">
-        <v>15</v>
+      <c r="A67">
+        <v>0.5</v>
       </c>
       <c r="B67" s="5"/>
       <c r="C67" s="2">
         <v>3.1327203465188001E-3</v>
       </c>
       <c r="D67">
-        <v>2.9966209956305001E-3</v>
-      </c>
-      <c r="E67">
-        <v>3.14006419786265E-3</v>
-      </c>
-      <c r="F67" s="11">
-        <f t="shared" ref="F67:F76" si="6">E67/D67</f>
-        <v>1.0478683164942482</v>
+        <v>1.02051178015395E-4</v>
+      </c>
+      <c r="E67" s="2">
+        <v>9.4705678455829002E-5</v>
+      </c>
+      <c r="F67" s="10">
+        <f t="shared" ref="F67:F78" si="6">E67/D67</f>
+        <v>0.92802141334950694</v>
       </c>
       <c r="G67" s="4"/>
       <c r="I67">
-        <v>3.6561489620800698E-3</v>
+        <v>1.237590596311E-4</v>
       </c>
       <c r="J67">
-        <v>3.8583728177792702E-3</v>
+        <v>1.2781285534871299E-4</v>
       </c>
       <c r="K67" s="11">
-        <f t="shared" ref="K67:K76" si="7">J67/I67</f>
-        <v>1.0553106172085915</v>
+        <f t="shared" ref="K67:K78" si="7">J67/I67</f>
+        <v>1.0327555471873857</v>
       </c>
     </row>
     <row r="68" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A68">
-        <v>30</v>
+        <v>1</v>
       </c>
       <c r="B68" s="5"/>
       <c r="C68" s="2">
         <v>6.2691724987101998E-3</v>
       </c>
       <c r="D68">
-        <v>6.0122469256428399E-3</v>
+        <v>2.0004896550590901E-4</v>
       </c>
       <c r="E68">
-        <v>6.2971023902297701E-3</v>
+        <v>2.0519183351723301E-4</v>
       </c>
       <c r="F68" s="10">
         <f t="shared" si="6"/>
-        <v>1.0473792025028101</v>
+        <v>1.0257080460192236</v>
       </c>
       <c r="G68" s="4"/>
       <c r="I68">
-        <v>7.3167786817070497E-3</v>
+        <v>2.47009346021372E-4</v>
       </c>
       <c r="J68">
-        <v>7.7206053021012903E-3</v>
+        <v>2.5056736662623701E-4</v>
       </c>
       <c r="K68" s="10">
         <f t="shared" si="7"/>
-        <v>1.0551918594181156</v>
+        <v>1.0144043966844767</v>
       </c>
     </row>
     <row r="69" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A69" s="4">
-        <v>60</v>
+      <c r="A69">
+        <v>10</v>
       </c>
       <c r="B69" s="5"/>
       <c r="C69" s="2">
         <v>1.2558983712415E-2</v>
       </c>
       <c r="D69">
-        <v>1.2036181905772299E-2</v>
+        <v>1.9727739159685499E-3</v>
       </c>
       <c r="E69">
-        <v>1.26843202591898E-2</v>
-      </c>
-      <c r="F69" s="11">
+        <v>2.1002402963605799E-3</v>
+      </c>
+      <c r="F69" s="10">
         <f t="shared" si="6"/>
-        <v>1.053849165664958</v>
+        <v>1.0646127665011473</v>
       </c>
       <c r="G69" s="4"/>
       <c r="I69">
-        <v>1.4655010559957399E-2</v>
+        <v>2.41443999850058E-3</v>
       </c>
       <c r="J69">
-        <v>1.54708347850845E-2</v>
+        <v>2.5624129143282902E-3</v>
       </c>
       <c r="K69" s="11">
         <f t="shared" si="7"/>
-        <v>1.0556686207621178</v>
+        <v>1.0612866403470804</v>
       </c>
     </row>
     <row r="70" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A70">
-        <v>90</v>
+        <v>25</v>
       </c>
       <c r="B70" s="5"/>
       <c r="C70" s="2">
         <v>1.8782496824776201E-2</v>
       </c>
       <c r="D70">
-        <v>1.81922730031659E-2</v>
+        <v>4.9269907229743297E-3</v>
       </c>
       <c r="E70">
-        <v>1.9125340454343599E-2</v>
+        <v>5.2981099306138504E-3</v>
       </c>
       <c r="F70" s="10">
         <f t="shared" si="6"/>
-        <v>1.051289217736306</v>
+        <v>1.0753237074121145</v>
       </c>
       <c r="G70" s="4"/>
       <c r="I70">
-        <v>2.20520227131588E-2</v>
+        <v>6.11270182240103E-3</v>
       </c>
       <c r="J70">
-        <v>2.3279563002525702E-2</v>
+        <v>6.4145321839513504E-3</v>
       </c>
       <c r="K70" s="10">
         <f t="shared" si="7"/>
-        <v>1.0556656550437167</v>
+        <v>1.0493775699060295</v>
       </c>
     </row>
     <row r="71" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A71" s="4">
-        <v>120</v>
+      <c r="A71">
+        <v>50</v>
       </c>
       <c r="B71" s="5"/>
       <c r="C71" s="2">
         <v>2.51046376970986E-2</v>
       </c>
       <c r="D71">
-        <v>2.42950363565053E-2</v>
+        <v>9.7820010092556295E-3</v>
       </c>
       <c r="E71">
-        <v>2.55954016873969E-2</v>
-      </c>
-      <c r="F71" s="11">
+        <v>1.0195154351149101E-2</v>
+      </c>
+      <c r="F71" s="10">
         <f t="shared" si="6"/>
-        <v>1.0535239096501048</v>
+        <v>1.0422360763919929</v>
       </c>
       <c r="G71" s="4"/>
       <c r="I71">
-        <v>2.9379142051595902E-2</v>
+        <v>1.20970549355645E-2</v>
       </c>
       <c r="J71">
-        <v>3.0966693098777899E-2</v>
+        <v>1.24175942421624E-2</v>
       </c>
       <c r="K71" s="11">
         <f t="shared" si="7"/>
-        <v>1.0540366714723639</v>
+        <v>1.0264973010625533</v>
       </c>
     </row>
     <row r="72" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A72">
-        <v>150</v>
+        <v>75</v>
       </c>
       <c r="B72" s="5"/>
       <c r="C72" s="2">
         <v>3.1476119846668899E-2</v>
       </c>
       <c r="D72">
-        <v>3.0568379602756501E-2</v>
+        <v>1.43763436727791E-2</v>
       </c>
       <c r="E72">
-        <v>3.2160454077141201E-2</v>
+        <v>1.5782984835099299E-2</v>
       </c>
       <c r="F72" s="10">
         <f t="shared" si="6"/>
-        <v>1.0520823967470339</v>
+        <v>1.0978441524727602</v>
       </c>
       <c r="G72" s="4"/>
       <c r="I72">
-        <v>3.6804448452257998E-2</v>
+        <v>1.8002551123509802E-2</v>
       </c>
       <c r="J72">
-        <v>3.8844686371276298E-2</v>
+        <v>1.8976376994297401E-2</v>
       </c>
       <c r="K72" s="10">
         <f t="shared" si="7"/>
-        <v>1.0554345467685748</v>
+        <v>1.0540937706054263</v>
       </c>
     </row>
     <row r="73" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A73" s="4">
-        <v>250</v>
+      <c r="A73">
+        <v>100</v>
       </c>
       <c r="B73" s="5"/>
       <c r="C73" s="2">
         <v>5.2878603388737497E-2</v>
       </c>
       <c r="D73">
-        <v>5.1688372196524002E-2</v>
+        <v>2.00458898906196E-2</v>
       </c>
       <c r="E73">
-        <v>5.4514904682317102E-2</v>
-      </c>
-      <c r="F73" s="11">
+        <v>2.0804120655568799E-2</v>
+      </c>
+      <c r="F73" s="10">
         <f t="shared" si="6"/>
-        <v>1.0546841071923558</v>
+        <v>1.0378247495664441</v>
       </c>
       <c r="G73" s="4"/>
       <c r="I73">
-        <v>6.1567552933483601E-2</v>
+        <v>2.4309982506840501E-2</v>
       </c>
       <c r="J73">
-        <v>6.4958585716827305E-2</v>
+        <v>2.56065505285916E-2</v>
       </c>
       <c r="K73" s="11">
         <f t="shared" si="7"/>
-        <v>1.0550782453057264</v>
+        <v>1.0533347986320543</v>
       </c>
     </row>
     <row r="74" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A74">
-        <v>500</v>
+        <v>150</v>
       </c>
       <c r="B74" s="5"/>
       <c r="C74" s="2">
         <v>0.107716927588289</v>
       </c>
       <c r="D74">
-        <v>0.107312205249392</v>
+        <v>3.0432830381329601E-2</v>
       </c>
       <c r="E74">
-        <v>0.11284726504879</v>
+        <v>3.14434702136525E-2</v>
       </c>
       <c r="F74" s="10">
         <f t="shared" si="6"/>
-        <v>1.0515790332193304</v>
+        <v>1.0332088675177227</v>
       </c>
       <c r="G74" s="4"/>
       <c r="I74">
-        <v>0.124585487877085</v>
+        <v>3.5308084946377202E-2</v>
       </c>
       <c r="J74">
-        <v>0.13088073929294</v>
+        <v>3.7911161854217702E-2</v>
       </c>
       <c r="K74" s="10">
         <f t="shared" si="7"/>
-        <v>1.0505295722890764</v>
+        <v>1.0737246699104135</v>
       </c>
     </row>
     <row r="75" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A75" s="4">
-        <v>750</v>
+      <c r="A75">
+        <v>250</v>
       </c>
       <c r="B75" s="5"/>
       <c r="C75" s="2">
         <v>0.16515386445267599</v>
       </c>
       <c r="D75">
-        <v>0.166593474221475</v>
+        <v>4.89210306757277E-2</v>
       </c>
       <c r="E75">
-        <v>0.17437302973664801</v>
-      </c>
-      <c r="F75" s="11">
+        <v>5.3975920537313898E-2</v>
+      </c>
+      <c r="F75" s="10">
         <f t="shared" si="6"/>
-        <v>1.0466978406658991</v>
+        <v>1.1033275421994369</v>
       </c>
       <c r="G75" s="4"/>
       <c r="I75">
-        <v>0.188315720076114</v>
+        <v>5.8808790512075798E-2</v>
       </c>
       <c r="J75">
-        <v>0.19671890522285099</v>
+        <v>6.2265324575410202E-2</v>
       </c>
       <c r="K75" s="11">
         <f t="shared" si="7"/>
-        <v>1.0446228554012409</v>
+        <v>1.0587758060187387</v>
       </c>
     </row>
     <row r="76" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A76">
-        <v>1000</v>
+        <v>500</v>
       </c>
       <c r="B76" s="5"/>
       <c r="C76" s="2">
         <v>0.22114304090137801</v>
       </c>
       <c r="D76">
-        <v>0.22843742858074301</v>
+        <v>9.6226590649767796E-2</v>
       </c>
       <c r="E76">
-        <v>0.23785710518924499</v>
+        <v>0.10212774105006001</v>
       </c>
       <c r="F76" s="10">
         <f t="shared" si="6"/>
-        <v>1.0412352593312988</v>
+        <v>1.0613255687481478</v>
       </c>
       <c r="G76" s="4"/>
       <c r="I76">
-        <v>0.25212873564071397</v>
+        <v>0.11146020972599301</v>
       </c>
       <c r="J76">
-        <v>0.26159631710660702</v>
+        <v>0.118001707852343</v>
       </c>
       <c r="K76" s="10">
         <f t="shared" si="7"/>
+        <v>1.0586890886212328</v>
+      </c>
+    </row>
+    <row r="77" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A77">
+        <v>750</v>
+      </c>
+      <c r="D77">
+        <v>0.140294088260282</v>
+      </c>
+      <c r="E77">
+        <v>0.15225875418305601</v>
+      </c>
+      <c r="F77" s="10">
+        <f t="shared" si="6"/>
+        <v>1.0852827519045309</v>
+      </c>
+      <c r="I77">
+        <v>0.164782092113922</v>
+      </c>
+      <c r="J77">
+        <v>0.171436913407884</v>
+      </c>
+      <c r="K77" s="11">
+        <f t="shared" si="7"/>
+        <v>1.0403855856458066</v>
+      </c>
+    </row>
+    <row r="78" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A78">
+        <v>999.99</v>
+      </c>
+      <c r="D78">
+        <v>0.181401571560247</v>
+      </c>
+      <c r="E78">
+        <v>0.20058148390920799</v>
+      </c>
+      <c r="F78" s="10">
+        <f t="shared" si="6"/>
+        <v>1.1057317871283765</v>
+      </c>
+      <c r="I78">
+        <v>0.211482254080264</v>
+      </c>
+      <c r="J78">
+        <v>0.22688990016688301</v>
+      </c>
+      <c r="K78" s="10">
+        <f t="shared" si="7"/>
+        <v>1.0728555034256981</v>
+      </c>
+    </row>
+    <row r="80" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="C80" s="12" t="s">
+        <v>10</v>
+      </c>
+      <c r="D80" s="12"/>
+      <c r="E80" s="13"/>
+      <c r="F80" s="13"/>
+      <c r="H80" s="2"/>
+      <c r="I80" s="2"/>
+      <c r="J80" s="2"/>
+      <c r="K80" s="2"/>
+    </row>
+    <row r="81" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="C81" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="D81" s="3"/>
+      <c r="E81" s="9"/>
+      <c r="F81" s="3"/>
+      <c r="H81" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="I81" s="3"/>
+      <c r="J81" s="9"/>
+      <c r="K81" s="9"/>
+    </row>
+    <row r="82" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A82" s="6" t="s">
+        <v>0</v>
+      </c>
+      <c r="B82" s="6"/>
+      <c r="C82" s="6" t="s">
+        <v>1</v>
+      </c>
+      <c r="D82" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="E82" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="F82" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="G82" s="8"/>
+      <c r="H82" s="6" t="s">
+        <v>1</v>
+      </c>
+      <c r="I82" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="J82" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="K82" s="7" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="83" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A83">
+        <v>0.1</v>
+      </c>
+      <c r="B83" s="5"/>
+      <c r="C83" s="2">
+        <v>2.0906018648200899E-5</v>
+      </c>
+      <c r="D83" s="2">
+        <v>2.8143173972499801E-7</v>
+      </c>
+      <c r="E83" s="2">
+        <v>1.46150091119403E-6</v>
+      </c>
+      <c r="F83" s="10">
+        <f t="shared" ref="F83:F94" si="8">F66*((E83/E66)^2 +(D83/D66)^2)^0.5</f>
+        <v>7.5175789820697683E-2</v>
+      </c>
+      <c r="G83" s="4"/>
+      <c r="H83" s="2"/>
+      <c r="I83" s="2">
+        <v>2.4434932696069799E-5</v>
+      </c>
+      <c r="J83" s="2">
+        <v>2.5518609602937599E-5</v>
+      </c>
+      <c r="K83" s="10">
+        <f>J83/I83</f>
+        <v>1.0443494942403546</v>
+      </c>
+    </row>
+    <row r="84" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A84">
+        <v>0.5</v>
+      </c>
+      <c r="B84" s="5"/>
+      <c r="C84" s="2">
+        <v>3.1327203465188001E-3</v>
+      </c>
+      <c r="D84" s="2">
+        <v>1.5222069872849199E-6</v>
+      </c>
+      <c r="E84" s="2">
+        <v>3.7622530224669299E-6</v>
+      </c>
+      <c r="F84" s="10">
+        <f t="shared" si="8"/>
+        <v>3.9379446327356661E-2</v>
+      </c>
+      <c r="G84" s="4"/>
+      <c r="I84">
+        <v>3.6561489620800698E-3</v>
+      </c>
+      <c r="J84">
+        <v>3.8583728177792702E-3</v>
+      </c>
+      <c r="K84" s="11">
+        <f t="shared" ref="K84:K93" si="9">J84/I84</f>
+        <v>1.0553106172085915</v>
+      </c>
+    </row>
+    <row r="85" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A85">
+        <v>1</v>
+      </c>
+      <c r="B85" s="5"/>
+      <c r="C85" s="2">
+        <v>6.2691724987101998E-3</v>
+      </c>
+      <c r="D85" s="2">
+        <v>2.33807312394273E-6</v>
+      </c>
+      <c r="E85" s="2">
+        <v>6.5127278910264096E-6</v>
+      </c>
+      <c r="F85" s="10">
+        <f t="shared" si="8"/>
+        <v>3.4692692812303069E-2</v>
+      </c>
+      <c r="G85" s="4"/>
+      <c r="I85">
+        <v>7.3167786817070497E-3</v>
+      </c>
+      <c r="J85">
+        <v>7.7206053021012903E-3</v>
+      </c>
+      <c r="K85" s="10">
+        <f t="shared" si="9"/>
+        <v>1.0551918594181156</v>
+      </c>
+    </row>
+    <row r="86" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A86">
+        <v>10</v>
+      </c>
+      <c r="B86" s="5"/>
+      <c r="C86" s="2">
+        <v>1.2558983712415E-2</v>
+      </c>
+      <c r="D86" s="2">
+        <v>2.7701090496064399E-5</v>
+      </c>
+      <c r="E86" s="2">
+        <v>3.8011060965548303E-5</v>
+      </c>
+      <c r="F86" s="10">
+        <f t="shared" si="8"/>
+        <v>2.4386896067040687E-2</v>
+      </c>
+      <c r="G86" s="4"/>
+      <c r="I86">
+        <v>1.4655010559957399E-2</v>
+      </c>
+      <c r="J86">
+        <v>1.54708347850845E-2</v>
+      </c>
+      <c r="K86" s="11">
+        <f t="shared" si="9"/>
+        <v>1.0556686207621178</v>
+      </c>
+    </row>
+    <row r="87" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A87">
+        <v>25</v>
+      </c>
+      <c r="B87" s="5"/>
+      <c r="C87" s="2">
+        <v>1.8782496824776201E-2</v>
+      </c>
+      <c r="D87" s="2">
+        <v>8.0985715172972504E-5</v>
+      </c>
+      <c r="E87" s="2">
+        <v>8.2936422592517207E-5</v>
+      </c>
+      <c r="F87" s="10">
+        <f t="shared" si="8"/>
+        <v>2.4408348565916203E-2</v>
+      </c>
+      <c r="G87" s="4"/>
+      <c r="I87">
+        <v>2.20520227131588E-2</v>
+      </c>
+      <c r="J87">
+        <v>2.3279563002525702E-2</v>
+      </c>
+      <c r="K87" s="10">
+        <f t="shared" si="9"/>
+        <v>1.0556656550437167</v>
+      </c>
+    </row>
+    <row r="88" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A88">
+        <v>50</v>
+      </c>
+      <c r="B88" s="5"/>
+      <c r="C88" s="2">
+        <v>2.51046376970986E-2</v>
+      </c>
+      <c r="D88">
+        <v>1.14857385321631E-4</v>
+      </c>
+      <c r="E88">
+        <v>1.40546480514001E-4</v>
+      </c>
+      <c r="F88" s="10">
+        <f t="shared" si="8"/>
+        <v>1.8873133491714433E-2</v>
+      </c>
+      <c r="G88" s="4"/>
+      <c r="I88">
+        <v>2.9379142051595902E-2</v>
+      </c>
+      <c r="J88">
+        <v>3.0966693098777899E-2</v>
+      </c>
+      <c r="K88" s="11">
+        <f t="shared" si="9"/>
+        <v>1.0540366714723639</v>
+      </c>
+    </row>
+    <row r="89" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A89">
+        <v>75</v>
+      </c>
+      <c r="B89" s="5"/>
+      <c r="C89" s="2">
+        <v>3.1476119846668899E-2</v>
+      </c>
+      <c r="D89">
+        <v>1.6692001786006801E-4</v>
+      </c>
+      <c r="E89">
+        <v>2.2355768083561999E-4</v>
+      </c>
+      <c r="F89" s="10">
+        <f t="shared" si="8"/>
+        <v>2.0107088599017175E-2</v>
+      </c>
+      <c r="G89" s="4"/>
+      <c r="I89">
+        <v>3.6804448452257998E-2</v>
+      </c>
+      <c r="J89">
+        <v>3.8844686371276298E-2</v>
+      </c>
+      <c r="K89" s="10">
+        <f t="shared" si="9"/>
+        <v>1.0554345467685748</v>
+      </c>
+    </row>
+    <row r="90" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A90">
+        <v>100</v>
+      </c>
+      <c r="B90" s="5"/>
+      <c r="C90" s="2">
+        <v>5.2878603388737497E-2</v>
+      </c>
+      <c r="D90">
+        <v>2.77931449091848E-4</v>
+      </c>
+      <c r="E90">
+        <v>2.1739476286188801E-4</v>
+      </c>
+      <c r="F90" s="10">
+        <f t="shared" si="8"/>
+        <v>1.8018315350781095E-2</v>
+      </c>
+      <c r="G90" s="4"/>
+      <c r="I90">
+        <v>6.1567552933483601E-2</v>
+      </c>
+      <c r="J90">
+        <v>6.4958585716827305E-2</v>
+      </c>
+      <c r="K90" s="11">
+        <f t="shared" si="9"/>
+        <v>1.0550782453057264</v>
+      </c>
+    </row>
+    <row r="91" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A91">
+        <v>150</v>
+      </c>
+      <c r="B91" s="5"/>
+      <c r="C91" s="2">
+        <v>0.107716927588289</v>
+      </c>
+      <c r="D91">
+        <v>3.3888866496247497E-4</v>
+      </c>
+      <c r="E91">
+        <v>4.2099807481717899E-4</v>
+      </c>
+      <c r="F91" s="10">
+        <f t="shared" si="8"/>
+        <v>1.7992932963347683E-2</v>
+      </c>
+      <c r="G91" s="4"/>
+      <c r="I91">
+        <v>0.124585487877085</v>
+      </c>
+      <c r="J91">
+        <v>0.13088073929294</v>
+      </c>
+      <c r="K91" s="10">
+        <f t="shared" si="9"/>
+        <v>1.0505295722890764</v>
+      </c>
+    </row>
+    <row r="92" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A92">
+        <v>250</v>
+      </c>
+      <c r="B92" s="5"/>
+      <c r="C92" s="2">
+        <v>0.16515386445267599</v>
+      </c>
+      <c r="D92">
+        <v>6.0844630496931901E-4</v>
+      </c>
+      <c r="E92">
+        <v>7.1735921087181002E-4</v>
+      </c>
+      <c r="F92" s="10">
+        <f t="shared" si="8"/>
+        <v>2.0082997872230529E-2</v>
+      </c>
+      <c r="G92" s="4"/>
+      <c r="I92">
+        <v>0.188315720076114</v>
+      </c>
+      <c r="J92">
+        <v>0.19671890522285099</v>
+      </c>
+      <c r="K92" s="11">
+        <f t="shared" si="9"/>
+        <v>1.0446228554012409</v>
+      </c>
+    </row>
+    <row r="93" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A93">
+        <v>500</v>
+      </c>
+      <c r="B93" s="5"/>
+      <c r="C93" s="2">
+        <v>0.22114304090137801</v>
+      </c>
+      <c r="D93">
+        <v>1.3901143553867799E-3</v>
+      </c>
+      <c r="E93">
+        <v>1.45703989958587E-3</v>
+      </c>
+      <c r="F93" s="10">
+        <f t="shared" si="8"/>
+        <v>2.1548753693625213E-2</v>
+      </c>
+      <c r="G93" s="4"/>
+      <c r="I93">
+        <v>0.25212873564071397</v>
+      </c>
+      <c r="J93">
+        <v>0.26159631710660702</v>
+      </c>
+      <c r="K93" s="10">
+        <f t="shared" si="9"/>
         <v>1.0375505847908761</v>
+      </c>
+    </row>
+    <row r="94" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A94">
+        <v>750</v>
+      </c>
+      <c r="D94">
+        <v>1.59024586083695E-3</v>
+      </c>
+      <c r="E94">
+        <v>1.88927153592098E-3</v>
+      </c>
+      <c r="F94" s="10">
+        <f t="shared" si="8"/>
+        <v>1.8239532257896197E-2</v>
+      </c>
+    </row>
+    <row r="95" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A95">
+        <v>999.99</v>
+      </c>
+      <c r="D95">
+        <v>2.0916951916344802E-3</v>
+      </c>
+      <c r="E95">
+        <v>2.14759074882869E-3</v>
+      </c>
+      <c r="F95" s="10">
+        <f>F78*((E95/E78)^2 +(D95/D78)^2)^0.5</f>
+        <v>1.7398828006913617E-2</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
hcpb renamed and data updated
</commit_message>
<xml_diff>
--- a/Jupyter/Wedge/wedge_data_2026-03-25.xlsx
+++ b/Jupyter/Wedge/wedge_data_2026-03-25.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\patri\projects\emma-openmc\Jupyter\Wedge\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7B184866-94F8-47FB-9604-EE9CD1C46C89}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BDAEB268-8B64-460D-9E40-EF1FACC7331B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="17496" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -274,10 +274,10 @@
           </c:marker>
           <c:xVal>
             <c:numRef>
-              <c:f>'Sheet 1'!$A$26:$A$40</c:f>
+              <c:f>'Sheet 1'!$A$24:$A$36</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="15"/>
+                <c:ptCount val="13"/>
                 <c:pt idx="0">
                   <c:v>0.1</c:v>
                 </c:pt>
@@ -285,97 +285,85 @@
                   <c:v>0.5</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>1.5</c:v>
+                  <c:v>1</c:v>
                 </c:pt>
                 <c:pt idx="3">
                   <c:v>10</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>15</c:v>
+                  <c:v>25</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>30</c:v>
+                  <c:v>50</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>60</c:v>
+                  <c:v>75</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>90</c:v>
+                  <c:v>100</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>100</c:v>
+                  <c:v>150</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>120</c:v>
+                  <c:v>250</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>150</c:v>
+                  <c:v>500</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>250</c:v>
+                  <c:v>750</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>500</c:v>
-                </c:pt>
-                <c:pt idx="13">
-                  <c:v>750</c:v>
-                </c:pt>
-                <c:pt idx="14">
-                  <c:v>1000</c:v>
+                  <c:v>999.99</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>'Sheet 1'!$F$26:$F$40</c:f>
+              <c:f>'Sheet 1'!$F$24:$F$36</c:f>
               <c:numCache>
                 <c:formatCode>0.000000</c:formatCode>
-                <c:ptCount val="15"/>
+                <c:ptCount val="13"/>
                 <c:pt idx="0">
-                  <c:v>0.7274775745944605</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0.64347975683918834</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>0.49583688440425344</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>0.66859607525333198</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>0.73291562987349301</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>0.74746751893992558</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>0.78627670393149318</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>0.87619376520123537</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>0.86809490045634352</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>0.79255474288640204</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>0.90551396638088599</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>0.92837643974491146</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>0.93787715524054671</c:v>
-                </c:pt>
-                <c:pt idx="13">
-                  <c:v>1.0174259839976012</c:v>
-                </c:pt>
-                <c:pt idx="14">
-                  <c:v>1.0246283267351703</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -414,10 +402,10 @@
           </c:marker>
           <c:xVal>
             <c:numRef>
-              <c:f>'Sheet 1'!$A$26:$A$40</c:f>
+              <c:f>'Sheet 1'!$A$24:$A$36</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="15"/>
+                <c:ptCount val="13"/>
                 <c:pt idx="0">
                   <c:v>0.1</c:v>
                 </c:pt>
@@ -425,97 +413,85 @@
                   <c:v>0.5</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>1.5</c:v>
+                  <c:v>1</c:v>
                 </c:pt>
                 <c:pt idx="3">
                   <c:v>10</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>15</c:v>
+                  <c:v>25</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>30</c:v>
+                  <c:v>50</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>60</c:v>
+                  <c:v>75</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>90</c:v>
+                  <c:v>100</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>100</c:v>
+                  <c:v>150</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>120</c:v>
+                  <c:v>250</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>150</c:v>
+                  <c:v>500</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>250</c:v>
+                  <c:v>750</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>500</c:v>
-                </c:pt>
-                <c:pt idx="13">
-                  <c:v>750</c:v>
-                </c:pt>
-                <c:pt idx="14">
-                  <c:v>1000</c:v>
+                  <c:v>999.99</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>'Sheet 1'!$K$26:$K$40</c:f>
+              <c:f>'Sheet 1'!$K$24:$K$36</c:f>
               <c:numCache>
                 <c:formatCode>0.000000</c:formatCode>
-                <c:ptCount val="15"/>
+                <c:ptCount val="13"/>
                 <c:pt idx="0">
-                  <c:v>0.29264705217301878</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>1.3315375295667062</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>0.8971337860952534</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>0.86727127408207016</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>0.96019947785672299</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>0.82054207267800461</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>0.89620098412984728</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>0.99789498609321658</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>0.92546657383389286</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>0.95340718196328889</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>0.94899688560909901</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>0.9624346474925255</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>1.0215461604572156</c:v>
-                </c:pt>
-                <c:pt idx="13">
-                  <c:v>1.0753115641669349</c:v>
-                </c:pt>
-                <c:pt idx="14">
-                  <c:v>1.0025476893384362</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -874,10 +850,10 @@
           </c:trendline>
           <c:xVal>
             <c:numRef>
-              <c:f>'Sheet 1'!$A$5:$A$19</c:f>
+              <c:f>'Sheet 1'!$A$5:$A$17</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="15"/>
+                <c:ptCount val="13"/>
                 <c:pt idx="0">
                   <c:v>0.1</c:v>
                 </c:pt>
@@ -885,42 +861,36 @@
                   <c:v>0.5</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>1.5</c:v>
+                  <c:v>1</c:v>
                 </c:pt>
                 <c:pt idx="3">
                   <c:v>10</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>15</c:v>
+                  <c:v>25</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>30</c:v>
+                  <c:v>50</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>60</c:v>
+                  <c:v>75</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>90</c:v>
+                  <c:v>100</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>100</c:v>
+                  <c:v>150</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>120</c:v>
+                  <c:v>250</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>150</c:v>
+                  <c:v>500</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>250</c:v>
+                  <c:v>750</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>500</c:v>
-                </c:pt>
-                <c:pt idx="13">
-                  <c:v>750</c:v>
-                </c:pt>
-                <c:pt idx="14">
                   <c:v>999.99</c:v>
                 </c:pt>
               </c:numCache>
@@ -928,54 +898,48 @@
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>'Sheet 1'!$F$5:$F$19</c:f>
+              <c:f>'Sheet 1'!$F$5:$F$17</c:f>
               <c:numCache>
                 <c:formatCode>0.000000</c:formatCode>
-                <c:ptCount val="15"/>
+                <c:ptCount val="13"/>
                 <c:pt idx="0">
-                  <c:v>1.0120583199660715</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0.98723674640081305</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>0.97352011835670349</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>0.98670947182667379</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>1.0274179661023068</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>0.9995818870330847</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>1.0035538292803527</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>1.0225693897940391</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>1.0133855529616367</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>1.0168926589087053</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>1.0023371440138709</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>0.99143857028386306</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>0.99628894469879192</c:v>
-                </c:pt>
-                <c:pt idx="13">
-                  <c:v>1.0133076136706871</c:v>
-                </c:pt>
-                <c:pt idx="14">
-                  <c:v>0.98894242420015732</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1065,10 +1029,10 @@
           </c:trendline>
           <c:xVal>
             <c:numRef>
-              <c:f>'Sheet 1'!$A$5:$A$19</c:f>
+              <c:f>'Sheet 1'!$A$5:$A$17</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="15"/>
+                <c:ptCount val="13"/>
                 <c:pt idx="0">
                   <c:v>0.1</c:v>
                 </c:pt>
@@ -1076,42 +1040,36 @@
                   <c:v>0.5</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>1.5</c:v>
+                  <c:v>1</c:v>
                 </c:pt>
                 <c:pt idx="3">
                   <c:v>10</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>15</c:v>
+                  <c:v>25</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>30</c:v>
+                  <c:v>50</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>60</c:v>
+                  <c:v>75</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>90</c:v>
+                  <c:v>100</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>100</c:v>
+                  <c:v>150</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>120</c:v>
+                  <c:v>250</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>150</c:v>
+                  <c:v>500</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>250</c:v>
+                  <c:v>750</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>500</c:v>
-                </c:pt>
-                <c:pt idx="13">
-                  <c:v>750</c:v>
-                </c:pt>
-                <c:pt idx="14">
                   <c:v>999.99</c:v>
                 </c:pt>
               </c:numCache>
@@ -1119,54 +1077,48 @@
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>'Sheet 1'!$K$5:$K$19</c:f>
+              <c:f>'Sheet 1'!$K$5:$K$17</c:f>
               <c:numCache>
                 <c:formatCode>0.000000</c:formatCode>
-                <c:ptCount val="15"/>
+                <c:ptCount val="13"/>
                 <c:pt idx="0">
-                  <c:v>1.0124595607074192</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0.98955684846579572</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>0.97266576371713243</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>0.99532217045916183</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>1.0246126531897757</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>0.99123212311197628</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>1.0019803232436455</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>1.0235838898658773</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>1.0328136474978709</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>0.99238859087523068</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>1.0068419602917082</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>1.0041778550412717</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>1.0147327958753034</c:v>
-                </c:pt>
-                <c:pt idx="13">
-                  <c:v>1.0192489706741765</c:v>
-                </c:pt>
-                <c:pt idx="14">
-                  <c:v>0.9824392574158276</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1451,7 +1403,7 @@
           <c:order val="0"/>
           <c:tx>
             <c:strRef>
-              <c:f>'Sheet 1'!$F$65</c:f>
+              <c:f>'Sheet 1'!$F$61</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -1484,7 +1436,7 @@
           </c:marker>
           <c:xVal>
             <c:numRef>
-              <c:f>'Sheet 1'!$A$66:$A$76</c:f>
+              <c:f>'Sheet 1'!$A$62:$A$72</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="11"/>
@@ -1526,7 +1478,7 @@
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>'Sheet 1'!$F$66:$F$76</c:f>
+              <c:f>'Sheet 1'!$F$62:$F$72</c:f>
               <c:numCache>
                 <c:formatCode>0.000000</c:formatCode>
                 <c:ptCount val="11"/>
@@ -1815,7 +1767,7 @@
           <c:order val="0"/>
           <c:tx>
             <c:strRef>
-              <c:f>'Sheet 1'!$F$47</c:f>
+              <c:f>'Sheet 1'!$F$43</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -1848,7 +1800,7 @@
           </c:marker>
           <c:xVal>
             <c:numRef>
-              <c:f>'Sheet 1'!$A$48:$A$58</c:f>
+              <c:f>'Sheet 1'!$A$44:$A$54</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="11"/>
@@ -1890,7 +1842,7 @@
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>'Sheet 1'!$F$48:$F$58</c:f>
+              <c:f>'Sheet 1'!$F$44:$F$54</c:f>
               <c:numCache>
                 <c:formatCode>0.000000</c:formatCode>
                 <c:ptCount val="11"/>
@@ -4354,13 +4306,13 @@
     <xdr:from>
       <xdr:col>12</xdr:col>
       <xdr:colOff>132179</xdr:colOff>
-      <xdr:row>22</xdr:row>
+      <xdr:row>20</xdr:row>
       <xdr:rowOff>56857</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>19</xdr:col>
       <xdr:colOff>436979</xdr:colOff>
-      <xdr:row>41</xdr:row>
+      <xdr:row>37</xdr:row>
       <xdr:rowOff>56857</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
@@ -4396,8 +4348,8 @@
     <xdr:to>
       <xdr:col>19</xdr:col>
       <xdr:colOff>605790</xdr:colOff>
-      <xdr:row>18</xdr:row>
-      <xdr:rowOff>99060</xdr:rowOff>
+      <xdr:row>17</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
@@ -4426,13 +4378,13 @@
     <xdr:from>
       <xdr:col>11</xdr:col>
       <xdr:colOff>868680</xdr:colOff>
-      <xdr:row>61</xdr:row>
+      <xdr:row>57</xdr:row>
       <xdr:rowOff>76200</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>19</xdr:col>
       <xdr:colOff>198120</xdr:colOff>
-      <xdr:row>76</xdr:row>
+      <xdr:row>72</xdr:row>
       <xdr:rowOff>76200</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
@@ -4462,13 +4414,13 @@
     <xdr:from>
       <xdr:col>11</xdr:col>
       <xdr:colOff>929640</xdr:colOff>
-      <xdr:row>44</xdr:row>
+      <xdr:row>40</xdr:row>
       <xdr:rowOff>7620</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>19</xdr:col>
       <xdr:colOff>259080</xdr:colOff>
-      <xdr:row>60</xdr:row>
+      <xdr:row>56</xdr:row>
       <xdr:rowOff>7620</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
@@ -4760,7 +4712,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C22416C2-1180-4450-A3B0-0B08DD9AEC85}">
-  <dimension ref="A1:L95"/>
+  <dimension ref="A1:L91"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="12.33203125" customWidth="1"/>
@@ -4842,32 +4794,17 @@
         <v>0.1</v>
       </c>
       <c r="B5" s="5"/>
-      <c r="C5">
-        <v>1.4063862998066801</v>
-      </c>
-      <c r="D5">
-        <v>1.3686193553583801</v>
-      </c>
       <c r="E5">
-        <v>1.38512260545705</v>
-      </c>
-      <c r="F5" s="10">
+        <v>1.38933589370449</v>
+      </c>
+      <c r="F5" s="10" t="e">
         <f>E5/D5</f>
-        <v>1.0120583199660715</v>
+        <v>#DIV/0!</v>
       </c>
       <c r="G5" s="4"/>
-      <c r="H5">
-        <v>1.4074651112049299</v>
-      </c>
-      <c r="I5">
-        <v>1.3681177802680899</v>
-      </c>
-      <c r="J5">
-        <v>1.3851639268062399</v>
-      </c>
-      <c r="K5" s="10">
+      <c r="K5" s="10" t="e">
         <f>J5/I5</f>
-        <v>1.0124595607074192</v>
+        <v>#DIV/0!</v>
       </c>
       <c r="L5" s="10"/>
     </row>
@@ -4876,66 +4813,36 @@
         <v>0.5</v>
       </c>
       <c r="B6" s="5"/>
-      <c r="C6">
-        <v>1.4065448393936499</v>
-      </c>
-      <c r="D6">
-        <v>1.3922831524096599</v>
-      </c>
       <c r="E6">
-        <v>1.37451308945358</v>
-      </c>
-      <c r="F6" s="10">
-        <f t="shared" ref="F6:F19" si="0">E6/D6</f>
-        <v>0.98723674640081305</v>
+        <v>1.3891670563732801</v>
+      </c>
+      <c r="F6" s="10" t="e">
+        <f t="shared" ref="F6:F17" si="0">E6/D6</f>
+        <v>#DIV/0!</v>
       </c>
       <c r="G6" s="4"/>
-      <c r="H6">
-        <v>1.4079920998080599</v>
-      </c>
-      <c r="I6">
-        <v>1.3884228746446901</v>
-      </c>
-      <c r="J6">
-        <v>1.3739233641712201</v>
-      </c>
-      <c r="K6" s="10">
-        <f t="shared" ref="K6:K19" si="1">J6/I6</f>
-        <v>0.98955684846579572</v>
+      <c r="K6" s="10" t="e">
+        <f t="shared" ref="K6:K17" si="1">J6/I6</f>
+        <v>#DIV/0!</v>
       </c>
       <c r="L6" s="10"/>
     </row>
     <row r="7" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A7">
-        <v>1.5</v>
+        <v>1</v>
       </c>
       <c r="B7" s="5"/>
-      <c r="C7">
-        <v>1.40593053429746</v>
-      </c>
-      <c r="D7">
-        <v>1.4141178954362701</v>
-      </c>
       <c r="E7">
-        <v>1.3766722209354501</v>
-      </c>
-      <c r="F7" s="10">
+        <v>1.3888589124812201</v>
+      </c>
+      <c r="F7" s="10" t="e">
         <f t="shared" si="0"/>
-        <v>0.97352011835670349</v>
+        <v>#DIV/0!</v>
       </c>
       <c r="G7" s="4"/>
-      <c r="H7">
-        <v>1.4079445884292401</v>
-      </c>
-      <c r="I7">
-        <v>1.4147283449213399</v>
-      </c>
-      <c r="J7">
-        <v>1.3760578260651899</v>
-      </c>
-      <c r="K7" s="10">
+      <c r="K7" s="10" t="e">
         <f t="shared" si="1"/>
-        <v>0.97266576371713243</v>
+        <v>#DIV/0!</v>
       </c>
       <c r="L7" s="10"/>
     </row>
@@ -4944,2264 +4851,1809 @@
         <v>10</v>
       </c>
       <c r="B8" s="5"/>
-      <c r="C8">
-        <v>1.39838837861919</v>
-      </c>
-      <c r="D8">
-        <v>1.4052374449883001</v>
-      </c>
       <c r="E8">
-        <v>1.38656109713547</v>
-      </c>
-      <c r="F8" s="10">
+        <v>1.3868055893142199</v>
+      </c>
+      <c r="F8" s="10" t="e">
         <f t="shared" si="0"/>
-        <v>0.98670947182667379</v>
+        <v>#DIV/0!</v>
       </c>
       <c r="G8" s="4"/>
-      <c r="H8">
-        <v>1.4018754625880101</v>
-      </c>
-      <c r="I8">
-        <v>1.3952787310994501</v>
-      </c>
-      <c r="J8">
-        <v>1.3887518550334099</v>
-      </c>
-      <c r="K8" s="10">
+      <c r="K8" s="10" t="e">
         <f t="shared" si="1"/>
-        <v>0.99532217045916183</v>
+        <v>#DIV/0!</v>
       </c>
       <c r="L8" s="10"/>
     </row>
     <row r="9" spans="1:12" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A9">
-        <v>15</v>
+        <v>25</v>
       </c>
       <c r="B9" s="5"/>
-      <c r="C9">
-        <v>1.39742877901721</v>
-      </c>
-      <c r="D9">
-        <v>1.3588321367490299</v>
-      </c>
+      <c r="C9"/>
+      <c r="D9"/>
       <c r="E9">
-        <v>1.3960885502131399</v>
-      </c>
-      <c r="F9" s="10">
+        <v>1.3820193582140401</v>
+      </c>
+      <c r="F9" s="10" t="e">
         <f t="shared" si="0"/>
-        <v>1.0274179661023068</v>
-      </c>
-      <c r="H9">
-        <v>1.4018991482118599</v>
-      </c>
-      <c r="I9">
-        <v>1.36086238814935</v>
-      </c>
-      <c r="J9">
-        <v>1.3943568221478799</v>
-      </c>
-      <c r="K9" s="10">
+        <v>#DIV/0!</v>
+      </c>
+      <c r="H9"/>
+      <c r="I9"/>
+      <c r="J9"/>
+      <c r="K9" s="10" t="e">
         <f t="shared" si="1"/>
-        <v>1.0246126531897757</v>
+        <v>#DIV/0!</v>
       </c>
       <c r="L9" s="11"/>
     </row>
     <row r="10" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A10">
-        <v>30</v>
+        <v>50</v>
       </c>
       <c r="B10" s="5"/>
-      <c r="C10">
-        <v>1.3977734656963801</v>
-      </c>
-      <c r="D10">
-        <v>1.38084479180245</v>
-      </c>
       <c r="E10">
-        <v>1.3802674426896999</v>
-      </c>
-      <c r="F10" s="10">
+        <v>1.3754575654543499</v>
+      </c>
+      <c r="F10" s="10" t="e">
         <f t="shared" si="0"/>
-        <v>0.9995818870330847</v>
+        <v>#DIV/0!</v>
       </c>
       <c r="G10" s="4"/>
-      <c r="H10">
-        <v>1.3914317207496001</v>
-      </c>
-      <c r="I10">
-        <v>1.3852911212816701</v>
-      </c>
-      <c r="J10">
-        <v>1.3731450592762</v>
-      </c>
-      <c r="K10" s="10">
+      <c r="K10" s="10" t="e">
         <f t="shared" si="1"/>
-        <v>0.99123212311197628</v>
+        <v>#DIV/0!</v>
       </c>
       <c r="L10" s="10"/>
     </row>
     <row r="11" spans="1:12" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A11">
-        <v>60</v>
+        <v>75</v>
       </c>
       <c r="B11" s="5"/>
-      <c r="C11">
-        <v>1.39314164652525</v>
-      </c>
-      <c r="D11">
-        <v>1.35391575819657</v>
-      </c>
+      <c r="C11"/>
+      <c r="D11"/>
       <c r="E11">
-        <v>1.35872734366118</v>
-      </c>
-      <c r="F11" s="10">
+        <v>1.37040384545697</v>
+      </c>
+      <c r="F11" s="10" t="e">
         <f t="shared" si="0"/>
-        <v>1.0035538292803527</v>
-      </c>
-      <c r="H11">
-        <v>1.3881975250755401</v>
-      </c>
-      <c r="I11">
-        <v>1.3558315843768101</v>
-      </c>
-      <c r="J11">
-        <v>1.35851656917782</v>
-      </c>
-      <c r="K11" s="10">
+        <v>#DIV/0!</v>
+      </c>
+      <c r="H11"/>
+      <c r="I11"/>
+      <c r="J11"/>
+      <c r="K11" s="10" t="e">
         <f t="shared" si="1"/>
-        <v>1.0019803232436455</v>
+        <v>#DIV/0!</v>
       </c>
       <c r="L11" s="11"/>
     </row>
     <row r="12" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A12">
-        <v>90</v>
+        <v>100</v>
       </c>
       <c r="B12" s="5"/>
-      <c r="C12">
-        <v>1.3818447189929399</v>
-      </c>
-      <c r="D12">
-        <v>1.3540665504448699</v>
-      </c>
       <c r="E12">
-        <v>1.3846270062289301</v>
-      </c>
-      <c r="F12" s="10">
+        <v>1.3649754350071801</v>
+      </c>
+      <c r="F12" s="10" t="e">
         <f t="shared" si="0"/>
-        <v>1.0225693897940391</v>
+        <v>#DIV/0!</v>
       </c>
       <c r="G12" s="4"/>
-      <c r="H12">
-        <v>1.3733638983322201</v>
-      </c>
-      <c r="I12">
-        <v>1.34423803647162</v>
-      </c>
-      <c r="J12">
-        <v>1.37594039827729</v>
-      </c>
-      <c r="K12" s="10">
+      <c r="K12" s="10" t="e">
         <f t="shared" si="1"/>
-        <v>1.0235838898658773</v>
+        <v>#DIV/0!</v>
       </c>
       <c r="L12" s="10"/>
     </row>
     <row r="13" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A13">
-        <v>100</v>
+        <v>150</v>
       </c>
       <c r="B13" s="5"/>
-      <c r="C13">
-        <v>1.37950613179578</v>
-      </c>
-      <c r="D13">
-        <v>1.3565730983264299</v>
-      </c>
       <c r="E13">
-        <v>1.37473157938041</v>
-      </c>
-      <c r="F13" s="10">
+        <v>1.35044101904588</v>
+      </c>
+      <c r="F13" s="10" t="e">
         <f t="shared" si="0"/>
-        <v>1.0133855529616367</v>
+        <v>#DIV/0!</v>
       </c>
       <c r="G13" s="4"/>
-      <c r="H13">
-        <v>1.3697423426526301</v>
-      </c>
-      <c r="I13">
-        <v>1.3294388930292</v>
-      </c>
-      <c r="J13">
-        <v>1.3730626322350199</v>
-      </c>
-      <c r="K13" s="10">
+      <c r="K13" s="10" t="e">
         <f t="shared" si="1"/>
-        <v>1.0328136474978709</v>
+        <v>#DIV/0!</v>
       </c>
       <c r="L13" s="10"/>
     </row>
     <row r="14" spans="1:12" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A14">
-        <v>120</v>
+        <v>250</v>
       </c>
       <c r="B14" s="5"/>
-      <c r="C14">
-        <v>1.37505741757767</v>
-      </c>
-      <c r="D14">
-        <v>1.34077916991197</v>
-      </c>
+      <c r="C14"/>
+      <c r="D14"/>
       <c r="E14">
-        <v>1.3634284951011899</v>
-      </c>
-      <c r="F14" s="10">
+        <v>1.3309639224463901</v>
+      </c>
+      <c r="F14" s="10" t="e">
         <f t="shared" si="0"/>
-        <v>1.0168926589087053</v>
-      </c>
-      <c r="H14">
-        <v>1.36267435359262</v>
-      </c>
-      <c r="I14">
-        <v>1.35581073898229</v>
-      </c>
-      <c r="J14">
-        <v>1.34549110875214</v>
-      </c>
-      <c r="K14" s="10">
+        <v>#DIV/0!</v>
+      </c>
+      <c r="H14"/>
+      <c r="I14"/>
+      <c r="J14"/>
+      <c r="K14" s="10" t="e">
         <f t="shared" si="1"/>
-        <v>0.99238859087523068</v>
+        <v>#DIV/0!</v>
       </c>
       <c r="L14" s="11"/>
     </row>
     <row r="15" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A15">
-        <v>150</v>
+        <v>500</v>
       </c>
       <c r="B15" s="5"/>
-      <c r="C15">
-        <v>1.3614670031018901</v>
-      </c>
-      <c r="D15">
-        <v>1.3628583617894401</v>
-      </c>
       <c r="E15">
-        <v>1.3660435580514501</v>
-      </c>
-      <c r="F15" s="10">
+        <v>1.2901507582212099</v>
+      </c>
+      <c r="F15" s="10" t="e">
         <f t="shared" si="0"/>
-        <v>1.0023371440138709</v>
+        <v>#DIV/0!</v>
       </c>
       <c r="G15" s="4"/>
-      <c r="H15">
-        <v>1.3561935884492</v>
-      </c>
-      <c r="I15">
-        <v>1.34642475596859</v>
-      </c>
-      <c r="J15">
-        <v>1.3556369406847</v>
-      </c>
-      <c r="K15" s="10">
+      <c r="K15" s="10" t="e">
         <f t="shared" si="1"/>
-        <v>1.0068419602917082</v>
+        <v>#DIV/0!</v>
       </c>
       <c r="L15" s="10"/>
     </row>
     <row r="16" spans="1:12" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A16">
-        <v>250</v>
+        <v>750</v>
       </c>
       <c r="B16" s="5"/>
-      <c r="C16">
-        <v>1.3422623387583901</v>
-      </c>
-      <c r="D16">
-        <v>1.31238054231434</v>
-      </c>
+      <c r="C16"/>
+      <c r="D16"/>
       <c r="E16">
-        <v>1.30114468854049</v>
-      </c>
-      <c r="F16" s="10">
+        <v>1.2537253487050199</v>
+      </c>
+      <c r="F16" s="10" t="e">
         <f t="shared" si="0"/>
-        <v>0.99143857028386306</v>
-      </c>
-      <c r="H16">
-        <v>1.3247863550055301</v>
-      </c>
-      <c r="I16">
-        <v>1.2854468687873799</v>
-      </c>
-      <c r="J16">
-        <v>1.2908172794684301</v>
-      </c>
-      <c r="K16" s="10">
+        <v>#DIV/0!</v>
+      </c>
+      <c r="H16"/>
+      <c r="I16"/>
+      <c r="J16"/>
+      <c r="K16" s="10" t="e">
         <f t="shared" si="1"/>
-        <v>1.0041778550412717</v>
+        <v>#DIV/0!</v>
       </c>
       <c r="L16" s="11"/>
     </row>
     <row r="17" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A17">
-        <v>500</v>
+        <v>999.99</v>
       </c>
       <c r="B17" s="5"/>
-      <c r="C17">
-        <v>1.3014014859735601</v>
-      </c>
-      <c r="D17">
-        <v>1.27106900787611</v>
-      </c>
       <c r="E17">
-        <v>1.2663520004962301</v>
-      </c>
-      <c r="F17" s="10">
+        <v>1.2163442531022399</v>
+      </c>
+      <c r="F17" s="10" t="e">
         <f t="shared" si="0"/>
-        <v>0.99628894469879192</v>
+        <v>#DIV/0!</v>
       </c>
       <c r="G17" s="4"/>
-      <c r="H17">
-        <v>1.26268865444005</v>
-      </c>
-      <c r="I17">
-        <v>1.24215702849295</v>
-      </c>
-      <c r="J17">
-        <v>1.26045747443881</v>
-      </c>
-      <c r="K17" s="10">
+      <c r="K17" s="10" t="e">
         <f t="shared" si="1"/>
-        <v>1.0147327958753034</v>
+        <v>#DIV/0!</v>
       </c>
       <c r="L17" s="10"/>
     </row>
-    <row r="18" spans="1:12" s="4" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A18">
-        <v>750</v>
-      </c>
-      <c r="B18" s="5"/>
-      <c r="C18">
-        <v>1.2615551433943699</v>
-      </c>
-      <c r="D18">
-        <v>1.2502327359779</v>
-      </c>
-      <c r="E18">
-        <v>1.26687035022674</v>
-      </c>
-      <c r="F18" s="10">
-        <f t="shared" si="0"/>
-        <v>1.0133076136706871</v>
-      </c>
-      <c r="H18">
-        <v>1.2096572387659299</v>
-      </c>
-      <c r="I18">
-        <v>1.20261020085431</v>
-      </c>
-      <c r="J18">
-        <v>1.2257592093430201</v>
-      </c>
-      <c r="K18" s="10">
-        <f t="shared" si="1"/>
-        <v>1.0192489706741765</v>
-      </c>
-      <c r="L18" s="11"/>
-    </row>
-    <row r="19" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A19">
-        <v>999.99</v>
-      </c>
-      <c r="B19" s="5"/>
-      <c r="C19">
-        <v>1.2295679722156101</v>
-      </c>
-      <c r="D19">
-        <v>1.2216766905077201</v>
-      </c>
-      <c r="E19">
-        <v>1.20816790789953</v>
-      </c>
-      <c r="F19" s="10">
-        <f t="shared" si="0"/>
-        <v>0.98894242420015732</v>
-      </c>
-      <c r="G19" s="4"/>
-      <c r="H19">
-        <v>1.15612158785918</v>
-      </c>
-      <c r="I19">
-        <v>1.1553240194424299</v>
-      </c>
-      <c r="J19">
-        <v>1.13503567173569</v>
-      </c>
-      <c r="K19" s="10">
-        <f t="shared" si="1"/>
-        <v>0.9824392574158276</v>
-      </c>
-      <c r="L19" s="10"/>
+    <row r="21" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="C21" s="12" t="s">
+        <v>5</v>
+      </c>
+      <c r="D21" s="12"/>
+      <c r="E21" s="13"/>
+      <c r="F21" s="13"/>
+      <c r="H21" s="2"/>
+      <c r="I21" s="2"/>
+      <c r="J21" s="2"/>
+      <c r="K21" s="2"/>
+    </row>
+    <row r="22" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="C22" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="D22" s="3"/>
+      <c r="E22" s="9"/>
+      <c r="F22" s="3"/>
+      <c r="H22" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="I22" s="3"/>
+      <c r="J22" s="9"/>
+      <c r="K22" s="9"/>
+      <c r="L22" s="3"/>
     </row>
     <row r="23" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="C23" s="12" t="s">
-        <v>5</v>
-      </c>
-      <c r="D23" s="12"/>
-      <c r="E23" s="13"/>
-      <c r="F23" s="13"/>
-      <c r="H23" s="2"/>
-      <c r="I23" s="2"/>
-      <c r="J23" s="2"/>
-      <c r="K23" s="2"/>
+      <c r="A23" s="6" t="s">
+        <v>0</v>
+      </c>
+      <c r="B23" s="6"/>
+      <c r="C23" s="6" t="s">
+        <v>1</v>
+      </c>
+      <c r="D23" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="E23" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="F23" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="G23" s="8"/>
+      <c r="H23" s="6" t="s">
+        <v>1</v>
+      </c>
+      <c r="I23" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="J23" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="K23" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="L23" s="7"/>
     </row>
     <row r="24" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="C24" s="3" t="s">
-        <v>4</v>
-      </c>
-      <c r="D24" s="3"/>
-      <c r="E24" s="9"/>
-      <c r="F24" s="3"/>
-      <c r="H24" s="3" t="s">
-        <v>3</v>
-      </c>
-      <c r="I24" s="3"/>
-      <c r="J24" s="9"/>
-      <c r="K24" s="9"/>
-      <c r="L24" s="3"/>
+      <c r="A24">
+        <v>0.1</v>
+      </c>
+      <c r="B24" s="5"/>
+      <c r="C24" s="2"/>
+      <c r="D24" s="2"/>
+      <c r="E24" s="2">
+        <v>2.3188386654289999E-5</v>
+      </c>
+      <c r="F24" s="10" t="e">
+        <f>E24/D24</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="G24" s="4"/>
+      <c r="H24" s="2"/>
+      <c r="I24" s="2"/>
+      <c r="J24" s="2"/>
+      <c r="K24" s="10" t="e">
+        <f>J24/I24</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="L24" s="10"/>
     </row>
     <row r="25" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A25" s="6" t="s">
-        <v>0</v>
-      </c>
-      <c r="B25" s="6"/>
-      <c r="C25" s="6" t="s">
-        <v>1</v>
-      </c>
-      <c r="D25" s="6" t="s">
-        <v>7</v>
-      </c>
-      <c r="E25" s="6" t="s">
-        <v>6</v>
-      </c>
-      <c r="F25" s="7" t="s">
-        <v>8</v>
-      </c>
-      <c r="G25" s="8"/>
-      <c r="H25" s="6" t="s">
-        <v>1</v>
-      </c>
-      <c r="I25" s="6" t="s">
-        <v>7</v>
-      </c>
-      <c r="J25" s="6" t="s">
-        <v>6</v>
-      </c>
-      <c r="K25" s="7" t="s">
-        <v>8</v>
-      </c>
-      <c r="L25" s="7"/>
+      <c r="A25">
+        <v>0.5</v>
+      </c>
+      <c r="B25" s="5"/>
+      <c r="E25">
+        <v>1.16379113471186E-4</v>
+      </c>
+      <c r="F25" s="10" t="e">
+        <f t="shared" ref="F25:F36" si="2">E25/D25</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="G25" s="4"/>
+      <c r="K25" s="10" t="e">
+        <f t="shared" ref="K25:K36" si="3">J25/I25</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="L25" s="10"/>
     </row>
     <row r="26" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A26">
-        <v>0.1</v>
+        <v>1</v>
       </c>
       <c r="B26" s="5"/>
-      <c r="C26" s="2">
-        <v>3.53760968083747E-5</v>
-      </c>
-      <c r="D26" s="2">
-        <v>3.4283030439073703E-5</v>
-      </c>
-      <c r="E26" s="2">
-        <v>2.4940135833565399E-5</v>
-      </c>
-      <c r="F26" s="10">
-        <f>E26/D26</f>
-        <v>0.7274775745944605</v>
+      <c r="E26">
+        <v>2.31665379952172E-4</v>
+      </c>
+      <c r="F26" s="10" t="e">
+        <f t="shared" si="2"/>
+        <v>#DIV/0!</v>
       </c>
       <c r="G26" s="4"/>
-      <c r="H26" s="2">
-        <v>3.2455422398815998E-5</v>
-      </c>
-      <c r="I26" s="2">
-        <v>3.06037506527904E-5</v>
-      </c>
-      <c r="J26" s="2">
-        <v>8.9560974139772096E-6</v>
-      </c>
-      <c r="K26" s="10">
-        <f>J26/I26</f>
-        <v>0.29264705217301878</v>
+      <c r="K26" s="10" t="e">
+        <f t="shared" si="3"/>
+        <v>#DIV/0!</v>
       </c>
       <c r="L26" s="10"/>
     </row>
     <row r="27" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A27">
-        <v>0.5</v>
+        <v>10</v>
       </c>
       <c r="B27" s="5"/>
-      <c r="C27">
-        <v>1.769377952569E-4</v>
-      </c>
-      <c r="D27">
-        <v>1.7795710468822501E-4</v>
-      </c>
       <c r="E27">
-        <v>1.1451179445258501E-4</v>
-      </c>
-      <c r="F27" s="10">
-        <f t="shared" ref="F27:F40" si="2">E27/D27</f>
-        <v>0.64347975683918834</v>
+        <v>2.3274949085023899E-3</v>
+      </c>
+      <c r="F27" s="10" t="e">
+        <f t="shared" si="2"/>
+        <v>#DIV/0!</v>
       </c>
       <c r="G27" s="4"/>
-      <c r="H27">
-        <v>1.622082823178E-4</v>
-      </c>
-      <c r="I27">
-        <v>1.51128498783429E-4</v>
-      </c>
-      <c r="J27">
-        <v>2.0123326791721201E-4</v>
-      </c>
-      <c r="K27" s="10">
-        <f t="shared" ref="K27:K40" si="3">J27/I27</f>
-        <v>1.3315375295667062</v>
+      <c r="K27" s="10" t="e">
+        <f t="shared" si="3"/>
+        <v>#DIV/0!</v>
       </c>
       <c r="L27" s="10"/>
     </row>
     <row r="28" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A28">
-        <v>1.5</v>
+        <v>25</v>
       </c>
       <c r="B28" s="5"/>
-      <c r="C28">
-        <v>5.2503514596129999E-4</v>
-      </c>
-      <c r="D28">
-        <v>5.6289187437775004E-4</v>
-      </c>
       <c r="E28">
-        <v>2.79102553247934E-4</v>
-      </c>
-      <c r="F28" s="10">
+        <v>5.7868683352336496E-3</v>
+      </c>
+      <c r="F28" s="10" t="e">
         <f t="shared" si="2"/>
-        <v>0.49583688440425344</v>
+        <v>#DIV/0!</v>
       </c>
       <c r="G28" s="4"/>
-      <c r="H28">
-        <v>4.8498345014689998E-4</v>
-      </c>
-      <c r="I28">
-        <v>4.4989314990682798E-4</v>
-      </c>
-      <c r="J28">
-        <v>4.03614344914232E-4</v>
-      </c>
-      <c r="K28" s="10">
+      <c r="K28" s="10" t="e">
         <f t="shared" si="3"/>
-        <v>0.8971337860952534</v>
-      </c>
-      <c r="L28" s="10"/>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="L28" s="11"/>
     </row>
     <row r="29" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A29">
-        <v>10</v>
+        <v>50</v>
       </c>
       <c r="B29" s="5"/>
-      <c r="C29">
-        <v>3.3839428456904001E-3</v>
-      </c>
-      <c r="D29">
-        <v>3.3365070331695802E-3</v>
-      </c>
       <c r="E29">
-        <v>2.2307755074323201E-3</v>
-      </c>
-      <c r="F29" s="10">
+        <v>1.1357972286110201E-2</v>
+      </c>
+      <c r="F29" s="10" t="e">
         <f t="shared" si="2"/>
-        <v>0.66859607525333198</v>
+        <v>#DIV/0!</v>
       </c>
       <c r="G29" s="4"/>
-      <c r="H29">
-        <v>3.1626406186310001E-3</v>
-      </c>
-      <c r="I29">
-        <v>3.0155921421882699E-3</v>
-      </c>
-      <c r="J29">
-        <v>2.6153364392675002E-3</v>
-      </c>
-      <c r="K29" s="10">
+      <c r="K29" s="10" t="e">
         <f t="shared" si="3"/>
-        <v>0.86727127408207016</v>
+        <v>#DIV/0!</v>
       </c>
       <c r="L29" s="10"/>
     </row>
     <row r="30" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A30" s="4">
-        <v>15</v>
+      <c r="A30">
+        <v>75</v>
       </c>
       <c r="B30" s="5"/>
-      <c r="C30">
-        <v>4.9687340175238997E-3</v>
-      </c>
-      <c r="D30">
-        <v>4.9536689812130401E-3</v>
-      </c>
       <c r="E30">
-        <v>3.6306214215505398E-3</v>
-      </c>
-      <c r="F30" s="10">
+        <v>1.6724313084056999E-2</v>
+      </c>
+      <c r="F30" s="10" t="e">
         <f t="shared" si="2"/>
-        <v>0.73291562987349301</v>
+        <v>#DIV/0!</v>
       </c>
       <c r="G30" s="4"/>
-      <c r="H30">
-        <v>4.7034313826145001E-3</v>
-      </c>
-      <c r="I30">
-        <v>4.2298917106053102E-3</v>
-      </c>
-      <c r="J30">
-        <v>4.0615398119136998E-3</v>
-      </c>
-      <c r="K30" s="10">
+      <c r="K30" s="10" t="e">
         <f t="shared" si="3"/>
-        <v>0.96019947785672299</v>
+        <v>#DIV/0!</v>
       </c>
       <c r="L30" s="11"/>
     </row>
     <row r="31" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A31">
-        <v>30</v>
+        <v>100</v>
       </c>
       <c r="B31" s="5"/>
-      <c r="C31">
-        <v>9.6668811570342003E-3</v>
-      </c>
-      <c r="D31">
-        <v>9.8049806314099101E-3</v>
-      </c>
       <c r="E31">
-        <v>7.3289045458139902E-3</v>
-      </c>
-      <c r="F31" s="10">
+        <v>2.2149757308928399E-2</v>
+      </c>
+      <c r="F31" s="10" t="e">
         <f t="shared" si="2"/>
-        <v>0.74746751893992558</v>
+        <v>#DIV/0!</v>
       </c>
       <c r="G31" s="4"/>
-      <c r="H31">
-        <v>9.2377761797262006E-3</v>
-      </c>
-      <c r="I31">
-        <v>8.8658994417866593E-3</v>
-      </c>
-      <c r="J31">
-        <v>7.2748435041183898E-3</v>
-      </c>
-      <c r="K31" s="10">
+      <c r="K31" s="10" t="e">
         <f t="shared" si="3"/>
-        <v>0.82054207267800461</v>
+        <v>#DIV/0!</v>
       </c>
       <c r="L31" s="10"/>
     </row>
     <row r="32" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A32" s="4">
-        <v>60</v>
+      <c r="A32">
+        <v>150</v>
       </c>
       <c r="B32" s="5"/>
-      <c r="C32">
-        <v>1.7647794082264599E-2</v>
-      </c>
-      <c r="D32">
-        <v>1.6929482364304901E-2</v>
-      </c>
       <c r="E32">
-        <v>1.3311257592672E-2</v>
-      </c>
-      <c r="F32" s="10">
+        <v>3.2103137598192298E-2</v>
+      </c>
+      <c r="F32" s="10" t="e">
         <f t="shared" si="2"/>
-        <v>0.78627670393149318</v>
+        <v>#DIV/0!</v>
       </c>
       <c r="G32" s="4"/>
-      <c r="H32">
-        <v>1.79734898063151E-2</v>
-      </c>
-      <c r="I32">
-        <v>1.57606335049696E-2</v>
-      </c>
-      <c r="J32">
-        <v>1.41246952576636E-2</v>
-      </c>
-      <c r="K32" s="10">
+      <c r="K32" s="10" t="e">
         <f t="shared" si="3"/>
-        <v>0.89620098412984728</v>
-      </c>
-      <c r="L32" s="11"/>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="L32" s="10"/>
     </row>
     <row r="33" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A33">
-        <v>90</v>
+        <v>250</v>
       </c>
       <c r="B33" s="5"/>
-      <c r="C33">
-        <v>2.5054917938694E-2</v>
-      </c>
-      <c r="D33">
-        <v>2.3458449507632401E-2</v>
-      </c>
       <c r="E33">
-        <v>2.05541471998755E-2</v>
-      </c>
-      <c r="F33" s="10">
+        <v>5.1114734736025402E-2</v>
+      </c>
+      <c r="F33" s="10" t="e">
         <f t="shared" si="2"/>
-        <v>0.87619376520123537</v>
+        <v>#DIV/0!</v>
       </c>
       <c r="G33" s="4"/>
-      <c r="H33">
-        <v>2.6164917465571601E-2</v>
-      </c>
-      <c r="I33">
-        <v>2.3818302176688601E-2</v>
-      </c>
-      <c r="J33">
-        <v>2.3768164319370701E-2</v>
-      </c>
-      <c r="K33" s="10">
+      <c r="K33" s="10" t="e">
         <f t="shared" si="3"/>
-        <v>0.99789498609321658</v>
-      </c>
-      <c r="L33" s="10"/>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="L33" s="11"/>
     </row>
     <row r="34" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A34" s="4">
-        <v>100</v>
+      <c r="A34">
+        <v>500</v>
       </c>
       <c r="B34" s="5"/>
-      <c r="C34">
-        <v>2.73242514617307E-2</v>
-      </c>
-      <c r="D34">
-        <v>2.5947125661509699E-2</v>
-      </c>
       <c r="E34">
-        <v>2.2524567468256498E-2</v>
-      </c>
-      <c r="F34" s="10">
+        <v>9.1445222619505398E-2</v>
+      </c>
+      <c r="F34" s="10" t="e">
         <f t="shared" si="2"/>
-        <v>0.86809490045634352</v>
+        <v>#DIV/0!</v>
       </c>
       <c r="G34" s="4"/>
-      <c r="H34">
-        <v>2.8758676699886999E-2</v>
-      </c>
-      <c r="I34">
-        <v>2.6060698692637999E-2</v>
-      </c>
-      <c r="J34">
-        <v>2.41183055307931E-2</v>
-      </c>
-      <c r="K34" s="10">
+      <c r="K34" s="10" t="e">
         <f t="shared" si="3"/>
-        <v>0.92546657383389286</v>
+        <v>#DIV/0!</v>
       </c>
       <c r="L34" s="10"/>
     </row>
     <row r="35" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A35" s="4">
-        <v>120</v>
+      <c r="A35">
+        <v>750</v>
       </c>
       <c r="B35" s="5"/>
-      <c r="C35">
-        <v>3.1756367537968302E-2</v>
-      </c>
-      <c r="D35">
-        <v>3.2193504593870201E-2</v>
-      </c>
       <c r="E35">
-        <v>2.5515114756006999E-2</v>
-      </c>
-      <c r="F35" s="10">
+        <v>0.12725844081883</v>
+      </c>
+      <c r="F35" s="10" t="e">
         <f t="shared" si="2"/>
-        <v>0.79255474288640204</v>
+        <v>#DIV/0!</v>
       </c>
       <c r="G35" s="4"/>
-      <c r="H35">
-        <v>3.3831181126573399E-2</v>
-      </c>
-      <c r="I35">
-        <v>3.0884672634417399E-2</v>
-      </c>
-      <c r="J35">
-        <v>2.9445668702238598E-2</v>
-      </c>
-      <c r="K35" s="10">
+      <c r="K35" s="10" t="e">
         <f t="shared" si="3"/>
-        <v>0.95340718196328889</v>
+        <v>#DIV/0!</v>
       </c>
       <c r="L35" s="11"/>
     </row>
     <row r="36" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A36">
-        <v>150</v>
+        <v>999.99</v>
       </c>
       <c r="B36" s="5"/>
-      <c r="C36">
-        <v>3.79760832406765E-2</v>
-      </c>
-      <c r="D36">
-        <v>3.6337278414827603E-2</v>
-      </c>
       <c r="E36">
-        <v>3.2903913104897098E-2</v>
-      </c>
-      <c r="F36" s="10">
+        <v>0.157583868759714</v>
+      </c>
+      <c r="F36" s="10" t="e">
         <f t="shared" si="2"/>
-        <v>0.90551396638088599</v>
+        <v>#DIV/0!</v>
       </c>
       <c r="G36" s="4"/>
-      <c r="H36">
-        <v>4.0827391559504302E-2</v>
-      </c>
-      <c r="I36">
-        <v>3.8123585674305099E-2</v>
-      </c>
-      <c r="J36">
-        <v>3.6179164073167201E-2</v>
-      </c>
-      <c r="K36" s="10">
+      <c r="K36" s="10" t="e">
         <f t="shared" si="3"/>
-        <v>0.94899688560909901</v>
+        <v>#DIV/0!</v>
       </c>
       <c r="L36" s="10"/>
     </row>
-    <row r="37" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A37" s="4">
-        <v>250</v>
-      </c>
-      <c r="B37" s="5"/>
-      <c r="C37">
-        <v>5.6477544791410803E-2</v>
-      </c>
-      <c r="D37">
-        <v>5.5465836690505303E-2</v>
-      </c>
-      <c r="E37">
-        <v>5.1493175994203999E-2</v>
-      </c>
-      <c r="F37" s="10">
-        <f t="shared" si="2"/>
-        <v>0.92837643974491146</v>
-      </c>
-      <c r="G37" s="4"/>
-      <c r="H37">
-        <v>6.2587066941841005E-2</v>
-      </c>
-      <c r="I37">
-        <v>5.8814448863946898E-2</v>
-      </c>
-      <c r="J37">
-        <v>5.6605063359839898E-2</v>
-      </c>
-      <c r="K37" s="10">
-        <f t="shared" si="3"/>
-        <v>0.9624346474925255</v>
-      </c>
-      <c r="L37" s="11"/>
-    </row>
-    <row r="38" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A38">
-        <v>500</v>
-      </c>
-      <c r="B38" s="5"/>
-      <c r="C38">
-        <v>9.6749839749360703E-2</v>
-      </c>
-      <c r="D38">
-        <v>9.2698744321603202E-2</v>
-      </c>
-      <c r="E38">
-        <v>8.6940034618715994E-2</v>
-      </c>
-      <c r="F38" s="10">
-        <f t="shared" si="2"/>
-        <v>0.93787715524054671</v>
-      </c>
-      <c r="G38" s="4"/>
-      <c r="H38">
-        <v>0.10941310652236901</v>
-      </c>
-      <c r="I38">
-        <v>0.101328636998795</v>
-      </c>
-      <c r="J38">
-        <v>0.103511880070482</v>
-      </c>
-      <c r="K38" s="10">
-        <f t="shared" si="3"/>
-        <v>1.0215461604572156</v>
-      </c>
-      <c r="L38" s="10"/>
-    </row>
-    <row r="39" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A39" s="4">
-        <v>750</v>
-      </c>
-      <c r="B39" s="5"/>
-      <c r="C39">
-        <v>0.12913289428404701</v>
-      </c>
-      <c r="D39">
-        <v>0.12658460512460301</v>
-      </c>
-      <c r="E39">
-        <v>0.128790466427847</v>
-      </c>
-      <c r="F39" s="10">
-        <f t="shared" si="2"/>
-        <v>1.0174259839976012</v>
-      </c>
-      <c r="G39" s="4"/>
-      <c r="H39">
-        <v>0.14632252761592299</v>
-      </c>
-      <c r="I39">
-        <v>0.13858937862319001</v>
-      </c>
-      <c r="J39">
-        <v>0.149026761504226</v>
-      </c>
-      <c r="K39" s="10">
-        <f t="shared" si="3"/>
-        <v>1.0753115641669349</v>
-      </c>
-      <c r="L39" s="11"/>
-    </row>
     <row r="40" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A40">
-        <v>1000</v>
-      </c>
-      <c r="B40" s="5"/>
-      <c r="C40">
-        <v>0.157828985100924</v>
-      </c>
-      <c r="D40">
-        <v>0.15157133316674601</v>
-      </c>
-      <c r="E40">
-        <v>0.15530428148366199</v>
-      </c>
-      <c r="F40" s="10">
-        <f t="shared" si="2"/>
-        <v>1.0246283267351703</v>
-      </c>
-      <c r="G40" s="4"/>
-      <c r="H40">
-        <v>0.178362496787381</v>
-      </c>
-      <c r="I40">
-        <v>0.17072801306535401</v>
-      </c>
-      <c r="J40">
-        <v>0.17116297500401301</v>
-      </c>
-      <c r="K40" s="10">
-        <f t="shared" si="3"/>
-        <v>1.0025476893384362</v>
-      </c>
-      <c r="L40" s="10"/>
+      <c r="C40" s="1" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="41" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="C41" s="14" t="s">
+        <v>2</v>
+      </c>
+      <c r="D41" s="14"/>
+      <c r="E41" s="15"/>
+      <c r="H41" s="2"/>
+      <c r="I41" s="2"/>
+      <c r="J41" s="2"/>
+      <c r="K41" s="2"/>
+    </row>
+    <row r="42" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="C42" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="D42" s="3"/>
+      <c r="E42" s="9"/>
+      <c r="F42" s="3"/>
+      <c r="H42" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="I42" s="3"/>
+      <c r="J42" s="9"/>
+      <c r="K42" s="9"/>
+    </row>
+    <row r="43" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A43" s="6" t="s">
+        <v>0</v>
+      </c>
+      <c r="B43" s="6"/>
+      <c r="C43" s="6" t="s">
+        <v>1</v>
+      </c>
+      <c r="D43" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="E43" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="F43" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="G43" s="8"/>
+      <c r="H43" s="6" t="s">
+        <v>1</v>
+      </c>
+      <c r="I43" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="J43" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="K43" s="7" t="s">
+        <v>8</v>
+      </c>
     </row>
     <row r="44" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="C44" s="1" t="s">
-        <v>9</v>
+      <c r="A44">
+        <v>0.1</v>
+      </c>
+      <c r="B44" s="5"/>
+      <c r="C44">
+        <v>1.38755773111088</v>
+      </c>
+      <c r="D44">
+        <v>1.33146077610654</v>
+      </c>
+      <c r="E44">
+        <v>1.3294682945082299</v>
+      </c>
+      <c r="F44" s="10">
+        <f>E44/D44</f>
+        <v>0.9985035371420129</v>
+      </c>
+      <c r="G44" s="4"/>
+      <c r="I44">
+        <v>1.33422182541257</v>
+      </c>
+      <c r="J44">
+        <v>1.3288821396550801</v>
+      </c>
+      <c r="K44" s="10">
+        <f>J44/I44</f>
+        <v>0.99599790255579224</v>
       </c>
     </row>
     <row r="45" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="C45" s="14" t="s">
-        <v>2</v>
-      </c>
-      <c r="D45" s="14"/>
-      <c r="E45" s="15"/>
-      <c r="H45" s="2"/>
-      <c r="I45" s="2"/>
-      <c r="J45" s="2"/>
-      <c r="K45" s="2"/>
+      <c r="A45">
+        <v>0.5</v>
+      </c>
+      <c r="B45" s="5"/>
+      <c r="C45">
+        <v>1.38409520401011</v>
+      </c>
+      <c r="D45">
+        <v>1.35765661048369</v>
+      </c>
+      <c r="E45">
+        <v>1.3402135659025001</v>
+      </c>
+      <c r="F45" s="10">
+        <f t="shared" ref="F45:F56" si="4">E45/D45</f>
+        <v>0.98715209394887005</v>
+      </c>
+      <c r="G45" s="4"/>
+      <c r="H45" s="4"/>
+      <c r="I45">
+        <v>1.3552315082948401</v>
+      </c>
+      <c r="J45">
+        <v>1.34024384554322</v>
+      </c>
+      <c r="K45" s="11">
+        <f t="shared" ref="K45:K54" si="5">J45/I45</f>
+        <v>0.98894088378266998</v>
+      </c>
     </row>
     <row r="46" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="C46" s="3" t="s">
-        <v>4</v>
-      </c>
-      <c r="D46" s="3"/>
-      <c r="E46" s="9"/>
-      <c r="F46" s="3"/>
-      <c r="H46" s="3" t="s">
-        <v>3</v>
-      </c>
-      <c r="I46" s="3"/>
-      <c r="J46" s="9"/>
-      <c r="K46" s="9"/>
+      <c r="A46">
+        <v>1</v>
+      </c>
+      <c r="B46" s="5"/>
+      <c r="C46">
+        <v>1.3811622398640599</v>
+      </c>
+      <c r="D46">
+        <v>1.33903476392587</v>
+      </c>
+      <c r="E46">
+        <v>1.3294539841566</v>
+      </c>
+      <c r="F46" s="10">
+        <f t="shared" si="4"/>
+        <v>0.99284501043036377</v>
+      </c>
+      <c r="G46" s="4"/>
+      <c r="I46">
+        <v>1.3461367977004299</v>
+      </c>
+      <c r="J46">
+        <v>1.32904261090945</v>
+      </c>
+      <c r="K46" s="10">
+        <f t="shared" si="5"/>
+        <v>0.98730130041747499</v>
+      </c>
     </row>
     <row r="47" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A47" s="6" t="s">
-        <v>0</v>
-      </c>
-      <c r="B47" s="6"/>
-      <c r="C47" s="6" t="s">
-        <v>1</v>
-      </c>
-      <c r="D47" s="6" t="s">
-        <v>7</v>
-      </c>
-      <c r="E47" s="6" t="s">
-        <v>6</v>
-      </c>
-      <c r="F47" s="7" t="s">
-        <v>8</v>
-      </c>
-      <c r="G47" s="8"/>
-      <c r="H47" s="6" t="s">
-        <v>1</v>
-      </c>
-      <c r="I47" s="6" t="s">
-        <v>7</v>
-      </c>
-      <c r="J47" s="6" t="s">
-        <v>6</v>
-      </c>
-      <c r="K47" s="7" t="s">
-        <v>8</v>
+      <c r="A47">
+        <v>10</v>
+      </c>
+      <c r="B47" s="5"/>
+      <c r="C47">
+        <v>1.37486493369789</v>
+      </c>
+      <c r="D47">
+        <v>1.31789010731641</v>
+      </c>
+      <c r="E47">
+        <v>1.3448930260504799</v>
+      </c>
+      <c r="F47" s="10">
+        <f t="shared" si="4"/>
+        <v>1.0204895071175968</v>
+      </c>
+      <c r="G47" s="4"/>
+      <c r="H47" s="4"/>
+      <c r="I47">
+        <v>1.31846450590491</v>
+      </c>
+      <c r="J47">
+        <v>1.3511493506913199</v>
+      </c>
+      <c r="K47" s="11">
+        <f t="shared" si="5"/>
+        <v>1.0247900831914902</v>
       </c>
     </row>
     <row r="48" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A48">
-        <v>0.1</v>
+        <v>25</v>
       </c>
       <c r="B48" s="5"/>
       <c r="C48">
-        <v>1.38755773111088</v>
+        <v>1.36350384779266</v>
       </c>
       <c r="D48">
-        <v>1.33146077610654</v>
+        <v>1.32036564820574</v>
       </c>
       <c r="E48">
-        <v>1.3294682945082299</v>
+        <v>1.3268512139816999</v>
       </c>
       <c r="F48" s="10">
-        <f>E48/D48</f>
-        <v>0.9985035371420129</v>
+        <f t="shared" si="4"/>
+        <v>1.0049119467662411</v>
       </c>
       <c r="G48" s="4"/>
       <c r="I48">
-        <v>1.33422182541257</v>
+        <v>1.33152629750905</v>
       </c>
       <c r="J48">
-        <v>1.3288821396550801</v>
+        <v>1.33015612015508</v>
       </c>
       <c r="K48" s="10">
-        <f>J48/I48</f>
-        <v>0.99599790255579224</v>
+        <f t="shared" si="5"/>
+        <v>0.99897097236717491</v>
       </c>
     </row>
     <row r="49" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A49">
-        <v>0.5</v>
+        <v>50</v>
       </c>
       <c r="B49" s="5"/>
       <c r="C49">
-        <v>1.38409520401011</v>
+        <v>1.3571706170428599</v>
       </c>
       <c r="D49">
-        <v>1.35765661048369</v>
+        <v>1.3197738196808499</v>
       </c>
       <c r="E49">
-        <v>1.3402135659025001</v>
+        <v>1.3126564921716899</v>
       </c>
       <c r="F49" s="10">
-        <f t="shared" ref="F49:F60" si="4">E49/D49</f>
-        <v>0.98715209394887005</v>
+        <f t="shared" si="4"/>
+        <v>0.99460716116426584</v>
       </c>
       <c r="G49" s="4"/>
       <c r="H49" s="4"/>
       <c r="I49">
-        <v>1.3552315082948401</v>
+        <v>1.32005527665466</v>
       </c>
       <c r="J49">
-        <v>1.34024384554322</v>
+        <v>1.30244954906179</v>
       </c>
       <c r="K49" s="11">
-        <f t="shared" ref="K49:K58" si="5">J49/I49</f>
-        <v>0.98894088378266998</v>
+        <f t="shared" si="5"/>
+        <v>0.98666288608952257</v>
       </c>
     </row>
     <row r="50" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A50">
-        <v>1</v>
+        <v>75</v>
       </c>
       <c r="B50" s="5"/>
       <c r="C50">
-        <v>1.3811622398640599</v>
+        <v>1.35109721915133</v>
       </c>
       <c r="D50">
-        <v>1.33903476392587</v>
+        <v>1.29935652652886</v>
       </c>
       <c r="E50">
-        <v>1.3294539841566</v>
+        <v>1.32473430230751</v>
       </c>
       <c r="F50" s="10">
         <f t="shared" si="4"/>
-        <v>0.99284501043036377</v>
+        <v>1.0195310334465668</v>
       </c>
       <c r="G50" s="4"/>
       <c r="I50">
-        <v>1.3461367977004299</v>
+        <v>1.30908256842566</v>
       </c>
       <c r="J50">
-        <v>1.32904261090945</v>
+        <v>1.30672475018709</v>
       </c>
       <c r="K50" s="10">
         <f t="shared" si="5"/>
-        <v>0.98730130041747499</v>
+        <v>0.99819887736996948</v>
       </c>
     </row>
     <row r="51" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A51">
-        <v>10</v>
+        <v>100</v>
       </c>
       <c r="B51" s="5"/>
       <c r="C51">
-        <v>1.37486493369789</v>
+        <v>1.32844051248484</v>
       </c>
       <c r="D51">
-        <v>1.31789010731641</v>
+        <v>1.33910590256307</v>
       </c>
       <c r="E51">
-        <v>1.3448930260504799</v>
+        <v>1.3167897334910501</v>
       </c>
       <c r="F51" s="10">
         <f t="shared" si="4"/>
-        <v>1.0204895071175968</v>
+        <v>0.98333502299608533</v>
       </c>
       <c r="G51" s="4"/>
       <c r="H51" s="4"/>
       <c r="I51">
-        <v>1.31846450590491</v>
+        <v>1.3171859836539099</v>
       </c>
       <c r="J51">
-        <v>1.3511493506913199</v>
+        <v>1.31060168409573</v>
       </c>
       <c r="K51" s="11">
         <f t="shared" si="5"/>
-        <v>1.0247900831914902</v>
+        <v>0.99500123775997451</v>
       </c>
     </row>
     <row r="52" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A52">
-        <v>25</v>
+        <v>150</v>
       </c>
       <c r="B52" s="5"/>
       <c r="C52">
-        <v>1.36350384779266</v>
+        <v>1.26939305918802</v>
       </c>
       <c r="D52">
-        <v>1.32036564820574</v>
+        <v>1.3346899335651701</v>
       </c>
       <c r="E52">
-        <v>1.3268512139816999</v>
+        <v>1.3164282135057199</v>
       </c>
       <c r="F52" s="10">
         <f t="shared" si="4"/>
-        <v>1.0049119467662411</v>
+        <v>0.98631763108404502</v>
       </c>
       <c r="G52" s="4"/>
       <c r="I52">
-        <v>1.33152629750905</v>
+        <v>1.28924587434467</v>
       </c>
       <c r="J52">
-        <v>1.33015612015508</v>
+        <v>1.3011790803332</v>
       </c>
       <c r="K52" s="10">
         <f t="shared" si="5"/>
-        <v>0.99897097236717491</v>
+        <v>1.0092559582512495</v>
       </c>
     </row>
     <row r="53" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A53">
-        <v>50</v>
+        <v>250</v>
       </c>
       <c r="B53" s="5"/>
       <c r="C53">
-        <v>1.3571706170428599</v>
+        <v>1.2146497361047901</v>
       </c>
       <c r="D53">
-        <v>1.3197738196808499</v>
+        <v>1.29678717701069</v>
       </c>
       <c r="E53">
-        <v>1.3126564921716899</v>
+        <v>1.33451901185347</v>
       </c>
       <c r="F53" s="10">
         <f t="shared" si="4"/>
-        <v>0.99460716116426584</v>
+        <v>1.0290963972436542</v>
       </c>
       <c r="G53" s="4"/>
       <c r="H53" s="4"/>
       <c r="I53">
-        <v>1.32005527665466</v>
+        <v>1.2845821783281699</v>
       </c>
       <c r="J53">
-        <v>1.30244954906179</v>
+        <v>1.27732476166037</v>
       </c>
       <c r="K53" s="11">
         <f t="shared" si="5"/>
-        <v>0.98666288608952257</v>
+        <v>0.99435036793267273</v>
       </c>
     </row>
     <row r="54" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A54">
-        <v>75</v>
+        <v>500</v>
       </c>
       <c r="B54" s="5"/>
       <c r="C54">
-        <v>1.35109721915133</v>
+        <v>1.1436421352186501</v>
       </c>
       <c r="D54">
-        <v>1.29935652652886</v>
+        <v>1.2662694099393199</v>
       </c>
       <c r="E54">
-        <v>1.32473430230751</v>
+        <v>1.2620512370753201</v>
       </c>
       <c r="F54" s="10">
         <f t="shared" si="4"/>
-        <v>1.0195310334465668</v>
+        <v>0.99666881879093805</v>
       </c>
       <c r="G54" s="4"/>
       <c r="I54">
-        <v>1.30908256842566</v>
+        <v>1.2051198250164299</v>
       </c>
       <c r="J54">
-        <v>1.30672475018709</v>
+        <v>1.19710463230099</v>
       </c>
       <c r="K54" s="10">
         <f t="shared" si="5"/>
-        <v>0.99819887736996948</v>
+        <v>0.99334904915755518</v>
       </c>
     </row>
     <row r="55" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A55">
-        <v>100</v>
-      </c>
-      <c r="B55" s="5"/>
-      <c r="C55">
-        <v>1.32844051248484</v>
+        <v>750</v>
       </c>
       <c r="D55">
-        <v>1.33910590256307</v>
+        <v>1.23279071771682</v>
       </c>
       <c r="E55">
-        <v>1.3167897334910501</v>
+        <v>1.23649350366719</v>
       </c>
       <c r="F55" s="10">
         <f t="shared" si="4"/>
-        <v>0.98333502299608533</v>
-      </c>
-      <c r="G55" s="4"/>
-      <c r="H55" s="4"/>
+        <v>1.0030035803296993</v>
+      </c>
       <c r="I55">
-        <v>1.3171859836539099</v>
+        <v>1.1807532343395699</v>
       </c>
       <c r="J55">
-        <v>1.31060168409573</v>
-      </c>
-      <c r="K55" s="11">
-        <f t="shared" si="5"/>
-        <v>0.99500123775997451</v>
+        <v>1.1563239206929501</v>
       </c>
     </row>
     <row r="56" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A56">
-        <v>150</v>
-      </c>
-      <c r="B56" s="5"/>
-      <c r="C56">
-        <v>1.26939305918802</v>
+        <v>999.99</v>
       </c>
       <c r="D56">
-        <v>1.3346899335651701</v>
+        <v>1.1928852496040101</v>
       </c>
       <c r="E56">
-        <v>1.3164282135057199</v>
+        <v>1.2106403902979499</v>
       </c>
       <c r="F56" s="10">
         <f t="shared" si="4"/>
-        <v>0.98631763108404502</v>
-      </c>
-      <c r="G56" s="4"/>
+        <v>1.0148841983751864</v>
+      </c>
       <c r="I56">
-        <v>1.28924587434467</v>
+        <v>1.13357719050286</v>
       </c>
       <c r="J56">
-        <v>1.3011790803332</v>
-      </c>
-      <c r="K56" s="10">
-        <f t="shared" si="5"/>
-        <v>1.0092559582512495</v>
-      </c>
-    </row>
-    <row r="57" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A57">
-        <v>250</v>
-      </c>
-      <c r="B57" s="5"/>
-      <c r="C57">
-        <v>1.2146497361047901</v>
-      </c>
-      <c r="D57">
-        <v>1.29678717701069</v>
-      </c>
-      <c r="E57">
-        <v>1.33451901185347</v>
-      </c>
-      <c r="F57" s="10">
-        <f t="shared" si="4"/>
-        <v>1.0290963972436542</v>
-      </c>
-      <c r="G57" s="4"/>
-      <c r="H57" s="4"/>
-      <c r="I57">
-        <v>1.2845821783281699</v>
-      </c>
-      <c r="J57">
-        <v>1.27732476166037</v>
-      </c>
-      <c r="K57" s="11">
-        <f t="shared" si="5"/>
-        <v>0.99435036793267273</v>
-      </c>
-    </row>
-    <row r="58" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A58">
-        <v>500</v>
-      </c>
-      <c r="B58" s="5"/>
-      <c r="C58">
-        <v>1.1436421352186501</v>
-      </c>
-      <c r="D58">
-        <v>1.2662694099393199</v>
-      </c>
-      <c r="E58">
-        <v>1.2620512370753201</v>
-      </c>
-      <c r="F58" s="10">
-        <f t="shared" si="4"/>
-        <v>0.99666881879093805</v>
-      </c>
-      <c r="G58" s="4"/>
-      <c r="I58">
-        <v>1.2051198250164299</v>
-      </c>
-      <c r="J58">
-        <v>1.19710463230099</v>
-      </c>
-      <c r="K58" s="10">
-        <f t="shared" si="5"/>
-        <v>0.99334904915755518</v>
+        <v>1.1342010761596699</v>
       </c>
     </row>
     <row r="59" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A59">
-        <v>750</v>
-      </c>
-      <c r="D59">
-        <v>1.23279071771682</v>
-      </c>
-      <c r="E59">
-        <v>1.23649350366719</v>
-      </c>
-      <c r="F59" s="10">
-        <f t="shared" si="4"/>
-        <v>1.0030035803296993</v>
-      </c>
-      <c r="I59">
-        <v>1.1807532343395699</v>
-      </c>
-      <c r="J59">
-        <v>1.1563239206929501</v>
-      </c>
+      <c r="C59" s="12" t="s">
+        <v>5</v>
+      </c>
+      <c r="D59" s="12"/>
+      <c r="E59" s="13"/>
+      <c r="F59" s="13"/>
+      <c r="H59" s="2"/>
+      <c r="I59" s="2"/>
+      <c r="J59" s="2"/>
+      <c r="K59" s="2"/>
     </row>
     <row r="60" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A60">
-        <v>999.99</v>
-      </c>
-      <c r="D60">
-        <v>1.1928852496040101</v>
-      </c>
-      <c r="E60">
-        <v>1.2106403902979499</v>
-      </c>
-      <c r="F60" s="10">
-        <f t="shared" si="4"/>
-        <v>1.0148841983751864</v>
-      </c>
-      <c r="I60">
-        <v>1.13357719050286</v>
-      </c>
-      <c r="J60">
-        <v>1.1342010761596699</v>
+      <c r="C60" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="D60" s="3"/>
+      <c r="E60" s="9"/>
+      <c r="F60" s="3"/>
+      <c r="H60" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="I60" s="3"/>
+      <c r="J60" s="9"/>
+      <c r="K60" s="9"/>
+    </row>
+    <row r="61" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A61" s="6" t="s">
+        <v>0</v>
+      </c>
+      <c r="B61" s="6"/>
+      <c r="C61" s="6" t="s">
+        <v>1</v>
+      </c>
+      <c r="D61" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="E61" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="F61" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="G61" s="8"/>
+      <c r="H61" s="6" t="s">
+        <v>1</v>
+      </c>
+      <c r="I61" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="J61" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="K61" s="7" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="62" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A62">
+        <v>0.1</v>
+      </c>
+      <c r="B62" s="5"/>
+      <c r="C62" s="2">
+        <v>2.0906018648200899E-5</v>
+      </c>
+      <c r="D62" s="2">
+        <v>1.9785240862768899E-5</v>
+      </c>
+      <c r="E62" s="2">
+        <v>1.9417624590728801E-5</v>
+      </c>
+      <c r="F62" s="10">
+        <f>E62/D62</f>
+        <v>0.98141967163352228</v>
+      </c>
+      <c r="G62" s="4"/>
+      <c r="H62" s="2"/>
+      <c r="I62" s="2">
+        <v>2.44555572729164E-5</v>
+      </c>
+      <c r="J62" s="2">
+        <v>2.3173152783100001E-5</v>
+      </c>
+      <c r="K62" s="10">
+        <f>J62/I62</f>
+        <v>0.94756183735642718</v>
       </c>
     </row>
     <row r="63" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="C63" s="12" t="s">
-        <v>5</v>
-      </c>
-      <c r="D63" s="12"/>
-      <c r="E63" s="13"/>
-      <c r="F63" s="13"/>
-      <c r="H63" s="2"/>
-      <c r="I63" s="2"/>
-      <c r="J63" s="2"/>
-      <c r="K63" s="2"/>
+      <c r="A63">
+        <v>0.5</v>
+      </c>
+      <c r="B63" s="5"/>
+      <c r="C63" s="2">
+        <v>3.1327203465188001E-3</v>
+      </c>
+      <c r="D63">
+        <v>1.02051178015395E-4</v>
+      </c>
+      <c r="E63" s="2">
+        <v>9.4705678455829002E-5</v>
+      </c>
+      <c r="F63" s="10">
+        <f t="shared" ref="F63:F74" si="6">E63/D63</f>
+        <v>0.92802141334950694</v>
+      </c>
+      <c r="G63" s="4"/>
+      <c r="I63">
+        <v>1.237590596311E-4</v>
+      </c>
+      <c r="J63">
+        <v>1.2781285534871299E-4</v>
+      </c>
+      <c r="K63" s="11">
+        <f t="shared" ref="K63:K74" si="7">J63/I63</f>
+        <v>1.0327555471873857</v>
+      </c>
     </row>
     <row r="64" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="C64" s="3" t="s">
-        <v>4</v>
-      </c>
-      <c r="D64" s="3"/>
-      <c r="E64" s="9"/>
-      <c r="F64" s="3"/>
-      <c r="H64" s="3" t="s">
-        <v>3</v>
-      </c>
-      <c r="I64" s="3"/>
-      <c r="J64" s="9"/>
-      <c r="K64" s="9"/>
+      <c r="A64">
+        <v>1</v>
+      </c>
+      <c r="B64" s="5"/>
+      <c r="C64" s="2">
+        <v>6.2691724987101998E-3</v>
+      </c>
+      <c r="D64">
+        <v>2.0004896550590901E-4</v>
+      </c>
+      <c r="E64">
+        <v>2.0519183351723301E-4</v>
+      </c>
+      <c r="F64" s="10">
+        <f t="shared" si="6"/>
+        <v>1.0257080460192236</v>
+      </c>
+      <c r="G64" s="4"/>
+      <c r="I64">
+        <v>2.47009346021372E-4</v>
+      </c>
+      <c r="J64">
+        <v>2.5056736662623701E-4</v>
+      </c>
+      <c r="K64" s="10">
+        <f t="shared" si="7"/>
+        <v>1.0144043966844767</v>
+      </c>
     </row>
     <row r="65" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A65" s="6" t="s">
-        <v>0</v>
-      </c>
-      <c r="B65" s="6"/>
-      <c r="C65" s="6" t="s">
-        <v>1</v>
-      </c>
-      <c r="D65" s="6" t="s">
-        <v>7</v>
-      </c>
-      <c r="E65" s="6" t="s">
-        <v>6</v>
-      </c>
-      <c r="F65" s="7" t="s">
-        <v>8</v>
-      </c>
-      <c r="G65" s="8"/>
-      <c r="H65" s="6" t="s">
-        <v>1</v>
-      </c>
-      <c r="I65" s="6" t="s">
-        <v>7</v>
-      </c>
-      <c r="J65" s="6" t="s">
-        <v>6</v>
-      </c>
-      <c r="K65" s="7" t="s">
-        <v>8</v>
+      <c r="A65">
+        <v>10</v>
+      </c>
+      <c r="B65" s="5"/>
+      <c r="C65" s="2">
+        <v>1.2558983712415E-2</v>
+      </c>
+      <c r="D65">
+        <v>1.9727739159685499E-3</v>
+      </c>
+      <c r="E65">
+        <v>2.1002402963605799E-3</v>
+      </c>
+      <c r="F65" s="10">
+        <f t="shared" si="6"/>
+        <v>1.0646127665011473</v>
+      </c>
+      <c r="G65" s="4"/>
+      <c r="I65">
+        <v>2.41443999850058E-3</v>
+      </c>
+      <c r="J65">
+        <v>2.5624129143282902E-3</v>
+      </c>
+      <c r="K65" s="11">
+        <f t="shared" si="7"/>
+        <v>1.0612866403470804</v>
       </c>
     </row>
     <row r="66" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A66">
-        <v>0.1</v>
+        <v>25</v>
       </c>
       <c r="B66" s="5"/>
       <c r="C66" s="2">
-        <v>2.0906018648200899E-5</v>
-      </c>
-      <c r="D66" s="2">
-        <v>1.9785240862768899E-5</v>
-      </c>
-      <c r="E66" s="2">
-        <v>1.9417624590728801E-5</v>
+        <v>1.8782496824776201E-2</v>
+      </c>
+      <c r="D66">
+        <v>4.9269907229743297E-3</v>
+      </c>
+      <c r="E66">
+        <v>5.2981099306138504E-3</v>
       </c>
       <c r="F66" s="10">
-        <f>E66/D66</f>
-        <v>0.98141967163352228</v>
+        <f t="shared" si="6"/>
+        <v>1.0753237074121145</v>
       </c>
       <c r="G66" s="4"/>
-      <c r="H66" s="2"/>
-      <c r="I66" s="2">
-        <v>2.44555572729164E-5</v>
-      </c>
-      <c r="J66" s="2">
-        <v>2.3173152783100001E-5</v>
+      <c r="I66">
+        <v>6.11270182240103E-3</v>
+      </c>
+      <c r="J66">
+        <v>6.4145321839513504E-3</v>
       </c>
       <c r="K66" s="10">
-        <f>J66/I66</f>
-        <v>0.94756183735642718</v>
+        <f t="shared" si="7"/>
+        <v>1.0493775699060295</v>
       </c>
     </row>
     <row r="67" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A67">
-        <v>0.5</v>
+        <v>50</v>
       </c>
       <c r="B67" s="5"/>
       <c r="C67" s="2">
-        <v>3.1327203465188001E-3</v>
+        <v>2.51046376970986E-2</v>
       </c>
       <c r="D67">
-        <v>1.02051178015395E-4</v>
-      </c>
-      <c r="E67" s="2">
-        <v>9.4705678455829002E-5</v>
+        <v>9.7820010092556295E-3</v>
+      </c>
+      <c r="E67">
+        <v>1.0195154351149101E-2</v>
       </c>
       <c r="F67" s="10">
-        <f t="shared" ref="F67:F78" si="6">E67/D67</f>
-        <v>0.92802141334950694</v>
+        <f t="shared" si="6"/>
+        <v>1.0422360763919929</v>
       </c>
       <c r="G67" s="4"/>
       <c r="I67">
-        <v>1.237590596311E-4</v>
+        <v>1.20970549355645E-2</v>
       </c>
       <c r="J67">
-        <v>1.2781285534871299E-4</v>
+        <v>1.24175942421624E-2</v>
       </c>
       <c r="K67" s="11">
-        <f t="shared" ref="K67:K78" si="7">J67/I67</f>
-        <v>1.0327555471873857</v>
+        <f t="shared" si="7"/>
+        <v>1.0264973010625533</v>
       </c>
     </row>
     <row r="68" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A68">
-        <v>1</v>
+        <v>75</v>
       </c>
       <c r="B68" s="5"/>
       <c r="C68" s="2">
-        <v>6.2691724987101998E-3</v>
+        <v>3.1476119846668899E-2</v>
       </c>
       <c r="D68">
-        <v>2.0004896550590901E-4</v>
+        <v>1.43763436727791E-2</v>
       </c>
       <c r="E68">
-        <v>2.0519183351723301E-4</v>
+        <v>1.5782984835099299E-2</v>
       </c>
       <c r="F68" s="10">
         <f t="shared" si="6"/>
-        <v>1.0257080460192236</v>
+        <v>1.0978441524727602</v>
       </c>
       <c r="G68" s="4"/>
       <c r="I68">
-        <v>2.47009346021372E-4</v>
+        <v>1.8002551123509802E-2</v>
       </c>
       <c r="J68">
-        <v>2.5056736662623701E-4</v>
+        <v>1.8976376994297401E-2</v>
       </c>
       <c r="K68" s="10">
         <f t="shared" si="7"/>
-        <v>1.0144043966844767</v>
+        <v>1.0540937706054263</v>
       </c>
     </row>
     <row r="69" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A69">
-        <v>10</v>
+        <v>100</v>
       </c>
       <c r="B69" s="5"/>
       <c r="C69" s="2">
-        <v>1.2558983712415E-2</v>
+        <v>5.2878603388737497E-2</v>
       </c>
       <c r="D69">
-        <v>1.9727739159685499E-3</v>
+        <v>2.00458898906196E-2</v>
       </c>
       <c r="E69">
-        <v>2.1002402963605799E-3</v>
+        <v>2.0804120655568799E-2</v>
       </c>
       <c r="F69" s="10">
         <f t="shared" si="6"/>
-        <v>1.0646127665011473</v>
+        <v>1.0378247495664441</v>
       </c>
       <c r="G69" s="4"/>
       <c r="I69">
-        <v>2.41443999850058E-3</v>
+        <v>2.4309982506840501E-2</v>
       </c>
       <c r="J69">
-        <v>2.5624129143282902E-3</v>
+        <v>2.56065505285916E-2</v>
       </c>
       <c r="K69" s="11">
         <f t="shared" si="7"/>
-        <v>1.0612866403470804</v>
+        <v>1.0533347986320543</v>
       </c>
     </row>
     <row r="70" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A70">
-        <v>25</v>
+        <v>150</v>
       </c>
       <c r="B70" s="5"/>
       <c r="C70" s="2">
-        <v>1.8782496824776201E-2</v>
+        <v>0.107716927588289</v>
       </c>
       <c r="D70">
-        <v>4.9269907229743297E-3</v>
+        <v>3.0432830381329601E-2</v>
       </c>
       <c r="E70">
-        <v>5.2981099306138504E-3</v>
+        <v>3.14434702136525E-2</v>
       </c>
       <c r="F70" s="10">
         <f t="shared" si="6"/>
-        <v>1.0753237074121145</v>
+        <v>1.0332088675177227</v>
       </c>
       <c r="G70" s="4"/>
       <c r="I70">
-        <v>6.11270182240103E-3</v>
+        <v>3.5308084946377202E-2</v>
       </c>
       <c r="J70">
-        <v>6.4145321839513504E-3</v>
+        <v>3.7911161854217702E-2</v>
       </c>
       <c r="K70" s="10">
         <f t="shared" si="7"/>
-        <v>1.0493775699060295</v>
+        <v>1.0737246699104135</v>
       </c>
     </row>
     <row r="71" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A71">
-        <v>50</v>
+        <v>250</v>
       </c>
       <c r="B71" s="5"/>
       <c r="C71" s="2">
-        <v>2.51046376970986E-2</v>
+        <v>0.16515386445267599</v>
       </c>
       <c r="D71">
-        <v>9.7820010092556295E-3</v>
+        <v>4.89210306757277E-2</v>
       </c>
       <c r="E71">
-        <v>1.0195154351149101E-2</v>
+        <v>5.3975920537313898E-2</v>
       </c>
       <c r="F71" s="10">
         <f t="shared" si="6"/>
-        <v>1.0422360763919929</v>
+        <v>1.1033275421994369</v>
       </c>
       <c r="G71" s="4"/>
       <c r="I71">
-        <v>1.20970549355645E-2</v>
+        <v>5.8808790512075798E-2</v>
       </c>
       <c r="J71">
-        <v>1.24175942421624E-2</v>
+        <v>6.2265324575410202E-2</v>
       </c>
       <c r="K71" s="11">
         <f t="shared" si="7"/>
-        <v>1.0264973010625533</v>
+        <v>1.0587758060187387</v>
       </c>
     </row>
     <row r="72" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A72">
-        <v>75</v>
+        <v>500</v>
       </c>
       <c r="B72" s="5"/>
       <c r="C72" s="2">
-        <v>3.1476119846668899E-2</v>
+        <v>0.22114304090137801</v>
       </c>
       <c r="D72">
-        <v>1.43763436727791E-2</v>
+        <v>9.6226590649767796E-2</v>
       </c>
       <c r="E72">
-        <v>1.5782984835099299E-2</v>
+        <v>0.10212774105006001</v>
       </c>
       <c r="F72" s="10">
         <f t="shared" si="6"/>
-        <v>1.0978441524727602</v>
+        <v>1.0613255687481478</v>
       </c>
       <c r="G72" s="4"/>
       <c r="I72">
-        <v>1.8002551123509802E-2</v>
+        <v>0.11146020972599301</v>
       </c>
       <c r="J72">
-        <v>1.8976376994297401E-2</v>
+        <v>0.118001707852343</v>
       </c>
       <c r="K72" s="10">
         <f t="shared" si="7"/>
-        <v>1.0540937706054263</v>
+        <v>1.0586890886212328</v>
       </c>
     </row>
     <row r="73" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A73">
-        <v>100</v>
-      </c>
-      <c r="B73" s="5"/>
-      <c r="C73" s="2">
-        <v>5.2878603388737497E-2</v>
+        <v>750</v>
       </c>
       <c r="D73">
-        <v>2.00458898906196E-2</v>
+        <v>0.140294088260282</v>
       </c>
       <c r="E73">
-        <v>2.0804120655568799E-2</v>
+        <v>0.15225875418305601</v>
       </c>
       <c r="F73" s="10">
         <f t="shared" si="6"/>
-        <v>1.0378247495664441</v>
-      </c>
-      <c r="G73" s="4"/>
+        <v>1.0852827519045309</v>
+      </c>
       <c r="I73">
-        <v>2.4309982506840501E-2</v>
+        <v>0.164782092113922</v>
       </c>
       <c r="J73">
-        <v>2.56065505285916E-2</v>
+        <v>0.171436913407884</v>
       </c>
       <c r="K73" s="11">
         <f t="shared" si="7"/>
-        <v>1.0533347986320543</v>
+        <v>1.0403855856458066</v>
       </c>
     </row>
     <row r="74" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A74">
-        <v>150</v>
-      </c>
-      <c r="B74" s="5"/>
-      <c r="C74" s="2">
-        <v>0.107716927588289</v>
+        <v>999.99</v>
       </c>
       <c r="D74">
-        <v>3.0432830381329601E-2</v>
+        <v>0.181401571560247</v>
       </c>
       <c r="E74">
-        <v>3.14434702136525E-2</v>
+        <v>0.20058148390920799</v>
       </c>
       <c r="F74" s="10">
         <f t="shared" si="6"/>
-        <v>1.0332088675177227</v>
-      </c>
-      <c r="G74" s="4"/>
+        <v>1.1057317871283765</v>
+      </c>
       <c r="I74">
-        <v>3.5308084946377202E-2</v>
+        <v>0.211482254080264</v>
       </c>
       <c r="J74">
-        <v>3.7911161854217702E-2</v>
+        <v>0.22688990016688301</v>
       </c>
       <c r="K74" s="10">
         <f t="shared" si="7"/>
-        <v>1.0737246699104135</v>
-      </c>
-    </row>
-    <row r="75" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A75">
-        <v>250</v>
-      </c>
-      <c r="B75" s="5"/>
-      <c r="C75" s="2">
-        <v>0.16515386445267599</v>
-      </c>
-      <c r="D75">
-        <v>4.89210306757277E-2</v>
-      </c>
-      <c r="E75">
-        <v>5.3975920537313898E-2</v>
-      </c>
-      <c r="F75" s="10">
-        <f t="shared" si="6"/>
-        <v>1.1033275421994369</v>
-      </c>
-      <c r="G75" s="4"/>
-      <c r="I75">
-        <v>5.8808790512075798E-2</v>
-      </c>
-      <c r="J75">
-        <v>6.2265324575410202E-2</v>
-      </c>
-      <c r="K75" s="11">
-        <f t="shared" si="7"/>
-        <v>1.0587758060187387</v>
+        <v>1.0728555034256981</v>
       </c>
     </row>
     <row r="76" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A76">
-        <v>500</v>
-      </c>
-      <c r="B76" s="5"/>
-      <c r="C76" s="2">
-        <v>0.22114304090137801</v>
-      </c>
-      <c r="D76">
-        <v>9.6226590649767796E-2</v>
-      </c>
-      <c r="E76">
-        <v>0.10212774105006001</v>
-      </c>
-      <c r="F76" s="10">
-        <f t="shared" si="6"/>
-        <v>1.0613255687481478</v>
-      </c>
-      <c r="G76" s="4"/>
-      <c r="I76">
-        <v>0.11146020972599301</v>
-      </c>
-      <c r="J76">
-        <v>0.118001707852343</v>
-      </c>
-      <c r="K76" s="10">
-        <f t="shared" si="7"/>
-        <v>1.0586890886212328</v>
-      </c>
+      <c r="C76" s="12" t="s">
+        <v>10</v>
+      </c>
+      <c r="D76" s="12"/>
+      <c r="E76" s="13"/>
+      <c r="F76" s="13"/>
+      <c r="H76" s="2"/>
+      <c r="I76" s="2"/>
+      <c r="J76" s="2"/>
+      <c r="K76" s="2"/>
     </row>
     <row r="77" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A77">
-        <v>750</v>
-      </c>
-      <c r="D77">
-        <v>0.140294088260282</v>
-      </c>
-      <c r="E77">
-        <v>0.15225875418305601</v>
-      </c>
-      <c r="F77" s="10">
-        <f t="shared" si="6"/>
-        <v>1.0852827519045309</v>
-      </c>
-      <c r="I77">
-        <v>0.164782092113922</v>
-      </c>
-      <c r="J77">
-        <v>0.171436913407884</v>
-      </c>
-      <c r="K77" s="11">
-        <f t="shared" si="7"/>
-        <v>1.0403855856458066</v>
-      </c>
+      <c r="C77" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="D77" s="3"/>
+      <c r="E77" s="9"/>
+      <c r="F77" s="3"/>
+      <c r="H77" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="I77" s="3"/>
+      <c r="J77" s="9"/>
+      <c r="K77" s="9"/>
     </row>
     <row r="78" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A78">
-        <v>999.99</v>
-      </c>
-      <c r="D78">
-        <v>0.181401571560247</v>
-      </c>
-      <c r="E78">
-        <v>0.20058148390920799</v>
-      </c>
-      <c r="F78" s="10">
-        <f t="shared" si="6"/>
-        <v>1.1057317871283765</v>
-      </c>
-      <c r="I78">
-        <v>0.211482254080264</v>
-      </c>
-      <c r="J78">
-        <v>0.22688990016688301</v>
-      </c>
-      <c r="K78" s="10">
-        <f t="shared" si="7"/>
-        <v>1.0728555034256981</v>
+      <c r="A78" s="6" t="s">
+        <v>0</v>
+      </c>
+      <c r="B78" s="6"/>
+      <c r="C78" s="6" t="s">
+        <v>1</v>
+      </c>
+      <c r="D78" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="E78" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="F78" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="G78" s="8"/>
+      <c r="H78" s="6" t="s">
+        <v>1</v>
+      </c>
+      <c r="I78" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="J78" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="K78" s="7" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="79" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A79">
+        <v>0.1</v>
+      </c>
+      <c r="B79" s="5"/>
+      <c r="C79" s="2">
+        <v>2.0906018648200899E-5</v>
+      </c>
+      <c r="D79" s="2">
+        <v>2.8143173972499801E-7</v>
+      </c>
+      <c r="E79" s="2">
+        <v>1.46150091119403E-6</v>
+      </c>
+      <c r="F79" s="10">
+        <f t="shared" ref="F79:F90" si="8">F62*((E79/E62)^2 +(D79/D62)^2)^0.5</f>
+        <v>7.5175789820697683E-2</v>
+      </c>
+      <c r="G79" s="4"/>
+      <c r="H79" s="2"/>
+      <c r="I79" s="2">
+        <v>2.4434932696069799E-5</v>
+      </c>
+      <c r="J79" s="2">
+        <v>2.5518609602937599E-5</v>
+      </c>
+      <c r="K79" s="10">
+        <f>J79/I79</f>
+        <v>1.0443494942403546</v>
       </c>
     </row>
     <row r="80" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="C80" s="12" t="s">
+      <c r="A80">
+        <v>0.5</v>
+      </c>
+      <c r="B80" s="5"/>
+      <c r="C80" s="2">
+        <v>3.1327203465188001E-3</v>
+      </c>
+      <c r="D80" s="2">
+        <v>1.5222069872849199E-6</v>
+      </c>
+      <c r="E80" s="2">
+        <v>3.7622530224669299E-6</v>
+      </c>
+      <c r="F80" s="10">
+        <f t="shared" si="8"/>
+        <v>3.9379446327356661E-2</v>
+      </c>
+      <c r="G80" s="4"/>
+      <c r="I80">
+        <v>3.6561489620800698E-3</v>
+      </c>
+      <c r="J80">
+        <v>3.8583728177792702E-3</v>
+      </c>
+      <c r="K80" s="11">
+        <f t="shared" ref="K80:K89" si="9">J80/I80</f>
+        <v>1.0553106172085915</v>
+      </c>
+    </row>
+    <row r="81" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A81">
+        <v>1</v>
+      </c>
+      <c r="B81" s="5"/>
+      <c r="C81" s="2">
+        <v>6.2691724987101998E-3</v>
+      </c>
+      <c r="D81" s="2">
+        <v>2.33807312394273E-6</v>
+      </c>
+      <c r="E81" s="2">
+        <v>6.5127278910264096E-6</v>
+      </c>
+      <c r="F81" s="10">
+        <f t="shared" si="8"/>
+        <v>3.4692692812303069E-2</v>
+      </c>
+      <c r="G81" s="4"/>
+      <c r="I81">
+        <v>7.3167786817070497E-3</v>
+      </c>
+      <c r="J81">
+        <v>7.7206053021012903E-3</v>
+      </c>
+      <c r="K81" s="10">
+        <f t="shared" si="9"/>
+        <v>1.0551918594181156</v>
+      </c>
+    </row>
+    <row r="82" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A82">
         <v>10</v>
       </c>
-      <c r="D80" s="12"/>
-      <c r="E80" s="13"/>
-      <c r="F80" s="13"/>
-      <c r="H80" s="2"/>
-      <c r="I80" s="2"/>
-      <c r="J80" s="2"/>
-      <c r="K80" s="2"/>
-    </row>
-    <row r="81" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="C81" s="3" t="s">
-        <v>4</v>
-      </c>
-      <c r="D81" s="3"/>
-      <c r="E81" s="9"/>
-      <c r="F81" s="3"/>
-      <c r="H81" s="3" t="s">
-        <v>3</v>
-      </c>
-      <c r="I81" s="3"/>
-      <c r="J81" s="9"/>
-      <c r="K81" s="9"/>
-    </row>
-    <row r="82" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A82" s="6" t="s">
-        <v>0</v>
-      </c>
-      <c r="B82" s="6"/>
-      <c r="C82" s="6" t="s">
-        <v>1</v>
-      </c>
-      <c r="D82" s="6" t="s">
-        <v>7</v>
-      </c>
-      <c r="E82" s="6" t="s">
-        <v>6</v>
-      </c>
-      <c r="F82" s="7" t="s">
-        <v>8</v>
-      </c>
-      <c r="G82" s="8"/>
-      <c r="H82" s="6" t="s">
-        <v>1</v>
-      </c>
-      <c r="I82" s="6" t="s">
-        <v>7</v>
-      </c>
-      <c r="J82" s="6" t="s">
-        <v>6</v>
-      </c>
-      <c r="K82" s="7" t="s">
-        <v>8</v>
+      <c r="B82" s="5"/>
+      <c r="C82" s="2">
+        <v>1.2558983712415E-2</v>
+      </c>
+      <c r="D82" s="2">
+        <v>2.7701090496064399E-5</v>
+      </c>
+      <c r="E82" s="2">
+        <v>3.8011060965548303E-5</v>
+      </c>
+      <c r="F82" s="10">
+        <f t="shared" si="8"/>
+        <v>2.4386896067040687E-2</v>
+      </c>
+      <c r="G82" s="4"/>
+      <c r="I82">
+        <v>1.4655010559957399E-2</v>
+      </c>
+      <c r="J82">
+        <v>1.54708347850845E-2</v>
+      </c>
+      <c r="K82" s="11">
+        <f t="shared" si="9"/>
+        <v>1.0556686207621178</v>
       </c>
     </row>
     <row r="83" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A83">
-        <v>0.1</v>
+        <v>25</v>
       </c>
       <c r="B83" s="5"/>
       <c r="C83" s="2">
-        <v>2.0906018648200899E-5</v>
+        <v>1.8782496824776201E-2</v>
       </c>
       <c r="D83" s="2">
-        <v>2.8143173972499801E-7</v>
+        <v>8.0985715172972504E-5</v>
       </c>
       <c r="E83" s="2">
-        <v>1.46150091119403E-6</v>
+        <v>8.2936422592517207E-5</v>
       </c>
       <c r="F83" s="10">
-        <f t="shared" ref="F83:F94" si="8">F66*((E83/E66)^2 +(D83/D66)^2)^0.5</f>
-        <v>7.5175789820697683E-2</v>
+        <f t="shared" si="8"/>
+        <v>2.4408348565916203E-2</v>
       </c>
       <c r="G83" s="4"/>
-      <c r="H83" s="2"/>
-      <c r="I83" s="2">
-        <v>2.4434932696069799E-5</v>
-      </c>
-      <c r="J83" s="2">
-        <v>2.5518609602937599E-5</v>
+      <c r="I83">
+        <v>2.20520227131588E-2</v>
+      </c>
+      <c r="J83">
+        <v>2.3279563002525702E-2</v>
       </c>
       <c r="K83" s="10">
-        <f>J83/I83</f>
-        <v>1.0443494942403546</v>
+        <f t="shared" si="9"/>
+        <v>1.0556656550437167</v>
       </c>
     </row>
     <row r="84" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A84">
-        <v>0.5</v>
+        <v>50</v>
       </c>
       <c r="B84" s="5"/>
       <c r="C84" s="2">
-        <v>3.1327203465188001E-3</v>
-      </c>
-      <c r="D84" s="2">
-        <v>1.5222069872849199E-6</v>
-      </c>
-      <c r="E84" s="2">
-        <v>3.7622530224669299E-6</v>
+        <v>2.51046376970986E-2</v>
+      </c>
+      <c r="D84">
+        <v>1.14857385321631E-4</v>
+      </c>
+      <c r="E84">
+        <v>1.40546480514001E-4</v>
       </c>
       <c r="F84" s="10">
         <f t="shared" si="8"/>
-        <v>3.9379446327356661E-2</v>
+        <v>1.8873133491714433E-2</v>
       </c>
       <c r="G84" s="4"/>
       <c r="I84">
-        <v>3.6561489620800698E-3</v>
+        <v>2.9379142051595902E-2</v>
       </c>
       <c r="J84">
-        <v>3.8583728177792702E-3</v>
+        <v>3.0966693098777899E-2</v>
       </c>
       <c r="K84" s="11">
-        <f t="shared" ref="K84:K93" si="9">J84/I84</f>
-        <v>1.0553106172085915</v>
+        <f t="shared" si="9"/>
+        <v>1.0540366714723639</v>
       </c>
     </row>
     <row r="85" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A85">
-        <v>1</v>
+        <v>75</v>
       </c>
       <c r="B85" s="5"/>
       <c r="C85" s="2">
-        <v>6.2691724987101998E-3</v>
-      </c>
-      <c r="D85" s="2">
-        <v>2.33807312394273E-6</v>
-      </c>
-      <c r="E85" s="2">
-        <v>6.5127278910264096E-6</v>
+        <v>3.1476119846668899E-2</v>
+      </c>
+      <c r="D85">
+        <v>1.6692001786006801E-4</v>
+      </c>
+      <c r="E85">
+        <v>2.2355768083561999E-4</v>
       </c>
       <c r="F85" s="10">
         <f t="shared" si="8"/>
-        <v>3.4692692812303069E-2</v>
+        <v>2.0107088599017175E-2</v>
       </c>
       <c r="G85" s="4"/>
       <c r="I85">
-        <v>7.3167786817070497E-3</v>
+        <v>3.6804448452257998E-2</v>
       </c>
       <c r="J85">
-        <v>7.7206053021012903E-3</v>
+        <v>3.8844686371276298E-2</v>
       </c>
       <c r="K85" s="10">
         <f t="shared" si="9"/>
-        <v>1.0551918594181156</v>
+        <v>1.0554345467685748</v>
       </c>
     </row>
     <row r="86" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A86">
-        <v>10</v>
+        <v>100</v>
       </c>
       <c r="B86" s="5"/>
       <c r="C86" s="2">
-        <v>1.2558983712415E-2</v>
-      </c>
-      <c r="D86" s="2">
-        <v>2.7701090496064399E-5</v>
-      </c>
-      <c r="E86" s="2">
-        <v>3.8011060965548303E-5</v>
+        <v>5.2878603388737497E-2</v>
+      </c>
+      <c r="D86">
+        <v>2.77931449091848E-4</v>
+      </c>
+      <c r="E86">
+        <v>2.1739476286188801E-4</v>
       </c>
       <c r="F86" s="10">
         <f t="shared" si="8"/>
-        <v>2.4386896067040687E-2</v>
+        <v>1.8018315350781095E-2</v>
       </c>
       <c r="G86" s="4"/>
       <c r="I86">
-        <v>1.4655010559957399E-2</v>
+        <v>6.1567552933483601E-2</v>
       </c>
       <c r="J86">
-        <v>1.54708347850845E-2</v>
+        <v>6.4958585716827305E-2</v>
       </c>
       <c r="K86" s="11">
         <f t="shared" si="9"/>
-        <v>1.0556686207621178</v>
+        <v>1.0550782453057264</v>
       </c>
     </row>
     <row r="87" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A87">
-        <v>25</v>
+        <v>150</v>
       </c>
       <c r="B87" s="5"/>
       <c r="C87" s="2">
-        <v>1.8782496824776201E-2</v>
-      </c>
-      <c r="D87" s="2">
-        <v>8.0985715172972504E-5</v>
-      </c>
-      <c r="E87" s="2">
-        <v>8.2936422592517207E-5</v>
+        <v>0.107716927588289</v>
+      </c>
+      <c r="D87">
+        <v>3.3888866496247497E-4</v>
+      </c>
+      <c r="E87">
+        <v>4.2099807481717899E-4</v>
       </c>
       <c r="F87" s="10">
         <f t="shared" si="8"/>
-        <v>2.4408348565916203E-2</v>
+        <v>1.7992932963347683E-2</v>
       </c>
       <c r="G87" s="4"/>
       <c r="I87">
-        <v>2.20520227131588E-2</v>
+        <v>0.124585487877085</v>
       </c>
       <c r="J87">
-        <v>2.3279563002525702E-2</v>
+        <v>0.13088073929294</v>
       </c>
       <c r="K87" s="10">
         <f t="shared" si="9"/>
-        <v>1.0556656550437167</v>
+        <v>1.0505295722890764</v>
       </c>
     </row>
     <row r="88" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A88">
-        <v>50</v>
+        <v>250</v>
       </c>
       <c r="B88" s="5"/>
       <c r="C88" s="2">
-        <v>2.51046376970986E-2</v>
+        <v>0.16515386445267599</v>
       </c>
       <c r="D88">
-        <v>1.14857385321631E-4</v>
+        <v>6.0844630496931901E-4</v>
       </c>
       <c r="E88">
-        <v>1.40546480514001E-4</v>
+        <v>7.1735921087181002E-4</v>
       </c>
       <c r="F88" s="10">
         <f t="shared" si="8"/>
-        <v>1.8873133491714433E-2</v>
+        <v>2.0082997872230529E-2</v>
       </c>
       <c r="G88" s="4"/>
       <c r="I88">
-        <v>2.9379142051595902E-2</v>
+        <v>0.188315720076114</v>
       </c>
       <c r="J88">
-        <v>3.0966693098777899E-2</v>
+        <v>0.19671890522285099</v>
       </c>
       <c r="K88" s="11">
         <f t="shared" si="9"/>
-        <v>1.0540366714723639</v>
+        <v>1.0446228554012409</v>
       </c>
     </row>
     <row r="89" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A89">
-        <v>75</v>
+        <v>500</v>
       </c>
       <c r="B89" s="5"/>
       <c r="C89" s="2">
-        <v>3.1476119846668899E-2</v>
+        <v>0.22114304090137801</v>
       </c>
       <c r="D89">
-        <v>1.6692001786006801E-4</v>
+        <v>1.3901143553867799E-3</v>
       </c>
       <c r="E89">
-        <v>2.2355768083561999E-4</v>
+        <v>1.45703989958587E-3</v>
       </c>
       <c r="F89" s="10">
         <f t="shared" si="8"/>
-        <v>2.0107088599017175E-2</v>
+        <v>2.1548753693625213E-2</v>
       </c>
       <c r="G89" s="4"/>
       <c r="I89">
-        <v>3.6804448452257998E-2</v>
+        <v>0.25212873564071397</v>
       </c>
       <c r="J89">
-        <v>3.8844686371276298E-2</v>
+        <v>0.26159631710660702</v>
       </c>
       <c r="K89" s="10">
         <f t="shared" si="9"/>
-        <v>1.0554345467685748</v>
+        <v>1.0375505847908761</v>
       </c>
     </row>
     <row r="90" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A90">
-        <v>100</v>
-      </c>
-      <c r="B90" s="5"/>
-      <c r="C90" s="2">
-        <v>5.2878603388737497E-2</v>
+        <v>750</v>
       </c>
       <c r="D90">
-        <v>2.77931449091848E-4</v>
+        <v>1.59024586083695E-3</v>
       </c>
       <c r="E90">
-        <v>2.1739476286188801E-4</v>
+        <v>1.88927153592098E-3</v>
       </c>
       <c r="F90" s="10">
         <f t="shared" si="8"/>
-        <v>1.8018315350781095E-2</v>
-      </c>
-      <c r="G90" s="4"/>
-      <c r="I90">
-        <v>6.1567552933483601E-2</v>
-      </c>
-      <c r="J90">
-        <v>6.4958585716827305E-2</v>
-      </c>
-      <c r="K90" s="11">
-        <f t="shared" si="9"/>
-        <v>1.0550782453057264</v>
+        <v>1.8239532257896197E-2</v>
       </c>
     </row>
     <row r="91" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A91">
-        <v>150</v>
-      </c>
-      <c r="B91" s="5"/>
-      <c r="C91" s="2">
-        <v>0.107716927588289</v>
+        <v>999.99</v>
       </c>
       <c r="D91">
-        <v>3.3888866496247497E-4</v>
+        <v>2.0916951916344802E-3</v>
       </c>
       <c r="E91">
-        <v>4.2099807481717899E-4</v>
+        <v>2.14759074882869E-3</v>
       </c>
       <c r="F91" s="10">
-        <f t="shared" si="8"/>
-        <v>1.7992932963347683E-2</v>
-      </c>
-      <c r="G91" s="4"/>
-      <c r="I91">
-        <v>0.124585487877085</v>
-      </c>
-      <c r="J91">
-        <v>0.13088073929294</v>
-      </c>
-      <c r="K91" s="10">
-        <f t="shared" si="9"/>
-        <v>1.0505295722890764</v>
-      </c>
-    </row>
-    <row r="92" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A92">
-        <v>250</v>
-      </c>
-      <c r="B92" s="5"/>
-      <c r="C92" s="2">
-        <v>0.16515386445267599</v>
-      </c>
-      <c r="D92">
-        <v>6.0844630496931901E-4</v>
-      </c>
-      <c r="E92">
-        <v>7.1735921087181002E-4</v>
-      </c>
-      <c r="F92" s="10">
-        <f t="shared" si="8"/>
-        <v>2.0082997872230529E-2</v>
-      </c>
-      <c r="G92" s="4"/>
-      <c r="I92">
-        <v>0.188315720076114</v>
-      </c>
-      <c r="J92">
-        <v>0.19671890522285099</v>
-      </c>
-      <c r="K92" s="11">
-        <f t="shared" si="9"/>
-        <v>1.0446228554012409</v>
-      </c>
-    </row>
-    <row r="93" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A93">
-        <v>500</v>
-      </c>
-      <c r="B93" s="5"/>
-      <c r="C93" s="2">
-        <v>0.22114304090137801</v>
-      </c>
-      <c r="D93">
-        <v>1.3901143553867799E-3</v>
-      </c>
-      <c r="E93">
-        <v>1.45703989958587E-3</v>
-      </c>
-      <c r="F93" s="10">
-        <f t="shared" si="8"/>
-        <v>2.1548753693625213E-2</v>
-      </c>
-      <c r="G93" s="4"/>
-      <c r="I93">
-        <v>0.25212873564071397</v>
-      </c>
-      <c r="J93">
-        <v>0.26159631710660702</v>
-      </c>
-      <c r="K93" s="10">
-        <f t="shared" si="9"/>
-        <v>1.0375505847908761</v>
-      </c>
-    </row>
-    <row r="94" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A94">
-        <v>750</v>
-      </c>
-      <c r="D94">
-        <v>1.59024586083695E-3</v>
-      </c>
-      <c r="E94">
-        <v>1.88927153592098E-3</v>
-      </c>
-      <c r="F94" s="10">
-        <f t="shared" si="8"/>
-        <v>1.8239532257896197E-2</v>
-      </c>
-    </row>
-    <row r="95" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A95">
-        <v>999.99</v>
-      </c>
-      <c r="D95">
-        <v>2.0916951916344802E-3</v>
-      </c>
-      <c r="E95">
-        <v>2.14759074882869E-3</v>
-      </c>
-      <c r="F95" s="10">
-        <f>F78*((E95/E78)^2 +(D95/D78)^2)^0.5</f>
+        <f>F74*((E91/E74)^2 +(D91/D74)^2)^0.5</f>
         <v>1.7398828006913617E-2</v>
       </c>
     </row>

</xml_diff>

<commit_message>
porting dcll runs to della
</commit_message>
<xml_diff>
--- a/Jupyter/Wedge/wedge_data_2026-03-25.xlsx
+++ b/Jupyter/Wedge/wedge_data_2026-03-25.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\patri\projects\emma-openmc\Jupyter\Wedge\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BDAEB268-8B64-460D-9E40-EF1FACC7331B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9AB2CA5D-4A5C-4C3D-AD30-BA95464744A9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="17496" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -327,16 +327,16 @@
                 <c:formatCode>0.000000</c:formatCode>
                 <c:ptCount val="13"/>
                 <c:pt idx="0">
-                  <c:v>0</c:v>
+                  <c:v>0.67015864678428949</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0</c:v>
+                  <c:v>0.67399433743759052</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>0</c:v>
+                  <c:v>0.67258163487423628</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>0</c:v>
+                  <c:v>0.69883311557825745</c:v>
                 </c:pt>
                 <c:pt idx="4">
                   <c:v>0</c:v>
@@ -903,16 +903,16 @@
                 <c:formatCode>0.000000</c:formatCode>
                 <c:ptCount val="13"/>
                 <c:pt idx="0">
-                  <c:v>0</c:v>
+                  <c:v>1.0001629351709587</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0</c:v>
+                  <c:v>1.0000650261216626</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>0</c:v>
+                  <c:v>0.99996036360746876</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>0</c:v>
+                  <c:v>1.0005266084564297</c:v>
                 </c:pt>
                 <c:pt idx="4">
                   <c:v>0</c:v>
@@ -1436,10 +1436,10 @@
           </c:marker>
           <c:xVal>
             <c:numRef>
-              <c:f>'Sheet 1'!$A$62:$A$72</c:f>
+              <c:f>'Sheet 1'!$A$62:$A$74</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="11"/>
+                <c:ptCount val="13"/>
                 <c:pt idx="0">
                   <c:v>0.1</c:v>
                 </c:pt>
@@ -1472,16 +1472,22 @@
                 </c:pt>
                 <c:pt idx="10">
                   <c:v>500</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>750</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>999.99</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>'Sheet 1'!$F$62:$F$72</c:f>
+              <c:f>'Sheet 1'!$F$62:$F$74</c:f>
               <c:numCache>
                 <c:formatCode>0.000000</c:formatCode>
-                <c:ptCount val="11"/>
+                <c:ptCount val="13"/>
                 <c:pt idx="0">
                   <c:v>0.98141967163352228</c:v>
                 </c:pt>
@@ -1514,6 +1520,12 @@
                 </c:pt>
                 <c:pt idx="10">
                   <c:v>1.0613255687481478</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>1.0852827519045309</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>1.1057317871283765</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1800,10 +1812,10 @@
           </c:marker>
           <c:xVal>
             <c:numRef>
-              <c:f>'Sheet 1'!$A$44:$A$54</c:f>
+              <c:f>'Sheet 1'!$A$44:$A$56</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="11"/>
+                <c:ptCount val="13"/>
                 <c:pt idx="0">
                   <c:v>0.1</c:v>
                 </c:pt>
@@ -1836,16 +1848,22 @@
                 </c:pt>
                 <c:pt idx="10">
                   <c:v>500</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>750</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>999.99</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>'Sheet 1'!$F$44:$F$54</c:f>
+              <c:f>'Sheet 1'!$F$44:$F$56</c:f>
               <c:numCache>
                 <c:formatCode>0.000000</c:formatCode>
-                <c:ptCount val="11"/>
+                <c:ptCount val="13"/>
                 <c:pt idx="0">
                   <c:v>0.9985035371420129</c:v>
                 </c:pt>
@@ -1878,6 +1896,12 @@
                 </c:pt>
                 <c:pt idx="10">
                   <c:v>0.99666881879093805</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>1.0030035803296993</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>1.0148841983751864</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -4305,15 +4329,15 @@
   <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>12</xdr:col>
-      <xdr:colOff>132179</xdr:colOff>
+      <xdr:colOff>383970</xdr:colOff>
       <xdr:row>20</xdr:row>
-      <xdr:rowOff>56857</xdr:rowOff>
+      <xdr:rowOff>103240</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>19</xdr:col>
-      <xdr:colOff>436979</xdr:colOff>
+      <xdr:col>20</xdr:col>
+      <xdr:colOff>79170</xdr:colOff>
       <xdr:row>37</xdr:row>
-      <xdr:rowOff>56857</xdr:rowOff>
+      <xdr:rowOff>103240</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
@@ -4341,13 +4365,13 @@
   <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>12</xdr:col>
-      <xdr:colOff>300990</xdr:colOff>
+      <xdr:colOff>373877</xdr:colOff>
       <xdr:row>2</xdr:row>
       <xdr:rowOff>99060</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>19</xdr:col>
-      <xdr:colOff>605790</xdr:colOff>
+      <xdr:col>20</xdr:col>
+      <xdr:colOff>69077</xdr:colOff>
       <xdr:row>17</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:to>
@@ -4376,16 +4400,16 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>11</xdr:col>
-      <xdr:colOff>868680</xdr:colOff>
-      <xdr:row>57</xdr:row>
-      <xdr:rowOff>76200</xdr:rowOff>
+      <xdr:col>12</xdr:col>
+      <xdr:colOff>7289</xdr:colOff>
+      <xdr:row>59</xdr:row>
+      <xdr:rowOff>9939</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>19</xdr:col>
-      <xdr:colOff>198120</xdr:colOff>
-      <xdr:row>72</xdr:row>
-      <xdr:rowOff>76200</xdr:rowOff>
+      <xdr:colOff>310764</xdr:colOff>
+      <xdr:row>74</xdr:row>
+      <xdr:rowOff>9939</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
@@ -4412,16 +4436,16 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>11</xdr:col>
-      <xdr:colOff>929640</xdr:colOff>
-      <xdr:row>40</xdr:row>
-      <xdr:rowOff>7620</xdr:rowOff>
+      <xdr:col>12</xdr:col>
+      <xdr:colOff>8614</xdr:colOff>
+      <xdr:row>41</xdr:row>
+      <xdr:rowOff>20871</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>19</xdr:col>
-      <xdr:colOff>259080</xdr:colOff>
-      <xdr:row>56</xdr:row>
-      <xdr:rowOff>7620</xdr:rowOff>
+      <xdr:colOff>312089</xdr:colOff>
+      <xdr:row>57</xdr:row>
+      <xdr:rowOff>20871</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
@@ -4794,12 +4818,15 @@
         <v>0.1</v>
       </c>
       <c r="B5" s="5"/>
+      <c r="D5">
+        <v>1.3891095589010301</v>
+      </c>
       <c r="E5">
         <v>1.38933589370449</v>
       </c>
-      <c r="F5" s="10" t="e">
+      <c r="F5" s="10">
         <f>E5/D5</f>
-        <v>#DIV/0!</v>
+        <v>1.0001629351709587</v>
       </c>
       <c r="G5" s="4"/>
       <c r="K5" s="10" t="e">
@@ -4813,12 +4840,15 @@
         <v>0.5</v>
       </c>
       <c r="B6" s="5"/>
+      <c r="D6">
+        <v>1.38907673010083</v>
+      </c>
       <c r="E6">
         <v>1.3891670563732801</v>
       </c>
-      <c r="F6" s="10" t="e">
+      <c r="F6" s="10">
         <f t="shared" ref="F6:F17" si="0">E6/D6</f>
-        <v>#DIV/0!</v>
+        <v>1.0000650261216626</v>
       </c>
       <c r="G6" s="4"/>
       <c r="K6" s="10" t="e">
@@ -4832,12 +4862,15 @@
         <v>1</v>
       </c>
       <c r="B7" s="5"/>
+      <c r="D7">
+        <v>1.3889139640202901</v>
+      </c>
       <c r="E7">
         <v>1.3888589124812201</v>
       </c>
-      <c r="F7" s="10" t="e">
+      <c r="F7" s="10">
         <f t="shared" si="0"/>
-        <v>#DIV/0!</v>
+        <v>0.99996036360746876</v>
       </c>
       <c r="G7" s="4"/>
       <c r="K7" s="10" t="e">
@@ -4851,12 +4884,15 @@
         <v>10</v>
       </c>
       <c r="B8" s="5"/>
+      <c r="D8">
+        <v>1.38607567014507</v>
+      </c>
       <c r="E8">
         <v>1.3868055893142199</v>
       </c>
-      <c r="F8" s="10" t="e">
+      <c r="F8" s="10">
         <f t="shared" si="0"/>
-        <v>#DIV/0!</v>
+        <v>1.0005266084564297</v>
       </c>
       <c r="G8" s="4"/>
       <c r="K8" s="10" t="e">
@@ -5117,13 +5153,15 @@
       </c>
       <c r="B24" s="5"/>
       <c r="C24" s="2"/>
-      <c r="D24" s="2"/>
+      <c r="D24" s="2">
+        <v>3.4601339198647797E-5</v>
+      </c>
       <c r="E24" s="2">
         <v>2.3188386654289999E-5</v>
       </c>
-      <c r="F24" s="10" t="e">
+      <c r="F24" s="10">
         <f>E24/D24</f>
-        <v>#DIV/0!</v>
+        <v>0.67015864678428949</v>
       </c>
       <c r="G24" s="4"/>
       <c r="H24" s="2"/>
@@ -5140,12 +5178,15 @@
         <v>0.5</v>
       </c>
       <c r="B25" s="5"/>
+      <c r="D25">
+        <v>1.7267075850167999E-4</v>
+      </c>
       <c r="E25">
         <v>1.16379113471186E-4</v>
       </c>
-      <c r="F25" s="10" t="e">
+      <c r="F25" s="10">
         <f t="shared" ref="F25:F36" si="2">E25/D25</f>
-        <v>#DIV/0!</v>
+        <v>0.67399433743759052</v>
       </c>
       <c r="G25" s="4"/>
       <c r="K25" s="10" t="e">
@@ -5159,12 +5200,15 @@
         <v>1</v>
       </c>
       <c r="B26" s="5"/>
+      <c r="D26">
+        <v>3.4444202449192702E-4</v>
+      </c>
       <c r="E26">
         <v>2.31665379952172E-4</v>
       </c>
-      <c r="F26" s="10" t="e">
+      <c r="F26" s="10">
         <f t="shared" si="2"/>
-        <v>#DIV/0!</v>
+        <v>0.67258163487423628</v>
       </c>
       <c r="G26" s="4"/>
       <c r="K26" s="10" t="e">
@@ -5178,12 +5222,15 @@
         <v>10</v>
       </c>
       <c r="B27" s="5"/>
+      <c r="D27">
+        <v>3.33054467027722E-3</v>
+      </c>
       <c r="E27">
         <v>2.3274949085023899E-3</v>
       </c>
-      <c r="F27" s="10" t="e">
+      <c r="F27" s="10">
         <f t="shared" si="2"/>
-        <v>#DIV/0!</v>
+        <v>0.69883311557825745</v>
       </c>
       <c r="G27" s="4"/>
       <c r="K27" s="10" t="e">
@@ -5429,9 +5476,6 @@
         <v>0.1</v>
       </c>
       <c r="B44" s="5"/>
-      <c r="C44">
-        <v>1.38755773111088</v>
-      </c>
       <c r="D44">
         <v>1.33146077610654</v>
       </c>
@@ -5459,9 +5503,6 @@
         <v>0.5</v>
       </c>
       <c r="B45" s="5"/>
-      <c r="C45">
-        <v>1.38409520401011</v>
-      </c>
       <c r="D45">
         <v>1.35765661048369</v>
       </c>
@@ -5490,9 +5531,6 @@
         <v>1</v>
       </c>
       <c r="B46" s="5"/>
-      <c r="C46">
-        <v>1.3811622398640599</v>
-      </c>
       <c r="D46">
         <v>1.33903476392587</v>
       </c>
@@ -5520,9 +5558,6 @@
         <v>10</v>
       </c>
       <c r="B47" s="5"/>
-      <c r="C47">
-        <v>1.37486493369789</v>
-      </c>
       <c r="D47">
         <v>1.31789010731641</v>
       </c>
@@ -5551,9 +5586,6 @@
         <v>25</v>
       </c>
       <c r="B48" s="5"/>
-      <c r="C48">
-        <v>1.36350384779266</v>
-      </c>
       <c r="D48">
         <v>1.32036564820574</v>
       </c>
@@ -5581,9 +5613,6 @@
         <v>50</v>
       </c>
       <c r="B49" s="5"/>
-      <c r="C49">
-        <v>1.3571706170428599</v>
-      </c>
       <c r="D49">
         <v>1.3197738196808499</v>
       </c>
@@ -5612,9 +5641,6 @@
         <v>75</v>
       </c>
       <c r="B50" s="5"/>
-      <c r="C50">
-        <v>1.35109721915133</v>
-      </c>
       <c r="D50">
         <v>1.29935652652886</v>
       </c>
@@ -5642,9 +5668,6 @@
         <v>100</v>
       </c>
       <c r="B51" s="5"/>
-      <c r="C51">
-        <v>1.32844051248484</v>
-      </c>
       <c r="D51">
         <v>1.33910590256307</v>
       </c>
@@ -5673,9 +5696,6 @@
         <v>150</v>
       </c>
       <c r="B52" s="5"/>
-      <c r="C52">
-        <v>1.26939305918802</v>
-      </c>
       <c r="D52">
         <v>1.3346899335651701</v>
       </c>
@@ -5703,9 +5723,6 @@
         <v>250</v>
       </c>
       <c r="B53" s="5"/>
-      <c r="C53">
-        <v>1.2146497361047901</v>
-      </c>
       <c r="D53">
         <v>1.29678717701069</v>
       </c>
@@ -5734,9 +5751,6 @@
         <v>500</v>
       </c>
       <c r="B54" s="5"/>
-      <c r="C54">
-        <v>1.1436421352186501</v>
-      </c>
       <c r="D54">
         <v>1.2662694099393199</v>
       </c>
@@ -5763,6 +5777,7 @@
       <c r="A55">
         <v>750</v>
       </c>
+      <c r="B55" s="5"/>
       <c r="D55">
         <v>1.23279071771682</v>
       </c>
@@ -5773,6 +5788,7 @@
         <f t="shared" si="4"/>
         <v>1.0030035803296993</v>
       </c>
+      <c r="G55" s="5"/>
       <c r="I55">
         <v>1.1807532343395699</v>
       </c>
@@ -5784,6 +5800,7 @@
       <c r="A56">
         <v>999.99</v>
       </c>
+      <c r="B56" s="5"/>
       <c r="D56">
         <v>1.1928852496040101</v>
       </c>
@@ -5794,6 +5811,7 @@
         <f t="shared" si="4"/>
         <v>1.0148841983751864</v>
       </c>
+      <c r="G56" s="5"/>
       <c r="I56">
         <v>1.13357719050286</v>
       </c>
@@ -6193,6 +6211,7 @@
       <c r="A73">
         <v>750</v>
       </c>
+      <c r="B73" s="5"/>
       <c r="D73">
         <v>0.140294088260282</v>
       </c>
@@ -6203,6 +6222,7 @@
         <f t="shared" si="6"/>
         <v>1.0852827519045309</v>
       </c>
+      <c r="G73" s="5"/>
       <c r="I73">
         <v>0.164782092113922</v>
       </c>
@@ -6218,6 +6238,7 @@
       <c r="A74">
         <v>999.99</v>
       </c>
+      <c r="B74" s="5"/>
       <c r="D74">
         <v>0.181401571560247</v>
       </c>
@@ -6228,6 +6249,7 @@
         <f t="shared" si="6"/>
         <v>1.1057317871283765</v>
       </c>
+      <c r="G74" s="5"/>
       <c r="I74">
         <v>0.211482254080264</v>
       </c>

</xml_diff>

<commit_message>
prism hcpb u238 and th232
</commit_message>
<xml_diff>
--- a/Jupyter/Wedge/wedge_data_2026-03-25.xlsx
+++ b/Jupyter/Wedge/wedge_data_2026-03-25.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\patri\projects\emma-openmc\Jupyter\Wedge\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9AB2CA5D-4A5C-4C3D-AD30-BA95464744A9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2727A53E-B710-49C1-8960-17B14C6CB01B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="17496" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="61" uniqueCount="11">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="67" uniqueCount="14">
   <si>
     <t>Fertile kg/m3</t>
   </si>
@@ -70,13 +70,23 @@
   <si>
     <t>FISSILE PRODUCTION RATE ERROR PROPAGATION [ RXNS/SRC-N ]</t>
   </si>
+  <si>
+    <t>A-err</t>
+  </si>
+  <si>
+    <t>C-err</t>
+  </si>
+  <si>
+    <t>=C/A err</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="1">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="0.000000"/>
+    <numFmt numFmtId="173" formatCode="0.00000000"/>
   </numFmts>
   <fonts count="6" x14ac:knownFonts="1">
     <font>
@@ -163,7 +173,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="11" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -180,6 +190,7 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="11" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="173" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -322,7 +333,7 @@
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>'Sheet 1'!$F$24:$F$36</c:f>
+              <c:f>'Sheet 1'!$H$24:$H$36</c:f>
               <c:numCache>
                 <c:formatCode>0.000000</c:formatCode>
                 <c:ptCount val="13"/>
@@ -339,31 +350,31 @@
                   <c:v>0.69883311557825745</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>0</c:v>
+                  <c:v>0.73244907600666376</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>0</c:v>
+                  <c:v>0.76691398093902452</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>0</c:v>
+                  <c:v>0.79412199858198884</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>0</c:v>
+                  <c:v>0.82771654679092965</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>0</c:v>
+                  <c:v>0.87277793951821403</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>0</c:v>
+                  <c:v>0.90774216971761523</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>0</c:v>
+                  <c:v>0.96885985849430767</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>0</c:v>
+                  <c:v>1.0035052756769365</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>0</c:v>
+                  <c:v>1.0159556160581653</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -450,7 +461,7 @@
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>'Sheet 1'!$K$24:$K$36</c:f>
+              <c:f>'Sheet 1'!$N$24:$N$36</c:f>
               <c:numCache>
                 <c:formatCode>0.000000</c:formatCode>
                 <c:ptCount val="13"/>
@@ -898,7 +909,7 @@
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>'Sheet 1'!$F$5:$F$17</c:f>
+              <c:f>'Sheet 1'!$H$5:$H$17</c:f>
               <c:numCache>
                 <c:formatCode>0.000000</c:formatCode>
                 <c:ptCount val="13"/>
@@ -915,31 +926,31 @@
                   <c:v>1.0005266084564297</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>0</c:v>
+                  <c:v>1.0018467149465879</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>0</c:v>
+                  <c:v>1.002287048308576</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>0</c:v>
+                  <c:v>1.0038025582102672</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>0</c:v>
+                  <c:v>1.0036838050286592</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>0</c:v>
+                  <c:v>1.002467577491776</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>0</c:v>
+                  <c:v>1.000596548769378</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>0</c:v>
+                  <c:v>1.0015290596941282</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>0</c:v>
+                  <c:v>1.0029865814925498</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>0</c:v>
+                  <c:v>1.0003513071302839</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1077,7 +1088,7 @@
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>'Sheet 1'!$K$5:$K$17</c:f>
+              <c:f>'Sheet 1'!$N$5:$N$17</c:f>
               <c:numCache>
                 <c:formatCode>0.000000</c:formatCode>
                 <c:ptCount val="13"/>
@@ -1403,7 +1414,7 @@
           <c:order val="0"/>
           <c:tx>
             <c:strRef>
-              <c:f>'Sheet 1'!$F$61</c:f>
+              <c:f>'Sheet 1'!$I$61</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -1484,7 +1495,7 @@
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>'Sheet 1'!$F$62:$F$74</c:f>
+              <c:f>'Sheet 1'!$I$62:$I$74</c:f>
               <c:numCache>
                 <c:formatCode>0.000000</c:formatCode>
                 <c:ptCount val="13"/>
@@ -1779,7 +1790,7 @@
           <c:order val="0"/>
           <c:tx>
             <c:strRef>
-              <c:f>'Sheet 1'!$F$43</c:f>
+              <c:f>'Sheet 1'!$I$43</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -1860,7 +1871,7 @@
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>'Sheet 1'!$F$44:$F$56</c:f>
+              <c:f>'Sheet 1'!$I$44:$I$56</c:f>
               <c:numCache>
                 <c:formatCode>0.000000</c:formatCode>
                 <c:ptCount val="13"/>
@@ -4328,13 +4339,13 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>12</xdr:col>
+      <xdr:col>15</xdr:col>
       <xdr:colOff>383970</xdr:colOff>
       <xdr:row>20</xdr:row>
       <xdr:rowOff>103240</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>20</xdr:col>
+      <xdr:col>23</xdr:col>
       <xdr:colOff>79170</xdr:colOff>
       <xdr:row>37</xdr:row>
       <xdr:rowOff>103240</xdr:rowOff>
@@ -4364,13 +4375,13 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>12</xdr:col>
+      <xdr:col>15</xdr:col>
       <xdr:colOff>373877</xdr:colOff>
       <xdr:row>2</xdr:row>
       <xdr:rowOff>99060</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>20</xdr:col>
+      <xdr:col>23</xdr:col>
       <xdr:colOff>69077</xdr:colOff>
       <xdr:row>17</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
@@ -4400,13 +4411,13 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>12</xdr:col>
+      <xdr:col>15</xdr:col>
       <xdr:colOff>7289</xdr:colOff>
       <xdr:row>59</xdr:row>
       <xdr:rowOff>9939</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>19</xdr:col>
+      <xdr:col>22</xdr:col>
       <xdr:colOff>310764</xdr:colOff>
       <xdr:row>74</xdr:row>
       <xdr:rowOff>9939</xdr:rowOff>
@@ -4436,13 +4447,13 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>12</xdr:col>
+      <xdr:col>15</xdr:col>
       <xdr:colOff>8614</xdr:colOff>
       <xdr:row>41</xdr:row>
       <xdr:rowOff>20871</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>19</xdr:col>
+      <xdr:col>22</xdr:col>
       <xdr:colOff>312089</xdr:colOff>
       <xdr:row>57</xdr:row>
       <xdr:rowOff>20871</xdr:rowOff>
@@ -4736,52 +4747,58 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C22416C2-1180-4450-A3B0-0B08DD9AEC85}">
-  <dimension ref="A1:L91"/>
+  <dimension ref="A1:O91"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="12.33203125" customWidth="1"/>
     <col min="2" max="2" width="2.109375" customWidth="1"/>
-    <col min="3" max="4" width="12.21875" customWidth="1"/>
-    <col min="5" max="5" width="15.88671875" customWidth="1"/>
-    <col min="6" max="6" width="15.6640625" customWidth="1"/>
-    <col min="7" max="7" width="2.77734375" customWidth="1"/>
-    <col min="8" max="11" width="13.33203125" customWidth="1"/>
-    <col min="12" max="12" width="14.21875" customWidth="1"/>
+    <col min="3" max="5" width="12.21875" customWidth="1"/>
+    <col min="6" max="8" width="15.88671875" customWidth="1"/>
+    <col min="9" max="9" width="15.109375" customWidth="1"/>
+    <col min="10" max="10" width="2.77734375" customWidth="1"/>
+    <col min="11" max="14" width="13.33203125" customWidth="1"/>
+    <col min="15" max="15" width="14.21875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="H1" s="1"/>
-      <c r="I1" s="1"/>
-      <c r="J1" s="1"/>
+    <row r="1" spans="1:15" x14ac:dyDescent="0.3">
       <c r="K1" s="1"/>
-    </row>
-    <row r="2" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="L1" s="1"/>
+      <c r="M1" s="1"/>
+      <c r="N1" s="1"/>
+    </row>
+    <row r="2" spans="1:15" x14ac:dyDescent="0.3">
       <c r="C2" s="14" t="s">
         <v>2</v>
       </c>
       <c r="D2" s="14"/>
-      <c r="E2" s="15"/>
-      <c r="H2" s="2"/>
-      <c r="I2" s="2"/>
-      <c r="J2" s="2"/>
+      <c r="E2" s="14"/>
+      <c r="F2" s="15"/>
+      <c r="G2" s="15"/>
+      <c r="H2" s="15"/>
       <c r="K2" s="2"/>
-    </row>
-    <row r="3" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="L2" s="2"/>
+      <c r="M2" s="2"/>
+      <c r="N2" s="2"/>
+    </row>
+    <row r="3" spans="1:15" x14ac:dyDescent="0.3">
       <c r="C3" s="3" t="s">
         <v>4</v>
       </c>
       <c r="D3" s="3"/>
-      <c r="E3" s="9"/>
-      <c r="F3" s="3"/>
-      <c r="H3" s="3" t="s">
+      <c r="E3" s="3"/>
+      <c r="F3" s="9"/>
+      <c r="G3" s="9"/>
+      <c r="H3" s="9"/>
+      <c r="I3" s="3"/>
+      <c r="K3" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="I3" s="3"/>
-      <c r="J3" s="9"/>
-      <c r="K3" s="9"/>
       <c r="L3" s="3"/>
-    </row>
-    <row r="4" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="M3" s="9"/>
+      <c r="N3" s="9"/>
+      <c r="O3" s="3"/>
+    </row>
+    <row r="4" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A4" s="6" t="s">
         <v>0</v>
       </c>
@@ -4793,27 +4810,36 @@
         <v>7</v>
       </c>
       <c r="E4" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="F4" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="F4" s="7" t="s">
+      <c r="G4" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="H4" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="G4" s="8"/>
-      <c r="H4" s="6" t="s">
+      <c r="I4" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="J4" s="8"/>
+      <c r="K4" s="6" t="s">
         <v>1</v>
       </c>
-      <c r="I4" s="6" t="s">
+      <c r="L4" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="J4" s="6" t="s">
+      <c r="M4" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="K4" s="7" t="s">
+      <c r="N4" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="L4" s="7"/>
-    </row>
-    <row r="5" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="O4" s="7"/>
+    </row>
+    <row r="5" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A5">
         <v>0.1</v>
       </c>
@@ -4822,20 +4848,33 @@
         <v>1.3891095589010301</v>
       </c>
       <c r="E5">
+        <v>1.02494314460544E-4</v>
+      </c>
+      <c r="F5">
         <v>1.38933589370449</v>
       </c>
-      <c r="F5" s="10">
-        <f>E5/D5</f>
+      <c r="G5">
+        <v>1.1377551521665301E-4</v>
+      </c>
+      <c r="H5" s="10">
+        <f>F5/D5</f>
         <v>1.0001629351709587</v>
       </c>
-      <c r="G5" s="4"/>
-      <c r="K5" s="10" t="e">
-        <f>J5/I5</f>
+      <c r="I5">
+        <f>H5*((E5/D5)^2 +(G5/F5)^2)^0.5</f>
+        <v>1.1024684824037706E-4</v>
+      </c>
+      <c r="J5" s="4"/>
+      <c r="M5">
+        <v>1.38932778213898</v>
+      </c>
+      <c r="N5" s="10" t="e">
+        <f>M5/L5</f>
         <v>#DIV/0!</v>
       </c>
-      <c r="L5" s="10"/>
-    </row>
-    <row r="6" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="O5" s="10"/>
+    </row>
+    <row r="6" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A6">
         <v>0.5</v>
       </c>
@@ -4844,20 +4883,33 @@
         <v>1.38907673010083</v>
       </c>
       <c r="E6">
+        <v>1.52707495750366E-4</v>
+      </c>
+      <c r="F6">
         <v>1.3891670563732801</v>
       </c>
-      <c r="F6" s="10">
-        <f t="shared" ref="F6:F17" si="0">E6/D6</f>
+      <c r="G6">
+        <v>1.6878154642812701E-4</v>
+      </c>
+      <c r="H6" s="10">
+        <f>F6/D6</f>
         <v>1.0000650261216626</v>
       </c>
-      <c r="G6" s="4"/>
-      <c r="K6" s="10" t="e">
-        <f t="shared" ref="K6:K17" si="1">J6/I6</f>
+      <c r="I6">
+        <f t="shared" ref="I6:I16" si="0">H6*((E6/D6)^2 +(G6/F6)^2)^0.5</f>
+        <v>1.6386259048946993E-4</v>
+      </c>
+      <c r="J6" s="4"/>
+      <c r="M6">
+        <v>1.38912815811046</v>
+      </c>
+      <c r="N6" s="10" t="e">
+        <f t="shared" ref="N6:N17" si="1">M6/L6</f>
         <v>#DIV/0!</v>
       </c>
-      <c r="L6" s="10"/>
-    </row>
-    <row r="7" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="O6" s="10"/>
+    </row>
+    <row r="7" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A7">
         <v>1</v>
       </c>
@@ -4866,20 +4918,33 @@
         <v>1.3889139640202901</v>
       </c>
       <c r="E7">
+        <v>1.8201886596701201E-4</v>
+      </c>
+      <c r="F7">
         <v>1.3888589124812201</v>
       </c>
-      <c r="F7" s="10">
+      <c r="G7">
+        <v>1.54337152453701E-4</v>
+      </c>
+      <c r="H7" s="10">
+        <f>F7/D7</f>
+        <v>0.99996036360746876</v>
+      </c>
+      <c r="I7">
         <f t="shared" si="0"/>
-        <v>0.99996036360746876</v>
-      </c>
-      <c r="G7" s="4"/>
-      <c r="K7" s="10" t="e">
+        <v>1.7181641313147609E-4</v>
+      </c>
+      <c r="J7" s="4"/>
+      <c r="M7">
+        <v>1.38877619043423</v>
+      </c>
+      <c r="N7" s="10" t="e">
         <f t="shared" si="1"/>
         <v>#DIV/0!</v>
       </c>
-      <c r="L7" s="10"/>
-    </row>
-    <row r="8" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="O7" s="10"/>
+    </row>
+    <row r="8" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A8">
         <v>10</v>
       </c>
@@ -4888,234 +4953,389 @@
         <v>1.38607567014507</v>
       </c>
       <c r="E8">
+        <v>3.8958612319318502E-4</v>
+      </c>
+      <c r="F8">
         <v>1.3868055893142199</v>
       </c>
-      <c r="F8" s="10">
+      <c r="G8">
+        <v>4.0944327607914799E-4</v>
+      </c>
+      <c r="H8" s="10">
+        <f>F8/D8</f>
+        <v>1.0005266084564297</v>
+      </c>
+      <c r="I8">
         <f t="shared" si="0"/>
-        <v>1.0005266084564297</v>
-      </c>
-      <c r="G8" s="4"/>
-      <c r="K8" s="10" t="e">
+        <v>4.0785290749755253E-4</v>
+      </c>
+      <c r="J8" s="4"/>
+      <c r="M8">
+        <v>1.38594397488493</v>
+      </c>
+      <c r="N8" s="10" t="e">
         <f t="shared" si="1"/>
         <v>#DIV/0!</v>
       </c>
-      <c r="L8" s="10"/>
-    </row>
-    <row r="9" spans="1:12" s="4" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="O8" s="10"/>
+    </row>
+    <row r="9" spans="1:15" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A9">
         <v>25</v>
       </c>
       <c r="B9" s="5"/>
       <c r="C9"/>
-      <c r="D9"/>
+      <c r="D9">
+        <v>1.37947186689904</v>
+      </c>
       <c r="E9">
+        <v>8.86091661857925E-4</v>
+      </c>
+      <c r="F9">
         <v>1.3820193582140401</v>
       </c>
-      <c r="F9" s="10" t="e">
+      <c r="G9">
+        <v>1.17898543365087E-3</v>
+      </c>
+      <c r="H9" s="10">
+        <f>F9/D9</f>
+        <v>1.0018467149465879</v>
+      </c>
+      <c r="I9">
         <f t="shared" si="0"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="H9"/>
-      <c r="I9"/>
-      <c r="J9"/>
-      <c r="K9" s="10" t="e">
+        <v>1.0698498708561776E-3</v>
+      </c>
+      <c r="K9"/>
+      <c r="L9"/>
+      <c r="M9">
+        <v>1.3801396333334499</v>
+      </c>
+      <c r="N9" s="10" t="e">
         <f t="shared" si="1"/>
         <v>#DIV/0!</v>
       </c>
-      <c r="L9" s="11"/>
-    </row>
-    <row r="10" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="O9" s="11"/>
+    </row>
+    <row r="10" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A10">
         <v>50</v>
       </c>
       <c r="B10" s="5"/>
+      <c r="D10">
+        <v>1.37231900559378</v>
+      </c>
       <c r="E10">
+        <v>9.8135892237590492E-4</v>
+      </c>
+      <c r="F10">
         <v>1.3754575654543499</v>
       </c>
-      <c r="F10" s="10" t="e">
+      <c r="G10">
+        <v>7.1929329253824501E-4</v>
+      </c>
+      <c r="H10" s="10">
+        <f>F10/D10</f>
+        <v>1.002287048308576</v>
+      </c>
+      <c r="I10">
         <f t="shared" si="0"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="G10" s="4"/>
-      <c r="K10" s="10" t="e">
+        <v>8.8794780325578441E-4</v>
+      </c>
+      <c r="J10" s="4"/>
+      <c r="M10">
+        <v>1.3711659238629099</v>
+      </c>
+      <c r="N10" s="10" t="e">
         <f t="shared" si="1"/>
         <v>#DIV/0!</v>
       </c>
-      <c r="L10" s="10"/>
-    </row>
-    <row r="11" spans="1:12" s="4" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="O10" s="10"/>
+    </row>
+    <row r="11" spans="1:15" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A11">
         <v>75</v>
       </c>
       <c r="B11" s="5"/>
       <c r="C11"/>
-      <c r="D11"/>
+      <c r="D11">
+        <v>1.3652125452841399</v>
+      </c>
       <c r="E11">
+        <v>9.36891207849102E-4</v>
+      </c>
+      <c r="F11">
         <v>1.37040384545697</v>
       </c>
-      <c r="F11" s="10" t="e">
+      <c r="G11">
+        <v>1.1043763633645899E-3</v>
+      </c>
+      <c r="H11" s="10">
+        <f>F11/D11</f>
+        <v>1.0038025582102672</v>
+      </c>
+      <c r="I11">
         <f t="shared" si="0"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="H11"/>
-      <c r="I11"/>
-      <c r="J11"/>
-      <c r="K11" s="10" t="e">
+        <v>1.0625098571799413E-3</v>
+      </c>
+      <c r="K11"/>
+      <c r="L11"/>
+      <c r="M11">
+        <v>1.36351969550464</v>
+      </c>
+      <c r="N11" s="10" t="e">
         <f t="shared" si="1"/>
         <v>#DIV/0!</v>
       </c>
-      <c r="L11" s="11"/>
-    </row>
-    <row r="12" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="O11" s="11"/>
+    </row>
+    <row r="12" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A12">
         <v>100</v>
       </c>
       <c r="B12" s="5"/>
+      <c r="D12">
+        <v>1.35996558693921</v>
+      </c>
       <c r="E12">
+        <v>8.2269713778889005E-4</v>
+      </c>
+      <c r="F12">
         <v>1.3649754350071801</v>
       </c>
-      <c r="F12" s="10" t="e">
+      <c r="G12">
+        <v>1.0934621564654399E-3</v>
+      </c>
+      <c r="H12" s="10">
+        <f>F12/D12</f>
+        <v>1.0036838050286592</v>
+      </c>
+      <c r="I12">
         <f t="shared" si="0"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="G12" s="4"/>
-      <c r="K12" s="10" t="e">
+        <v>1.0075356465859516E-3</v>
+      </c>
+      <c r="J12" s="4"/>
+      <c r="M12">
+        <v>1.35608844560886</v>
+      </c>
+      <c r="N12" s="10" t="e">
         <f t="shared" si="1"/>
         <v>#DIV/0!</v>
       </c>
-      <c r="L12" s="10"/>
-    </row>
-    <row r="13" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="O12" s="10"/>
+    </row>
+    <row r="13" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A13">
         <v>150</v>
       </c>
       <c r="B13" s="5"/>
+      <c r="D13">
+        <v>1.3471169036955299</v>
+      </c>
       <c r="E13">
+        <v>3.4192473007070602E-3</v>
+      </c>
+      <c r="F13">
         <v>1.35044101904588</v>
       </c>
-      <c r="F13" s="10" t="e">
+      <c r="G13">
+        <v>3.6209913911154899E-3</v>
+      </c>
+      <c r="H13" s="10">
+        <f>F13/D13</f>
+        <v>1.002467577491776</v>
+      </c>
+      <c r="I13">
         <f t="shared" si="0"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="G13" s="4"/>
-      <c r="K13" s="10" t="e">
+        <v>3.7012678767904027E-3</v>
+      </c>
+      <c r="J13" s="4"/>
+      <c r="M13">
+        <v>1.3448593643039499</v>
+      </c>
+      <c r="N13" s="10" t="e">
         <f t="shared" si="1"/>
         <v>#DIV/0!</v>
       </c>
-      <c r="L13" s="10"/>
-    </row>
-    <row r="14" spans="1:12" s="4" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="O13" s="10"/>
+    </row>
+    <row r="14" spans="1:15" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A14">
         <v>250</v>
       </c>
       <c r="B14" s="5"/>
       <c r="C14"/>
-      <c r="D14"/>
+      <c r="D14">
+        <v>1.3301704109246899</v>
+      </c>
       <c r="E14">
+        <v>2.6701333301032298E-3</v>
+      </c>
+      <c r="F14">
         <v>1.3309639224463901</v>
       </c>
-      <c r="F14" s="10" t="e">
+      <c r="G14">
+        <v>2.6466416072152398E-3</v>
+      </c>
+      <c r="H14" s="10">
+        <f>F14/D14</f>
+        <v>1.000596548769378</v>
+      </c>
+      <c r="I14">
         <f t="shared" si="0"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="H14"/>
-      <c r="I14"/>
-      <c r="J14"/>
-      <c r="K14" s="10" t="e">
+        <v>2.8272285541985462E-3</v>
+      </c>
+      <c r="K14"/>
+      <c r="L14"/>
+      <c r="M14">
+        <v>1.3096995917960299</v>
+      </c>
+      <c r="N14" s="10" t="e">
         <f t="shared" si="1"/>
         <v>#DIV/0!</v>
       </c>
-      <c r="L14" s="11"/>
-    </row>
-    <row r="15" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="O14" s="11"/>
+    </row>
+    <row r="15" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A15">
         <v>500</v>
       </c>
       <c r="B15" s="5"/>
+      <c r="D15">
+        <v>1.2881810524951001</v>
+      </c>
       <c r="E15">
+        <v>2.82817615567389E-3</v>
+      </c>
+      <c r="F15">
         <v>1.2901507582212099</v>
       </c>
-      <c r="F15" s="10" t="e">
+      <c r="G15">
+        <v>3.6382982434454399E-3</v>
+      </c>
+      <c r="H15" s="10">
+        <f>F15/D15</f>
+        <v>1.0015290596941282</v>
+      </c>
+      <c r="I15">
         <f t="shared" si="0"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="G15" s="4"/>
-      <c r="K15" s="10" t="e">
+        <v>3.579377630249193E-3</v>
+      </c>
+      <c r="J15" s="4"/>
+      <c r="M15">
+        <v>1.2497624884637799</v>
+      </c>
+      <c r="N15" s="10" t="e">
         <f t="shared" si="1"/>
         <v>#DIV/0!</v>
       </c>
-      <c r="L15" s="10"/>
-    </row>
-    <row r="16" spans="1:12" s="4" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="O15" s="10"/>
+    </row>
+    <row r="16" spans="1:15" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A16">
         <v>750</v>
       </c>
       <c r="B16" s="5"/>
       <c r="C16"/>
-      <c r="D16"/>
+      <c r="D16">
+        <v>1.24999214529804</v>
+      </c>
       <c r="E16">
+        <v>2.36320017159778E-3</v>
+      </c>
+      <c r="F16">
         <v>1.2537253487050199</v>
       </c>
-      <c r="F16" s="10" t="e">
+      <c r="G16">
+        <v>3.5797440463882701E-3</v>
+      </c>
+      <c r="H16" s="10">
+        <f>F16/D16</f>
+        <v>1.0029865814925498</v>
+      </c>
+      <c r="I16">
         <f t="shared" si="0"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="H16"/>
-      <c r="I16"/>
-      <c r="J16"/>
-      <c r="K16" s="10" t="e">
+        <v>3.4346863492251559E-3</v>
+      </c>
+      <c r="K16"/>
+      <c r="L16"/>
+      <c r="M16">
+        <v>1.20221749175355</v>
+      </c>
+      <c r="N16" s="10" t="e">
         <f t="shared" si="1"/>
         <v>#DIV/0!</v>
       </c>
-      <c r="L16" s="11"/>
-    </row>
-    <row r="17" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="O16" s="11"/>
+    </row>
+    <row r="17" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A17">
         <v>999.99</v>
       </c>
       <c r="B17" s="5"/>
+      <c r="D17">
+        <v>1.2159170927577201</v>
+      </c>
       <c r="E17">
+        <v>3.1109769949112399E-3</v>
+      </c>
+      <c r="F17">
         <v>1.2163442531022399</v>
       </c>
-      <c r="F17" s="10" t="e">
-        <f t="shared" si="0"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="G17" s="4"/>
-      <c r="K17" s="10" t="e">
+      <c r="G17">
+        <v>3.18424238805618E-3</v>
+      </c>
+      <c r="H17" s="10">
+        <f>F17/D17</f>
+        <v>1.0003513071302839</v>
+      </c>
+      <c r="I17">
+        <f>H17*((E17/D17)^2 +(G17/F17)^2)^0.5</f>
+        <v>3.6618101886275135E-3</v>
+      </c>
+      <c r="J17" s="4"/>
+      <c r="M17">
+        <v>1.1524770375920901</v>
+      </c>
+      <c r="N17" s="10" t="e">
         <f t="shared" si="1"/>
         <v>#DIV/0!</v>
       </c>
-      <c r="L17" s="10"/>
-    </row>
-    <row r="21" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="O17" s="10"/>
+    </row>
+    <row r="21" spans="1:15" x14ac:dyDescent="0.3">
       <c r="C21" s="12" t="s">
         <v>5</v>
       </c>
       <c r="D21" s="12"/>
-      <c r="E21" s="13"/>
+      <c r="E21" s="12"/>
       <c r="F21" s="13"/>
-      <c r="H21" s="2"/>
-      <c r="I21" s="2"/>
-      <c r="J21" s="2"/>
+      <c r="G21" s="13"/>
+      <c r="H21" s="13"/>
+      <c r="I21" s="13"/>
       <c r="K21" s="2"/>
-    </row>
-    <row r="22" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="L21" s="2"/>
+      <c r="M21" s="2"/>
+      <c r="N21" s="2"/>
+    </row>
+    <row r="22" spans="1:15" x14ac:dyDescent="0.3">
       <c r="C22" s="3" t="s">
         <v>4</v>
       </c>
       <c r="D22" s="3"/>
-      <c r="E22" s="9"/>
-      <c r="F22" s="3"/>
-      <c r="H22" s="3" t="s">
+      <c r="E22" s="3"/>
+      <c r="F22" s="9"/>
+      <c r="G22" s="9"/>
+      <c r="H22" s="9"/>
+      <c r="I22" s="3"/>
+      <c r="K22" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="I22" s="3"/>
-      <c r="J22" s="9"/>
-      <c r="K22" s="9"/>
       <c r="L22" s="3"/>
-    </row>
-    <row r="23" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="M22" s="9"/>
+      <c r="N22" s="9"/>
+      <c r="O22" s="3"/>
+    </row>
+    <row r="23" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A23" s="6" t="s">
         <v>0</v>
       </c>
@@ -5127,27 +5347,36 @@
         <v>7</v>
       </c>
       <c r="E23" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="F23" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="F23" s="7" t="s">
+      <c r="G23" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="H23" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="G23" s="8"/>
-      <c r="H23" s="6" t="s">
+      <c r="I23" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="J23" s="8"/>
+      <c r="K23" s="6" t="s">
         <v>1</v>
       </c>
-      <c r="I23" s="6" t="s">
+      <c r="L23" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="J23" s="6" t="s">
+      <c r="M23" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="K23" s="7" t="s">
+      <c r="N23" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="L23" s="7"/>
-    </row>
-    <row r="24" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="O23" s="7"/>
+    </row>
+    <row r="24" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A24">
         <v>0.1</v>
       </c>
@@ -5156,24 +5385,36 @@
       <c r="D24" s="2">
         <v>3.4601339198647797E-5</v>
       </c>
-      <c r="E24" s="2">
+      <c r="E24" s="16">
+        <v>1.22883732368375E-8</v>
+      </c>
+      <c r="F24" s="16">
         <v>2.3188386654289999E-5</v>
       </c>
-      <c r="F24" s="10">
-        <f>E24/D24</f>
+      <c r="G24" s="16">
+        <v>2.5713213345718999E-7</v>
+      </c>
+      <c r="H24" s="10">
+        <f>F24/D24</f>
         <v>0.67015864678428949</v>
       </c>
-      <c r="G24" s="4"/>
-      <c r="H24" s="2"/>
-      <c r="I24" s="2"/>
-      <c r="J24" s="2"/>
-      <c r="K24" s="10" t="e">
-        <f>J24/I24</f>
+      <c r="I24">
+        <f>H24*((E24/D24)^2 +(G24/F24)^2)^0.5</f>
+        <v>7.4350871718769813E-3</v>
+      </c>
+      <c r="J24" s="4"/>
+      <c r="K24" s="2"/>
+      <c r="L24" s="2"/>
+      <c r="M24" s="2">
+        <v>2.5899175434190999E-5</v>
+      </c>
+      <c r="N24" s="10" t="e">
+        <f>M24/L24</f>
         <v>#DIV/0!</v>
       </c>
-      <c r="L24" s="10"/>
-    </row>
-    <row r="25" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="O24" s="10"/>
+    </row>
+    <row r="25" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A25">
         <v>0.5</v>
       </c>
@@ -5181,21 +5422,34 @@
       <c r="D25">
         <v>1.7267075850167999E-4</v>
       </c>
-      <c r="E25">
+      <c r="E25" s="16">
+        <v>7.3730405114227898E-8</v>
+      </c>
+      <c r="F25" s="16">
         <v>1.16379113471186E-4</v>
       </c>
-      <c r="F25" s="10">
-        <f t="shared" ref="F25:F36" si="2">E25/D25</f>
+      <c r="G25" s="16">
+        <v>4.9685826902563597E-7</v>
+      </c>
+      <c r="H25" s="10">
+        <f>F25/D25</f>
         <v>0.67399433743759052</v>
       </c>
-      <c r="G25" s="4"/>
-      <c r="K25" s="10" t="e">
-        <f t="shared" ref="K25:K36" si="3">J25/I25</f>
+      <c r="I25">
+        <f t="shared" ref="I25:I35" si="2">H25*((E25/D25)^2 +(G25/F25)^2)^0.5</f>
+        <v>2.8918456475792078E-3</v>
+      </c>
+      <c r="J25" s="4"/>
+      <c r="M25">
+        <v>1.3026224043386099E-4</v>
+      </c>
+      <c r="N25" s="10" t="e">
+        <f t="shared" ref="N25:N36" si="3">M25/L25</f>
         <v>#DIV/0!</v>
       </c>
-      <c r="L25" s="10"/>
-    </row>
-    <row r="26" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="O25" s="10"/>
+    </row>
+    <row r="26" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A26">
         <v>1</v>
       </c>
@@ -5203,21 +5457,34 @@
       <c r="D26">
         <v>3.4444202449192702E-4</v>
       </c>
-      <c r="E26">
+      <c r="E26" s="16">
+        <v>1.02701859340892E-7</v>
+      </c>
+      <c r="F26" s="16">
         <v>2.31665379952172E-4</v>
       </c>
-      <c r="F26" s="10">
+      <c r="G26" s="16">
+        <v>6.9232886194979901E-7</v>
+      </c>
+      <c r="H26" s="10">
+        <f>F26/D26</f>
+        <v>0.67258163487423628</v>
+      </c>
+      <c r="I26">
         <f t="shared" si="2"/>
-        <v>0.67258163487423628</v>
-      </c>
-      <c r="G26" s="4"/>
-      <c r="K26" s="10" t="e">
+        <v>2.0199806972425911E-3</v>
+      </c>
+      <c r="J26" s="4"/>
+      <c r="M26">
+        <v>2.6089565621297098E-4</v>
+      </c>
+      <c r="N26" s="10" t="e">
         <f t="shared" si="3"/>
         <v>#DIV/0!</v>
       </c>
-      <c r="L26" s="10"/>
-    </row>
-    <row r="27" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="O26" s="10"/>
+    </row>
+    <row r="27" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A27">
         <v>10</v>
       </c>
@@ -5225,222 +5492,385 @@
       <c r="D27">
         <v>3.33054467027722E-3</v>
       </c>
-      <c r="E27">
+      <c r="E27" s="16">
+        <v>3.1023196230951202E-6</v>
+      </c>
+      <c r="F27" s="16">
         <v>2.3274949085023899E-3</v>
       </c>
-      <c r="F27" s="10">
+      <c r="G27" s="16">
+        <v>7.3576810457546899E-6</v>
+      </c>
+      <c r="H27" s="10">
+        <f>F27/D27</f>
+        <v>0.69883311557825745</v>
+      </c>
+      <c r="I27">
         <f t="shared" si="2"/>
-        <v>0.69883311557825745</v>
-      </c>
-      <c r="G27" s="4"/>
-      <c r="K27" s="10" t="e">
+        <v>2.3030599218682355E-3</v>
+      </c>
+      <c r="J27" s="4"/>
+      <c r="M27">
+        <v>2.5949076799098498E-3</v>
+      </c>
+      <c r="N27" s="10" t="e">
         <f t="shared" si="3"/>
         <v>#DIV/0!</v>
       </c>
-      <c r="L27" s="10"/>
-    </row>
-    <row r="28" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="O27" s="10"/>
+    </row>
+    <row r="28" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A28">
         <v>25</v>
       </c>
       <c r="B28" s="5"/>
-      <c r="E28">
+      <c r="D28">
+        <v>7.9007108136224906E-3</v>
+      </c>
+      <c r="E28" s="16">
+        <v>2.1579374269995798E-5</v>
+      </c>
+      <c r="F28" s="16">
         <v>5.7868683352336496E-3</v>
       </c>
-      <c r="F28" s="10" t="e">
+      <c r="G28" s="16">
+        <v>2.2153397083295701E-5</v>
+      </c>
+      <c r="H28" s="10">
+        <f>F28/D28</f>
+        <v>0.73244907600666376</v>
+      </c>
+      <c r="I28">
         <f t="shared" si="2"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="G28" s="4"/>
-      <c r="K28" s="10" t="e">
+        <v>3.444486925796071E-3</v>
+      </c>
+      <c r="J28" s="4"/>
+      <c r="M28">
+        <v>6.4419405380797103E-3</v>
+      </c>
+      <c r="N28" s="10" t="e">
         <f t="shared" si="3"/>
         <v>#DIV/0!</v>
       </c>
-      <c r="L28" s="11"/>
-    </row>
-    <row r="29" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="O28" s="11"/>
+    </row>
+    <row r="29" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A29">
         <v>50</v>
       </c>
       <c r="B29" s="5"/>
-      <c r="E29">
+      <c r="D29">
+        <v>1.48099690035684E-2</v>
+      </c>
+      <c r="E29" s="16">
+        <v>3.5619384608241799E-5</v>
+      </c>
+      <c r="F29" s="16">
         <v>1.1357972286110201E-2</v>
       </c>
-      <c r="F29" s="10" t="e">
+      <c r="G29" s="16">
+        <v>3.9960656049596501E-5</v>
+      </c>
+      <c r="H29" s="10">
+        <f>F29/D29</f>
+        <v>0.76691398093902452</v>
+      </c>
+      <c r="I29">
         <f t="shared" si="2"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="G29" s="4"/>
-      <c r="K29" s="10" t="e">
+        <v>3.2684265997479276E-3</v>
+      </c>
+      <c r="J29" s="4"/>
+      <c r="M29">
+        <v>1.26690225425122E-2</v>
+      </c>
+      <c r="N29" s="10" t="e">
         <f t="shared" si="3"/>
         <v>#DIV/0!</v>
       </c>
-      <c r="L29" s="10"/>
-    </row>
-    <row r="30" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="O29" s="10"/>
+    </row>
+    <row r="30" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A30">
         <v>75</v>
       </c>
       <c r="B30" s="5"/>
-      <c r="E30">
+      <c r="D30">
+        <v>2.1060130702738999E-2</v>
+      </c>
+      <c r="E30" s="16">
+        <v>3.0830038687911403E-5</v>
+      </c>
+      <c r="F30" s="16">
         <v>1.6724313084056999E-2</v>
       </c>
-      <c r="F30" s="10" t="e">
+      <c r="G30" s="16">
+        <v>4.6773312275541899E-5</v>
+      </c>
+      <c r="H30" s="10">
+        <f>F30/D30</f>
+        <v>0.79412199858198884</v>
+      </c>
+      <c r="I30">
         <f t="shared" si="2"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="G30" s="4"/>
-      <c r="K30" s="10" t="e">
+        <v>2.506797039006772E-3</v>
+      </c>
+      <c r="J30" s="4"/>
+      <c r="M30">
+        <v>1.8873120984925901E-2</v>
+      </c>
+      <c r="N30" s="10" t="e">
         <f t="shared" si="3"/>
         <v>#DIV/0!</v>
       </c>
-      <c r="L30" s="11"/>
-    </row>
-    <row r="31" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="O30" s="11"/>
+    </row>
+    <row r="31" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A31">
         <v>100</v>
       </c>
       <c r="B31" s="5"/>
-      <c r="E31">
+      <c r="D31">
+        <v>2.67600755292417E-2</v>
+      </c>
+      <c r="E31" s="16">
+        <v>6.1301138330409899E-5</v>
+      </c>
+      <c r="F31" s="16">
         <v>2.2149757308928399E-2</v>
       </c>
-      <c r="F31" s="10" t="e">
+      <c r="G31" s="16">
+        <v>5.1020148947823797E-5</v>
+      </c>
+      <c r="H31" s="10">
+        <f>F31/D31</f>
+        <v>0.82771654679092965</v>
+      </c>
+      <c r="I31">
         <f t="shared" si="2"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="G31" s="4"/>
-      <c r="K31" s="10" t="e">
+        <v>2.6889139523652702E-3</v>
+      </c>
+      <c r="J31" s="4"/>
+      <c r="M31">
+        <v>2.4681477633588599E-2</v>
+      </c>
+      <c r="N31" s="10" t="e">
         <f t="shared" si="3"/>
         <v>#DIV/0!</v>
       </c>
-      <c r="L31" s="10"/>
-    </row>
-    <row r="32" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="O31" s="10"/>
+    </row>
+    <row r="32" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A32">
         <v>150</v>
       </c>
       <c r="B32" s="5"/>
-      <c r="E32">
+      <c r="D32">
+        <v>3.6782709718709998E-2</v>
+      </c>
+      <c r="E32" s="16">
+        <v>1.97489580151579E-4</v>
+      </c>
+      <c r="F32" s="16">
         <v>3.2103137598192298E-2</v>
       </c>
-      <c r="F32" s="10" t="e">
+      <c r="G32" s="16">
+        <v>2.08831333646651E-4</v>
+      </c>
+      <c r="H32" s="10">
+        <f>F32/D32</f>
+        <v>0.87277793951821403</v>
+      </c>
+      <c r="I32">
         <f t="shared" si="2"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="G32" s="4"/>
-      <c r="K32" s="10" t="e">
+        <v>7.3615233968889766E-3</v>
+      </c>
+      <c r="J32" s="4"/>
+      <c r="M32">
+        <v>3.6134840661020101E-2</v>
+      </c>
+      <c r="N32" s="10" t="e">
         <f t="shared" si="3"/>
         <v>#DIV/0!</v>
       </c>
-      <c r="L32" s="10"/>
-    </row>
-    <row r="33" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="O32" s="10"/>
+    </row>
+    <row r="33" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A33">
         <v>250</v>
       </c>
       <c r="B33" s="5"/>
-      <c r="E33">
+      <c r="D33">
+        <v>5.6309750104400702E-2</v>
+      </c>
+      <c r="E33" s="16">
+        <v>2.51687827781958E-4</v>
+      </c>
+      <c r="F33" s="16">
         <v>5.1114734736025402E-2</v>
       </c>
-      <c r="F33" s="10" t="e">
+      <c r="G33" s="16">
+        <v>2.8833834514146198E-4</v>
+      </c>
+      <c r="H33" s="10">
+        <f>F33/D33</f>
+        <v>0.90774216971761523</v>
+      </c>
+      <c r="I33">
         <f t="shared" si="2"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="G33" s="4"/>
-      <c r="K33" s="10" t="e">
+        <v>6.5331679556135417E-3</v>
+      </c>
+      <c r="J33" s="4"/>
+      <c r="M33">
+        <v>5.7361502212218099E-2</v>
+      </c>
+      <c r="N33" s="10" t="e">
         <f t="shared" si="3"/>
         <v>#DIV/0!</v>
       </c>
-      <c r="L33" s="11"/>
-    </row>
-    <row r="34" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="O33" s="11"/>
+    </row>
+    <row r="34" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A34">
         <v>500</v>
       </c>
       <c r="B34" s="5"/>
-      <c r="E34">
+      <c r="D34">
+        <v>9.4384365104793602E-2</v>
+      </c>
+      <c r="E34" s="16">
+        <v>3.7802904257795602E-4</v>
+      </c>
+      <c r="F34" s="16">
         <v>9.1445222619505398E-2</v>
       </c>
-      <c r="F34" s="10" t="e">
+      <c r="G34" s="16">
+        <v>4.4906828447954003E-4</v>
+      </c>
+      <c r="H34" s="10">
+        <f>F34/D34</f>
+        <v>0.96885985849430767</v>
+      </c>
+      <c r="I34">
         <f t="shared" si="2"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="G34" s="4"/>
-      <c r="K34" s="10" t="e">
+        <v>6.1396636178584303E-3</v>
+      </c>
+      <c r="J34" s="4"/>
+      <c r="M34">
+        <v>0.102092586065974</v>
+      </c>
+      <c r="N34" s="10" t="e">
         <f t="shared" si="3"/>
         <v>#DIV/0!</v>
       </c>
-      <c r="L34" s="10"/>
-    </row>
-    <row r="35" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="O34" s="10"/>
+    </row>
+    <row r="35" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A35">
         <v>750</v>
       </c>
       <c r="B35" s="5"/>
-      <c r="E35">
+      <c r="D35">
+        <v>0.12681392305883499</v>
+      </c>
+      <c r="E35" s="16">
+        <v>3.7117560576619898E-4</v>
+      </c>
+      <c r="F35" s="16">
         <v>0.12725844081883</v>
       </c>
-      <c r="F35" s="10" t="e">
+      <c r="G35" s="16">
+        <v>3.9277512684765298E-4</v>
+      </c>
+      <c r="H35" s="10">
+        <f>F35/D35</f>
+        <v>1.0035052756769365</v>
+      </c>
+      <c r="I35">
         <f t="shared" si="2"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="G35" s="4"/>
-      <c r="K35" s="10" t="e">
+        <v>4.2684987159538603E-3</v>
+      </c>
+      <c r="J35" s="4"/>
+      <c r="M35">
+        <v>0.14105605143254499</v>
+      </c>
+      <c r="N35" s="10" t="e">
         <f t="shared" si="3"/>
         <v>#DIV/0!</v>
       </c>
-      <c r="L35" s="11"/>
-    </row>
-    <row r="36" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="O35" s="11"/>
+    </row>
+    <row r="36" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A36">
         <v>999.99</v>
       </c>
       <c r="B36" s="5"/>
-      <c r="E36">
+      <c r="D36">
+        <v>0.15510900896549801</v>
+      </c>
+      <c r="E36" s="16">
+        <v>5.7851797067085496E-4</v>
+      </c>
+      <c r="F36" s="16">
         <v>0.157583868759714</v>
       </c>
-      <c r="F36" s="10" t="e">
-        <f t="shared" si="2"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="G36" s="4"/>
-      <c r="K36" s="10" t="e">
+      <c r="G36" s="16">
+        <v>5.8700051779191705E-4</v>
+      </c>
+      <c r="H36" s="10">
+        <f>F36/D36</f>
+        <v>1.0159556160581653</v>
+      </c>
+      <c r="I36">
+        <f>H36*((E36/D36)^2 +(G36/F36)^2)^0.5</f>
+        <v>5.3554157048239367E-3</v>
+      </c>
+      <c r="J36" s="4"/>
+      <c r="M36">
+        <v>0.17395996323018501</v>
+      </c>
+      <c r="N36" s="10" t="e">
         <f t="shared" si="3"/>
         <v>#DIV/0!</v>
       </c>
-      <c r="L36" s="10"/>
-    </row>
-    <row r="40" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="O36" s="10"/>
+    </row>
+    <row r="40" spans="1:15" x14ac:dyDescent="0.3">
       <c r="C40" s="1" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="41" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:15" x14ac:dyDescent="0.3">
       <c r="C41" s="14" t="s">
         <v>2</v>
       </c>
       <c r="D41" s="14"/>
-      <c r="E41" s="15"/>
-      <c r="H41" s="2"/>
-      <c r="I41" s="2"/>
-      <c r="J41" s="2"/>
+      <c r="E41" s="14"/>
+      <c r="F41" s="15"/>
+      <c r="G41" s="15"/>
+      <c r="H41" s="15"/>
       <c r="K41" s="2"/>
-    </row>
-    <row r="42" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="L41" s="2"/>
+      <c r="M41" s="2"/>
+      <c r="N41" s="2"/>
+    </row>
+    <row r="42" spans="1:15" x14ac:dyDescent="0.3">
       <c r="C42" s="3" t="s">
         <v>4</v>
       </c>
       <c r="D42" s="3"/>
-      <c r="E42" s="9"/>
-      <c r="F42" s="3"/>
-      <c r="H42" s="3" t="s">
+      <c r="E42" s="3"/>
+      <c r="F42" s="9"/>
+      <c r="G42" s="9"/>
+      <c r="H42" s="9"/>
+      <c r="I42" s="3"/>
+      <c r="K42" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="I42" s="3"/>
-      <c r="J42" s="9"/>
-      <c r="K42" s="9"/>
-    </row>
-    <row r="43" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="L42" s="3"/>
+      <c r="M42" s="9"/>
+      <c r="N42" s="9"/>
+    </row>
+    <row r="43" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A43" s="6" t="s">
         <v>0</v>
       </c>
@@ -5451,27 +5881,30 @@
       <c r="D43" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="E43" s="6" t="s">
+      <c r="E43" s="6"/>
+      <c r="F43" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="F43" s="7" t="s">
+      <c r="G43" s="6"/>
+      <c r="H43" s="6"/>
+      <c r="I43" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="G43" s="8"/>
-      <c r="H43" s="6" t="s">
+      <c r="J43" s="8"/>
+      <c r="K43" s="6" t="s">
         <v>1</v>
       </c>
-      <c r="I43" s="6" t="s">
+      <c r="L43" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="J43" s="6" t="s">
+      <c r="M43" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="K43" s="7" t="s">
+      <c r="N43" s="7" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="44" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A44">
         <v>0.1</v>
       </c>
@@ -5479,26 +5912,26 @@
       <c r="D44">
         <v>1.33146077610654</v>
       </c>
-      <c r="E44">
+      <c r="F44">
         <v>1.3294682945082299</v>
       </c>
-      <c r="F44" s="10">
-        <f>E44/D44</f>
+      <c r="I44" s="10">
+        <f>F44/D44</f>
         <v>0.9985035371420129</v>
       </c>
-      <c r="G44" s="4"/>
-      <c r="I44">
+      <c r="J44" s="4"/>
+      <c r="L44">
         <v>1.33422182541257</v>
       </c>
-      <c r="J44">
+      <c r="M44">
         <v>1.3288821396550801</v>
       </c>
-      <c r="K44" s="10">
-        <f>J44/I44</f>
+      <c r="N44" s="10">
+        <f>M44/L44</f>
         <v>0.99599790255579224</v>
       </c>
     </row>
-    <row r="45" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A45">
         <v>0.5</v>
       </c>
@@ -5506,27 +5939,27 @@
       <c r="D45">
         <v>1.35765661048369</v>
       </c>
-      <c r="E45">
+      <c r="F45">
         <v>1.3402135659025001</v>
       </c>
-      <c r="F45" s="10">
-        <f t="shared" ref="F45:F56" si="4">E45/D45</f>
+      <c r="I45" s="10">
+        <f t="shared" ref="I45:I56" si="4">F45/D45</f>
         <v>0.98715209394887005</v>
       </c>
-      <c r="G45" s="4"/>
-      <c r="H45" s="4"/>
-      <c r="I45">
+      <c r="J45" s="4"/>
+      <c r="K45" s="4"/>
+      <c r="L45">
         <v>1.3552315082948401</v>
       </c>
-      <c r="J45">
+      <c r="M45">
         <v>1.34024384554322</v>
       </c>
-      <c r="K45" s="11">
-        <f t="shared" ref="K45:K54" si="5">J45/I45</f>
+      <c r="N45" s="11">
+        <f t="shared" ref="N45:N56" si="5">M45/L45</f>
         <v>0.98894088378266998</v>
       </c>
     </row>
-    <row r="46" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A46">
         <v>1</v>
       </c>
@@ -5534,26 +5967,26 @@
       <c r="D46">
         <v>1.33903476392587</v>
       </c>
-      <c r="E46">
+      <c r="F46">
         <v>1.3294539841566</v>
       </c>
-      <c r="F46" s="10">
+      <c r="I46" s="10">
         <f t="shared" si="4"/>
         <v>0.99284501043036377</v>
       </c>
-      <c r="G46" s="4"/>
-      <c r="I46">
+      <c r="J46" s="4"/>
+      <c r="L46">
         <v>1.3461367977004299</v>
       </c>
-      <c r="J46">
+      <c r="M46">
         <v>1.32904261090945</v>
       </c>
-      <c r="K46" s="10">
+      <c r="N46" s="10">
         <f t="shared" si="5"/>
         <v>0.98730130041747499</v>
       </c>
     </row>
-    <row r="47" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A47">
         <v>10</v>
       </c>
@@ -5561,27 +5994,27 @@
       <c r="D47">
         <v>1.31789010731641</v>
       </c>
-      <c r="E47">
+      <c r="F47">
         <v>1.3448930260504799</v>
       </c>
-      <c r="F47" s="10">
+      <c r="I47" s="10">
         <f t="shared" si="4"/>
         <v>1.0204895071175968</v>
       </c>
-      <c r="G47" s="4"/>
-      <c r="H47" s="4"/>
-      <c r="I47">
+      <c r="J47" s="4"/>
+      <c r="K47" s="4"/>
+      <c r="L47">
         <v>1.31846450590491</v>
       </c>
-      <c r="J47">
+      <c r="M47">
         <v>1.3511493506913199</v>
       </c>
-      <c r="K47" s="11">
+      <c r="N47" s="11">
         <f t="shared" si="5"/>
         <v>1.0247900831914902</v>
       </c>
     </row>
-    <row r="48" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A48">
         <v>25</v>
       </c>
@@ -5589,26 +6022,26 @@
       <c r="D48">
         <v>1.32036564820574</v>
       </c>
-      <c r="E48">
+      <c r="F48">
         <v>1.3268512139816999</v>
       </c>
-      <c r="F48" s="10">
+      <c r="I48" s="10">
         <f t="shared" si="4"/>
         <v>1.0049119467662411</v>
       </c>
-      <c r="G48" s="4"/>
-      <c r="I48">
+      <c r="J48" s="4"/>
+      <c r="L48">
         <v>1.33152629750905</v>
       </c>
-      <c r="J48">
+      <c r="M48">
         <v>1.33015612015508</v>
       </c>
-      <c r="K48" s="10">
+      <c r="N48" s="10">
         <f t="shared" si="5"/>
         <v>0.99897097236717491</v>
       </c>
     </row>
-    <row r="49" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A49">
         <v>50</v>
       </c>
@@ -5616,27 +6049,27 @@
       <c r="D49">
         <v>1.3197738196808499</v>
       </c>
-      <c r="E49">
+      <c r="F49">
         <v>1.3126564921716899</v>
       </c>
-      <c r="F49" s="10">
+      <c r="I49" s="10">
         <f t="shared" si="4"/>
         <v>0.99460716116426584</v>
       </c>
-      <c r="G49" s="4"/>
-      <c r="H49" s="4"/>
-      <c r="I49">
+      <c r="J49" s="4"/>
+      <c r="K49" s="4"/>
+      <c r="L49">
         <v>1.32005527665466</v>
       </c>
-      <c r="J49">
+      <c r="M49">
         <v>1.30244954906179</v>
       </c>
-      <c r="K49" s="11">
+      <c r="N49" s="11">
         <f t="shared" si="5"/>
         <v>0.98666288608952257</v>
       </c>
     </row>
-    <row r="50" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A50">
         <v>75</v>
       </c>
@@ -5644,26 +6077,26 @@
       <c r="D50">
         <v>1.29935652652886</v>
       </c>
-      <c r="E50">
+      <c r="F50">
         <v>1.32473430230751</v>
       </c>
-      <c r="F50" s="10">
+      <c r="I50" s="10">
         <f t="shared" si="4"/>
         <v>1.0195310334465668</v>
       </c>
-      <c r="G50" s="4"/>
-      <c r="I50">
+      <c r="J50" s="4"/>
+      <c r="L50">
         <v>1.30908256842566</v>
       </c>
-      <c r="J50">
+      <c r="M50">
         <v>1.30672475018709</v>
       </c>
-      <c r="K50" s="10">
+      <c r="N50" s="10">
         <f t="shared" si="5"/>
         <v>0.99819887736996948</v>
       </c>
     </row>
-    <row r="51" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A51">
         <v>100</v>
       </c>
@@ -5671,27 +6104,27 @@
       <c r="D51">
         <v>1.33910590256307</v>
       </c>
-      <c r="E51">
+      <c r="F51">
         <v>1.3167897334910501</v>
       </c>
-      <c r="F51" s="10">
+      <c r="I51" s="10">
         <f t="shared" si="4"/>
         <v>0.98333502299608533</v>
       </c>
-      <c r="G51" s="4"/>
-      <c r="H51" s="4"/>
-      <c r="I51">
+      <c r="J51" s="4"/>
+      <c r="K51" s="4"/>
+      <c r="L51">
         <v>1.3171859836539099</v>
       </c>
-      <c r="J51">
+      <c r="M51">
         <v>1.31060168409573</v>
       </c>
-      <c r="K51" s="11">
+      <c r="N51" s="11">
         <f t="shared" si="5"/>
         <v>0.99500123775997451</v>
       </c>
     </row>
-    <row r="52" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A52">
         <v>150</v>
       </c>
@@ -5699,26 +6132,26 @@
       <c r="D52">
         <v>1.3346899335651701</v>
       </c>
-      <c r="E52">
+      <c r="F52">
         <v>1.3164282135057199</v>
       </c>
-      <c r="F52" s="10">
+      <c r="I52" s="10">
         <f t="shared" si="4"/>
         <v>0.98631763108404502</v>
       </c>
-      <c r="G52" s="4"/>
-      <c r="I52">
+      <c r="J52" s="4"/>
+      <c r="L52">
         <v>1.28924587434467</v>
       </c>
-      <c r="J52">
+      <c r="M52">
         <v>1.3011790803332</v>
       </c>
-      <c r="K52" s="10">
+      <c r="N52" s="10">
         <f t="shared" si="5"/>
         <v>1.0092559582512495</v>
       </c>
     </row>
-    <row r="53" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A53">
         <v>250</v>
       </c>
@@ -5726,27 +6159,27 @@
       <c r="D53">
         <v>1.29678717701069</v>
       </c>
-      <c r="E53">
+      <c r="F53">
         <v>1.33451901185347</v>
       </c>
-      <c r="F53" s="10">
+      <c r="I53" s="10">
         <f t="shared" si="4"/>
         <v>1.0290963972436542</v>
       </c>
-      <c r="G53" s="4"/>
-      <c r="H53" s="4"/>
-      <c r="I53">
+      <c r="J53" s="4"/>
+      <c r="K53" s="4"/>
+      <c r="L53">
         <v>1.2845821783281699</v>
       </c>
-      <c r="J53">
+      <c r="M53">
         <v>1.27732476166037</v>
       </c>
-      <c r="K53" s="11">
+      <c r="N53" s="11">
         <f t="shared" si="5"/>
         <v>0.99435036793267273</v>
       </c>
     </row>
-    <row r="54" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A54">
         <v>500</v>
       </c>
@@ -5754,26 +6187,26 @@
       <c r="D54">
         <v>1.2662694099393199</v>
       </c>
-      <c r="E54">
+      <c r="F54">
         <v>1.2620512370753201</v>
       </c>
-      <c r="F54" s="10">
+      <c r="I54" s="10">
         <f t="shared" si="4"/>
         <v>0.99666881879093805</v>
       </c>
-      <c r="G54" s="4"/>
-      <c r="I54">
+      <c r="J54" s="4"/>
+      <c r="L54">
         <v>1.2051198250164299</v>
       </c>
-      <c r="J54">
+      <c r="M54">
         <v>1.19710463230099</v>
       </c>
-      <c r="K54" s="10">
+      <c r="N54" s="10">
         <f t="shared" si="5"/>
         <v>0.99334904915755518</v>
       </c>
     </row>
-    <row r="55" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A55">
         <v>750</v>
       </c>
@@ -5781,22 +6214,26 @@
       <c r="D55">
         <v>1.23279071771682</v>
       </c>
-      <c r="E55">
+      <c r="F55">
         <v>1.23649350366719</v>
       </c>
-      <c r="F55" s="10">
+      <c r="I55" s="10">
         <f t="shared" si="4"/>
         <v>1.0030035803296993</v>
       </c>
-      <c r="G55" s="5"/>
-      <c r="I55">
+      <c r="J55" s="5"/>
+      <c r="L55">
         <v>1.1807532343395699</v>
       </c>
-      <c r="J55">
+      <c r="M55">
         <v>1.1563239206929501</v>
       </c>
-    </row>
-    <row r="56" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="N55" s="10">
+        <f t="shared" si="5"/>
+        <v>0.97931039870470149</v>
+      </c>
+    </row>
+    <row r="56" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A56">
         <v>999.99</v>
       </c>
@@ -5804,48 +6241,58 @@
       <c r="D56">
         <v>1.1928852496040101</v>
       </c>
-      <c r="E56">
+      <c r="F56">
         <v>1.2106403902979499</v>
       </c>
-      <c r="F56" s="10">
+      <c r="I56" s="10">
         <f t="shared" si="4"/>
         <v>1.0148841983751864</v>
       </c>
-      <c r="G56" s="5"/>
-      <c r="I56">
+      <c r="J56" s="5"/>
+      <c r="L56">
         <v>1.13357719050286</v>
       </c>
-      <c r="J56">
+      <c r="M56">
         <v>1.1342010761596699</v>
       </c>
-    </row>
-    <row r="59" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="N56" s="11">
+        <f t="shared" si="5"/>
+        <v>1.0005503689224138</v>
+      </c>
+    </row>
+    <row r="59" spans="1:14" x14ac:dyDescent="0.3">
       <c r="C59" s="12" t="s">
         <v>5</v>
       </c>
       <c r="D59" s="12"/>
-      <c r="E59" s="13"/>
+      <c r="E59" s="12"/>
       <c r="F59" s="13"/>
-      <c r="H59" s="2"/>
-      <c r="I59" s="2"/>
-      <c r="J59" s="2"/>
+      <c r="G59" s="13"/>
+      <c r="H59" s="13"/>
+      <c r="I59" s="13"/>
       <c r="K59" s="2"/>
-    </row>
-    <row r="60" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L59" s="2"/>
+      <c r="M59" s="2"/>
+      <c r="N59" s="2"/>
+    </row>
+    <row r="60" spans="1:14" x14ac:dyDescent="0.3">
       <c r="C60" s="3" t="s">
         <v>4</v>
       </c>
       <c r="D60" s="3"/>
-      <c r="E60" s="9"/>
-      <c r="F60" s="3"/>
-      <c r="H60" s="3" t="s">
+      <c r="E60" s="3"/>
+      <c r="F60" s="9"/>
+      <c r="G60" s="9"/>
+      <c r="H60" s="9"/>
+      <c r="I60" s="3"/>
+      <c r="K60" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="I60" s="3"/>
-      <c r="J60" s="9"/>
-      <c r="K60" s="9"/>
-    </row>
-    <row r="61" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L60" s="3"/>
+      <c r="M60" s="9"/>
+      <c r="N60" s="9"/>
+    </row>
+    <row r="61" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A61" s="6" t="s">
         <v>0</v>
       </c>
@@ -5856,27 +6303,30 @@
       <c r="D61" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="E61" s="6" t="s">
+      <c r="E61" s="6"/>
+      <c r="F61" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="F61" s="7" t="s">
+      <c r="G61" s="6"/>
+      <c r="H61" s="6"/>
+      <c r="I61" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="G61" s="8"/>
-      <c r="H61" s="6" t="s">
+      <c r="J61" s="8"/>
+      <c r="K61" s="6" t="s">
         <v>1</v>
       </c>
-      <c r="I61" s="6" t="s">
+      <c r="L61" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="J61" s="6" t="s">
+      <c r="M61" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="K61" s="7" t="s">
+      <c r="N61" s="7" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="62" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="62" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A62">
         <v>0.1</v>
       </c>
@@ -5887,27 +6337,30 @@
       <c r="D62" s="2">
         <v>1.9785240862768899E-5</v>
       </c>
-      <c r="E62" s="2">
+      <c r="E62" s="2"/>
+      <c r="F62" s="2">
         <v>1.9417624590728801E-5</v>
       </c>
-      <c r="F62" s="10">
-        <f>E62/D62</f>
+      <c r="G62" s="2"/>
+      <c r="H62" s="2"/>
+      <c r="I62" s="10">
+        <f>F62/D62</f>
         <v>0.98141967163352228</v>
       </c>
-      <c r="G62" s="4"/>
-      <c r="H62" s="2"/>
-      <c r="I62" s="2">
+      <c r="J62" s="4"/>
+      <c r="K62" s="2"/>
+      <c r="L62" s="2">
         <v>2.44555572729164E-5</v>
       </c>
-      <c r="J62" s="2">
+      <c r="M62" s="2">
         <v>2.3173152783100001E-5</v>
       </c>
-      <c r="K62" s="10">
-        <f>J62/I62</f>
+      <c r="N62" s="10">
+        <f>M62/L62</f>
         <v>0.94756183735642718</v>
       </c>
     </row>
-    <row r="63" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A63">
         <v>0.5</v>
       </c>
@@ -5918,26 +6371,28 @@
       <c r="D63">
         <v>1.02051178015395E-4</v>
       </c>
-      <c r="E63" s="2">
+      <c r="F63" s="2">
         <v>9.4705678455829002E-5</v>
       </c>
-      <c r="F63" s="10">
-        <f t="shared" ref="F63:F74" si="6">E63/D63</f>
+      <c r="G63" s="2"/>
+      <c r="H63" s="2"/>
+      <c r="I63" s="10">
+        <f t="shared" ref="I63:I74" si="6">F63/D63</f>
         <v>0.92802141334950694</v>
       </c>
-      <c r="G63" s="4"/>
-      <c r="I63">
+      <c r="J63" s="4"/>
+      <c r="L63">
         <v>1.237590596311E-4</v>
       </c>
-      <c r="J63">
+      <c r="M63">
         <v>1.2781285534871299E-4</v>
       </c>
-      <c r="K63" s="11">
-        <f t="shared" ref="K63:K74" si="7">J63/I63</f>
+      <c r="N63" s="11">
+        <f t="shared" ref="N63:N74" si="7">M63/L63</f>
         <v>1.0327555471873857</v>
       </c>
     </row>
-    <row r="64" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A64">
         <v>1</v>
       </c>
@@ -5948,26 +6403,26 @@
       <c r="D64">
         <v>2.0004896550590901E-4</v>
       </c>
-      <c r="E64">
+      <c r="F64">
         <v>2.0519183351723301E-4</v>
       </c>
-      <c r="F64" s="10">
+      <c r="I64" s="10">
         <f t="shared" si="6"/>
         <v>1.0257080460192236</v>
       </c>
-      <c r="G64" s="4"/>
-      <c r="I64">
+      <c r="J64" s="4"/>
+      <c r="L64">
         <v>2.47009346021372E-4</v>
       </c>
-      <c r="J64">
+      <c r="M64">
         <v>2.5056736662623701E-4</v>
       </c>
-      <c r="K64" s="10">
+      <c r="N64" s="10">
         <f t="shared" si="7"/>
         <v>1.0144043966844767</v>
       </c>
     </row>
-    <row r="65" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="65" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A65">
         <v>10</v>
       </c>
@@ -5978,26 +6433,26 @@
       <c r="D65">
         <v>1.9727739159685499E-3</v>
       </c>
-      <c r="E65">
+      <c r="F65">
         <v>2.1002402963605799E-3</v>
       </c>
-      <c r="F65" s="10">
+      <c r="I65" s="10">
         <f t="shared" si="6"/>
         <v>1.0646127665011473</v>
       </c>
-      <c r="G65" s="4"/>
-      <c r="I65">
+      <c r="J65" s="4"/>
+      <c r="L65">
         <v>2.41443999850058E-3</v>
       </c>
-      <c r="J65">
+      <c r="M65">
         <v>2.5624129143282902E-3</v>
       </c>
-      <c r="K65" s="11">
+      <c r="N65" s="11">
         <f t="shared" si="7"/>
         <v>1.0612866403470804</v>
       </c>
     </row>
-    <row r="66" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A66">
         <v>25</v>
       </c>
@@ -6008,26 +6463,26 @@
       <c r="D66">
         <v>4.9269907229743297E-3</v>
       </c>
-      <c r="E66">
+      <c r="F66">
         <v>5.2981099306138504E-3</v>
       </c>
-      <c r="F66" s="10">
+      <c r="I66" s="10">
         <f t="shared" si="6"/>
         <v>1.0753237074121145</v>
       </c>
-      <c r="G66" s="4"/>
-      <c r="I66">
+      <c r="J66" s="4"/>
+      <c r="L66">
         <v>6.11270182240103E-3</v>
       </c>
-      <c r="J66">
+      <c r="M66">
         <v>6.4145321839513504E-3</v>
       </c>
-      <c r="K66" s="10">
+      <c r="N66" s="10">
         <f t="shared" si="7"/>
         <v>1.0493775699060295</v>
       </c>
     </row>
-    <row r="67" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="67" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A67">
         <v>50</v>
       </c>
@@ -6038,26 +6493,26 @@
       <c r="D67">
         <v>9.7820010092556295E-3</v>
       </c>
-      <c r="E67">
+      <c r="F67">
         <v>1.0195154351149101E-2</v>
       </c>
-      <c r="F67" s="10">
+      <c r="I67" s="10">
         <f t="shared" si="6"/>
         <v>1.0422360763919929</v>
       </c>
-      <c r="G67" s="4"/>
-      <c r="I67">
+      <c r="J67" s="4"/>
+      <c r="L67">
         <v>1.20970549355645E-2</v>
       </c>
-      <c r="J67">
+      <c r="M67">
         <v>1.24175942421624E-2</v>
       </c>
-      <c r="K67" s="11">
+      <c r="N67" s="11">
         <f t="shared" si="7"/>
         <v>1.0264973010625533</v>
       </c>
     </row>
-    <row r="68" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="68" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A68">
         <v>75</v>
       </c>
@@ -6068,26 +6523,26 @@
       <c r="D68">
         <v>1.43763436727791E-2</v>
       </c>
-      <c r="E68">
+      <c r="F68">
         <v>1.5782984835099299E-2</v>
       </c>
-      <c r="F68" s="10">
+      <c r="I68" s="10">
         <f t="shared" si="6"/>
         <v>1.0978441524727602</v>
       </c>
-      <c r="G68" s="4"/>
-      <c r="I68">
+      <c r="J68" s="4"/>
+      <c r="L68">
         <v>1.8002551123509802E-2</v>
       </c>
-      <c r="J68">
+      <c r="M68">
         <v>1.8976376994297401E-2</v>
       </c>
-      <c r="K68" s="10">
+      <c r="N68" s="10">
         <f t="shared" si="7"/>
         <v>1.0540937706054263</v>
       </c>
     </row>
-    <row r="69" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="69" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A69">
         <v>100</v>
       </c>
@@ -6098,26 +6553,26 @@
       <c r="D69">
         <v>2.00458898906196E-2</v>
       </c>
-      <c r="E69">
+      <c r="F69">
         <v>2.0804120655568799E-2</v>
       </c>
-      <c r="F69" s="10">
+      <c r="I69" s="10">
         <f t="shared" si="6"/>
         <v>1.0378247495664441</v>
       </c>
-      <c r="G69" s="4"/>
-      <c r="I69">
+      <c r="J69" s="4"/>
+      <c r="L69">
         <v>2.4309982506840501E-2</v>
       </c>
-      <c r="J69">
+      <c r="M69">
         <v>2.56065505285916E-2</v>
       </c>
-      <c r="K69" s="11">
+      <c r="N69" s="11">
         <f t="shared" si="7"/>
         <v>1.0533347986320543</v>
       </c>
     </row>
-    <row r="70" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="70" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A70">
         <v>150</v>
       </c>
@@ -6128,26 +6583,26 @@
       <c r="D70">
         <v>3.0432830381329601E-2</v>
       </c>
-      <c r="E70">
+      <c r="F70">
         <v>3.14434702136525E-2</v>
       </c>
-      <c r="F70" s="10">
+      <c r="I70" s="10">
         <f t="shared" si="6"/>
         <v>1.0332088675177227</v>
       </c>
-      <c r="G70" s="4"/>
-      <c r="I70">
+      <c r="J70" s="4"/>
+      <c r="L70">
         <v>3.5308084946377202E-2</v>
       </c>
-      <c r="J70">
+      <c r="M70">
         <v>3.7911161854217702E-2</v>
       </c>
-      <c r="K70" s="10">
+      <c r="N70" s="10">
         <f t="shared" si="7"/>
         <v>1.0737246699104135</v>
       </c>
     </row>
-    <row r="71" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="71" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A71">
         <v>250</v>
       </c>
@@ -6158,26 +6613,26 @@
       <c r="D71">
         <v>4.89210306757277E-2</v>
       </c>
-      <c r="E71">
+      <c r="F71">
         <v>5.3975920537313898E-2</v>
       </c>
-      <c r="F71" s="10">
+      <c r="I71" s="10">
         <f t="shared" si="6"/>
         <v>1.1033275421994369</v>
       </c>
-      <c r="G71" s="4"/>
-      <c r="I71">
+      <c r="J71" s="4"/>
+      <c r="L71">
         <v>5.8808790512075798E-2</v>
       </c>
-      <c r="J71">
+      <c r="M71">
         <v>6.2265324575410202E-2</v>
       </c>
-      <c r="K71" s="11">
+      <c r="N71" s="11">
         <f t="shared" si="7"/>
         <v>1.0587758060187387</v>
       </c>
     </row>
-    <row r="72" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="72" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A72">
         <v>500</v>
       </c>
@@ -6188,26 +6643,26 @@
       <c r="D72">
         <v>9.6226590649767796E-2</v>
       </c>
-      <c r="E72">
+      <c r="F72">
         <v>0.10212774105006001</v>
       </c>
-      <c r="F72" s="10">
+      <c r="I72" s="10">
         <f t="shared" si="6"/>
         <v>1.0613255687481478</v>
       </c>
-      <c r="G72" s="4"/>
-      <c r="I72">
+      <c r="J72" s="4"/>
+      <c r="L72">
         <v>0.11146020972599301</v>
       </c>
-      <c r="J72">
+      <c r="M72">
         <v>0.118001707852343</v>
       </c>
-      <c r="K72" s="10">
+      <c r="N72" s="10">
         <f t="shared" si="7"/>
         <v>1.0586890886212328</v>
       </c>
     </row>
-    <row r="73" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="73" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A73">
         <v>750</v>
       </c>
@@ -6215,26 +6670,26 @@
       <c r="D73">
         <v>0.140294088260282</v>
       </c>
-      <c r="E73">
+      <c r="F73">
         <v>0.15225875418305601</v>
       </c>
-      <c r="F73" s="10">
+      <c r="I73" s="10">
         <f t="shared" si="6"/>
         <v>1.0852827519045309</v>
       </c>
-      <c r="G73" s="5"/>
-      <c r="I73">
+      <c r="J73" s="5"/>
+      <c r="L73">
         <v>0.164782092113922</v>
       </c>
-      <c r="J73">
+      <c r="M73">
         <v>0.171436913407884</v>
       </c>
-      <c r="K73" s="11">
+      <c r="N73" s="11">
         <f t="shared" si="7"/>
         <v>1.0403855856458066</v>
       </c>
     </row>
-    <row r="74" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="74" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A74">
         <v>999.99</v>
       </c>
@@ -6242,52 +6697,58 @@
       <c r="D74">
         <v>0.181401571560247</v>
       </c>
-      <c r="E74">
+      <c r="F74">
         <v>0.20058148390920799</v>
       </c>
-      <c r="F74" s="10">
+      <c r="I74" s="10">
         <f t="shared" si="6"/>
         <v>1.1057317871283765</v>
       </c>
-      <c r="G74" s="5"/>
-      <c r="I74">
+      <c r="J74" s="5"/>
+      <c r="L74">
         <v>0.211482254080264</v>
       </c>
-      <c r="J74">
+      <c r="M74">
         <v>0.22688990016688301</v>
       </c>
-      <c r="K74" s="10">
+      <c r="N74" s="10">
         <f t="shared" si="7"/>
         <v>1.0728555034256981</v>
       </c>
     </row>
-    <row r="76" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="76" spans="1:14" x14ac:dyDescent="0.3">
       <c r="C76" s="12" t="s">
         <v>10</v>
       </c>
       <c r="D76" s="12"/>
-      <c r="E76" s="13"/>
+      <c r="E76" s="12"/>
       <c r="F76" s="13"/>
-      <c r="H76" s="2"/>
-      <c r="I76" s="2"/>
-      <c r="J76" s="2"/>
+      <c r="G76" s="13"/>
+      <c r="H76" s="13"/>
+      <c r="I76" s="13"/>
       <c r="K76" s="2"/>
-    </row>
-    <row r="77" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L76" s="2"/>
+      <c r="M76" s="2"/>
+      <c r="N76" s="2"/>
+    </row>
+    <row r="77" spans="1:14" x14ac:dyDescent="0.3">
       <c r="C77" s="3" t="s">
         <v>4</v>
       </c>
       <c r="D77" s="3"/>
-      <c r="E77" s="9"/>
-      <c r="F77" s="3"/>
-      <c r="H77" s="3" t="s">
+      <c r="E77" s="3"/>
+      <c r="F77" s="9"/>
+      <c r="G77" s="9"/>
+      <c r="H77" s="9"/>
+      <c r="I77" s="3"/>
+      <c r="K77" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="I77" s="3"/>
-      <c r="J77" s="9"/>
-      <c r="K77" s="9"/>
-    </row>
-    <row r="78" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L77" s="3"/>
+      <c r="M77" s="9"/>
+      <c r="N77" s="9"/>
+    </row>
+    <row r="78" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A78" s="6" t="s">
         <v>0</v>
       </c>
@@ -6298,27 +6759,30 @@
       <c r="D78" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="E78" s="6" t="s">
+      <c r="E78" s="6"/>
+      <c r="F78" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="F78" s="7" t="s">
+      <c r="G78" s="6"/>
+      <c r="H78" s="6"/>
+      <c r="I78" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="G78" s="8"/>
-      <c r="H78" s="6" t="s">
+      <c r="J78" s="8"/>
+      <c r="K78" s="6" t="s">
         <v>1</v>
       </c>
-      <c r="I78" s="6" t="s">
+      <c r="L78" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="J78" s="6" t="s">
+      <c r="M78" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="K78" s="7" t="s">
+      <c r="N78" s="7" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="79" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="79" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A79">
         <v>0.1</v>
       </c>
@@ -6329,27 +6793,30 @@
       <c r="D79" s="2">
         <v>2.8143173972499801E-7</v>
       </c>
-      <c r="E79" s="2">
+      <c r="E79" s="2"/>
+      <c r="F79" s="2">
         <v>1.46150091119403E-6</v>
       </c>
-      <c r="F79" s="10">
-        <f t="shared" ref="F79:F90" si="8">F62*((E79/E62)^2 +(D79/D62)^2)^0.5</f>
+      <c r="G79" s="2"/>
+      <c r="H79" s="2"/>
+      <c r="I79" s="10">
+        <f t="shared" ref="I79:I90" si="8">I62*((F79/F62)^2 +(D79/D62)^2)^0.5</f>
         <v>7.5175789820697683E-2</v>
       </c>
-      <c r="G79" s="4"/>
-      <c r="H79" s="2"/>
-      <c r="I79" s="2">
+      <c r="J79" s="4"/>
+      <c r="K79" s="2"/>
+      <c r="L79" s="2">
         <v>2.4434932696069799E-5</v>
       </c>
-      <c r="J79" s="2">
+      <c r="M79" s="2">
         <v>2.5518609602937599E-5</v>
       </c>
-      <c r="K79" s="10">
-        <f>J79/I79</f>
+      <c r="N79" s="10">
+        <f>M79/L79</f>
         <v>1.0443494942403546</v>
       </c>
     </row>
-    <row r="80" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="80" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A80">
         <v>0.5</v>
       </c>
@@ -6360,26 +6827,29 @@
       <c r="D80" s="2">
         <v>1.5222069872849199E-6</v>
       </c>
-      <c r="E80" s="2">
+      <c r="E80" s="2"/>
+      <c r="F80" s="2">
         <v>3.7622530224669299E-6</v>
       </c>
-      <c r="F80" s="10">
+      <c r="G80" s="2"/>
+      <c r="H80" s="2"/>
+      <c r="I80" s="10">
         <f t="shared" si="8"/>
         <v>3.9379446327356661E-2</v>
       </c>
-      <c r="G80" s="4"/>
-      <c r="I80">
+      <c r="J80" s="4"/>
+      <c r="L80">
         <v>3.6561489620800698E-3</v>
       </c>
-      <c r="J80">
+      <c r="M80">
         <v>3.8583728177792702E-3</v>
       </c>
-      <c r="K80" s="11">
-        <f t="shared" ref="K80:K89" si="9">J80/I80</f>
+      <c r="N80" s="11">
+        <f t="shared" ref="N80:N89" si="9">M80/L80</f>
         <v>1.0553106172085915</v>
       </c>
     </row>
-    <row r="81" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="81" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A81">
         <v>1</v>
       </c>
@@ -6390,26 +6860,29 @@
       <c r="D81" s="2">
         <v>2.33807312394273E-6</v>
       </c>
-      <c r="E81" s="2">
+      <c r="E81" s="2"/>
+      <c r="F81" s="2">
         <v>6.5127278910264096E-6</v>
       </c>
-      <c r="F81" s="10">
+      <c r="G81" s="2"/>
+      <c r="H81" s="2"/>
+      <c r="I81" s="10">
         <f t="shared" si="8"/>
         <v>3.4692692812303069E-2</v>
       </c>
-      <c r="G81" s="4"/>
-      <c r="I81">
+      <c r="J81" s="4"/>
+      <c r="L81">
         <v>7.3167786817070497E-3</v>
       </c>
-      <c r="J81">
+      <c r="M81">
         <v>7.7206053021012903E-3</v>
       </c>
-      <c r="K81" s="10">
+      <c r="N81" s="10">
         <f t="shared" si="9"/>
         <v>1.0551918594181156</v>
       </c>
     </row>
-    <row r="82" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="82" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A82">
         <v>10</v>
       </c>
@@ -6420,26 +6893,29 @@
       <c r="D82" s="2">
         <v>2.7701090496064399E-5</v>
       </c>
-      <c r="E82" s="2">
+      <c r="E82" s="2"/>
+      <c r="F82" s="2">
         <v>3.8011060965548303E-5</v>
       </c>
-      <c r="F82" s="10">
+      <c r="G82" s="2"/>
+      <c r="H82" s="2"/>
+      <c r="I82" s="10">
         <f t="shared" si="8"/>
         <v>2.4386896067040687E-2</v>
       </c>
-      <c r="G82" s="4"/>
-      <c r="I82">
+      <c r="J82" s="4"/>
+      <c r="L82">
         <v>1.4655010559957399E-2</v>
       </c>
-      <c r="J82">
+      <c r="M82">
         <v>1.54708347850845E-2</v>
       </c>
-      <c r="K82" s="11">
+      <c r="N82" s="11">
         <f t="shared" si="9"/>
         <v>1.0556686207621178</v>
       </c>
     </row>
-    <row r="83" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="83" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A83">
         <v>25</v>
       </c>
@@ -6450,26 +6926,29 @@
       <c r="D83" s="2">
         <v>8.0985715172972504E-5</v>
       </c>
-      <c r="E83" s="2">
+      <c r="E83" s="2"/>
+      <c r="F83" s="2">
         <v>8.2936422592517207E-5</v>
       </c>
-      <c r="F83" s="10">
+      <c r="G83" s="2"/>
+      <c r="H83" s="2"/>
+      <c r="I83" s="10">
         <f t="shared" si="8"/>
         <v>2.4408348565916203E-2</v>
       </c>
-      <c r="G83" s="4"/>
-      <c r="I83">
+      <c r="J83" s="4"/>
+      <c r="L83">
         <v>2.20520227131588E-2</v>
       </c>
-      <c r="J83">
+      <c r="M83">
         <v>2.3279563002525702E-2</v>
       </c>
-      <c r="K83" s="10">
+      <c r="N83" s="10">
         <f t="shared" si="9"/>
         <v>1.0556656550437167</v>
       </c>
     </row>
-    <row r="84" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="84" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A84">
         <v>50</v>
       </c>
@@ -6480,26 +6959,26 @@
       <c r="D84">
         <v>1.14857385321631E-4</v>
       </c>
-      <c r="E84">
+      <c r="F84">
         <v>1.40546480514001E-4</v>
       </c>
-      <c r="F84" s="10">
+      <c r="I84" s="10">
         <f t="shared" si="8"/>
         <v>1.8873133491714433E-2</v>
       </c>
-      <c r="G84" s="4"/>
-      <c r="I84">
+      <c r="J84" s="4"/>
+      <c r="L84">
         <v>2.9379142051595902E-2</v>
       </c>
-      <c r="J84">
+      <c r="M84">
         <v>3.0966693098777899E-2</v>
       </c>
-      <c r="K84" s="11">
+      <c r="N84" s="11">
         <f t="shared" si="9"/>
         <v>1.0540366714723639</v>
       </c>
     </row>
-    <row r="85" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="85" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A85">
         <v>75</v>
       </c>
@@ -6510,26 +6989,26 @@
       <c r="D85">
         <v>1.6692001786006801E-4</v>
       </c>
-      <c r="E85">
+      <c r="F85">
         <v>2.2355768083561999E-4</v>
       </c>
-      <c r="F85" s="10">
+      <c r="I85" s="10">
         <f t="shared" si="8"/>
         <v>2.0107088599017175E-2</v>
       </c>
-      <c r="G85" s="4"/>
-      <c r="I85">
+      <c r="J85" s="4"/>
+      <c r="L85">
         <v>3.6804448452257998E-2</v>
       </c>
-      <c r="J85">
+      <c r="M85">
         <v>3.8844686371276298E-2</v>
       </c>
-      <c r="K85" s="10">
+      <c r="N85" s="10">
         <f t="shared" si="9"/>
         <v>1.0554345467685748</v>
       </c>
     </row>
-    <row r="86" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="86" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A86">
         <v>100</v>
       </c>
@@ -6540,26 +7019,26 @@
       <c r="D86">
         <v>2.77931449091848E-4</v>
       </c>
-      <c r="E86">
+      <c r="F86">
         <v>2.1739476286188801E-4</v>
       </c>
-      <c r="F86" s="10">
+      <c r="I86" s="10">
         <f t="shared" si="8"/>
         <v>1.8018315350781095E-2</v>
       </c>
-      <c r="G86" s="4"/>
-      <c r="I86">
+      <c r="J86" s="4"/>
+      <c r="L86">
         <v>6.1567552933483601E-2</v>
       </c>
-      <c r="J86">
+      <c r="M86">
         <v>6.4958585716827305E-2</v>
       </c>
-      <c r="K86" s="11">
+      <c r="N86" s="11">
         <f t="shared" si="9"/>
         <v>1.0550782453057264</v>
       </c>
     </row>
-    <row r="87" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="87" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A87">
         <v>150</v>
       </c>
@@ -6570,26 +7049,26 @@
       <c r="D87">
         <v>3.3888866496247497E-4</v>
       </c>
-      <c r="E87">
+      <c r="F87">
         <v>4.2099807481717899E-4</v>
       </c>
-      <c r="F87" s="10">
+      <c r="I87" s="10">
         <f t="shared" si="8"/>
         <v>1.7992932963347683E-2</v>
       </c>
-      <c r="G87" s="4"/>
-      <c r="I87">
+      <c r="J87" s="4"/>
+      <c r="L87">
         <v>0.124585487877085</v>
       </c>
-      <c r="J87">
+      <c r="M87">
         <v>0.13088073929294</v>
       </c>
-      <c r="K87" s="10">
+      <c r="N87" s="10">
         <f t="shared" si="9"/>
         <v>1.0505295722890764</v>
       </c>
     </row>
-    <row r="88" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="88" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A88">
         <v>250</v>
       </c>
@@ -6600,26 +7079,26 @@
       <c r="D88">
         <v>6.0844630496931901E-4</v>
       </c>
-      <c r="E88">
+      <c r="F88">
         <v>7.1735921087181002E-4</v>
       </c>
-      <c r="F88" s="10">
+      <c r="I88" s="10">
         <f t="shared" si="8"/>
         <v>2.0082997872230529E-2</v>
       </c>
-      <c r="G88" s="4"/>
-      <c r="I88">
+      <c r="J88" s="4"/>
+      <c r="L88">
         <v>0.188315720076114</v>
       </c>
-      <c r="J88">
+      <c r="M88">
         <v>0.19671890522285099</v>
       </c>
-      <c r="K88" s="11">
+      <c r="N88" s="11">
         <f t="shared" si="9"/>
         <v>1.0446228554012409</v>
       </c>
     </row>
-    <row r="89" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="89" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A89">
         <v>500</v>
       </c>
@@ -6630,52 +7109,52 @@
       <c r="D89">
         <v>1.3901143553867799E-3</v>
       </c>
-      <c r="E89">
+      <c r="F89">
         <v>1.45703989958587E-3</v>
       </c>
-      <c r="F89" s="10">
+      <c r="I89" s="10">
         <f t="shared" si="8"/>
         <v>2.1548753693625213E-2</v>
       </c>
-      <c r="G89" s="4"/>
-      <c r="I89">
+      <c r="J89" s="4"/>
+      <c r="L89">
         <v>0.25212873564071397</v>
       </c>
-      <c r="J89">
+      <c r="M89">
         <v>0.26159631710660702</v>
       </c>
-      <c r="K89" s="10">
+      <c r="N89" s="10">
         <f t="shared" si="9"/>
         <v>1.0375505847908761</v>
       </c>
     </row>
-    <row r="90" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="90" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A90">
         <v>750</v>
       </c>
       <c r="D90">
         <v>1.59024586083695E-3</v>
       </c>
-      <c r="E90">
+      <c r="F90">
         <v>1.88927153592098E-3</v>
       </c>
-      <c r="F90" s="10">
+      <c r="I90" s="10">
         <f t="shared" si="8"/>
         <v>1.8239532257896197E-2</v>
       </c>
     </row>
-    <row r="91" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="91" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A91">
         <v>999.99</v>
       </c>
       <c r="D91">
         <v>2.0916951916344802E-3</v>
       </c>
-      <c r="E91">
+      <c r="F91">
         <v>2.14759074882869E-3</v>
       </c>
-      <c r="F91" s="10">
-        <f>F74*((E91/E74)^2 +(D91/D74)^2)^0.5</f>
+      <c r="I91" s="10">
+        <f>I74*((F91/F74)^2 +(D91/D74)^2)^0.5</f>
         <v>1.7398828006913617E-2</v>
       </c>
     </row>

</xml_diff>

<commit_message>
update with dcll from delta-pc
</commit_message>
<xml_diff>
--- a/Jupyter/Wedge/wedge_data_2026-03-25.xlsx
+++ b/Jupyter/Wedge/wedge_data_2026-03-25.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\patri\projects\emma-openmc\Jupyter\Wedge\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2727A53E-B710-49C1-8960-17B14C6CB01B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{44F889C1-F7F7-41B5-8112-3ECB99FD4818}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="17496" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -84,8 +84,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="2">
+  <numFmts count="3">
     <numFmt numFmtId="164" formatCode="0.000000"/>
+    <numFmt numFmtId="169" formatCode="0.000"/>
     <numFmt numFmtId="173" formatCode="0.00000000"/>
   </numFmts>
   <fonts count="6" x14ac:knownFonts="1">
@@ -173,7 +174,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="11" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -190,6 +191,7 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="11" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="169" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="173" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -335,7 +337,7 @@
             <c:numRef>
               <c:f>'Sheet 1'!$H$24:$H$36</c:f>
               <c:numCache>
-                <c:formatCode>0.000000</c:formatCode>
+                <c:formatCode>0.000</c:formatCode>
                 <c:ptCount val="13"/>
                 <c:pt idx="0">
                   <c:v>0.67015864678428949</c:v>
@@ -609,7 +611,7 @@
             <a:effectLst/>
           </c:spPr>
         </c:majorGridlines>
-        <c:numFmt formatCode="0.000000" sourceLinked="1"/>
+        <c:numFmt formatCode="0.000" sourceLinked="1"/>
         <c:majorTickMark val="none"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
@@ -4753,7 +4755,8 @@
     <col min="1" max="1" width="12.33203125" customWidth="1"/>
     <col min="2" max="2" width="2.109375" customWidth="1"/>
     <col min="3" max="5" width="12.21875" customWidth="1"/>
-    <col min="6" max="8" width="15.88671875" customWidth="1"/>
+    <col min="6" max="7" width="15.88671875" customWidth="1"/>
+    <col min="8" max="8" width="12.5546875" customWidth="1"/>
     <col min="9" max="9" width="15.109375" customWidth="1"/>
     <col min="10" max="10" width="2.77734375" customWidth="1"/>
     <col min="11" max="14" width="13.33203125" customWidth="1"/>
@@ -5385,16 +5388,16 @@
       <c r="D24" s="2">
         <v>3.4601339198647797E-5</v>
       </c>
-      <c r="E24" s="16">
+      <c r="E24" s="17">
         <v>1.22883732368375E-8</v>
       </c>
-      <c r="F24" s="16">
+      <c r="F24" s="17">
         <v>2.3188386654289999E-5</v>
       </c>
-      <c r="G24" s="16">
+      <c r="G24" s="17">
         <v>2.5713213345718999E-7</v>
       </c>
-      <c r="H24" s="10">
+      <c r="H24" s="16">
         <f>F24/D24</f>
         <v>0.67015864678428949</v>
       </c>
@@ -5422,16 +5425,16 @@
       <c r="D25">
         <v>1.7267075850167999E-4</v>
       </c>
-      <c r="E25" s="16">
+      <c r="E25" s="17">
         <v>7.3730405114227898E-8</v>
       </c>
-      <c r="F25" s="16">
+      <c r="F25" s="17">
         <v>1.16379113471186E-4</v>
       </c>
-      <c r="G25" s="16">
+      <c r="G25" s="17">
         <v>4.9685826902563597E-7</v>
       </c>
-      <c r="H25" s="10">
+      <c r="H25" s="16">
         <f>F25/D25</f>
         <v>0.67399433743759052</v>
       </c>
@@ -5457,16 +5460,16 @@
       <c r="D26">
         <v>3.4444202449192702E-4</v>
       </c>
-      <c r="E26" s="16">
+      <c r="E26" s="17">
         <v>1.02701859340892E-7</v>
       </c>
-      <c r="F26" s="16">
+      <c r="F26" s="17">
         <v>2.31665379952172E-4</v>
       </c>
-      <c r="G26" s="16">
+      <c r="G26" s="17">
         <v>6.9232886194979901E-7</v>
       </c>
-      <c r="H26" s="10">
+      <c r="H26" s="16">
         <f>F26/D26</f>
         <v>0.67258163487423628</v>
       </c>
@@ -5492,16 +5495,16 @@
       <c r="D27">
         <v>3.33054467027722E-3</v>
       </c>
-      <c r="E27" s="16">
+      <c r="E27" s="17">
         <v>3.1023196230951202E-6</v>
       </c>
-      <c r="F27" s="16">
+      <c r="F27" s="17">
         <v>2.3274949085023899E-3</v>
       </c>
-      <c r="G27" s="16">
+      <c r="G27" s="17">
         <v>7.3576810457546899E-6</v>
       </c>
-      <c r="H27" s="10">
+      <c r="H27" s="16">
         <f>F27/D27</f>
         <v>0.69883311557825745</v>
       </c>
@@ -5527,16 +5530,16 @@
       <c r="D28">
         <v>7.9007108136224906E-3</v>
       </c>
-      <c r="E28" s="16">
+      <c r="E28" s="17">
         <v>2.1579374269995798E-5</v>
       </c>
-      <c r="F28" s="16">
+      <c r="F28" s="17">
         <v>5.7868683352336496E-3</v>
       </c>
-      <c r="G28" s="16">
+      <c r="G28" s="17">
         <v>2.2153397083295701E-5</v>
       </c>
-      <c r="H28" s="10">
+      <c r="H28" s="16">
         <f>F28/D28</f>
         <v>0.73244907600666376</v>
       </c>
@@ -5562,16 +5565,16 @@
       <c r="D29">
         <v>1.48099690035684E-2</v>
       </c>
-      <c r="E29" s="16">
+      <c r="E29" s="17">
         <v>3.5619384608241799E-5</v>
       </c>
-      <c r="F29" s="16">
+      <c r="F29" s="17">
         <v>1.1357972286110201E-2</v>
       </c>
-      <c r="G29" s="16">
+      <c r="G29" s="17">
         <v>3.9960656049596501E-5</v>
       </c>
-      <c r="H29" s="10">
+      <c r="H29" s="16">
         <f>F29/D29</f>
         <v>0.76691398093902452</v>
       </c>
@@ -5597,16 +5600,16 @@
       <c r="D30">
         <v>2.1060130702738999E-2</v>
       </c>
-      <c r="E30" s="16">
+      <c r="E30" s="17">
         <v>3.0830038687911403E-5</v>
       </c>
-      <c r="F30" s="16">
+      <c r="F30" s="17">
         <v>1.6724313084056999E-2</v>
       </c>
-      <c r="G30" s="16">
+      <c r="G30" s="17">
         <v>4.6773312275541899E-5</v>
       </c>
-      <c r="H30" s="10">
+      <c r="H30" s="16">
         <f>F30/D30</f>
         <v>0.79412199858198884</v>
       </c>
@@ -5632,16 +5635,16 @@
       <c r="D31">
         <v>2.67600755292417E-2</v>
       </c>
-      <c r="E31" s="16">
+      <c r="E31" s="17">
         <v>6.1301138330409899E-5</v>
       </c>
-      <c r="F31" s="16">
+      <c r="F31" s="17">
         <v>2.2149757308928399E-2</v>
       </c>
-      <c r="G31" s="16">
+      <c r="G31" s="17">
         <v>5.1020148947823797E-5</v>
       </c>
-      <c r="H31" s="10">
+      <c r="H31" s="16">
         <f>F31/D31</f>
         <v>0.82771654679092965</v>
       </c>
@@ -5667,16 +5670,16 @@
       <c r="D32">
         <v>3.6782709718709998E-2</v>
       </c>
-      <c r="E32" s="16">
+      <c r="E32" s="17">
         <v>1.97489580151579E-4</v>
       </c>
-      <c r="F32" s="16">
+      <c r="F32" s="17">
         <v>3.2103137598192298E-2</v>
       </c>
-      <c r="G32" s="16">
+      <c r="G32" s="17">
         <v>2.08831333646651E-4</v>
       </c>
-      <c r="H32" s="10">
+      <c r="H32" s="16">
         <f>F32/D32</f>
         <v>0.87277793951821403</v>
       </c>
@@ -5702,16 +5705,16 @@
       <c r="D33">
         <v>5.6309750104400702E-2</v>
       </c>
-      <c r="E33" s="16">
+      <c r="E33" s="17">
         <v>2.51687827781958E-4</v>
       </c>
-      <c r="F33" s="16">
+      <c r="F33" s="17">
         <v>5.1114734736025402E-2</v>
       </c>
-      <c r="G33" s="16">
+      <c r="G33" s="17">
         <v>2.8833834514146198E-4</v>
       </c>
-      <c r="H33" s="10">
+      <c r="H33" s="16">
         <f>F33/D33</f>
         <v>0.90774216971761523</v>
       </c>
@@ -5737,16 +5740,16 @@
       <c r="D34">
         <v>9.4384365104793602E-2</v>
       </c>
-      <c r="E34" s="16">
+      <c r="E34" s="17">
         <v>3.7802904257795602E-4</v>
       </c>
-      <c r="F34" s="16">
+      <c r="F34" s="17">
         <v>9.1445222619505398E-2</v>
       </c>
-      <c r="G34" s="16">
+      <c r="G34" s="17">
         <v>4.4906828447954003E-4</v>
       </c>
-      <c r="H34" s="10">
+      <c r="H34" s="16">
         <f>F34/D34</f>
         <v>0.96885985849430767</v>
       </c>
@@ -5772,16 +5775,16 @@
       <c r="D35">
         <v>0.12681392305883499</v>
       </c>
-      <c r="E35" s="16">
+      <c r="E35" s="17">
         <v>3.7117560576619898E-4</v>
       </c>
-      <c r="F35" s="16">
+      <c r="F35" s="17">
         <v>0.12725844081883</v>
       </c>
-      <c r="G35" s="16">
+      <c r="G35" s="17">
         <v>3.9277512684765298E-4</v>
       </c>
-      <c r="H35" s="10">
+      <c r="H35" s="16">
         <f>F35/D35</f>
         <v>1.0035052756769365</v>
       </c>
@@ -5807,16 +5810,16 @@
       <c r="D36">
         <v>0.15510900896549801</v>
       </c>
-      <c r="E36" s="16">
+      <c r="E36" s="17">
         <v>5.7851797067085496E-4</v>
       </c>
-      <c r="F36" s="16">
+      <c r="F36" s="17">
         <v>0.157583868759714</v>
       </c>
-      <c r="G36" s="16">
+      <c r="G36" s="17">
         <v>5.8700051779191705E-4</v>
       </c>
-      <c r="H36" s="10">
+      <c r="H36" s="16">
         <f>F36/D36</f>
         <v>1.0159556160581653</v>
       </c>

</xml_diff>